<commit_message>
vault backup: 2026-04-22 22:03:46
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -1749,7 +1749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2068,7 +2068,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Δ Receivables</t>
+          <t>Receivables</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
@@ -2093,7 +2093,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Δ Inventories</t>
+          <t>Inventories</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
@@ -2118,7 +2118,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Δ Prepaids</t>
+          <t>Prepaids</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
@@ -2168,7 +2168,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Delta Accrued Expenses (change)</t>
+          <t>Accrued Expenses</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
@@ -2193,20 +2193,20 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Δ Accrued Promo Allowance</t>
+          <t>Accrued Promo</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>374</v>
+        <v>13379</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>2610</v>
+        <v>16940</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>7305</v>
+        <v>63810</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>4920</v>
+        <v>36161</v>
       </c>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="n"/>
@@ -2218,20 +2218,20 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Δ ROU/Lease</t>
+          <t>Other Current Liabilities</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>29</v>
+        <v>374</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>-183</v>
+        <v>2610</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>-102</v>
+        <v>7305</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>535</v>
+        <v>4920</v>
       </c>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="5" t="n"/>
@@ -2243,20 +2243,20 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Δ Deferred Revenue</t>
+          <t>ROU/Lease</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>189463</v>
+        <v>-183</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>-12723</v>
+        <v>-102</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>-9513</v>
+        <v>535</v>
       </c>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="5" t="n"/>
@@ -2268,20 +2268,20 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow from Operations</t>
+          <t>Deferred Revenue</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>-96586</v>
+        <v>0</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>108182</v>
+        <v>189463</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>141218</v>
+        <v>-12723</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>262898</v>
+        <v>-9513</v>
       </c>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="5" t="n"/>
@@ -2293,20 +2293,20 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Collections from Note Receivable</t>
+          <t>Cash Flow from Operations</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>1886</v>
+        <v>-96586</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>2592</v>
+        <v>108182</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>3233</v>
+        <v>141218</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0</v>
+        <v>262898</v>
       </c>
       <c r="F21" s="5" t="n"/>
       <c r="G21" s="5" t="n"/>
@@ -2318,20 +2318,20 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Purchase of PP&amp;E</t>
+          <t>Collections from Note Receivable</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>-3150</v>
+        <v>1886</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>-8264</v>
+        <v>2592</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>-17433</v>
+        <v>3233</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>-23390</v>
+        <v>0</v>
       </c>
       <c r="F22" s="5" t="n"/>
       <c r="G22" s="5" t="n"/>
@@ -2343,20 +2343,20 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow from Investing</t>
+          <t>Purchase of PP&amp;E</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>-1264</v>
+        <v>-3150</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>-5672</v>
+        <v>-8264</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>-14200</v>
+        <v>-17433</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>-101726</v>
+        <v>-23390</v>
       </c>
       <c r="F23" s="5" t="n"/>
       <c r="G23" s="5" t="n"/>
@@ -2368,20 +2368,20 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Finance Lease Payments</t>
+          <t>Cash Flow from Investing</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>-94</v>
+        <v>-1264</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>-63</v>
+        <v>-5672</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>-44</v>
+        <v>-14200</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>-61</v>
+        <v>-101726</v>
       </c>
       <c r="F24" s="5" t="n"/>
       <c r="G24" s="5" t="n"/>
@@ -2393,20 +2393,20 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Stock Options</t>
+          <t>Finance Lease Payments</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>3720</v>
+        <v>-94</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>3683</v>
+        <v>-63</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>2285</v>
+        <v>-44</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>3856</v>
+        <v>-61</v>
       </c>
       <c r="F25" s="5" t="n"/>
       <c r="G25" s="5" t="n"/>
@@ -2418,20 +2418,20 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Preferred</t>
+          <t>Proceeds from Stock Options</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>0</v>
+        <v>3720</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>542018</v>
+        <v>3683</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>0</v>
+        <v>2285</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>0</v>
+        <v>3856</v>
       </c>
       <c r="F26" s="5" t="n"/>
       <c r="G26" s="5" t="n"/>
@@ -2443,20 +2443,20 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Dividends Paid on Preferred</t>
+          <t>Proceeds from Preferred</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>-11526</v>
+        <v>542018</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>-27462</v>
+        <v>0</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>-27500</v>
+        <v>0</v>
       </c>
       <c r="F27" s="5" t="n"/>
       <c r="G27" s="5" t="n"/>
@@ -2468,20 +2468,20 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow from Financing</t>
+          <t>Dividends Paid on Preferred</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
-        <v>71395</v>
+        <v>0</v>
       </c>
       <c r="C28" s="4" t="n">
-        <v>534112</v>
+        <v>-11526</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>-25221</v>
+        <v>-27462</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>-25966</v>
+        <v>-27500</v>
       </c>
       <c r="F28" s="5" t="n"/>
       <c r="G28" s="5" t="n"/>
@@ -2493,20 +2493,20 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>FX Effect on Cash</t>
+          <t>Cash Flow from Financing</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>-538</v>
+        <v>71395</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>50</v>
+        <v>534112</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>1257</v>
+        <v>-25221</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>-997</v>
+        <v>-25966</v>
       </c>
       <c r="F29" s="5" t="n"/>
       <c r="G29" s="5" t="n"/>
@@ -2518,20 +2518,20 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Net Change in Cash</t>
+          <t>FX Effect on Cash</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>-26993</v>
+        <v>-538</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>636672</v>
+        <v>50</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>103054</v>
+        <v>1257</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>134209</v>
+        <v>-997</v>
       </c>
       <c r="F30" s="5" t="n"/>
       <c r="G30" s="5" t="n"/>
@@ -2543,20 +2543,20 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Cash at Beginning</t>
+          <t>Net Change in Cash</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>43248</v>
+        <v>-26993</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>16255</v>
+        <v>636672</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>652927</v>
+        <v>103054</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>755981</v>
+        <v>134209</v>
       </c>
       <c r="F31" s="5" t="n"/>
       <c r="G31" s="5" t="n"/>
@@ -2568,20 +2568,20 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Cash at End</t>
+          <t>Cash at Beginning</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
+        <v>43248</v>
+      </c>
+      <c r="C32" s="4" t="n">
         <v>16255</v>
       </c>
-      <c r="C32" s="4" t="n">
+      <c r="D32" s="4" t="n">
         <v>652927</v>
       </c>
-      <c r="D32" s="4" t="n">
+      <c r="E32" s="4" t="n">
         <v>755981</v>
-      </c>
-      <c r="E32" s="4" t="n">
-        <v>890190</v>
       </c>
       <c r="F32" s="5" t="n"/>
       <c r="G32" s="5" t="n"/>
@@ -2593,20 +2593,20 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Deferred Income Taxes-Net</t>
+          <t>Cash at End</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
-        <v>-9201</v>
+        <v>16255</v>
       </c>
       <c r="C33" s="4" t="n">
-        <v>20244</v>
+        <v>652927</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>-42055</v>
+        <v>755981</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>-9730</v>
+        <v>890190</v>
       </c>
       <c r="F33" s="5" t="n"/>
       <c r="G33" s="5" t="n"/>
@@ -2618,8 +2618,20 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Δ Note Receivable</t>
-        </is>
+          <t>Deferred Income Taxes-Net</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>-9201</v>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>20244</v>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>-42055</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>-9730</v>
       </c>
       <c r="F34" s="5" t="n"/>
       <c r="G34" s="5" t="n"/>
@@ -2631,7 +2643,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Δ Accounts Payable</t>
+          <t>Note Receivable</t>
         </is>
       </c>
       <c r="F35" s="5" t="n"/>
@@ -2644,7 +2656,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Δ Accrued Expenses</t>
+          <t>Accounts Payable</t>
         </is>
       </c>
       <c r="F36" s="5" t="n"/>
@@ -2657,17 +2669,8 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Δ Other Long-Term Assets</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="n">
-        <v>37</v>
-      </c>
-      <c r="D37" s="4" t="n">
-        <v>-28</v>
-      </c>
-      <c r="E37" s="4" t="n">
-        <v>-4862</v>
+          <t>Accrued Expenses</t>
+        </is>
       </c>
       <c r="F37" s="5" t="n"/>
       <c r="G37" s="5" t="n"/>
@@ -2679,17 +2682,17 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Purchase of Non-Marketable Equity Securities</t>
+          <t>Other Long-Term Assets</t>
         </is>
       </c>
       <c r="C38" s="4" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>0</v>
+        <v>-28</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>-3000</v>
+        <v>-4862</v>
       </c>
       <c r="F38" s="5" t="n"/>
       <c r="G38" s="5" t="n"/>
@@ -2701,8 +2704,17 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Acquisition of [entity]</t>
-        </is>
+          <t>Purchase of Non-Marketable Equity Securities</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>-3000</v>
       </c>
       <c r="F39" s="5" t="n"/>
       <c r="G39" s="5" t="n"/>
@@ -2714,17 +2726,8 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Acquisition of Big Beverages</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="4" t="n">
-        <v>-75336</v>
+          <t>Acquisition of [entity]</t>
+        </is>
       </c>
       <c r="F40" s="5" t="n"/>
       <c r="G40" s="5" t="n"/>
@@ -2736,7 +2739,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Delta Note Receivable</t>
+          <t>Acquisition of Big Beverages</t>
         </is>
       </c>
       <c r="C41" s="4" t="n">
@@ -2746,7 +2749,7 @@
         <v>0</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>2318</v>
+        <v>-75336</v>
       </c>
       <c r="F41" s="5" t="n"/>
       <c r="G41" s="5" t="n"/>
@@ -2758,8 +2761,17 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Common</t>
-        </is>
+          <t>Note Receivable</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>2318</v>
       </c>
       <c r="F42" s="5" t="n"/>
       <c r="G42" s="5" t="n"/>
@@ -2768,6 +2780,19 @@
       <c r="J42" s="5" t="n"/>
       <c r="K42" s="5" t="n"/>
     </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Proceeds from Common</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="n"/>
+      <c r="G43" s="5" t="n"/>
+      <c r="H43" s="5" t="n"/>
+      <c r="I43" s="5" t="n"/>
+      <c r="J43" s="5" t="n"/>
+      <c r="K43" s="5" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-04-22 22:19:05
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -690,20 +690,17 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Pre-Tax Income</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>-4059</v>
+          <t>Other Income</t>
+        </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>-152664</v>
+        <v>0</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>291749</v>
+        <v>0</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>195050</v>
+        <v>1793</v>
       </c>
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
@@ -715,20 +712,20 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Income Taxes</t>
+          <t>Pre-Tax Income</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>7996</v>
+        <v>-4059</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>-34618</v>
+        <v>-152664</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>-64948</v>
+        <v>291749</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>-49976</v>
+        <v>195050</v>
       </c>
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
@@ -740,20 +737,20 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Net Income</t>
+          <t>Income Taxes</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>3937</v>
+        <v>7996</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>-187282</v>
+        <v>-34618</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>226801</v>
+        <v>-64948</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>145074</v>
+        <v>-49976</v>
       </c>
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
@@ -765,20 +762,20 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Dividends on Series A Pref</t>
+          <t>Net Income</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>0</v>
+        <v>3937</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>-11526</v>
+        <v>-187282</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>-27462</v>
+        <v>226801</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-27500</v>
+        <v>145074</v>
       </c>
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
@@ -790,20 +787,20 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Net Income to Common Shareholders</t>
+          <t>Dividends on Series A Pref</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>3937</v>
+        <v>0</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>-198808</v>
+        <v>-11526</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>181991</v>
+        <v>-27462</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>107457</v>
+        <v>-27500</v>
       </c>
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="n"/>
@@ -815,20 +812,20 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Income Allocated to Participating</t>
+          <t>Net Income to Common Shareholders</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>0</v>
+        <v>3937</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>0</v>
+        <v>-198808</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>-17348</v>
+        <v>181991</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>-10117</v>
+        <v>107457</v>
       </c>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
@@ -840,20 +837,20 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>GAAP EPS (Basic)</t>
+          <t>Income Allocated to Participating</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>-0.88</v>
+        <v>0</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>0.79</v>
+        <v>-17348</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>0.46</v>
+        <v>-10117</v>
       </c>
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
@@ -865,7 +862,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>GAAP EPS (Diluted)</t>
+          <t>GAAP EPS (Basic)</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
@@ -875,10 +872,10 @@
         <v>-0.88</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>0.77</v>
+        <v>0.79</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
@@ -915,20 +912,20 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Weighted Avg Shares Outstanding (Diluted)</t>
+          <t>GAAP EPS (Diluted)</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>233067</v>
+        <v>0.02</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>226947</v>
+        <v>-0.88</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>236964</v>
+        <v>0.77</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>237404</v>
+        <v>0.45</v>
       </c>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="5" t="n"/>
@@ -940,17 +937,20 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Other Income</t>
-        </is>
+          <t>Weighted Avg Shares Outstanding (Diluted)</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>233067</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>0</v>
+        <v>226947</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>0</v>
+        <v>236964</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>1793</v>
+        <v>237404</v>
       </c>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="5" t="n"/>
@@ -1749,7 +1749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2018,20 +2018,20 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Foreign Exchange Loss</t>
+          <t>Deferred Income Taxes-Net</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>880</v>
+        <v>-9201</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>483</v>
+        <v>20244</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>1246</v>
+        <v>-42055</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>1734</v>
+        <v>-9730</v>
       </c>
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
@@ -2043,20 +2043,20 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Other Items</t>
+          <t>Foreign Exchange Loss</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>0</v>
+        <v>880</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>0</v>
+        <v>483</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0</v>
+        <v>1246</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>-324</v>
+        <v>1734</v>
       </c>
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
@@ -2068,20 +2068,20 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Receivables</t>
+          <t>Other Items</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>-25249</v>
+        <v>0</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>-26369</v>
+        <v>0</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>-121558</v>
+        <v>0</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-89665</v>
+        <v>-324</v>
       </c>
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
@@ -2093,20 +2093,20 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Inventories</t>
+          <t>Receivables</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>-175174</v>
+        <v>-25249</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>11802</v>
+        <v>-26369</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>-63299</v>
+        <v>-121558</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>77190</v>
+        <v>-89665</v>
       </c>
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="n"/>
@@ -2118,20 +2118,20 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Prepaids</t>
+          <t>Inventories</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>1072</v>
+        <v>-175174</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>2214</v>
+        <v>11802</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>-7980</v>
+        <v>-63299</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>1074</v>
+        <v>77190</v>
       </c>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
@@ -2143,20 +2143,20 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Change in A/P and Accrued (legacy)</t>
+          <t>Prepaids</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>23966</v>
+        <v>1072</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>428</v>
+        <v>2214</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>5249</v>
+        <v>-7980</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>-1170</v>
+        <v>1074</v>
       </c>
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
@@ -2168,20 +2168,20 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Accrued Expenses</t>
+          <t>Change in A/P and Accrued (legacy)</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>26484</v>
+        <v>23966</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>34644</v>
+        <v>428</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>-8025</v>
+        <v>5249</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>85398</v>
+        <v>-1170</v>
       </c>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
@@ -2193,20 +2193,20 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Accrued Promo</t>
+          <t>Accrued Expenses</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>13379</v>
+        <v>26484</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>16940</v>
+        <v>34644</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>63810</v>
+        <v>-8025</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>36161</v>
+        <v>85398</v>
       </c>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="n"/>
@@ -2218,20 +2218,20 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Other Current Liabilities</t>
+          <t>Accrued Promo</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>374</v>
+        <v>13379</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>2610</v>
+        <v>16940</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>7305</v>
+        <v>63810</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>4920</v>
+        <v>36161</v>
       </c>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="5" t="n"/>
@@ -2243,20 +2243,20 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>ROU/Lease</t>
+          <t>Other Current Liabilities</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>29</v>
+        <v>374</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>-183</v>
+        <v>2610</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>-102</v>
+        <v>7305</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>535</v>
+        <v>4920</v>
       </c>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="5" t="n"/>
@@ -2268,20 +2268,20 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Deferred Revenue</t>
+          <t>ROU/Lease</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>189463</v>
+        <v>-183</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>-12723</v>
+        <v>-102</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>-9513</v>
+        <v>535</v>
       </c>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="5" t="n"/>
@@ -2293,20 +2293,20 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow from Operations</t>
+          <t>Deferred Revenue</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>-96586</v>
+        <v>0</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>108182</v>
+        <v>189463</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>141218</v>
+        <v>-12723</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>262898</v>
+        <v>-9513</v>
       </c>
       <c r="F21" s="5" t="n"/>
       <c r="G21" s="5" t="n"/>
@@ -2318,20 +2318,17 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Collections from Note Receivable</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n">
-        <v>1886</v>
+          <t>Other Long-Term Assets</t>
+        </is>
       </c>
       <c r="C22" s="4" t="n">
-        <v>2592</v>
+        <v>37</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>3233</v>
+        <v>-28</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>0</v>
+        <v>-4862</v>
       </c>
       <c r="F22" s="5" t="n"/>
       <c r="G22" s="5" t="n"/>
@@ -2343,20 +2340,17 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Purchase of PP&amp;E</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n">
-        <v>-3150</v>
+          <t>Note Receivable</t>
+        </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>-8264</v>
+        <v>0</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>-17433</v>
+        <v>0</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>-23390</v>
+        <v>2318</v>
       </c>
       <c r="F23" s="5" t="n"/>
       <c r="G23" s="5" t="n"/>
@@ -2368,20 +2362,20 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow from Investing</t>
+          <t>Accrued Distributor Termination</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>-1264</v>
+        <v>0</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>-5672</v>
+        <v>3986</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>-14200</v>
+        <v>-3739</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>-101726</v>
+        <v>-248</v>
       </c>
       <c r="F24" s="5" t="n"/>
       <c r="G24" s="5" t="n"/>
@@ -2393,20 +2387,20 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Finance Lease Payments</t>
+          <t>Cash Flow from Operations</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>-94</v>
+        <v>-96586</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>-63</v>
+        <v>108182</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>-44</v>
+        <v>141218</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>-61</v>
+        <v>262898</v>
       </c>
       <c r="F25" s="5" t="n"/>
       <c r="G25" s="5" t="n"/>
@@ -2418,20 +2412,20 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Stock Options</t>
+          <t>Collections from Note Receivable</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>3720</v>
+        <v>1886</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>3683</v>
+        <v>2592</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>2285</v>
+        <v>3233</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>3856</v>
+        <v>0</v>
       </c>
       <c r="F26" s="5" t="n"/>
       <c r="G26" s="5" t="n"/>
@@ -2443,20 +2437,17 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Preferred</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="n">
-        <v>0</v>
+          <t>Purchase of Non-Marketable Equity Securities</t>
+        </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>542018</v>
+        <v>0</v>
       </c>
       <c r="D27" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>0</v>
+        <v>-3000</v>
       </c>
       <c r="F27" s="5" t="n"/>
       <c r="G27" s="5" t="n"/>
@@ -2468,20 +2459,8 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Dividends Paid on Preferred</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="4" t="n">
-        <v>-11526</v>
-      </c>
-      <c r="D28" s="4" t="n">
-        <v>-27462</v>
-      </c>
-      <c r="E28" s="4" t="n">
-        <v>-27500</v>
+          <t>Acquisition of [entity]</t>
+        </is>
       </c>
       <c r="F28" s="5" t="n"/>
       <c r="G28" s="5" t="n"/>
@@ -2493,20 +2472,17 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow from Financing</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="n">
-        <v>71395</v>
+          <t>Acquisition of Big Beverages</t>
+        </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>534112</v>
+        <v>0</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>-25221</v>
+        <v>0</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>-25966</v>
+        <v>-75336</v>
       </c>
       <c r="F29" s="5" t="n"/>
       <c r="G29" s="5" t="n"/>
@@ -2518,20 +2494,20 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>FX Effect on Cash</t>
+          <t>Purchase of PP&amp;E</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>-538</v>
+        <v>-3150</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>50</v>
+        <v>-8264</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>1257</v>
+        <v>-17433</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>-997</v>
+        <v>-23390</v>
       </c>
       <c r="F30" s="5" t="n"/>
       <c r="G30" s="5" t="n"/>
@@ -2543,20 +2519,20 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Net Change in Cash</t>
+          <t>Cash Flow from Investing</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>-26993</v>
+        <v>-1264</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>636672</v>
+        <v>-5672</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>103054</v>
+        <v>-14200</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>134209</v>
+        <v>-101726</v>
       </c>
       <c r="F31" s="5" t="n"/>
       <c r="G31" s="5" t="n"/>
@@ -2568,20 +2544,20 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Cash at Beginning</t>
+          <t>Finance Lease Payments</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>43248</v>
+        <v>-94</v>
       </c>
       <c r="C32" s="4" t="n">
-        <v>16255</v>
+        <v>-63</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>652927</v>
+        <v>-44</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>755981</v>
+        <v>-61</v>
       </c>
       <c r="F32" s="5" t="n"/>
       <c r="G32" s="5" t="n"/>
@@ -2593,20 +2569,17 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Cash at End</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="n">
-        <v>16255</v>
+          <t>Repurchase of Common Stock (Tax Withholdings)</t>
+        </is>
       </c>
       <c r="C33" s="4" t="n">
-        <v>652927</v>
+        <v>0</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>755981</v>
+        <v>0</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>890190</v>
+        <v>-2261</v>
       </c>
       <c r="F33" s="5" t="n"/>
       <c r="G33" s="5" t="n"/>
@@ -2618,20 +2591,20 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Deferred Income Taxes-Net</t>
+          <t>Proceeds from Stock Options</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>-9201</v>
+        <v>3720</v>
       </c>
       <c r="C34" s="4" t="n">
-        <v>20244</v>
+        <v>3683</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>-42055</v>
+        <v>2285</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>-9730</v>
+        <v>3856</v>
       </c>
       <c r="F34" s="5" t="n"/>
       <c r="G34" s="5" t="n"/>
@@ -2643,7 +2616,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Note Receivable</t>
+          <t>Proceeds from Common</t>
         </is>
       </c>
       <c r="F35" s="5" t="n"/>
@@ -2656,8 +2629,20 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Accounts Payable</t>
-        </is>
+          <t>Proceeds from Preferred</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>542018</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="F36" s="5" t="n"/>
       <c r="G36" s="5" t="n"/>
@@ -2669,8 +2654,20 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Accrued Expenses</t>
-        </is>
+          <t>Dividends Paid on Preferred</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>-11526</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>-27462</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>-27500</v>
       </c>
       <c r="F37" s="5" t="n"/>
       <c r="G37" s="5" t="n"/>
@@ -2682,17 +2679,20 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Other Long-Term Assets</t>
-        </is>
+          <t>Cash Flow from Financing</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>71395</v>
       </c>
       <c r="C38" s="4" t="n">
-        <v>37</v>
+        <v>534112</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>-28</v>
+        <v>-25221</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>-4862</v>
+        <v>-25966</v>
       </c>
       <c r="F38" s="5" t="n"/>
       <c r="G38" s="5" t="n"/>
@@ -2704,17 +2704,20 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Purchase of Non-Marketable Equity Securities</t>
-        </is>
+          <t>FX Effect on Cash</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="n">
+        <v>-538</v>
       </c>
       <c r="C39" s="4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>0</v>
+        <v>1257</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>-3000</v>
+        <v>-997</v>
       </c>
       <c r="F39" s="5" t="n"/>
       <c r="G39" s="5" t="n"/>
@@ -2726,8 +2729,20 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Acquisition of [entity]</t>
-        </is>
+          <t>Net Change in Cash</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>-26993</v>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>636672</v>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>103054</v>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>134209</v>
       </c>
       <c r="F40" s="5" t="n"/>
       <c r="G40" s="5" t="n"/>
@@ -2739,17 +2754,20 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Acquisition of Big Beverages</t>
-        </is>
+          <t>Cash at Beginning</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="n">
+        <v>43248</v>
       </c>
       <c r="C41" s="4" t="n">
-        <v>0</v>
+        <v>16255</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>0</v>
+        <v>652927</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>-75336</v>
+        <v>755981</v>
       </c>
       <c r="F41" s="5" t="n"/>
       <c r="G41" s="5" t="n"/>
@@ -2761,17 +2779,20 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Note Receivable</t>
-        </is>
+          <t>Cash at End</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="n">
+        <v>16255</v>
       </c>
       <c r="C42" s="4" t="n">
-        <v>0</v>
+        <v>652927</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>0</v>
+        <v>755981</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>2318</v>
+        <v>890190</v>
       </c>
       <c r="F42" s="5" t="n"/>
       <c r="G42" s="5" t="n"/>
@@ -2780,19 +2801,6 @@
       <c r="J42" s="5" t="n"/>
       <c r="K42" s="5" t="n"/>
     </row>
-    <row r="43">
-      <c r="A43" s="3" t="inlineStr">
-        <is>
-          <t>Proceeds from Common</t>
-        </is>
-      </c>
-      <c r="F43" s="5" t="n"/>
-      <c r="G43" s="5" t="n"/>
-      <c r="H43" s="5" t="n"/>
-      <c r="I43" s="5" t="n"/>
-      <c r="J43" s="5" t="n"/>
-      <c r="K43" s="5" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-04-22 23:04:55
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -693,6 +693,9 @@
           <t>Other Income</t>
         </is>
       </c>
+      <c r="B9" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="C9" s="4" t="n">
         <v>0</v>
       </c>
@@ -1067,6 +1070,9 @@
       <c r="C3" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="D3" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="5" t="n"/>
@@ -1520,6 +1526,15 @@
           <t>Lease Liability - Operating NC</t>
         </is>
       </c>
+      <c r="B24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="E24" s="5" t="n"/>
       <c r="F24" s="5" t="n"/>
       <c r="G24" s="5" t="n"/>
@@ -1533,6 +1548,9 @@
           <t>Lease Liability - Finance NC</t>
         </is>
       </c>
+      <c r="B25" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="C25" s="4" t="n">
         <v>193</v>
       </c>
@@ -1706,6 +1724,9 @@
           <t>Retained Earnings (Accumulated Deficit)</t>
         </is>
       </c>
+      <c r="B33" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="C33" s="4" t="n">
         <v>-12053</v>
       </c>
@@ -1729,6 +1750,9 @@
         <v>3986</v>
       </c>
       <c r="C34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E34" s="5" t="n"/>
@@ -1749,7 +1773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1999,6 +2023,9 @@
           <t>Loss on Disposal of PP&amp;E</t>
         </is>
       </c>
+      <c r="B9" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="C9" s="4" t="n">
         <v>0</v>
       </c>
@@ -2168,7 +2195,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Change in A/P and Accrued (legacy)</t>
+          <t>Accounts Payable</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
@@ -2321,6 +2348,9 @@
           <t>Other Long-Term Assets</t>
         </is>
       </c>
+      <c r="B22" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="C22" s="4" t="n">
         <v>37</v>
       </c>
@@ -2343,6 +2373,9 @@
           <t>Note Receivable</t>
         </is>
       </c>
+      <c r="B23" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="C23" s="4" t="n">
         <v>0</v>
       </c>
@@ -2440,6 +2473,9 @@
           <t>Purchase of Non-Marketable Equity Securities</t>
         </is>
       </c>
+      <c r="B27" s="4" t="n">
+        <v>0</v>
+      </c>
       <c r="C27" s="4" t="n">
         <v>0</v>
       </c>
@@ -2459,8 +2495,20 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Acquisition of [entity]</t>
-        </is>
+          <t>Acquisition of Big Beverages</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>-75336</v>
       </c>
       <c r="F28" s="5" t="n"/>
       <c r="G28" s="5" t="n"/>
@@ -2472,17 +2520,20 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Acquisition of Big Beverages</t>
-        </is>
+          <t>Purchase of PP&amp;E</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="n">
+        <v>-3150</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>0</v>
+        <v>-8264</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>0</v>
+        <v>-17433</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>-75336</v>
+        <v>-23390</v>
       </c>
       <c r="F29" s="5" t="n"/>
       <c r="G29" s="5" t="n"/>
@@ -2494,20 +2545,20 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Purchase of PP&amp;E</t>
+          <t>Cash Flow from Investing</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>-3150</v>
+        <v>-1264</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>-8264</v>
+        <v>-5672</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>-17433</v>
+        <v>-14200</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>-23390</v>
+        <v>-101726</v>
       </c>
       <c r="F30" s="5" t="n"/>
       <c r="G30" s="5" t="n"/>
@@ -2519,20 +2570,20 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow from Investing</t>
+          <t>Finance Lease Payments</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>-1264</v>
+        <v>-94</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>-5672</v>
+        <v>-63</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>-14200</v>
+        <v>-44</v>
       </c>
       <c r="E31" s="4" t="n">
-        <v>-101726</v>
+        <v>-61</v>
       </c>
       <c r="F31" s="5" t="n"/>
       <c r="G31" s="5" t="n"/>
@@ -2544,20 +2595,20 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Finance Lease Payments</t>
+          <t>Repurchase of Common Stock (Tax Withholdings)</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>-94</v>
+        <v>0</v>
       </c>
       <c r="C32" s="4" t="n">
-        <v>-63</v>
+        <v>0</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>-44</v>
+        <v>0</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>-61</v>
+        <v>-2261</v>
       </c>
       <c r="F32" s="5" t="n"/>
       <c r="G32" s="5" t="n"/>
@@ -2569,17 +2620,20 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Repurchase of Common Stock (Tax Withholdings)</t>
-        </is>
+          <t>Proceeds from Stock Options</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>3720</v>
       </c>
       <c r="C33" s="4" t="n">
-        <v>0</v>
+        <v>3683</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>0</v>
+        <v>2285</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>-2261</v>
+        <v>3856</v>
       </c>
       <c r="F33" s="5" t="n"/>
       <c r="G33" s="5" t="n"/>
@@ -2591,20 +2645,20 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Stock Options</t>
+          <t>Proceeds from Common</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>3720</v>
+        <v>0</v>
       </c>
       <c r="C34" s="4" t="n">
-        <v>3683</v>
+        <v>0</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>2285</v>
+        <v>0</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>3856</v>
+        <v>0</v>
       </c>
       <c r="F34" s="5" t="n"/>
       <c r="G34" s="5" t="n"/>
@@ -2616,8 +2670,20 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Common</t>
-        </is>
+          <t>Proceeds from Preferred</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>542018</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="F35" s="5" t="n"/>
       <c r="G35" s="5" t="n"/>
@@ -2629,20 +2695,20 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Preferred</t>
+          <t>Dividends Paid on Preferred</t>
         </is>
       </c>
       <c r="B36" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C36" s="4" t="n">
-        <v>542018</v>
+        <v>-11526</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>0</v>
+        <v>-27462</v>
       </c>
       <c r="E36" s="4" t="n">
-        <v>0</v>
+        <v>-27500</v>
       </c>
       <c r="F36" s="5" t="n"/>
       <c r="G36" s="5" t="n"/>
@@ -2654,20 +2720,20 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Dividends Paid on Preferred</t>
+          <t>Cash Flow from Financing</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>0</v>
+        <v>71395</v>
       </c>
       <c r="C37" s="4" t="n">
-        <v>-11526</v>
+        <v>534112</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>-27462</v>
+        <v>-25221</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>-27500</v>
+        <v>-25966</v>
       </c>
       <c r="F37" s="5" t="n"/>
       <c r="G37" s="5" t="n"/>
@@ -2679,20 +2745,20 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow from Financing</t>
+          <t>FX Effect on Cash</t>
         </is>
       </c>
       <c r="B38" s="4" t="n">
-        <v>71395</v>
+        <v>-538</v>
       </c>
       <c r="C38" s="4" t="n">
-        <v>534112</v>
+        <v>50</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>-25221</v>
+        <v>1257</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>-25966</v>
+        <v>-997</v>
       </c>
       <c r="F38" s="5" t="n"/>
       <c r="G38" s="5" t="n"/>
@@ -2704,20 +2770,20 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>FX Effect on Cash</t>
+          <t>Net Change in Cash</t>
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>-538</v>
+        <v>-26993</v>
       </c>
       <c r="C39" s="4" t="n">
-        <v>50</v>
+        <v>636672</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>1257</v>
+        <v>103054</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>-997</v>
+        <v>134209</v>
       </c>
       <c r="F39" s="5" t="n"/>
       <c r="G39" s="5" t="n"/>
@@ -2729,20 +2795,20 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Net Change in Cash</t>
+          <t>Cash at Beginning</t>
         </is>
       </c>
       <c r="B40" s="4" t="n">
-        <v>-26993</v>
+        <v>43248</v>
       </c>
       <c r="C40" s="4" t="n">
-        <v>636672</v>
+        <v>16255</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>103054</v>
+        <v>652927</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>134209</v>
+        <v>755981</v>
       </c>
       <c r="F40" s="5" t="n"/>
       <c r="G40" s="5" t="n"/>
@@ -2754,20 +2820,20 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Cash at Beginning</t>
+          <t>Cash at End</t>
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>43248</v>
+        <v>16255</v>
       </c>
       <c r="C41" s="4" t="n">
-        <v>16255</v>
+        <v>652927</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>652927</v>
+        <v>755981</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>755981</v>
+        <v>890190</v>
       </c>
       <c r="F41" s="5" t="n"/>
       <c r="G41" s="5" t="n"/>
@@ -2776,31 +2842,6 @@
       <c r="J41" s="5" t="n"/>
       <c r="K41" s="5" t="n"/>
     </row>
-    <row r="42">
-      <c r="A42" s="3" t="inlineStr">
-        <is>
-          <t>Cash at End</t>
-        </is>
-      </c>
-      <c r="B42" s="4" t="n">
-        <v>16255</v>
-      </c>
-      <c r="C42" s="4" t="n">
-        <v>652927</v>
-      </c>
-      <c r="D42" s="4" t="n">
-        <v>755981</v>
-      </c>
-      <c r="E42" s="4" t="n">
-        <v>890190</v>
-      </c>
-      <c r="F42" s="5" t="n"/>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="5" t="n"/>
-      <c r="I42" s="5" t="n"/>
-      <c r="J42" s="5" t="n"/>
-      <c r="K42" s="5" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-04-22 23:15:09
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -69,7 +69,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -78,6 +78,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2423,24 +2425,46 @@
           <t>Cash Flow from Operations</t>
         </is>
       </c>
-      <c r="B25" s="4" t="n">
-        <v>-96586</v>
-      </c>
-      <c r="C25" s="4" t="n">
-        <v>108182</v>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>141218</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>262898</v>
-      </c>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="5" t="n"/>
-      <c r="I25" s="5" t="n"/>
-      <c r="J25" s="5" t="n"/>
-      <c r="K25" s="5" t="n"/>
+      <c r="B25" s="6">
+        <f>SUM(B2:B24)</f>
+        <v/>
+      </c>
+      <c r="C25" s="6">
+        <f>SUM(C2:C24)</f>
+        <v/>
+      </c>
+      <c r="D25" s="6">
+        <f>SUM(D2:D24)</f>
+        <v/>
+      </c>
+      <c r="E25" s="6">
+        <f>SUM(E2:E24)</f>
+        <v/>
+      </c>
+      <c r="F25" s="7">
+        <f>SUM(F2:F24)</f>
+        <v/>
+      </c>
+      <c r="G25" s="7">
+        <f>SUM(G2:G24)</f>
+        <v/>
+      </c>
+      <c r="H25" s="7">
+        <f>SUM(H2:H24)</f>
+        <v/>
+      </c>
+      <c r="I25" s="7">
+        <f>SUM(I2:I24)</f>
+        <v/>
+      </c>
+      <c r="J25" s="7">
+        <f>SUM(J2:J24)</f>
+        <v/>
+      </c>
+      <c r="K25" s="7">
+        <f>SUM(K2:K24)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -2548,24 +2572,46 @@
           <t>Cash Flow from Investing</t>
         </is>
       </c>
-      <c r="B30" s="4" t="n">
-        <v>-1264</v>
-      </c>
-      <c r="C30" s="4" t="n">
-        <v>-5672</v>
-      </c>
-      <c r="D30" s="4" t="n">
-        <v>-14200</v>
-      </c>
-      <c r="E30" s="4" t="n">
-        <v>-101726</v>
-      </c>
-      <c r="F30" s="5" t="n"/>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="5" t="n"/>
-      <c r="I30" s="5" t="n"/>
-      <c r="J30" s="5" t="n"/>
-      <c r="K30" s="5" t="n"/>
+      <c r="B30" s="6">
+        <f>SUM(B26:B29)</f>
+        <v/>
+      </c>
+      <c r="C30" s="6">
+        <f>SUM(C26:C29)</f>
+        <v/>
+      </c>
+      <c r="D30" s="6">
+        <f>SUM(D26:D29)</f>
+        <v/>
+      </c>
+      <c r="E30" s="6">
+        <f>SUM(E26:E29)</f>
+        <v/>
+      </c>
+      <c r="F30" s="7">
+        <f>SUM(F26:F29)</f>
+        <v/>
+      </c>
+      <c r="G30" s="7">
+        <f>SUM(G26:G29)</f>
+        <v/>
+      </c>
+      <c r="H30" s="7">
+        <f>SUM(H26:H29)</f>
+        <v/>
+      </c>
+      <c r="I30" s="7">
+        <f>SUM(I26:I29)</f>
+        <v/>
+      </c>
+      <c r="J30" s="7">
+        <f>SUM(J26:J29)</f>
+        <v/>
+      </c>
+      <c r="K30" s="7">
+        <f>SUM(K26:K29)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -2723,24 +2769,46 @@
           <t>Cash Flow from Financing</t>
         </is>
       </c>
-      <c r="B37" s="4" t="n">
-        <v>71395</v>
-      </c>
-      <c r="C37" s="4" t="n">
-        <v>534112</v>
-      </c>
-      <c r="D37" s="4" t="n">
-        <v>-25221</v>
-      </c>
-      <c r="E37" s="4" t="n">
-        <v>-25966</v>
-      </c>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="5" t="n"/>
-      <c r="I37" s="5" t="n"/>
-      <c r="J37" s="5" t="n"/>
-      <c r="K37" s="5" t="n"/>
+      <c r="B37" s="6">
+        <f>SUM(B31:B36)</f>
+        <v/>
+      </c>
+      <c r="C37" s="6">
+        <f>SUM(C31:C36)</f>
+        <v/>
+      </c>
+      <c r="D37" s="6">
+        <f>SUM(D31:D36)</f>
+        <v/>
+      </c>
+      <c r="E37" s="6">
+        <f>SUM(E31:E36)</f>
+        <v/>
+      </c>
+      <c r="F37" s="7">
+        <f>SUM(F31:F36)</f>
+        <v/>
+      </c>
+      <c r="G37" s="7">
+        <f>SUM(G31:G36)</f>
+        <v/>
+      </c>
+      <c r="H37" s="7">
+        <f>SUM(H31:H36)</f>
+        <v/>
+      </c>
+      <c r="I37" s="7">
+        <f>SUM(I31:I36)</f>
+        <v/>
+      </c>
+      <c r="J37" s="7">
+        <f>SUM(J31:J36)</f>
+        <v/>
+      </c>
+      <c r="K37" s="7">
+        <f>SUM(K31:K36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">

</xml_diff>

<commit_message>
vault backup: 2026-04-23 00:57:03
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -57,13 +57,18 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -78,8 +83,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -975,7 +980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1195,39 +1200,60 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Net PP&amp;E</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>10185</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>24868</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>55602</v>
-      </c>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
+          <t>Total Current Assets</t>
+        </is>
+      </c>
+      <c r="B9" s="6">
+        <f>SUM(B2:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="6">
+        <f>SUM(C2:C8)</f>
+        <v/>
+      </c>
+      <c r="D9" s="6">
+        <f>SUM(D2:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="7">
+        <f>SUM(E2:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="7">
+        <f>SUM(F2:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="7">
+        <f>SUM(G2:G8)</f>
+        <v/>
+      </c>
+      <c r="H9" s="7">
+        <f>SUM(H2:H8)</f>
+        <v/>
+      </c>
+      <c r="I9" s="7">
+        <f>SUM(I2:I8)</f>
+        <v/>
+      </c>
+      <c r="J9" s="7">
+        <f>SUM(J2:J8)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Deferred Tax Assets</t>
+          <t>Net PP&amp;E</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>501</v>
+        <v>10185</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>29518</v>
+        <v>24868</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>38699</v>
+        <v>55602</v>
       </c>
       <c r="E10" s="5" t="n"/>
       <c r="F10" s="5" t="n"/>
@@ -1239,17 +1265,17 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>ROU Assets - Operating</t>
+          <t>Deferred Tax Assets</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>972</v>
+        <v>501</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1957</v>
+        <v>29518</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>21606</v>
+        <v>38699</v>
       </c>
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
@@ -1261,17 +1287,17 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>ROU Assets - Finance</t>
+          <t>ROU Assets - Operating</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>208</v>
+        <v>972</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>208</v>
+        <v>1957</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>230</v>
+        <v>21606</v>
       </c>
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="n"/>
@@ -1283,17 +1309,17 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Deferred Other Costs (NC)</t>
+          <t>ROU Assets - Finance</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>262462</v>
+        <v>208</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>248338</v>
+        <v>208</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>234215</v>
+        <v>230</v>
       </c>
       <c r="E13" s="5" t="n"/>
       <c r="F13" s="5" t="n"/>
@@ -1305,17 +1331,17 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Intangibles</t>
+          <t>Deferred Other Costs (NC)</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>12254</v>
+        <v>262462</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>12139</v>
+        <v>248338</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>12213</v>
+        <v>234215</v>
       </c>
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
@@ -1327,17 +1353,17 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Goodwill</t>
+          <t>Intangibles</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>13679</v>
+        <v>12254</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>14173</v>
+        <v>12139</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>71582</v>
+        <v>12213</v>
       </c>
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="n"/>
@@ -1349,17 +1375,17 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Other Long-Term Assets</t>
+          <t>Goodwill</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>263</v>
+        <v>13679</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>291</v>
+        <v>14173</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>8154</v>
+        <v>71582</v>
       </c>
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
@@ -1371,17 +1397,17 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Accounts Payable</t>
+          <t>Other Long-Term Assets</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>36248</v>
+        <v>263</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>42840</v>
+        <v>291</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>41287</v>
+        <v>8154</v>
       </c>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
@@ -1393,39 +1419,60 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Accrued Expenses</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>69899</v>
-      </c>
-      <c r="C18" s="4" t="n">
-        <v>62120</v>
-      </c>
-      <c r="D18" s="4" t="n">
-        <v>148780</v>
-      </c>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="5" t="n"/>
+          <t>Total Assets</t>
+        </is>
+      </c>
+      <c r="B18" s="6">
+        <f>B9+SUM(B10:B17)</f>
+        <v/>
+      </c>
+      <c r="C18" s="6">
+        <f>C9+SUM(C10:C17)</f>
+        <v/>
+      </c>
+      <c r="D18" s="6">
+        <f>D9+SUM(D10:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="7">
+        <f>E9+SUM(E10:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="7">
+        <f>F9+SUM(F10:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="7">
+        <f>G9+SUM(G10:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="7">
+        <f>H9+SUM(H10:H17)</f>
+        <v/>
+      </c>
+      <c r="I18" s="7">
+        <f>I9+SUM(I10:I17)</f>
+        <v/>
+      </c>
+      <c r="J18" s="7">
+        <f>J9+SUM(J10:J17)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Accrued Promotional Allowance</t>
+          <t>Accounts Payable</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>35977</v>
+        <v>36248</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>99787</v>
+        <v>42840</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>135948</v>
+        <v>41287</v>
       </c>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
@@ -1437,17 +1484,17 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Operating Current</t>
+          <t>Accrued Expenses</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>661</v>
+        <v>69899</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>980</v>
+        <v>62120</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>3265</v>
+        <v>148780</v>
       </c>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
@@ -1459,17 +1506,17 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Finance Current</t>
+          <t>Accrued Promotional Allowance</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>70</v>
+        <v>35977</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>59</v>
+        <v>99787</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>100</v>
+        <v>135948</v>
       </c>
       <c r="E21" s="5" t="n"/>
       <c r="F21" s="5" t="n"/>
@@ -1481,17 +1528,17 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Deferred Revenue (Current)</t>
+          <t>Lease Liability - Finance Current</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>9675</v>
+        <v>70</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>9513</v>
+        <v>59</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>9513</v>
+        <v>100</v>
       </c>
       <c r="E22" s="5" t="n"/>
       <c r="F22" s="5" t="n"/>
@@ -1503,17 +1550,17 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Other Current Liabilities</t>
+          <t>Deferred Revenue (Current)</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>3586</v>
+        <v>9675</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>10890</v>
+        <v>9513</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>15808</v>
+        <v>9513</v>
       </c>
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n"/>
@@ -1525,17 +1572,17 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Operating NC</t>
+          <t>Other Current Liabilities</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>0</v>
+        <v>3586</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>0</v>
+        <v>10890</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>0</v>
+        <v>15808</v>
       </c>
       <c r="E24" s="5" t="n"/>
       <c r="F24" s="5" t="n"/>
@@ -1547,17 +1594,17 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Finance NC</t>
+          <t>Income Taxes Payable</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>0</v>
+        <v>1193</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>193</v>
+        <v>50424</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>211</v>
+        <v>10834</v>
       </c>
       <c r="E25" s="5" t="n"/>
       <c r="F25" s="5" t="n"/>
@@ -1569,17 +1616,17 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Deferred Tax Liability</t>
+          <t>Accrued Distributor Termination Fees</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>15919</v>
+        <v>3986</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>2880</v>
+        <v>0</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>2330</v>
+        <v>0</v>
       </c>
       <c r="E26" s="5" t="n"/>
       <c r="F26" s="5" t="n"/>
@@ -1591,39 +1638,60 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Deferred Revenue (NC)</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="n">
-        <v>179788</v>
-      </c>
-      <c r="C27" s="4" t="n">
-        <v>167227</v>
-      </c>
-      <c r="D27" s="4" t="n">
-        <v>157714</v>
-      </c>
-      <c r="E27" s="5" t="n"/>
-      <c r="F27" s="5" t="n"/>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="5" t="n"/>
-      <c r="I27" s="5" t="n"/>
-      <c r="J27" s="5" t="n"/>
+          <t>Total Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B27" s="6">
+        <f>SUM(B19:B26)</f>
+        <v/>
+      </c>
+      <c r="C27" s="6">
+        <f>SUM(C19:C26)</f>
+        <v/>
+      </c>
+      <c r="D27" s="6">
+        <f>SUM(D19:D26)</f>
+        <v/>
+      </c>
+      <c r="E27" s="7">
+        <f>SUM(E19:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="7">
+        <f>SUM(F19:F26)</f>
+        <v/>
+      </c>
+      <c r="G27" s="7">
+        <f>SUM(G19:G26)</f>
+        <v/>
+      </c>
+      <c r="H27" s="7">
+        <f>SUM(H19:H26)</f>
+        <v/>
+      </c>
+      <c r="I27" s="7">
+        <f>SUM(I19:I26)</f>
+        <v/>
+      </c>
+      <c r="J27" s="7">
+        <f>SUM(J19:J26)</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Income Taxes Payable</t>
+          <t>Lease Liability - Operating Current</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
-        <v>1193</v>
+        <v>661</v>
       </c>
       <c r="C28" s="4" t="n">
-        <v>50424</v>
+        <v>980</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>10834</v>
+        <v>3265</v>
       </c>
       <c r="E28" s="5" t="n"/>
       <c r="F28" s="5" t="n"/>
@@ -1635,17 +1703,17 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Convertible Preferred Stock</t>
+          <t>Lease Liability - Finance NC</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>824488</v>
+        <v>0</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>824488</v>
+        <v>193</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>824488</v>
+        <v>211</v>
       </c>
       <c r="E29" s="5" t="n"/>
       <c r="F29" s="5" t="n"/>
@@ -1657,17 +1725,17 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Common Stock</t>
+          <t>Deferred Tax Liability</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>76</v>
+        <v>15919</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>77</v>
+        <v>2880</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>79</v>
+        <v>2330</v>
       </c>
       <c r="E30" s="5" t="n"/>
       <c r="F30" s="5" t="n"/>
@@ -1679,17 +1747,17 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Additional Paid-in Capital</t>
+          <t>Deferred Revenue (NC)</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>280668</v>
+        <v>179788</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>276717</v>
+        <v>167227</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>297579</v>
+        <v>157714</v>
       </c>
       <c r="E31" s="5" t="n"/>
       <c r="F31" s="5" t="n"/>
@@ -1701,39 +1769,60 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Accumulated Other Comprehensive Loss</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="n">
-        <v>-1881</v>
-      </c>
-      <c r="C32" s="4" t="n">
-        <v>-701</v>
-      </c>
-      <c r="D32" s="4" t="n">
-        <v>-3250</v>
-      </c>
-      <c r="E32" s="5" t="n"/>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="5" t="n"/>
-      <c r="H32" s="5" t="n"/>
-      <c r="I32" s="5" t="n"/>
-      <c r="J32" s="5" t="n"/>
+          <t>Total Liabilities</t>
+        </is>
+      </c>
+      <c r="B32" s="6">
+        <f>B27+SUM(B28:B31)</f>
+        <v/>
+      </c>
+      <c r="C32" s="6">
+        <f>C27+SUM(C28:C31)</f>
+        <v/>
+      </c>
+      <c r="D32" s="6">
+        <f>D27+SUM(D28:D31)</f>
+        <v/>
+      </c>
+      <c r="E32" s="7">
+        <f>E27+SUM(E28:E31)</f>
+        <v/>
+      </c>
+      <c r="F32" s="7">
+        <f>F27+SUM(F28:F31)</f>
+        <v/>
+      </c>
+      <c r="G32" s="7">
+        <f>G27+SUM(G28:G31)</f>
+        <v/>
+      </c>
+      <c r="H32" s="7">
+        <f>H27+SUM(H28:H31)</f>
+        <v/>
+      </c>
+      <c r="I32" s="7">
+        <f>I27+SUM(I28:I31)</f>
+        <v/>
+      </c>
+      <c r="J32" s="7">
+        <f>J27+SUM(J28:J31)</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Retained Earnings (Accumulated Deficit)</t>
+          <t>Convertible Preferred Stock</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
-        <v>0</v>
+        <v>824488</v>
       </c>
       <c r="C33" s="4" t="n">
-        <v>-12053</v>
+        <v>824488</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>105521</v>
+        <v>824488</v>
       </c>
       <c r="E33" s="5" t="n"/>
       <c r="F33" s="5" t="n"/>
@@ -1745,17 +1834,17 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Accrued Distributor Termination Fees</t>
+          <t>Common Stock</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>3986</v>
+        <v>76</v>
       </c>
       <c r="C34" s="4" t="n">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="E34" s="5" t="n"/>
       <c r="F34" s="5" t="n"/>
@@ -1763,6 +1852,180 @@
       <c r="H34" s="5" t="n"/>
       <c r="I34" s="5" t="n"/>
       <c r="J34" s="5" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Additional Paid-in Capital</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="n">
+        <v>280668</v>
+      </c>
+      <c r="C35" s="4" t="n">
+        <v>276717</v>
+      </c>
+      <c r="D35" s="4" t="n">
+        <v>297579</v>
+      </c>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="5" t="n"/>
+      <c r="G35" s="5" t="n"/>
+      <c r="H35" s="5" t="n"/>
+      <c r="I35" s="5" t="n"/>
+      <c r="J35" s="5" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Accumulated Other Comprehensive Loss</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>-1881</v>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>-701</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>-3250</v>
+      </c>
+      <c r="E36" s="5" t="n"/>
+      <c r="F36" s="5" t="n"/>
+      <c r="G36" s="5" t="n"/>
+      <c r="H36" s="5" t="n"/>
+      <c r="I36" s="5" t="n"/>
+      <c r="J36" s="5" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Retained Earnings (Accumulated Deficit)</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>-12053</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>105521</v>
+      </c>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="5" t="n"/>
+      <c r="I37" s="5" t="n"/>
+      <c r="J37" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Total Stockholders' Equity</t>
+        </is>
+      </c>
+      <c r="B38" s="6">
+        <f>SUM(B34:B37)</f>
+        <v/>
+      </c>
+      <c r="C38" s="6">
+        <f>SUM(C34:C37)</f>
+        <v/>
+      </c>
+      <c r="D38" s="6">
+        <f>SUM(D34:D37)</f>
+        <v/>
+      </c>
+      <c r="E38" s="7">
+        <f>SUM(E34:E37)</f>
+        <v/>
+      </c>
+      <c r="F38" s="7">
+        <f>SUM(F34:F37)</f>
+        <v/>
+      </c>
+      <c r="G38" s="7">
+        <f>SUM(G34:G37)</f>
+        <v/>
+      </c>
+      <c r="H38" s="7">
+        <f>SUM(H34:H37)</f>
+        <v/>
+      </c>
+      <c r="I38" s="7">
+        <f>SUM(I34:I37)</f>
+        <v/>
+      </c>
+      <c r="J38" s="7">
+        <f>SUM(J34:J37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Total Liabilities, Mezzanine &amp; Stockholders' Equity</t>
+        </is>
+      </c>
+      <c r="B39" s="6">
+        <f>B32+B33+B38</f>
+        <v/>
+      </c>
+      <c r="C39" s="6">
+        <f>C32+C33+C38</f>
+        <v/>
+      </c>
+      <c r="D39" s="6">
+        <f>D32+D33+D38</f>
+        <v/>
+      </c>
+      <c r="E39" s="7">
+        <f>E32+E33+E38</f>
+        <v/>
+      </c>
+      <c r="F39" s="7">
+        <f>F32+F33+F38</f>
+        <v/>
+      </c>
+      <c r="G39" s="7">
+        <f>G32+G33+G38</f>
+        <v/>
+      </c>
+      <c r="H39" s="7">
+        <f>H32+H33+H38</f>
+        <v/>
+      </c>
+      <c r="I39" s="7">
+        <f>I32+I33+I38</f>
+        <v/>
+      </c>
+      <c r="J39" s="7">
+        <f>J32+J33+J38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Lease Liability - Operating NC</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="5" t="n"/>
+      <c r="F40" s="5" t="n"/>
+      <c r="G40" s="5" t="n"/>
+      <c r="H40" s="5" t="n"/>
+      <c r="I40" s="5" t="n"/>
+      <c r="J40" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 01:07:18
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -1528,17 +1528,17 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Finance Current</t>
+          <t>Lease Liability - Operating Current</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>70</v>
+        <v>661</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>59</v>
+        <v>980</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>100</v>
+        <v>3265</v>
       </c>
       <c r="E22" s="5" t="n"/>
       <c r="F22" s="5" t="n"/>
@@ -1550,17 +1550,17 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Deferred Revenue (Current)</t>
+          <t>Lease Liability - Finance Current</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>9675</v>
+        <v>70</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>9513</v>
+        <v>59</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>9513</v>
+        <v>100</v>
       </c>
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n"/>
@@ -1572,17 +1572,17 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Other Current Liabilities</t>
+          <t>Deferred Revenue (Current)</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>3586</v>
+        <v>9675</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>10890</v>
+        <v>9513</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>15808</v>
+        <v>9513</v>
       </c>
       <c r="E24" s="5" t="n"/>
       <c r="F24" s="5" t="n"/>
@@ -1594,17 +1594,17 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Income Taxes Payable</t>
+          <t>Other Current Liabilities</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>1193</v>
+        <v>3586</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>50424</v>
+        <v>10890</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>10834</v>
+        <v>15808</v>
       </c>
       <c r="E25" s="5" t="n"/>
       <c r="F25" s="5" t="n"/>
@@ -1616,17 +1616,17 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Accrued Distributor Termination Fees</t>
+          <t>Income Taxes Payable</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>3986</v>
+        <v>1193</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>0</v>
+        <v>50424</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>0</v>
+        <v>10834</v>
       </c>
       <c r="E26" s="5" t="n"/>
       <c r="F26" s="5" t="n"/>
@@ -1638,82 +1638,82 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Total Current Liabilities</t>
-        </is>
-      </c>
-      <c r="B27" s="6">
-        <f>SUM(B19:B26)</f>
-        <v/>
-      </c>
-      <c r="C27" s="6">
-        <f>SUM(C19:C26)</f>
-        <v/>
-      </c>
-      <c r="D27" s="6">
-        <f>SUM(D19:D26)</f>
-        <v/>
-      </c>
-      <c r="E27" s="7">
-        <f>SUM(E19:E26)</f>
-        <v/>
-      </c>
-      <c r="F27" s="7">
-        <f>SUM(F19:F26)</f>
-        <v/>
-      </c>
-      <c r="G27" s="7">
-        <f>SUM(G19:G26)</f>
-        <v/>
-      </c>
-      <c r="H27" s="7">
-        <f>SUM(H19:H26)</f>
-        <v/>
-      </c>
-      <c r="I27" s="7">
-        <f>SUM(I19:I26)</f>
-        <v/>
-      </c>
-      <c r="J27" s="7">
-        <f>SUM(J19:J26)</f>
-        <v/>
-      </c>
+          <t>Accrued Distributor Termination Fees</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>3986</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
+      <c r="G27" s="5" t="n"/>
+      <c r="H27" s="5" t="n"/>
+      <c r="I27" s="5" t="n"/>
+      <c r="J27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Operating Current</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="n">
-        <v>661</v>
-      </c>
-      <c r="C28" s="4" t="n">
-        <v>980</v>
-      </c>
-      <c r="D28" s="4" t="n">
-        <v>3265</v>
-      </c>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="n"/>
-      <c r="I28" s="5" t="n"/>
-      <c r="J28" s="5" t="n"/>
+          <t>Total Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B28" s="6">
+        <f>SUM(B19:B27)</f>
+        <v/>
+      </c>
+      <c r="C28" s="6">
+        <f>SUM(C19:C27)</f>
+        <v/>
+      </c>
+      <c r="D28" s="6">
+        <f>SUM(D19:D27)</f>
+        <v/>
+      </c>
+      <c r="E28" s="7">
+        <f>SUM(E19:E27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="7">
+        <f>SUM(F19:F27)</f>
+        <v/>
+      </c>
+      <c r="G28" s="7">
+        <f>SUM(G19:G27)</f>
+        <v/>
+      </c>
+      <c r="H28" s="7">
+        <f>SUM(H19:H27)</f>
+        <v/>
+      </c>
+      <c r="I28" s="7">
+        <f>SUM(I19:I27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="7">
+        <f>SUM(J19:J27)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Finance NC</t>
+          <t>Lease Liability - Operating NC</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>193</v>
+        <v>955</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>211</v>
+        <v>16674</v>
       </c>
       <c r="E29" s="5" t="n"/>
       <c r="F29" s="5" t="n"/>
@@ -1725,17 +1725,17 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Deferred Tax Liability</t>
+          <t>Lease Liability - Finance NC</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>15919</v>
+        <v>0</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>2880</v>
+        <v>193</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>2330</v>
+        <v>211</v>
       </c>
       <c r="E30" s="5" t="n"/>
       <c r="F30" s="5" t="n"/>
@@ -1747,17 +1747,17 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Deferred Revenue (NC)</t>
+          <t>Deferred Tax Liability</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>179788</v>
+        <v>15919</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>167227</v>
+        <v>2880</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>157714</v>
+        <v>2330</v>
       </c>
       <c r="E31" s="5" t="n"/>
       <c r="F31" s="5" t="n"/>
@@ -1769,82 +1769,82 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Total Liabilities</t>
-        </is>
-      </c>
-      <c r="B32" s="6">
-        <f>B27+SUM(B28:B31)</f>
-        <v/>
-      </c>
-      <c r="C32" s="6">
-        <f>C27+SUM(C28:C31)</f>
-        <v/>
-      </c>
-      <c r="D32" s="6">
-        <f>D27+SUM(D28:D31)</f>
-        <v/>
-      </c>
-      <c r="E32" s="7">
-        <f>E27+SUM(E28:E31)</f>
-        <v/>
-      </c>
-      <c r="F32" s="7">
-        <f>F27+SUM(F28:F31)</f>
-        <v/>
-      </c>
-      <c r="G32" s="7">
-        <f>G27+SUM(G28:G31)</f>
-        <v/>
-      </c>
-      <c r="H32" s="7">
-        <f>H27+SUM(H28:H31)</f>
-        <v/>
-      </c>
-      <c r="I32" s="7">
-        <f>I27+SUM(I28:I31)</f>
-        <v/>
-      </c>
-      <c r="J32" s="7">
-        <f>J27+SUM(J28:J31)</f>
-        <v/>
-      </c>
+          <t>Deferred Revenue (NC)</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>179788</v>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>167227</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>157714</v>
+      </c>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="5" t="n"/>
+      <c r="H32" s="5" t="n"/>
+      <c r="I32" s="5" t="n"/>
+      <c r="J32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Convertible Preferred Stock</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="n">
-        <v>824488</v>
-      </c>
-      <c r="C33" s="4" t="n">
-        <v>824488</v>
-      </c>
-      <c r="D33" s="4" t="n">
-        <v>824488</v>
-      </c>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="5" t="n"/>
-      <c r="I33" s="5" t="n"/>
-      <c r="J33" s="5" t="n"/>
+          <t>Total Liabilities</t>
+        </is>
+      </c>
+      <c r="B33" s="6">
+        <f>B28+SUM(B29:B32)</f>
+        <v/>
+      </c>
+      <c r="C33" s="6">
+        <f>C28+SUM(C29:C32)</f>
+        <v/>
+      </c>
+      <c r="D33" s="6">
+        <f>D28+SUM(D29:D32)</f>
+        <v/>
+      </c>
+      <c r="E33" s="7">
+        <f>E28+SUM(E29:E32)</f>
+        <v/>
+      </c>
+      <c r="F33" s="7">
+        <f>F28+SUM(F29:F32)</f>
+        <v/>
+      </c>
+      <c r="G33" s="7">
+        <f>G28+SUM(G29:G32)</f>
+        <v/>
+      </c>
+      <c r="H33" s="7">
+        <f>H28+SUM(H29:H32)</f>
+        <v/>
+      </c>
+      <c r="I33" s="7">
+        <f>I28+SUM(I29:I32)</f>
+        <v/>
+      </c>
+      <c r="J33" s="7">
+        <f>J28+SUM(J29:J32)</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Common Stock</t>
+          <t>Convertible Preferred Stock</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
-        <v>76</v>
+        <v>824488</v>
       </c>
       <c r="C34" s="4" t="n">
-        <v>77</v>
+        <v>824488</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>79</v>
+        <v>824488</v>
       </c>
       <c r="E34" s="5" t="n"/>
       <c r="F34" s="5" t="n"/>
@@ -1856,17 +1856,17 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Additional Paid-in Capital</t>
+          <t>Common Stock</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
-        <v>280668</v>
+        <v>76</v>
       </c>
       <c r="C35" s="4" t="n">
-        <v>276717</v>
+        <v>77</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>297579</v>
+        <v>79</v>
       </c>
       <c r="E35" s="5" t="n"/>
       <c r="F35" s="5" t="n"/>
@@ -1878,17 +1878,17 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Accumulated Other Comprehensive Loss</t>
+          <t>Additional Paid-in Capital</t>
         </is>
       </c>
       <c r="B36" s="4" t="n">
-        <v>-1881</v>
+        <v>280668</v>
       </c>
       <c r="C36" s="4" t="n">
-        <v>-701</v>
+        <v>276717</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>-3250</v>
+        <v>297579</v>
       </c>
       <c r="E36" s="5" t="n"/>
       <c r="F36" s="5" t="n"/>
@@ -1900,17 +1900,17 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Retained Earnings (Accumulated Deficit)</t>
+          <t>Accumulated Other Comprehensive Loss</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>0</v>
+        <v>-1881</v>
       </c>
       <c r="C37" s="4" t="n">
-        <v>-12053</v>
+        <v>-701</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>105521</v>
+        <v>-3250</v>
       </c>
       <c r="E37" s="5" t="n"/>
       <c r="F37" s="5" t="n"/>
@@ -1922,110 +1922,110 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Total Stockholders' Equity</t>
-        </is>
-      </c>
-      <c r="B38" s="6">
-        <f>SUM(B34:B37)</f>
-        <v/>
-      </c>
-      <c r="C38" s="6">
-        <f>SUM(C34:C37)</f>
-        <v/>
-      </c>
-      <c r="D38" s="6">
-        <f>SUM(D34:D37)</f>
-        <v/>
-      </c>
-      <c r="E38" s="7">
-        <f>SUM(E34:E37)</f>
-        <v/>
-      </c>
-      <c r="F38" s="7">
-        <f>SUM(F34:F37)</f>
-        <v/>
-      </c>
-      <c r="G38" s="7">
-        <f>SUM(G34:G37)</f>
-        <v/>
-      </c>
-      <c r="H38" s="7">
-        <f>SUM(H34:H37)</f>
-        <v/>
-      </c>
-      <c r="I38" s="7">
-        <f>SUM(I34:I37)</f>
-        <v/>
-      </c>
-      <c r="J38" s="7">
-        <f>SUM(J34:J37)</f>
-        <v/>
-      </c>
+          <t>Retained Earnings (Accumulated Deficit)</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>-12053</v>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>105521</v>
+      </c>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="5" t="n"/>
+      <c r="G38" s="5" t="n"/>
+      <c r="H38" s="5" t="n"/>
+      <c r="I38" s="5" t="n"/>
+      <c r="J38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Total Liabilities, Mezzanine &amp; Stockholders' Equity</t>
+          <t>Total Stockholders' Equity</t>
         </is>
       </c>
       <c r="B39" s="6">
-        <f>B32+B33+B38</f>
+        <f>SUM(B35:B38)</f>
         <v/>
       </c>
       <c r="C39" s="6">
-        <f>C32+C33+C38</f>
+        <f>SUM(C35:C38)</f>
         <v/>
       </c>
       <c r="D39" s="6">
-        <f>D32+D33+D38</f>
+        <f>SUM(D35:D38)</f>
         <v/>
       </c>
       <c r="E39" s="7">
-        <f>E32+E33+E38</f>
+        <f>SUM(E35:E38)</f>
         <v/>
       </c>
       <c r="F39" s="7">
-        <f>F32+F33+F38</f>
+        <f>SUM(F35:F38)</f>
         <v/>
       </c>
       <c r="G39" s="7">
-        <f>G32+G33+G38</f>
+        <f>SUM(G35:G38)</f>
         <v/>
       </c>
       <c r="H39" s="7">
-        <f>H32+H33+H38</f>
+        <f>SUM(H35:H38)</f>
         <v/>
       </c>
       <c r="I39" s="7">
-        <f>I32+I33+I38</f>
+        <f>SUM(I35:I38)</f>
         <v/>
       </c>
       <c r="J39" s="7">
-        <f>J32+J33+J38</f>
+        <f>SUM(J35:J38)</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Operating NC</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" s="5" t="n"/>
-      <c r="F40" s="5" t="n"/>
-      <c r="G40" s="5" t="n"/>
-      <c r="H40" s="5" t="n"/>
-      <c r="I40" s="5" t="n"/>
-      <c r="J40" s="5" t="n"/>
+          <t>Total Liabilities, Mezzanine &amp; Stockholders' Equity</t>
+        </is>
+      </c>
+      <c r="B40" s="6">
+        <f>B33+B34+B39</f>
+        <v/>
+      </c>
+      <c r="C40" s="6">
+        <f>C33+C34+C39</f>
+        <v/>
+      </c>
+      <c r="D40" s="6">
+        <f>D33+D34+D39</f>
+        <v/>
+      </c>
+      <c r="E40" s="7">
+        <f>E33+E34+E39</f>
+        <v/>
+      </c>
+      <c r="F40" s="7">
+        <f>F33+F34+F39</f>
+        <v/>
+      </c>
+      <c r="G40" s="7">
+        <f>G33+G34+G39</f>
+        <v/>
+      </c>
+      <c r="H40" s="7">
+        <f>H33+H34+H39</f>
+        <v/>
+      </c>
+      <c r="I40" s="7">
+        <f>I33+I34+I39</f>
+        <v/>
+      </c>
+      <c r="J40" s="7">
+        <f>J33+J34+J39</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 12:08:05
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -575,24 +575,46 @@
           <t>Gross Profit</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
-        <v>128169</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>270869</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>633139</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>680207</v>
-      </c>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
+      <c r="B4" s="6">
+        <f>B2-B3</f>
+        <v/>
+      </c>
+      <c r="C4" s="6">
+        <f>C2-C3</f>
+        <v/>
+      </c>
+      <c r="D4" s="6">
+        <f>D2-D3</f>
+        <v/>
+      </c>
+      <c r="E4" s="6">
+        <f>E2-E3</f>
+        <v/>
+      </c>
+      <c r="F4" s="7">
+        <f>F2-F3</f>
+        <v/>
+      </c>
+      <c r="G4" s="7">
+        <f>G2-G3</f>
+        <v/>
+      </c>
+      <c r="H4" s="7">
+        <f>H2-H3</f>
+        <v/>
+      </c>
+      <c r="I4" s="7">
+        <f>I2-I3</f>
+        <v/>
+      </c>
+      <c r="J4" s="7">
+        <f>J2-J3</f>
+        <v/>
+      </c>
+      <c r="K4" s="7">
+        <f>K2-K3</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -625,24 +647,46 @@
           <t>Operating Profit</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>-4090</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>-157801</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>266366</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>155728</v>
-      </c>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
+      <c r="B6" s="6">
+        <f>B4-B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="6">
+        <f>C4-C5</f>
+        <v/>
+      </c>
+      <c r="D6" s="6">
+        <f>D4-D5</f>
+        <v/>
+      </c>
+      <c r="E6" s="6">
+        <f>E4-E5</f>
+        <v/>
+      </c>
+      <c r="F6" s="7">
+        <f>F4-F5</f>
+        <v/>
+      </c>
+      <c r="G6" s="7">
+        <f>G4-G5</f>
+        <v/>
+      </c>
+      <c r="H6" s="7">
+        <f>H4-H5</f>
+        <v/>
+      </c>
+      <c r="I6" s="7">
+        <f>I4-I5</f>
+        <v/>
+      </c>
+      <c r="J6" s="7">
+        <f>J4-J5</f>
+        <v/>
+      </c>
+      <c r="K6" s="7">
+        <f>K4-K5</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -725,24 +769,46 @@
           <t>Pre-Tax Income</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n">
-        <v>-4059</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>-152664</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>291749</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>195050</v>
-      </c>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
+      <c r="B10" s="6">
+        <f>B6+SUM(B7:B9)</f>
+        <v/>
+      </c>
+      <c r="C10" s="6">
+        <f>C6+SUM(C7:C9)</f>
+        <v/>
+      </c>
+      <c r="D10" s="6">
+        <f>D6+SUM(D7:D9)</f>
+        <v/>
+      </c>
+      <c r="E10" s="6">
+        <f>E6+SUM(E7:E9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="7">
+        <f>F6+SUM(F7:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="7">
+        <f>G6+SUM(G7:G9)</f>
+        <v/>
+      </c>
+      <c r="H10" s="7">
+        <f>H6+SUM(H7:H9)</f>
+        <v/>
+      </c>
+      <c r="I10" s="7">
+        <f>I6+SUM(I7:I9)</f>
+        <v/>
+      </c>
+      <c r="J10" s="7">
+        <f>J6+SUM(J7:J9)</f>
+        <v/>
+      </c>
+      <c r="K10" s="7">
+        <f>K6+SUM(K7:K9)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -775,24 +841,46 @@
           <t>Net Income</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n">
-        <v>3937</v>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>-187282</v>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>226801</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>145074</v>
-      </c>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
-      <c r="K12" s="5" t="n"/>
+      <c r="B12" s="6">
+        <f>B10+B11</f>
+        <v/>
+      </c>
+      <c r="C12" s="6">
+        <f>C10+C11</f>
+        <v/>
+      </c>
+      <c r="D12" s="6">
+        <f>D10+D11</f>
+        <v/>
+      </c>
+      <c r="E12" s="6">
+        <f>E10+E11</f>
+        <v/>
+      </c>
+      <c r="F12" s="7">
+        <f>F10+F11</f>
+        <v/>
+      </c>
+      <c r="G12" s="7">
+        <f>G10+G11</f>
+        <v/>
+      </c>
+      <c r="H12" s="7">
+        <f>H10+H11</f>
+        <v/>
+      </c>
+      <c r="I12" s="7">
+        <f>I10+I11</f>
+        <v/>
+      </c>
+      <c r="J12" s="7">
+        <f>J10+J11</f>
+        <v/>
+      </c>
+      <c r="K12" s="7">
+        <f>K10+K11</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">

</xml_diff>

<commit_message>
vault backup: 2026-04-23 12:18:22
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -695,13 +695,13 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>315</v>
+        <v>307</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>5292</v>
+        <v>10821</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>26501</v>
+        <v>53130</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>39263</v>
@@ -720,16 +720,16 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>817</v>
+        <v>-276</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>-2495</v>
+        <v>-392</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>1180</v>
+        <v>-1246</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>-2549</v>
+        <v>-1734</v>
       </c>
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
@@ -820,10 +820,10 @@
         <v>7996</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>-34618</v>
+        <v>-69236</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>-64948</v>
+        <v>-129896</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>-49976</v>
@@ -1204,10 +1204,10 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>3574</v>
+        <v>6553</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>2318</v>
+        <v>4636</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>0</v>
@@ -1623,7 +1623,7 @@
         <v>661</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>980</v>
+        <v>1960</v>
       </c>
       <c r="D22" s="4" t="n">
         <v>3265</v>
@@ -1645,7 +1645,7 @@
         <v>70</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>59</v>
+        <v>118</v>
       </c>
       <c r="D23" s="4" t="n">
         <v>100</v>
@@ -1667,7 +1667,7 @@
         <v>9675</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>9513</v>
+        <v>19026</v>
       </c>
       <c r="D24" s="4" t="n">
         <v>9513</v>
@@ -1864,7 +1864,7 @@
         <v>179788</v>
       </c>
       <c r="C32" s="4" t="n">
-        <v>167227</v>
+        <v>334454</v>
       </c>
       <c r="D32" s="4" t="n">
         <v>157714</v>
@@ -2455,10 +2455,10 @@
         <v>0</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>0</v>
+        <v>-28</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>-324</v>
@@ -2505,10 +2505,10 @@
         <v>-175174</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>11802</v>
+        <v>23604</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>-63299</v>
+        <v>-126598</v>
       </c>
       <c r="E14" s="4" t="n">
         <v>77190</v>
@@ -2627,16 +2627,16 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>374</v>
+        <v>1731</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>2610</v>
+        <v>2446</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>7305</v>
+        <v>55407</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>4920</v>
+        <v>-34616</v>
       </c>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="5" t="n"/>
@@ -2655,10 +2655,10 @@
         <v>29</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>-183</v>
+        <v>-366</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>-102</v>
+        <v>-204</v>
       </c>
       <c r="E20" s="4" t="n">
         <v>535</v>
@@ -3099,10 +3099,10 @@
         <v>0</v>
       </c>
       <c r="C36" s="4" t="n">
-        <v>-11526</v>
+        <v>-23052</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>-27462</v>
+        <v>-54924</v>
       </c>
       <c r="E36" s="4" t="n">
         <v>-27500</v>
@@ -3196,10 +3196,10 @@
         <v>-26993</v>
       </c>
       <c r="C39" s="4" t="n">
-        <v>636672</v>
+        <v>1273344</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>103054</v>
+        <v>206108</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>134209</v>
@@ -3221,10 +3221,10 @@
         <v>43248</v>
       </c>
       <c r="C40" s="4" t="n">
-        <v>16255</v>
+        <v>32510</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>652927</v>
+        <v>1305854</v>
       </c>
       <c r="E40" s="4" t="n">
         <v>755981</v>
@@ -3246,10 +3246,10 @@
         <v>16255</v>
       </c>
       <c r="C41" s="4" t="n">
-        <v>652927</v>
+        <v>1305854</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>755981</v>
+        <v>1511962</v>
       </c>
       <c r="E41" s="4" t="n">
         <v>890190</v>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 12:23:32
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -698,10 +698,10 @@
         <v>307</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>10821</v>
+        <v>5529</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>53130</v>
+        <v>26629</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>39263</v>
@@ -820,10 +820,10 @@
         <v>7996</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>-69236</v>
+        <v>-34618</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>-129896</v>
+        <v>-64948</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>-49976</v>
@@ -1207,7 +1207,7 @@
         <v>6553</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>4636</v>
+        <v>2318</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>0</v>
@@ -1620,10 +1620,10 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>661</v>
+        <v>987</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>1960</v>
+        <v>980</v>
       </c>
       <c r="D22" s="4" t="n">
         <v>3265</v>
@@ -1642,10 +1642,10 @@
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>70</v>
+        <v>232</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>118</v>
+        <v>59</v>
       </c>
       <c r="D23" s="4" t="n">
         <v>100</v>
@@ -1667,7 +1667,7 @@
         <v>9675</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>19026</v>
+        <v>9513</v>
       </c>
       <c r="D24" s="4" t="n">
         <v>9513</v>
@@ -1864,7 +1864,7 @@
         <v>179788</v>
       </c>
       <c r="C32" s="4" t="n">
-        <v>334454</v>
+        <v>167227</v>
       </c>
       <c r="D32" s="4" t="n">
         <v>157714</v>
@@ -2455,10 +2455,10 @@
         <v>0</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>-28</v>
+        <v>0</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>-324</v>
@@ -2505,10 +2505,10 @@
         <v>-175174</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>23604</v>
+        <v>11802</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>-126598</v>
+        <v>-63299</v>
       </c>
       <c r="E14" s="4" t="n">
         <v>77190</v>
@@ -2655,10 +2655,10 @@
         <v>29</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>-366</v>
+        <v>-183</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>-204</v>
+        <v>-102</v>
       </c>
       <c r="E20" s="4" t="n">
         <v>535</v>
@@ -3099,10 +3099,10 @@
         <v>0</v>
       </c>
       <c r="C36" s="4" t="n">
-        <v>-23052</v>
+        <v>-11526</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>-54924</v>
+        <v>-27462</v>
       </c>
       <c r="E36" s="4" t="n">
         <v>-27500</v>
@@ -3196,10 +3196,10 @@
         <v>-26993</v>
       </c>
       <c r="C39" s="4" t="n">
-        <v>1273344</v>
+        <v>636672</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>206108</v>
+        <v>103054</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>134209</v>
@@ -3221,10 +3221,10 @@
         <v>43248</v>
       </c>
       <c r="C40" s="4" t="n">
-        <v>32510</v>
+        <v>16255</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>1305854</v>
+        <v>652927</v>
       </c>
       <c r="E40" s="4" t="n">
         <v>755981</v>
@@ -3246,10 +3246,10 @@
         <v>16255</v>
       </c>
       <c r="C41" s="4" t="n">
-        <v>1305854</v>
+        <v>652927</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>1511962</v>
+        <v>755981</v>
       </c>
       <c r="E41" s="4" t="n">
         <v>890190</v>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 12:28:52
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -18,8 +18,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0;(#,##0)"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;--&quot;"/>
+    <numFmt numFmtId="165" formatCode="$#,##0_);($#,##0);&quot;$--&quot;_)"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00_);($#,##0.00)"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -74,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -83,8 +85,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -963,24 +967,24 @@
           <t>GAAP EPS (Basic)</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B16" s="8" t="n">
         <v>0.02</v>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="C16" s="8" t="n">
         <v>-0.88</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D16" s="8" t="n">
         <v>0.79</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" s="8" t="n">
         <v>0.46</v>
       </c>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
-      <c r="K16" s="5" t="n"/>
+      <c r="F16" s="9" t="n"/>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="9" t="n"/>
+      <c r="I16" s="9" t="n"/>
+      <c r="J16" s="9" t="n"/>
+      <c r="K16" s="9" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1013,24 +1017,24 @@
           <t>GAAP EPS (Diluted)</t>
         </is>
       </c>
-      <c r="B18" s="4" t="n">
+      <c r="B18" s="8" t="n">
         <v>0.02</v>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="C18" s="8" t="n">
         <v>-0.88</v>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="D18" s="8" t="n">
         <v>0.77</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" s="8" t="n">
         <v>0.45</v>
       </c>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="5" t="n"/>
-      <c r="K18" s="5" t="n"/>
+      <c r="F18" s="9" t="n"/>
+      <c r="G18" s="9" t="n"/>
+      <c r="H18" s="9" t="n"/>
+      <c r="I18" s="9" t="n"/>
+      <c r="J18" s="9" t="n"/>
+      <c r="K18" s="9" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">

</xml_diff>

<commit_message>
vault backup: 2026-04-23 13:05:04
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -2477,7 +2477,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Receivables</t>
+          <t>Accounts Receivable</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
@@ -2527,7 +2527,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Prepaids</t>
+          <t>Prepaid Expenses</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
@@ -2849,20 +2849,20 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Purchase of Non-Marketable Equity Securities</t>
+          <t>Purchase of PP&amp;E</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>0</v>
+        <v>-3150</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>0</v>
+        <v>-8264</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>0</v>
+        <v>-17433</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>-3000</v>
+        <v>-23390</v>
       </c>
       <c r="F27" s="5" t="n"/>
       <c r="G27" s="5" t="n"/>
@@ -2874,7 +2874,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Acquisition of Big Beverages</t>
+          <t>Purchase of Non-Marketable Equity Securities</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
@@ -2887,7 +2887,7 @@
         <v>0</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>-75336</v>
+        <v>-3000</v>
       </c>
       <c r="F28" s="5" t="n"/>
       <c r="G28" s="5" t="n"/>
@@ -2899,20 +2899,20 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Purchase of PP&amp;E</t>
+          <t>Acquisition of Big Beverages</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>-3150</v>
+        <v>0</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>-8264</v>
+        <v>0</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>-17433</v>
+        <v>0</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>-23390</v>
+        <v>-75336</v>
       </c>
       <c r="F29" s="5" t="n"/>
       <c r="G29" s="5" t="n"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 15:43:31
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -18,10 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;--&quot;"/>
     <numFmt numFmtId="165" formatCode="$#,##0_);($#,##0);&quot;$--&quot;_)"/>
-    <numFmt numFmtId="166" formatCode="$#,##0.00_);($#,##0.00)"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -76,7 +75,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -87,8 +86,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -526,7 +523,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Net Sales (Revenue)</t>
+          <t>Net Sales / Revenue</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
@@ -576,7 +573,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Gross Profit</t>
+          <t>Gross Profit (Loss)</t>
         </is>
       </c>
       <c r="B4" s="6">
@@ -623,7 +620,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Selling and Marketing Expenses</t>
+          <t>SG&amp;A</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
@@ -648,7 +645,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Operating Profit</t>
+          <t>Income (Loss) from Operations</t>
         </is>
       </c>
       <c r="B6" s="6">
@@ -695,7 +692,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Interest Income</t>
+          <t>Interest Income (Expense)</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
@@ -720,7 +717,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Foreign exchange gain (loss)</t>
+          <t>Foreign Currency Gain (Loss)</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
@@ -745,7 +742,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Other Income</t>
+          <t>Other Income (Expense)</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
@@ -770,7 +767,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Pre-Tax Income</t>
+          <t>Pre-Tax Income (Loss)</t>
         </is>
       </c>
       <c r="B10" s="6">
@@ -817,7 +814,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Income Taxes</t>
+          <t>Income Tax (Benefit) Expense</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
@@ -842,7 +839,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Net Income</t>
+          <t>Net Income (Loss)</t>
         </is>
       </c>
       <c r="B12" s="6">
@@ -889,7 +886,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Dividends on Series A Pref</t>
+          <t>Dividends</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
@@ -914,20 +911,20 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Net Income to Common Shareholders</t>
+          <t>Income Allocated to Participating Preferred</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>3937</v>
+        <v>0</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>-198808</v>
+        <v>0</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>181991</v>
+        <v>-17348</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>107457</v>
+        <v>-10117</v>
       </c>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
@@ -939,20 +936,20 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Income Allocated to Participating</t>
+          <t>Net Income (Loss) Attributable to Common Shareholders</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>0</v>
+        <v>3937</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>0</v>
+        <v>-198808</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>-17348</v>
+        <v>181991</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>-10117</v>
+        <v>107457</v>
       </c>
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
@@ -964,45 +961,45 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>GAAP EPS (Basic)</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="n">
+          <t>Basic Earnings (Loss) per Share</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
         <v>0.02</v>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16" s="4" t="n">
         <v>-0.88</v>
       </c>
-      <c r="D16" s="8" t="n">
+      <c r="D16" s="4" t="n">
         <v>0.79</v>
       </c>
-      <c r="E16" s="8" t="n">
+      <c r="E16" s="4" t="n">
         <v>0.46</v>
       </c>
-      <c r="F16" s="9" t="n"/>
-      <c r="G16" s="9" t="n"/>
-      <c r="H16" s="9" t="n"/>
-      <c r="I16" s="9" t="n"/>
-      <c r="J16" s="9" t="n"/>
-      <c r="K16" s="9" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="n"/>
+      <c r="J16" s="5" t="n"/>
+      <c r="K16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Weighted Avg Shares Outstanding (Basic)</t>
+          <t>Diluted Earnings (Loss) per Share</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>221343</v>
+        <v>0.02</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>226947</v>
+        <v>-0.88</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>230784</v>
+        <v>0.77</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>233667</v>
+        <v>0.45</v>
       </c>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="n"/>
@@ -1014,32 +1011,32 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>GAAP EPS (Diluted)</t>
-        </is>
-      </c>
-      <c r="B18" s="8" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="C18" s="8" t="n">
-        <v>-0.88</v>
-      </c>
-      <c r="D18" s="8" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="E18" s="8" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="F18" s="9" t="n"/>
-      <c r="G18" s="9" t="n"/>
-      <c r="H18" s="9" t="n"/>
-      <c r="I18" s="9" t="n"/>
-      <c r="J18" s="9" t="n"/>
-      <c r="K18" s="9" t="n"/>
+          <t>Weighted Average Shares Outstanding (Basic)</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>221343</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>226947</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>230784</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>233667</v>
+      </c>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="n"/>
+      <c r="K18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Weighted Avg Shares Outstanding (Diluted)</t>
+          <t>Weighted Average Shares Outstanding (Diluted)</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
@@ -1160,17 +1157,17 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Restricted Cash</t>
+          <t>Accounts Receivable</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>38768</v>
+        <v>63311</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>0</v>
+        <v>183703</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>0</v>
+        <v>270342</v>
       </c>
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="5" t="n"/>
@@ -1182,17 +1179,17 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Accounts Receivable</t>
+          <t>Note Receivable - Current</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>63311</v>
+        <v>6553</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>183703</v>
+        <v>2318</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>270342</v>
+        <v>0</v>
       </c>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
@@ -1204,17 +1201,17 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Note Receivable</t>
+          <t>Inventories</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>6553</v>
+        <v>173289</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>2318</v>
+        <v>229275</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0</v>
+        <v>131165</v>
       </c>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
@@ -1226,17 +1223,17 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Inventories</t>
+          <t>Deferred Other Costs - Current</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>173289</v>
+        <v>14124</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>229275</v>
+        <v>14124</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>131165</v>
+        <v>14124</v>
       </c>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
@@ -1248,17 +1245,17 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Deferred Other Costs (Current)</t>
+          <t>Prepaid Expenses</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>14124</v>
+        <v>11341</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>14124</v>
+        <v>19503</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>14124</v>
+        <v>18759</v>
       </c>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
@@ -1270,17 +1267,17 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Prepaid Expenses</t>
+          <t>Restricted Cash</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>11341</v>
+        <v>38768</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>19503</v>
+        <v>0</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>18759</v>
+        <v>0</v>
       </c>
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
@@ -1357,17 +1354,17 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Deferred Tax Assets</t>
+          <t>ROU Assets - Operating - Non-Current</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>501</v>
+        <v>972</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>29518</v>
+        <v>1957</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>38699</v>
+        <v>21606</v>
       </c>
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
@@ -1379,17 +1376,17 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>ROU Assets - Operating</t>
+          <t>ROU Assets - Finance - Non-Current</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>972</v>
+        <v>208</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>1957</v>
+        <v>208</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>21606</v>
+        <v>230</v>
       </c>
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="n"/>
@@ -1401,17 +1398,17 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>ROU Assets - Finance</t>
+          <t>Intangible Assets</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>208</v>
+        <v>12254</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>208</v>
+        <v>12139</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>230</v>
+        <v>12213</v>
       </c>
       <c r="E13" s="5" t="n"/>
       <c r="F13" s="5" t="n"/>
@@ -1423,17 +1420,17 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Deferred Other Costs (NC)</t>
+          <t>Goodwill</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>262462</v>
+        <v>13679</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>248338</v>
+        <v>14173</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>234215</v>
+        <v>71582</v>
       </c>
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
@@ -1445,17 +1442,17 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Intangibles</t>
+          <t>Deferred Other Costs - Non-Current</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>12254</v>
+        <v>262462</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>12139</v>
+        <v>248338</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>12213</v>
+        <v>234215</v>
       </c>
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="n"/>
@@ -1467,17 +1464,17 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Goodwill</t>
+          <t>Deferred Tax Assets</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>13679</v>
+        <v>501</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>14173</v>
+        <v>29518</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>71582</v>
+        <v>38699</v>
       </c>
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
@@ -1489,7 +1486,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Other Long-Term Assets</t>
+          <t>Other Non-Current Assets</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
@@ -1598,17 +1595,17 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Accrued Promotional Allowance</t>
+          <t>Income Taxes Payable</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>35977</v>
+        <v>1193</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>99787</v>
+        <v>50424</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>135948</v>
+        <v>10834</v>
       </c>
       <c r="E21" s="5" t="n"/>
       <c r="F21" s="5" t="n"/>
@@ -1620,17 +1617,17 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Operating Current</t>
+          <t>Accrued Promotional Allowance</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>987</v>
+        <v>35977</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>980</v>
+        <v>99787</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>3265</v>
+        <v>135948</v>
       </c>
       <c r="E22" s="5" t="n"/>
       <c r="F22" s="5" t="n"/>
@@ -1642,17 +1639,17 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Finance Current</t>
+          <t>Lease Liability - Operating - Current</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>232</v>
+        <v>987</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>59</v>
+        <v>980</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>100</v>
+        <v>3265</v>
       </c>
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n"/>
@@ -1664,17 +1661,17 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Deferred Revenue (Current)</t>
+          <t>Lease Liability - Finance - Current</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>9675</v>
+        <v>232</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>9513</v>
+        <v>59</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>9513</v>
+        <v>100</v>
       </c>
       <c r="E24" s="5" t="n"/>
       <c r="F24" s="5" t="n"/>
@@ -1686,17 +1683,17 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Other Current Liabilities</t>
+          <t>Deferred Revenue - Current</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>3586</v>
+        <v>9675</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>10890</v>
+        <v>9513</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>15808</v>
+        <v>9513</v>
       </c>
       <c r="E25" s="5" t="n"/>
       <c r="F25" s="5" t="n"/>
@@ -1708,17 +1705,17 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Income Taxes Payable</t>
+          <t>Other Current Liabilities</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>1193</v>
+        <v>3586</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>50424</v>
+        <v>10890</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>10834</v>
+        <v>15808</v>
       </c>
       <c r="E26" s="5" t="n"/>
       <c r="F26" s="5" t="n"/>
@@ -1795,7 +1792,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Operating NC</t>
+          <t>Lease Liability - Operating - Non-Current</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
@@ -1817,7 +1814,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Finance NC</t>
+          <t>Lease Liability - Finance - Non-Current</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
@@ -1861,7 +1858,7 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Deferred Revenue (NC)</t>
+          <t>Deferred Revenue - Non-Current</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
@@ -1992,7 +1989,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Accumulated Other Comprehensive Loss</t>
+          <t>Accumulated Other Comprehensive Income (Loss)</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
@@ -2018,7 +2015,7 @@
         </is>
       </c>
       <c r="B38" s="4" t="n">
-        <v>0</v>
+        <v>-238772</v>
       </c>
       <c r="C38" s="4" t="n">
         <v>-12053</v>
@@ -2130,7 +2127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2202,7 +2199,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Net Income</t>
+          <t>Net Income (Loss)</t>
         </is>
       </c>
       <c r="B2" s="4" t="n">
@@ -2327,7 +2324,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Inventory Obsolescence</t>
+          <t>Inventory Write-Down</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
@@ -2352,20 +2349,20 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Stock-Based Compensation</t>
+          <t>Gain (Loss) on Disposal of PP&amp;E</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>36475</v>
+        <v>0</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>20665</v>
+        <v>0</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>21226</v>
+        <v>198</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>19591</v>
+        <v>173</v>
       </c>
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
@@ -2377,20 +2374,20 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Loss on Disposal of PP&amp;E</t>
+          <t>Stock-Based Compensation</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>0</v>
+        <v>36475</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>0</v>
+        <v>20665</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>198</v>
+        <v>21226</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>173</v>
+        <v>19591</v>
       </c>
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
@@ -2402,7 +2399,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Deferred Income Taxes-Net</t>
+          <t>(Benefit) Provision for Deferred Income Taxes</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
@@ -2427,7 +2424,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Foreign Exchange Loss</t>
+          <t>Foreign Currency Gain (Loss)</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
@@ -2452,7 +2449,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Other Items</t>
+          <t>Other Operating Items</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
@@ -2502,20 +2499,20 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Inventories</t>
+          <t>Note Receivable</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>-175174</v>
+        <v>0</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>11802</v>
+        <v>0</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>-63299</v>
+        <v>0</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>77190</v>
+        <v>2318</v>
       </c>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
@@ -2527,20 +2524,20 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Prepaid Expenses</t>
+          <t>Inventories</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>1072</v>
+        <v>-175174</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>2214</v>
+        <v>11802</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>-7980</v>
+        <v>-63299</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>1074</v>
+        <v>77190</v>
       </c>
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
@@ -2552,20 +2549,20 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Accounts Payable</t>
+          <t>Prepaid Expenses</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>23966</v>
+        <v>1072</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>428</v>
+        <v>2214</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>5249</v>
+        <v>-7980</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>-1170</v>
+        <v>1074</v>
       </c>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
@@ -2577,20 +2574,20 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Accrued Expenses</t>
+          <t>Accounts Payable</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>26484</v>
+        <v>23966</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>34644</v>
+        <v>428</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>-8025</v>
+        <v>5249</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>85398</v>
+        <v>-1170</v>
       </c>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="n"/>
@@ -2602,20 +2599,20 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Accrued Promo</t>
+          <t>Accrued Expenses</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>13379</v>
+        <v>26484</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>16940</v>
+        <v>34644</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>63810</v>
+        <v>-8025</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>36161</v>
+        <v>85398</v>
       </c>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="5" t="n"/>
@@ -2652,20 +2649,20 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>ROU/Lease</t>
+          <t>Accrued Promotional Allowance</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>29</v>
+        <v>13379</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>-183</v>
+        <v>16940</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>-102</v>
+        <v>63810</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>535</v>
+        <v>36161</v>
       </c>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="5" t="n"/>
@@ -2677,20 +2674,20 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Deferred Revenue</t>
+          <t>Accrued Distributor Termination</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>189463</v>
+        <v>3986</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>-12723</v>
+        <v>-3739</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>-9513</v>
+        <v>-248</v>
       </c>
       <c r="F21" s="5" t="n"/>
       <c r="G21" s="5" t="n"/>
@@ -2702,20 +2699,20 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Other Long-Term Assets</t>
+          <t>ROU &amp; Lease Liability, Net</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>37</v>
+        <v>-183</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>-28</v>
+        <v>-102</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>-4862</v>
+        <v>535</v>
       </c>
       <c r="F22" s="5" t="n"/>
       <c r="G22" s="5" t="n"/>
@@ -2727,20 +2724,20 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Note Receivable</t>
+          <t>Deferred Revenue</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>0</v>
+        <v>189463</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0</v>
+        <v>-12723</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>2318</v>
+        <v>-9513</v>
       </c>
       <c r="F23" s="5" t="n"/>
       <c r="G23" s="5" t="n"/>
@@ -2752,20 +2749,20 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Accrued Distributor Termination</t>
+          <t>Other Non-Current Assets</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>3986</v>
+        <v>37</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>-3739</v>
+        <v>-28</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>-248</v>
+        <v>-4862</v>
       </c>
       <c r="F24" s="5" t="n"/>
       <c r="G24" s="5" t="n"/>
@@ -2996,20 +2993,20 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Repurchase of Common Stock (Tax Withholdings)</t>
+          <t>Proceeds from Exercise of Stock Options</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>0</v>
+        <v>3720</v>
       </c>
       <c r="C32" s="4" t="n">
-        <v>0</v>
+        <v>3683</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>0</v>
+        <v>2285</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>-2261</v>
+        <v>3856</v>
       </c>
       <c r="F32" s="5" t="n"/>
       <c r="G32" s="5" t="n"/>
@@ -3021,20 +3018,20 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Stock Options</t>
+          <t>Proceeds from Issuance of Preferred Stock</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
-        <v>3720</v>
+        <v>0</v>
       </c>
       <c r="C33" s="4" t="n">
-        <v>3683</v>
+        <v>542018</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>2285</v>
+        <v>0</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>3856</v>
+        <v>0</v>
       </c>
       <c r="F33" s="5" t="n"/>
       <c r="G33" s="5" t="n"/>
@@ -3046,20 +3043,20 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Common</t>
+          <t>Dividends Paid</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C34" s="4" t="n">
-        <v>0</v>
+        <v>-11526</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>0</v>
+        <v>-27462</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>0</v>
+        <v>-27500</v>
       </c>
       <c r="F34" s="5" t="n"/>
       <c r="G34" s="5" t="n"/>
@@ -3071,20 +3068,20 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Preferred</t>
+          <t>Share Repurchases</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C35" s="4" t="n">
-        <v>542018</v>
+        <v>0</v>
       </c>
       <c r="D35" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>0</v>
+        <v>-2261</v>
       </c>
       <c r="F35" s="5" t="n"/>
       <c r="G35" s="5" t="n"/>
@@ -3096,92 +3093,92 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Dividends Paid on Preferred</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C36" s="4" t="n">
-        <v>-11526</v>
-      </c>
-      <c r="D36" s="4" t="n">
-        <v>-27462</v>
-      </c>
-      <c r="E36" s="4" t="n">
-        <v>-27500</v>
-      </c>
-      <c r="F36" s="5" t="n"/>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="5" t="n"/>
-      <c r="I36" s="5" t="n"/>
-      <c r="J36" s="5" t="n"/>
-      <c r="K36" s="5" t="n"/>
+          <t>Cash Flow from Financing</t>
+        </is>
+      </c>
+      <c r="B36" s="6">
+        <f>SUM(B31:B35)</f>
+        <v/>
+      </c>
+      <c r="C36" s="6">
+        <f>SUM(C31:C35)</f>
+        <v/>
+      </c>
+      <c r="D36" s="6">
+        <f>SUM(D31:D35)</f>
+        <v/>
+      </c>
+      <c r="E36" s="6">
+        <f>SUM(E31:E35)</f>
+        <v/>
+      </c>
+      <c r="F36" s="7">
+        <f>SUM(F31:F35)</f>
+        <v/>
+      </c>
+      <c r="G36" s="7">
+        <f>SUM(G31:G35)</f>
+        <v/>
+      </c>
+      <c r="H36" s="7">
+        <f>SUM(H31:H35)</f>
+        <v/>
+      </c>
+      <c r="I36" s="7">
+        <f>SUM(I31:I35)</f>
+        <v/>
+      </c>
+      <c r="J36" s="7">
+        <f>SUM(J31:J35)</f>
+        <v/>
+      </c>
+      <c r="K36" s="7">
+        <f>SUM(K31:K35)</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow from Financing</t>
-        </is>
-      </c>
-      <c r="B37" s="6">
-        <f>SUM(B31:B36)</f>
-        <v/>
-      </c>
-      <c r="C37" s="6">
-        <f>SUM(C31:C36)</f>
-        <v/>
-      </c>
-      <c r="D37" s="6">
-        <f>SUM(D31:D36)</f>
-        <v/>
-      </c>
-      <c r="E37" s="6">
-        <f>SUM(E31:E36)</f>
-        <v/>
-      </c>
-      <c r="F37" s="7">
-        <f>SUM(F31:F36)</f>
-        <v/>
-      </c>
-      <c r="G37" s="7">
-        <f>SUM(G31:G36)</f>
-        <v/>
-      </c>
-      <c r="H37" s="7">
-        <f>SUM(H31:H36)</f>
-        <v/>
-      </c>
-      <c r="I37" s="7">
-        <f>SUM(I31:I36)</f>
-        <v/>
-      </c>
-      <c r="J37" s="7">
-        <f>SUM(J31:J36)</f>
-        <v/>
-      </c>
-      <c r="K37" s="7">
-        <f>SUM(K31:K36)</f>
-        <v/>
-      </c>
+          <t>FX Effect on Cash</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="n">
+        <v>-538</v>
+      </c>
+      <c r="C37" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="D37" s="4" t="n">
+        <v>1257</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>-997</v>
+      </c>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="5" t="n"/>
+      <c r="H37" s="5" t="n"/>
+      <c r="I37" s="5" t="n"/>
+      <c r="J37" s="5" t="n"/>
+      <c r="K37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>FX Effect on Cash</t>
+          <t>Net Change in Cash</t>
         </is>
       </c>
       <c r="B38" s="4" t="n">
-        <v>-538</v>
+        <v>-26993</v>
       </c>
       <c r="C38" s="4" t="n">
-        <v>50</v>
+        <v>636672</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>1257</v>
+        <v>103054</v>
       </c>
       <c r="E38" s="4" t="n">
-        <v>-997</v>
+        <v>134209</v>
       </c>
       <c r="F38" s="5" t="n"/>
       <c r="G38" s="5" t="n"/>
@@ -3193,20 +3190,20 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Net Change in Cash</t>
+          <t>Cash at Beginning of Period</t>
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>-26993</v>
+        <v>43248</v>
       </c>
       <c r="C39" s="4" t="n">
-        <v>636672</v>
+        <v>16255</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>103054</v>
+        <v>652927</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>134209</v>
+        <v>755981</v>
       </c>
       <c r="F39" s="5" t="n"/>
       <c r="G39" s="5" t="n"/>
@@ -3218,20 +3215,20 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Cash at Beginning</t>
+          <t>Cash at End of Period</t>
         </is>
       </c>
       <c r="B40" s="4" t="n">
-        <v>43248</v>
+        <v>16255</v>
       </c>
       <c r="C40" s="4" t="n">
-        <v>16255</v>
+        <v>652927</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>652927</v>
+        <v>755981</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>755981</v>
+        <v>890190</v>
       </c>
       <c r="F40" s="5" t="n"/>
       <c r="G40" s="5" t="n"/>
@@ -3243,20 +3240,20 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Cash at End</t>
+          <t>Gain (Loss) on Lease Cancellations</t>
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>16255</v>
+        <v>-28</v>
       </c>
       <c r="C41" s="4" t="n">
-        <v>652927</v>
+        <v>0</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>755981</v>
+        <v>0</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>890190</v>
+        <v>0</v>
       </c>
       <c r="F41" s="5" t="n"/>
       <c r="G41" s="5" t="n"/>
@@ -3265,6 +3262,31 @@
       <c r="J41" s="5" t="n"/>
       <c r="K41" s="5" t="n"/>
     </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Proceeds from Issuance of Common Stock</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="n">
+        <v>67769</v>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="5" t="n"/>
+      <c r="G42" s="5" t="n"/>
+      <c r="H42" s="5" t="n"/>
+      <c r="I42" s="5" t="n"/>
+      <c r="J42" s="5" t="n"/>
+      <c r="K42" s="5" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 15:48:41
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -696,16 +696,16 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>307</v>
+        <v>-307</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>5529</v>
+        <v>-5529</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>26629</v>
+        <v>-26629</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>39263</v>
+        <v>-39263</v>
       </c>
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
@@ -721,16 +721,16 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>-276</v>
+        <v>276</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>-392</v>
+        <v>392</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>-1246</v>
+        <v>1246</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>-1734</v>
+        <v>1734</v>
       </c>
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
@@ -755,7 +755,7 @@
         <v>0</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>1793</v>
+        <v>-1793</v>
       </c>
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
@@ -771,43 +771,43 @@
         </is>
       </c>
       <c r="B10" s="6">
-        <f>B6+SUM(B7:B9)</f>
+        <f>B6-SUM(B7:B9)</f>
         <v/>
       </c>
       <c r="C10" s="6">
-        <f>C6+SUM(C7:C9)</f>
+        <f>C6-SUM(C7:C9)</f>
         <v/>
       </c>
       <c r="D10" s="6">
-        <f>D6+SUM(D7:D9)</f>
+        <f>D6-SUM(D7:D9)</f>
         <v/>
       </c>
       <c r="E10" s="6">
-        <f>E6+SUM(E7:E9)</f>
+        <f>E6-SUM(E7:E9)</f>
         <v/>
       </c>
       <c r="F10" s="7">
-        <f>F6+SUM(F7:F9)</f>
+        <f>F6-SUM(F7:F9)</f>
         <v/>
       </c>
       <c r="G10" s="7">
-        <f>G6+SUM(G7:G9)</f>
+        <f>G6-SUM(G7:G9)</f>
         <v/>
       </c>
       <c r="H10" s="7">
-        <f>H6+SUM(H7:H9)</f>
+        <f>H6-SUM(H7:H9)</f>
         <v/>
       </c>
       <c r="I10" s="7">
-        <f>I6+SUM(I7:I9)</f>
+        <f>I6-SUM(I7:I9)</f>
         <v/>
       </c>
       <c r="J10" s="7">
-        <f>J6+SUM(J7:J9)</f>
+        <f>J6-SUM(J7:J9)</f>
         <v/>
       </c>
       <c r="K10" s="7">
-        <f>K6+SUM(K7:K9)</f>
+        <f>K6-SUM(K7:K9)</f>
         <v/>
       </c>
     </row>
@@ -818,16 +818,16 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>7996</v>
+        <v>-7996</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>-34618</v>
+        <v>34618</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>-64948</v>
+        <v>64948</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>-49976</v>
+        <v>49976</v>
       </c>
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
@@ -843,43 +843,43 @@
         </is>
       </c>
       <c r="B12" s="6">
-        <f>B10+B11</f>
+        <f>B10-B11</f>
         <v/>
       </c>
       <c r="C12" s="6">
-        <f>C10+C11</f>
+        <f>C10-C11</f>
         <v/>
       </c>
       <c r="D12" s="6">
-        <f>D10+D11</f>
+        <f>D10-D11</f>
         <v/>
       </c>
       <c r="E12" s="6">
-        <f>E10+E11</f>
+        <f>E10-E11</f>
         <v/>
       </c>
       <c r="F12" s="7">
-        <f>F10+F11</f>
+        <f>F10-F11</f>
         <v/>
       </c>
       <c r="G12" s="7">
-        <f>G10+G11</f>
+        <f>G10-G11</f>
         <v/>
       </c>
       <c r="H12" s="7">
-        <f>H10+H11</f>
+        <f>H10-H11</f>
         <v/>
       </c>
       <c r="I12" s="7">
-        <f>I10+I11</f>
+        <f>I10-I11</f>
         <v/>
       </c>
       <c r="J12" s="7">
-        <f>J10+J11</f>
+        <f>J10-J11</f>
         <v/>
       </c>
       <c r="K12" s="7">
-        <f>K10+K11</f>
+        <f>K10-K11</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 15:59:00
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -1157,17 +1157,17 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Accounts Receivable</t>
+          <t>Restricted Cash</t>
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>63311</v>
+        <v>38768</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>183703</v>
+        <v>0</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>270342</v>
+        <v>0</v>
       </c>
       <c r="E3" s="5" t="n"/>
       <c r="F3" s="5" t="n"/>
@@ -1179,17 +1179,17 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Note Receivable - Current</t>
+          <t>Accounts Receivable</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>6553</v>
+        <v>63311</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>2318</v>
+        <v>183703</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>0</v>
+        <v>270342</v>
       </c>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
@@ -1201,17 +1201,17 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Inventories</t>
+          <t>Note Receivable - Current</t>
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>173289</v>
+        <v>6553</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>229275</v>
+        <v>2318</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>131165</v>
+        <v>0</v>
       </c>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
@@ -1223,17 +1223,17 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Deferred Other Costs - Current</t>
+          <t>Inventories</t>
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>14124</v>
+        <v>173289</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>14124</v>
+        <v>229275</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>14124</v>
+        <v>131165</v>
       </c>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
@@ -1245,17 +1245,17 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Prepaid Expenses</t>
+          <t>Deferred Other Costs - Current</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>11341</v>
+        <v>14124</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>19503</v>
+        <v>14124</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>18759</v>
+        <v>14124</v>
       </c>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
@@ -1267,17 +1267,17 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Restricted Cash</t>
+          <t>Prepaid Expenses</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>38768</v>
+        <v>11341</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>0</v>
+        <v>19503</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>0</v>
+        <v>18759</v>
       </c>
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
@@ -1617,17 +1617,17 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Accrued Promotional Allowance</t>
+          <t>Accrued Distributor Termination Fees</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>35977</v>
+        <v>3986</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>99787</v>
+        <v>0</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>135948</v>
+        <v>0</v>
       </c>
       <c r="E22" s="5" t="n"/>
       <c r="F22" s="5" t="n"/>
@@ -1639,17 +1639,17 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Operating - Current</t>
+          <t>Accrued Promotional Allowance</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>987</v>
+        <v>35977</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>980</v>
+        <v>99787</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>3265</v>
+        <v>135948</v>
       </c>
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n"/>
@@ -1661,17 +1661,17 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Finance - Current</t>
+          <t>Lease Liability - Operating - Current</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>232</v>
+        <v>987</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>59</v>
+        <v>980</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>100</v>
+        <v>3265</v>
       </c>
       <c r="E24" s="5" t="n"/>
       <c r="F24" s="5" t="n"/>
@@ -1683,17 +1683,17 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Deferred Revenue - Current</t>
+          <t>Lease Liability - Finance - Current</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>9675</v>
+        <v>232</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>9513</v>
+        <v>59</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>9513</v>
+        <v>100</v>
       </c>
       <c r="E25" s="5" t="n"/>
       <c r="F25" s="5" t="n"/>
@@ -1705,17 +1705,17 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Other Current Liabilities</t>
+          <t>Deferred Revenue - Current</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>3586</v>
+        <v>9675</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>10890</v>
+        <v>9513</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>15808</v>
+        <v>9513</v>
       </c>
       <c r="E26" s="5" t="n"/>
       <c r="F26" s="5" t="n"/>
@@ -1727,17 +1727,17 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Accrued Distributor Termination Fees</t>
+          <t>Other Current Liabilities</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>3986</v>
+        <v>3586</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>0</v>
+        <v>10890</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>0</v>
+        <v>15808</v>
       </c>
       <c r="E27" s="5" t="n"/>
       <c r="F27" s="5" t="n"/>
@@ -2449,11 +2449,11 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Other Operating Items</t>
+          <t>Gain (Loss) on Lease Cancellations</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>0</v>
+        <v>-28</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>0</v>
@@ -2462,7 +2462,7 @@
         <v>0</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>-324</v>
+        <v>0</v>
       </c>
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
@@ -2474,20 +2474,20 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Accounts Receivable</t>
+          <t>Other Operating Items</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>-25249</v>
+        <v>0</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>-26369</v>
+        <v>0</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>-121558</v>
+        <v>0</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>-89665</v>
+        <v>-324</v>
       </c>
       <c r="F13" s="5" t="n"/>
       <c r="G13" s="5" t="n"/>
@@ -2499,20 +2499,20 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Note Receivable</t>
+          <t>Accounts Receivable</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>0</v>
+        <v>-25249</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>0</v>
+        <v>-26369</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>0</v>
+        <v>-121558</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>2318</v>
+        <v>-89665</v>
       </c>
       <c r="F14" s="5" t="n"/>
       <c r="G14" s="5" t="n"/>
@@ -2524,20 +2524,20 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Inventories</t>
+          <t>Note Receivable</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>-175174</v>
+        <v>0</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>11802</v>
+        <v>0</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>-63299</v>
+        <v>0</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>77190</v>
+        <v>2318</v>
       </c>
       <c r="F15" s="5" t="n"/>
       <c r="G15" s="5" t="n"/>
@@ -2549,20 +2549,20 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Prepaid Expenses</t>
+          <t>Inventories</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>1072</v>
+        <v>-175174</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>2214</v>
+        <v>11802</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>-7980</v>
+        <v>-63299</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>1074</v>
+        <v>77190</v>
       </c>
       <c r="F16" s="5" t="n"/>
       <c r="G16" s="5" t="n"/>
@@ -2574,20 +2574,20 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Accounts Payable</t>
+          <t>Prepaid Expenses</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>23966</v>
+        <v>1072</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>428</v>
+        <v>2214</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>5249</v>
+        <v>-7980</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>-1170</v>
+        <v>1074</v>
       </c>
       <c r="F17" s="5" t="n"/>
       <c r="G17" s="5" t="n"/>
@@ -2599,20 +2599,20 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Accrued Expenses</t>
+          <t>Accounts Payable</t>
         </is>
       </c>
       <c r="B18" s="4" t="n">
-        <v>26484</v>
+        <v>23966</v>
       </c>
       <c r="C18" s="4" t="n">
-        <v>34644</v>
+        <v>428</v>
       </c>
       <c r="D18" s="4" t="n">
-        <v>-8025</v>
+        <v>5249</v>
       </c>
       <c r="E18" s="4" t="n">
-        <v>85398</v>
+        <v>-1170</v>
       </c>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="5" t="n"/>
@@ -2624,20 +2624,20 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Other Current Liabilities</t>
+          <t>Accrued Expenses</t>
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>1731</v>
+        <v>26484</v>
       </c>
       <c r="C19" s="4" t="n">
-        <v>2446</v>
+        <v>34644</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>55407</v>
+        <v>-8025</v>
       </c>
       <c r="E19" s="4" t="n">
-        <v>-34616</v>
+        <v>85398</v>
       </c>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="5" t="n"/>
@@ -2649,20 +2649,20 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Accrued Promotional Allowance</t>
+          <t>Other Current Liabilities</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>13379</v>
+        <v>1731</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>16940</v>
+        <v>2446</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>63810</v>
+        <v>55407</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>36161</v>
+        <v>-34616</v>
       </c>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="5" t="n"/>
@@ -2674,20 +2674,20 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Accrued Distributor Termination</t>
+          <t>Accrued Promotional Allowance</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>0</v>
+        <v>13379</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>3986</v>
+        <v>16940</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>-3739</v>
+        <v>63810</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>-248</v>
+        <v>36161</v>
       </c>
       <c r="F21" s="5" t="n"/>
       <c r="G21" s="5" t="n"/>
@@ -2699,20 +2699,20 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>ROU &amp; Lease Liability, Net</t>
+          <t>Accrued Distributor Termination</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>-183</v>
+        <v>3986</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>-102</v>
+        <v>-3739</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>535</v>
+        <v>-248</v>
       </c>
       <c r="F22" s="5" t="n"/>
       <c r="G22" s="5" t="n"/>
@@ -2724,20 +2724,20 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Deferred Revenue</t>
+          <t>ROU &amp; Lease Liability, Net</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>189463</v>
+        <v>-183</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>-12723</v>
+        <v>-102</v>
       </c>
       <c r="E23" s="4" t="n">
-        <v>-9513</v>
+        <v>535</v>
       </c>
       <c r="F23" s="5" t="n"/>
       <c r="G23" s="5" t="n"/>
@@ -2749,20 +2749,20 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Other Non-Current Assets</t>
+          <t>Deferred Revenue</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>37</v>
+        <v>189463</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>-28</v>
+        <v>-12723</v>
       </c>
       <c r="E24" s="4" t="n">
-        <v>-4862</v>
+        <v>-9513</v>
       </c>
       <c r="F24" s="5" t="n"/>
       <c r="G24" s="5" t="n"/>
@@ -2774,92 +2774,92 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow from Operations</t>
-        </is>
-      </c>
-      <c r="B25" s="6">
-        <f>SUM(B2:B24)</f>
-        <v/>
-      </c>
-      <c r="C25" s="6">
-        <f>SUM(C2:C24)</f>
-        <v/>
-      </c>
-      <c r="D25" s="6">
-        <f>SUM(D2:D24)</f>
-        <v/>
-      </c>
-      <c r="E25" s="6">
-        <f>SUM(E2:E24)</f>
-        <v/>
-      </c>
-      <c r="F25" s="7">
-        <f>SUM(F2:F24)</f>
-        <v/>
-      </c>
-      <c r="G25" s="7">
-        <f>SUM(G2:G24)</f>
-        <v/>
-      </c>
-      <c r="H25" s="7">
-        <f>SUM(H2:H24)</f>
-        <v/>
-      </c>
-      <c r="I25" s="7">
-        <f>SUM(I2:I24)</f>
-        <v/>
-      </c>
-      <c r="J25" s="7">
-        <f>SUM(J2:J24)</f>
-        <v/>
-      </c>
-      <c r="K25" s="7">
-        <f>SUM(K2:K24)</f>
-        <v/>
-      </c>
+          <t>Other Non-Current Assets</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>-28</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>-4862</v>
+      </c>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="5" t="n"/>
+      <c r="I25" s="5" t="n"/>
+      <c r="J25" s="5" t="n"/>
+      <c r="K25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Collections from Note Receivable</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="n">
-        <v>1886</v>
-      </c>
-      <c r="C26" s="4" t="n">
-        <v>2592</v>
-      </c>
-      <c r="D26" s="4" t="n">
-        <v>3233</v>
-      </c>
-      <c r="E26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="5" t="n"/>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="5" t="n"/>
-      <c r="I26" s="5" t="n"/>
-      <c r="J26" s="5" t="n"/>
-      <c r="K26" s="5" t="n"/>
+          <t>Cash Flow from Operations</t>
+        </is>
+      </c>
+      <c r="B26" s="6">
+        <f>SUM(B2:B25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="6">
+        <f>SUM(C2:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="6">
+        <f>SUM(D2:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="6">
+        <f>SUM(E2:E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="7">
+        <f>SUM(F2:F25)</f>
+        <v/>
+      </c>
+      <c r="G26" s="7">
+        <f>SUM(G2:G25)</f>
+        <v/>
+      </c>
+      <c r="H26" s="7">
+        <f>SUM(H2:H25)</f>
+        <v/>
+      </c>
+      <c r="I26" s="7">
+        <f>SUM(I2:I25)</f>
+        <v/>
+      </c>
+      <c r="J26" s="7">
+        <f>SUM(J2:J25)</f>
+        <v/>
+      </c>
+      <c r="K26" s="7">
+        <f>SUM(K2:K25)</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Purchase of PP&amp;E</t>
+          <t>Collections from Note Receivable</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>-3150</v>
+        <v>1886</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>-8264</v>
+        <v>2592</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>-17433</v>
+        <v>3233</v>
       </c>
       <c r="E27" s="4" t="n">
-        <v>-23390</v>
+        <v>0</v>
       </c>
       <c r="F27" s="5" t="n"/>
       <c r="G27" s="5" t="n"/>
@@ -2871,20 +2871,20 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Purchase of Non-Marketable Equity Securities</t>
+          <t>Purchase of PP&amp;E</t>
         </is>
       </c>
       <c r="B28" s="4" t="n">
-        <v>0</v>
+        <v>-3150</v>
       </c>
       <c r="C28" s="4" t="n">
-        <v>0</v>
+        <v>-8264</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>0</v>
+        <v>-17433</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>-3000</v>
+        <v>-23390</v>
       </c>
       <c r="F28" s="5" t="n"/>
       <c r="G28" s="5" t="n"/>
@@ -2896,7 +2896,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Acquisition of Big Beverages</t>
+          <t>Purchase of Non-Marketable Equity Securities</t>
         </is>
       </c>
       <c r="B29" s="4" t="n">
@@ -2909,7 +2909,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>-75336</v>
+        <v>-3000</v>
       </c>
       <c r="F29" s="5" t="n"/>
       <c r="G29" s="5" t="n"/>
@@ -2921,92 +2921,92 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow from Investing</t>
-        </is>
-      </c>
-      <c r="B30" s="6">
-        <f>SUM(B26:B29)</f>
-        <v/>
-      </c>
-      <c r="C30" s="6">
-        <f>SUM(C26:C29)</f>
-        <v/>
-      </c>
-      <c r="D30" s="6">
-        <f>SUM(D26:D29)</f>
-        <v/>
-      </c>
-      <c r="E30" s="6">
-        <f>SUM(E26:E29)</f>
-        <v/>
-      </c>
-      <c r="F30" s="7">
-        <f>SUM(F26:F29)</f>
-        <v/>
-      </c>
-      <c r="G30" s="7">
-        <f>SUM(G26:G29)</f>
-        <v/>
-      </c>
-      <c r="H30" s="7">
-        <f>SUM(H26:H29)</f>
-        <v/>
-      </c>
-      <c r="I30" s="7">
-        <f>SUM(I26:I29)</f>
-        <v/>
-      </c>
-      <c r="J30" s="7">
-        <f>SUM(J26:J29)</f>
-        <v/>
-      </c>
-      <c r="K30" s="7">
-        <f>SUM(K26:K29)</f>
-        <v/>
-      </c>
+          <t>Acquisition of Big Beverages</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>-75336</v>
+      </c>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+      <c r="H30" s="5" t="n"/>
+      <c r="I30" s="5" t="n"/>
+      <c r="J30" s="5" t="n"/>
+      <c r="K30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Finance Lease Payments</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="n">
-        <v>-94</v>
-      </c>
-      <c r="C31" s="4" t="n">
-        <v>-63</v>
-      </c>
-      <c r="D31" s="4" t="n">
-        <v>-44</v>
-      </c>
-      <c r="E31" s="4" t="n">
-        <v>-61</v>
-      </c>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="5" t="n"/>
-      <c r="I31" s="5" t="n"/>
-      <c r="J31" s="5" t="n"/>
-      <c r="K31" s="5" t="n"/>
+          <t>Cash Flow from Investing</t>
+        </is>
+      </c>
+      <c r="B31" s="6">
+        <f>SUM(B27:B30)</f>
+        <v/>
+      </c>
+      <c r="C31" s="6">
+        <f>SUM(C27:C30)</f>
+        <v/>
+      </c>
+      <c r="D31" s="6">
+        <f>SUM(D27:D30)</f>
+        <v/>
+      </c>
+      <c r="E31" s="6">
+        <f>SUM(E27:E30)</f>
+        <v/>
+      </c>
+      <c r="F31" s="7">
+        <f>SUM(F27:F30)</f>
+        <v/>
+      </c>
+      <c r="G31" s="7">
+        <f>SUM(G27:G30)</f>
+        <v/>
+      </c>
+      <c r="H31" s="7">
+        <f>SUM(H27:H30)</f>
+        <v/>
+      </c>
+      <c r="I31" s="7">
+        <f>SUM(I27:I30)</f>
+        <v/>
+      </c>
+      <c r="J31" s="7">
+        <f>SUM(J27:J30)</f>
+        <v/>
+      </c>
+      <c r="K31" s="7">
+        <f>SUM(K27:K30)</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Exercise of Stock Options</t>
+          <t>Finance Lease Payments</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>3720</v>
+        <v>-94</v>
       </c>
       <c r="C32" s="4" t="n">
-        <v>3683</v>
+        <v>-63</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>2285</v>
+        <v>-44</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>3856</v>
+        <v>-61</v>
       </c>
       <c r="F32" s="5" t="n"/>
       <c r="G32" s="5" t="n"/>
@@ -3018,20 +3018,20 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Issuance of Preferred Stock</t>
+          <t>Proceeds from Exercise of Stock Options</t>
         </is>
       </c>
       <c r="B33" s="4" t="n">
-        <v>0</v>
+        <v>3720</v>
       </c>
       <c r="C33" s="4" t="n">
-        <v>542018</v>
+        <v>3683</v>
       </c>
       <c r="D33" s="4" t="n">
-        <v>0</v>
+        <v>2285</v>
       </c>
       <c r="E33" s="4" t="n">
-        <v>0</v>
+        <v>3856</v>
       </c>
       <c r="F33" s="5" t="n"/>
       <c r="G33" s="5" t="n"/>
@@ -3043,20 +3043,20 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Dividends Paid</t>
+          <t>Proceeds from Issuance of Preferred Stock</t>
         </is>
       </c>
       <c r="B34" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C34" s="4" t="n">
-        <v>-11526</v>
+        <v>542018</v>
       </c>
       <c r="D34" s="4" t="n">
-        <v>-27462</v>
+        <v>0</v>
       </c>
       <c r="E34" s="4" t="n">
-        <v>-27500</v>
+        <v>0</v>
       </c>
       <c r="F34" s="5" t="n"/>
       <c r="G34" s="5" t="n"/>
@@ -3068,20 +3068,20 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Share Repurchases</t>
+          <t>Dividends Paid</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C35" s="4" t="n">
-        <v>0</v>
+        <v>-11526</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>0</v>
+        <v>-27462</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>-2261</v>
+        <v>-27500</v>
       </c>
       <c r="F35" s="5" t="n"/>
       <c r="G35" s="5" t="n"/>
@@ -3093,67 +3093,45 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Cash Flow from Financing</t>
-        </is>
-      </c>
-      <c r="B36" s="6">
-        <f>SUM(B31:B35)</f>
-        <v/>
-      </c>
-      <c r="C36" s="6">
-        <f>SUM(C31:C35)</f>
-        <v/>
-      </c>
-      <c r="D36" s="6">
-        <f>SUM(D31:D35)</f>
-        <v/>
-      </c>
-      <c r="E36" s="6">
-        <f>SUM(E31:E35)</f>
-        <v/>
-      </c>
-      <c r="F36" s="7">
-        <f>SUM(F31:F35)</f>
-        <v/>
-      </c>
-      <c r="G36" s="7">
-        <f>SUM(G31:G35)</f>
-        <v/>
-      </c>
-      <c r="H36" s="7">
-        <f>SUM(H31:H35)</f>
-        <v/>
-      </c>
-      <c r="I36" s="7">
-        <f>SUM(I31:I35)</f>
-        <v/>
-      </c>
-      <c r="J36" s="7">
-        <f>SUM(J31:J35)</f>
-        <v/>
-      </c>
-      <c r="K36" s="7">
-        <f>SUM(K31:K35)</f>
-        <v/>
-      </c>
+          <t>Proceeds from Issuance of Common Stock</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>67769</v>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="5" t="n"/>
+      <c r="G36" s="5" t="n"/>
+      <c r="H36" s="5" t="n"/>
+      <c r="I36" s="5" t="n"/>
+      <c r="J36" s="5" t="n"/>
+      <c r="K36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>FX Effect on Cash</t>
+          <t>Share Repurchases</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>-538</v>
+        <v>0</v>
       </c>
       <c r="C37" s="4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>1257</v>
+        <v>0</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>-997</v>
+        <v>-2261</v>
       </c>
       <c r="F37" s="5" t="n"/>
       <c r="G37" s="5" t="n"/>
@@ -3165,45 +3143,67 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Net Change in Cash</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="n">
-        <v>-26993</v>
-      </c>
-      <c r="C38" s="4" t="n">
-        <v>636672</v>
-      </c>
-      <c r="D38" s="4" t="n">
-        <v>103054</v>
-      </c>
-      <c r="E38" s="4" t="n">
-        <v>134209</v>
-      </c>
-      <c r="F38" s="5" t="n"/>
-      <c r="G38" s="5" t="n"/>
-      <c r="H38" s="5" t="n"/>
-      <c r="I38" s="5" t="n"/>
-      <c r="J38" s="5" t="n"/>
-      <c r="K38" s="5" t="n"/>
+          <t>Cash Flow from Financing</t>
+        </is>
+      </c>
+      <c r="B38" s="6">
+        <f>SUM(B32:B37)</f>
+        <v/>
+      </c>
+      <c r="C38" s="6">
+        <f>SUM(C32:C37)</f>
+        <v/>
+      </c>
+      <c r="D38" s="6">
+        <f>SUM(D32:D37)</f>
+        <v/>
+      </c>
+      <c r="E38" s="6">
+        <f>SUM(E32:E37)</f>
+        <v/>
+      </c>
+      <c r="F38" s="7">
+        <f>SUM(F32:F37)</f>
+        <v/>
+      </c>
+      <c r="G38" s="7">
+        <f>SUM(G32:G37)</f>
+        <v/>
+      </c>
+      <c r="H38" s="7">
+        <f>SUM(H32:H37)</f>
+        <v/>
+      </c>
+      <c r="I38" s="7">
+        <f>SUM(I32:I37)</f>
+        <v/>
+      </c>
+      <c r="J38" s="7">
+        <f>SUM(J32:J37)</f>
+        <v/>
+      </c>
+      <c r="K38" s="7">
+        <f>SUM(K32:K37)</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Cash at Beginning of Period</t>
+          <t>FX Effect on Cash</t>
         </is>
       </c>
       <c r="B39" s="4" t="n">
-        <v>43248</v>
+        <v>-538</v>
       </c>
       <c r="C39" s="4" t="n">
-        <v>16255</v>
+        <v>50</v>
       </c>
       <c r="D39" s="4" t="n">
-        <v>652927</v>
+        <v>1257</v>
       </c>
       <c r="E39" s="4" t="n">
-        <v>755981</v>
+        <v>-997</v>
       </c>
       <c r="F39" s="5" t="n"/>
       <c r="G39" s="5" t="n"/>
@@ -3215,20 +3215,20 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Cash at End of Period</t>
+          <t>Net Change in Cash</t>
         </is>
       </c>
       <c r="B40" s="4" t="n">
-        <v>16255</v>
+        <v>-26993</v>
       </c>
       <c r="C40" s="4" t="n">
-        <v>652927</v>
+        <v>636672</v>
       </c>
       <c r="D40" s="4" t="n">
-        <v>755981</v>
+        <v>103054</v>
       </c>
       <c r="E40" s="4" t="n">
-        <v>890190</v>
+        <v>134209</v>
       </c>
       <c r="F40" s="5" t="n"/>
       <c r="G40" s="5" t="n"/>
@@ -3240,20 +3240,20 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>Gain (Loss) on Lease Cancellations</t>
+          <t>Cash at Beginning of Period</t>
         </is>
       </c>
       <c r="B41" s="4" t="n">
-        <v>-28</v>
+        <v>43248</v>
       </c>
       <c r="C41" s="4" t="n">
-        <v>0</v>
+        <v>16255</v>
       </c>
       <c r="D41" s="4" t="n">
-        <v>0</v>
+        <v>652927</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>0</v>
+        <v>755981</v>
       </c>
       <c r="F41" s="5" t="n"/>
       <c r="G41" s="5" t="n"/>
@@ -3265,20 +3265,20 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Proceeds from Issuance of Common Stock</t>
+          <t>Cash at End of Period</t>
         </is>
       </c>
       <c r="B42" s="4" t="n">
-        <v>67769</v>
+        <v>16255</v>
       </c>
       <c r="C42" s="4" t="n">
-        <v>0</v>
+        <v>652927</v>
       </c>
       <c r="D42" s="4" t="n">
-        <v>0</v>
+        <v>755981</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>0</v>
+        <v>890190</v>
       </c>
       <c r="F42" s="5" t="n"/>
       <c r="G42" s="5" t="n"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 16:04:10
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -1069,7 +1069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1205,7 +1205,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>6553</v>
+        <v>2979</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>2318</v>
@@ -1332,17 +1332,17 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Net PP&amp;E</t>
+          <t>Note Receivable - Non-Current</t>
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>10185</v>
+        <v>3574</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>24868</v>
+        <v>0</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>55602</v>
+        <v>0</v>
       </c>
       <c r="E10" s="5" t="n"/>
       <c r="F10" s="5" t="n"/>
@@ -1354,17 +1354,17 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>ROU Assets - Operating - Non-Current</t>
+          <t>Net PP&amp;E</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>972</v>
+        <v>10185</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>1957</v>
+        <v>24868</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>21606</v>
+        <v>55602</v>
       </c>
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
@@ -1376,17 +1376,17 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>ROU Assets - Finance - Non-Current</t>
+          <t>ROU Assets - Operating - Non-Current</t>
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>208</v>
+        <v>972</v>
       </c>
       <c r="C12" s="4" t="n">
-        <v>208</v>
+        <v>1957</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>230</v>
+        <v>21606</v>
       </c>
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="n"/>
@@ -1398,17 +1398,17 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Intangible Assets</t>
+          <t>ROU Assets - Finance - Non-Current</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>12254</v>
+        <v>208</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>12139</v>
+        <v>208</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>12213</v>
+        <v>230</v>
       </c>
       <c r="E13" s="5" t="n"/>
       <c r="F13" s="5" t="n"/>
@@ -1420,17 +1420,17 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Goodwill</t>
+          <t>Intangible Assets</t>
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>13679</v>
+        <v>12254</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>14173</v>
+        <v>12139</v>
       </c>
       <c r="D14" s="4" t="n">
-        <v>71582</v>
+        <v>12213</v>
       </c>
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
@@ -1442,17 +1442,17 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Deferred Other Costs - Non-Current</t>
+          <t>Goodwill</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>262462</v>
+        <v>13679</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>248338</v>
+        <v>14173</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>234215</v>
+        <v>71582</v>
       </c>
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="n"/>
@@ -1464,17 +1464,17 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Deferred Tax Assets</t>
+          <t>Deferred Other Costs - Non-Current</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>501</v>
+        <v>262462</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>29518</v>
+        <v>248338</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>38699</v>
+        <v>234215</v>
       </c>
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
@@ -1486,17 +1486,17 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Other Non-Current Assets</t>
+          <t>Deferred Tax Assets</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>263</v>
+        <v>501</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>291</v>
+        <v>29518</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>8154</v>
+        <v>38699</v>
       </c>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
@@ -1508,82 +1508,82 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Total Assets</t>
-        </is>
-      </c>
-      <c r="B18" s="6">
-        <f>B9+SUM(B10:B17)</f>
-        <v/>
-      </c>
-      <c r="C18" s="6">
-        <f>C9+SUM(C10:C17)</f>
-        <v/>
-      </c>
-      <c r="D18" s="6">
-        <f>D9+SUM(D10:D17)</f>
-        <v/>
-      </c>
-      <c r="E18" s="7">
-        <f>E9+SUM(E10:E17)</f>
-        <v/>
-      </c>
-      <c r="F18" s="7">
-        <f>F9+SUM(F10:F17)</f>
-        <v/>
-      </c>
-      <c r="G18" s="7">
-        <f>G9+SUM(G10:G17)</f>
-        <v/>
-      </c>
-      <c r="H18" s="7">
-        <f>H9+SUM(H10:H17)</f>
-        <v/>
-      </c>
-      <c r="I18" s="7">
-        <f>I9+SUM(I10:I17)</f>
-        <v/>
-      </c>
-      <c r="J18" s="7">
-        <f>J9+SUM(J10:J17)</f>
-        <v/>
-      </c>
+          <t>Other Non-Current Assets</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>263</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>291</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>8154</v>
+      </c>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="n"/>
+      <c r="J18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Accounts Payable</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="n">
-        <v>36248</v>
-      </c>
-      <c r="C19" s="4" t="n">
-        <v>42840</v>
-      </c>
-      <c r="D19" s="4" t="n">
-        <v>41287</v>
-      </c>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="n"/>
-      <c r="I19" s="5" t="n"/>
-      <c r="J19" s="5" t="n"/>
+          <t>Total Assets</t>
+        </is>
+      </c>
+      <c r="B19" s="6">
+        <f>B9+SUM(B10:B18)</f>
+        <v/>
+      </c>
+      <c r="C19" s="6">
+        <f>C9+SUM(C10:C18)</f>
+        <v/>
+      </c>
+      <c r="D19" s="6">
+        <f>D9+SUM(D10:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="7">
+        <f>E9+SUM(E10:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="7">
+        <f>F9+SUM(F10:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="7">
+        <f>G9+SUM(G10:G18)</f>
+        <v/>
+      </c>
+      <c r="H19" s="7">
+        <f>H9+SUM(H10:H18)</f>
+        <v/>
+      </c>
+      <c r="I19" s="7">
+        <f>I9+SUM(I10:I18)</f>
+        <v/>
+      </c>
+      <c r="J19" s="7">
+        <f>J9+SUM(J10:J18)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Accrued Expenses</t>
+          <t>Accounts Payable</t>
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>69899</v>
+        <v>36248</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>62120</v>
+        <v>42840</v>
       </c>
       <c r="D20" s="4" t="n">
-        <v>148780</v>
+        <v>41287</v>
       </c>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
@@ -1595,17 +1595,17 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Income Taxes Payable</t>
+          <t>Accrued Expenses</t>
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>1193</v>
+        <v>69899</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>50424</v>
+        <v>62120</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>10834</v>
+        <v>148780</v>
       </c>
       <c r="E21" s="5" t="n"/>
       <c r="F21" s="5" t="n"/>
@@ -1617,17 +1617,17 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Accrued Distributor Termination Fees</t>
+          <t>Income Taxes Payable</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>3986</v>
+        <v>1193</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>0</v>
+        <v>50424</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>0</v>
+        <v>10834</v>
       </c>
       <c r="E22" s="5" t="n"/>
       <c r="F22" s="5" t="n"/>
@@ -1639,17 +1639,17 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Accrued Promotional Allowance</t>
+          <t>Accrued Distributor Termination Fees</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>35977</v>
+        <v>3986</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>99787</v>
+        <v>0</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>135948</v>
+        <v>0</v>
       </c>
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n"/>
@@ -1661,17 +1661,17 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Operating - Current</t>
+          <t>Accrued Promotional Allowance</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>987</v>
+        <v>35977</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>980</v>
+        <v>99787</v>
       </c>
       <c r="D24" s="4" t="n">
-        <v>3265</v>
+        <v>135948</v>
       </c>
       <c r="E24" s="5" t="n"/>
       <c r="F24" s="5" t="n"/>
@@ -1683,17 +1683,17 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Finance - Current</t>
+          <t>Lease Liability - Operating - Current</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>232</v>
+        <v>661</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>59</v>
+        <v>980</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>100</v>
+        <v>3265</v>
       </c>
       <c r="E25" s="5" t="n"/>
       <c r="F25" s="5" t="n"/>
@@ -1705,17 +1705,17 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Deferred Revenue - Current</t>
+          <t>Lease Liability - Finance - Current</t>
         </is>
       </c>
       <c r="B26" s="4" t="n">
-        <v>9675</v>
+        <v>70</v>
       </c>
       <c r="C26" s="4" t="n">
-        <v>9513</v>
+        <v>59</v>
       </c>
       <c r="D26" s="4" t="n">
-        <v>9513</v>
+        <v>100</v>
       </c>
       <c r="E26" s="5" t="n"/>
       <c r="F26" s="5" t="n"/>
@@ -1727,17 +1727,17 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>Other Current Liabilities</t>
+          <t>Deferred Revenue - Current</t>
         </is>
       </c>
       <c r="B27" s="4" t="n">
-        <v>3586</v>
+        <v>9675</v>
       </c>
       <c r="C27" s="4" t="n">
-        <v>10890</v>
+        <v>9513</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>15808</v>
+        <v>9513</v>
       </c>
       <c r="E27" s="5" t="n"/>
       <c r="F27" s="5" t="n"/>
@@ -1749,82 +1749,82 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Total Current Liabilities</t>
-        </is>
-      </c>
-      <c r="B28" s="6">
-        <f>SUM(B19:B27)</f>
-        <v/>
-      </c>
-      <c r="C28" s="6">
-        <f>SUM(C19:C27)</f>
-        <v/>
-      </c>
-      <c r="D28" s="6">
-        <f>SUM(D19:D27)</f>
-        <v/>
-      </c>
-      <c r="E28" s="7">
-        <f>SUM(E19:E27)</f>
-        <v/>
-      </c>
-      <c r="F28" s="7">
-        <f>SUM(F19:F27)</f>
-        <v/>
-      </c>
-      <c r="G28" s="7">
-        <f>SUM(G19:G27)</f>
-        <v/>
-      </c>
-      <c r="H28" s="7">
-        <f>SUM(H19:H27)</f>
-        <v/>
-      </c>
-      <c r="I28" s="7">
-        <f>SUM(I19:I27)</f>
-        <v/>
-      </c>
-      <c r="J28" s="7">
-        <f>SUM(J19:J27)</f>
-        <v/>
-      </c>
+          <t>Other Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>3586</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>10890</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>15808</v>
+      </c>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
+      <c r="G28" s="5" t="n"/>
+      <c r="H28" s="5" t="n"/>
+      <c r="I28" s="5" t="n"/>
+      <c r="J28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Operating - Non-Current</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="C29" s="4" t="n">
-        <v>955</v>
-      </c>
-      <c r="D29" s="4" t="n">
-        <v>16674</v>
-      </c>
-      <c r="E29" s="5" t="n"/>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="5" t="n"/>
-      <c r="I29" s="5" t="n"/>
-      <c r="J29" s="5" t="n"/>
+          <t>Total Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B29" s="6">
+        <f>SUM(B20:B28)</f>
+        <v/>
+      </c>
+      <c r="C29" s="6">
+        <f>SUM(C20:C28)</f>
+        <v/>
+      </c>
+      <c r="D29" s="6">
+        <f>SUM(D20:D28)</f>
+        <v/>
+      </c>
+      <c r="E29" s="7">
+        <f>SUM(E20:E28)</f>
+        <v/>
+      </c>
+      <c r="F29" s="7">
+        <f>SUM(F20:F28)</f>
+        <v/>
+      </c>
+      <c r="G29" s="7">
+        <f>SUM(G20:G28)</f>
+        <v/>
+      </c>
+      <c r="H29" s="7">
+        <f>SUM(H20:H28)</f>
+        <v/>
+      </c>
+      <c r="I29" s="7">
+        <f>SUM(I20:I28)</f>
+        <v/>
+      </c>
+      <c r="J29" s="7">
+        <f>SUM(J20:J28)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Lease Liability - Finance - Non-Current</t>
+          <t>Lease Liability - Operating - Non-Current</t>
         </is>
       </c>
       <c r="B30" s="4" t="n">
-        <v>0</v>
+        <v>326</v>
       </c>
       <c r="C30" s="4" t="n">
-        <v>193</v>
+        <v>955</v>
       </c>
       <c r="D30" s="4" t="n">
-        <v>211</v>
+        <v>16674</v>
       </c>
       <c r="E30" s="5" t="n"/>
       <c r="F30" s="5" t="n"/>
@@ -1836,17 +1836,17 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Deferred Tax Liability</t>
+          <t>Lease Liability - Finance - Non-Current</t>
         </is>
       </c>
       <c r="B31" s="4" t="n">
-        <v>15919</v>
+        <v>162</v>
       </c>
       <c r="C31" s="4" t="n">
-        <v>2880</v>
+        <v>193</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>2330</v>
+        <v>211</v>
       </c>
       <c r="E31" s="5" t="n"/>
       <c r="F31" s="5" t="n"/>
@@ -1858,17 +1858,17 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Deferred Revenue - Non-Current</t>
+          <t>Deferred Tax Liability</t>
         </is>
       </c>
       <c r="B32" s="4" t="n">
-        <v>179788</v>
+        <v>15919</v>
       </c>
       <c r="C32" s="4" t="n">
-        <v>167227</v>
+        <v>2880</v>
       </c>
       <c r="D32" s="4" t="n">
-        <v>157714</v>
+        <v>2330</v>
       </c>
       <c r="E32" s="5" t="n"/>
       <c r="F32" s="5" t="n"/>
@@ -1880,82 +1880,82 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Total Liabilities</t>
-        </is>
-      </c>
-      <c r="B33" s="6">
-        <f>B28+SUM(B29:B32)</f>
-        <v/>
-      </c>
-      <c r="C33" s="6">
-        <f>C28+SUM(C29:C32)</f>
-        <v/>
-      </c>
-      <c r="D33" s="6">
-        <f>D28+SUM(D29:D32)</f>
-        <v/>
-      </c>
-      <c r="E33" s="7">
-        <f>E28+SUM(E29:E32)</f>
-        <v/>
-      </c>
-      <c r="F33" s="7">
-        <f>F28+SUM(F29:F32)</f>
-        <v/>
-      </c>
-      <c r="G33" s="7">
-        <f>G28+SUM(G29:G32)</f>
-        <v/>
-      </c>
-      <c r="H33" s="7">
-        <f>H28+SUM(H29:H32)</f>
-        <v/>
-      </c>
-      <c r="I33" s="7">
-        <f>I28+SUM(I29:I32)</f>
-        <v/>
-      </c>
-      <c r="J33" s="7">
-        <f>J28+SUM(J29:J32)</f>
-        <v/>
-      </c>
+          <t>Deferred Revenue - Non-Current</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>179788</v>
+      </c>
+      <c r="C33" s="4" t="n">
+        <v>167227</v>
+      </c>
+      <c r="D33" s="4" t="n">
+        <v>157714</v>
+      </c>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="n"/>
+      <c r="H33" s="5" t="n"/>
+      <c r="I33" s="5" t="n"/>
+      <c r="J33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Convertible Preferred Stock</t>
-        </is>
-      </c>
-      <c r="B34" s="4" t="n">
-        <v>824488</v>
-      </c>
-      <c r="C34" s="4" t="n">
-        <v>824488</v>
-      </c>
-      <c r="D34" s="4" t="n">
-        <v>824488</v>
-      </c>
-      <c r="E34" s="5" t="n"/>
-      <c r="F34" s="5" t="n"/>
-      <c r="G34" s="5" t="n"/>
-      <c r="H34" s="5" t="n"/>
-      <c r="I34" s="5" t="n"/>
-      <c r="J34" s="5" t="n"/>
+          <t>Total Liabilities</t>
+        </is>
+      </c>
+      <c r="B34" s="6">
+        <f>B29+SUM(B30:B33)</f>
+        <v/>
+      </c>
+      <c r="C34" s="6">
+        <f>C29+SUM(C30:C33)</f>
+        <v/>
+      </c>
+      <c r="D34" s="6">
+        <f>D29+SUM(D30:D33)</f>
+        <v/>
+      </c>
+      <c r="E34" s="7">
+        <f>E29+SUM(E30:E33)</f>
+        <v/>
+      </c>
+      <c r="F34" s="7">
+        <f>F29+SUM(F30:F33)</f>
+        <v/>
+      </c>
+      <c r="G34" s="7">
+        <f>G29+SUM(G30:G33)</f>
+        <v/>
+      </c>
+      <c r="H34" s="7">
+        <f>H29+SUM(H30:H33)</f>
+        <v/>
+      </c>
+      <c r="I34" s="7">
+        <f>I29+SUM(I30:I33)</f>
+        <v/>
+      </c>
+      <c r="J34" s="7">
+        <f>J29+SUM(J30:J33)</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Common Stock</t>
+          <t>Convertible Preferred Stock</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
-        <v>76</v>
+        <v>824488</v>
       </c>
       <c r="C35" s="4" t="n">
-        <v>77</v>
+        <v>824488</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>79</v>
+        <v>824488</v>
       </c>
       <c r="E35" s="5" t="n"/>
       <c r="F35" s="5" t="n"/>
@@ -1967,17 +1967,17 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>Additional Paid-in Capital</t>
+          <t>Common Stock</t>
         </is>
       </c>
       <c r="B36" s="4" t="n">
-        <v>280668</v>
+        <v>76</v>
       </c>
       <c r="C36" s="4" t="n">
-        <v>276717</v>
+        <v>77</v>
       </c>
       <c r="D36" s="4" t="n">
-        <v>297579</v>
+        <v>79</v>
       </c>
       <c r="E36" s="5" t="n"/>
       <c r="F36" s="5" t="n"/>
@@ -1989,17 +1989,17 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>Accumulated Other Comprehensive Income (Loss)</t>
+          <t>Additional Paid-in Capital</t>
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>-1881</v>
+        <v>280668</v>
       </c>
       <c r="C37" s="4" t="n">
-        <v>-701</v>
+        <v>276717</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>-3250</v>
+        <v>297579</v>
       </c>
       <c r="E37" s="5" t="n"/>
       <c r="F37" s="5" t="n"/>
@@ -2011,17 +2011,17 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>Retained Earnings (Accumulated Deficit)</t>
+          <t>Accumulated Other Comprehensive Income (Loss)</t>
         </is>
       </c>
       <c r="B38" s="4" t="n">
-        <v>-238772</v>
+        <v>-1881</v>
       </c>
       <c r="C38" s="4" t="n">
-        <v>-12053</v>
+        <v>-701</v>
       </c>
       <c r="D38" s="4" t="n">
-        <v>105521</v>
+        <v>-3250</v>
       </c>
       <c r="E38" s="5" t="n"/>
       <c r="F38" s="5" t="n"/>
@@ -2033,86 +2033,108 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>Total Stockholders' Equity</t>
-        </is>
-      </c>
-      <c r="B39" s="6">
-        <f>SUM(B35:B38)</f>
-        <v/>
-      </c>
-      <c r="C39" s="6">
-        <f>SUM(C35:C38)</f>
-        <v/>
-      </c>
-      <c r="D39" s="6">
-        <f>SUM(D35:D38)</f>
-        <v/>
-      </c>
-      <c r="E39" s="7">
-        <f>SUM(E35:E38)</f>
-        <v/>
-      </c>
-      <c r="F39" s="7">
-        <f>SUM(F35:F38)</f>
-        <v/>
-      </c>
-      <c r="G39" s="7">
-        <f>SUM(G35:G38)</f>
-        <v/>
-      </c>
-      <c r="H39" s="7">
-        <f>SUM(H35:H38)</f>
-        <v/>
-      </c>
-      <c r="I39" s="7">
-        <f>SUM(I35:I38)</f>
-        <v/>
-      </c>
-      <c r="J39" s="7">
-        <f>SUM(J35:J38)</f>
-        <v/>
-      </c>
+          <t>Retained Earnings (Accumulated Deficit)</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="n">
+        <v>-238772</v>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>-12053</v>
+      </c>
+      <c r="D39" s="4" t="n">
+        <v>105521</v>
+      </c>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="5" t="n"/>
+      <c r="H39" s="5" t="n"/>
+      <c r="I39" s="5" t="n"/>
+      <c r="J39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
+          <t>Total Stockholders' Equity</t>
+        </is>
+      </c>
+      <c r="B40" s="6">
+        <f>SUM(B36:B39)</f>
+        <v/>
+      </c>
+      <c r="C40" s="6">
+        <f>SUM(C36:C39)</f>
+        <v/>
+      </c>
+      <c r="D40" s="6">
+        <f>SUM(D36:D39)</f>
+        <v/>
+      </c>
+      <c r="E40" s="7">
+        <f>SUM(E36:E39)</f>
+        <v/>
+      </c>
+      <c r="F40" s="7">
+        <f>SUM(F36:F39)</f>
+        <v/>
+      </c>
+      <c r="G40" s="7">
+        <f>SUM(G36:G39)</f>
+        <v/>
+      </c>
+      <c r="H40" s="7">
+        <f>SUM(H36:H39)</f>
+        <v/>
+      </c>
+      <c r="I40" s="7">
+        <f>SUM(I36:I39)</f>
+        <v/>
+      </c>
+      <c r="J40" s="7">
+        <f>SUM(J36:J39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
           <t>Total Liabilities, Mezzanine &amp; Stockholders' Equity</t>
         </is>
       </c>
-      <c r="B40" s="6">
-        <f>B33+B34+B39</f>
-        <v/>
-      </c>
-      <c r="C40" s="6">
-        <f>C33+C34+C39</f>
-        <v/>
-      </c>
-      <c r="D40" s="6">
-        <f>D33+D34+D39</f>
-        <v/>
-      </c>
-      <c r="E40" s="7">
-        <f>E33+E34+E39</f>
-        <v/>
-      </c>
-      <c r="F40" s="7">
-        <f>F33+F34+F39</f>
-        <v/>
-      </c>
-      <c r="G40" s="7">
-        <f>G33+G34+G39</f>
-        <v/>
-      </c>
-      <c r="H40" s="7">
-        <f>H33+H34+H39</f>
-        <v/>
-      </c>
-      <c r="I40" s="7">
-        <f>I33+I34+I39</f>
-        <v/>
-      </c>
-      <c r="J40" s="7">
-        <f>J33+J34+J39</f>
+      <c r="B41" s="6">
+        <f>B34+B35+B40</f>
+        <v/>
+      </c>
+      <c r="C41" s="6">
+        <f>C34+C35+C40</f>
+        <v/>
+      </c>
+      <c r="D41" s="6">
+        <f>D34+D35+D40</f>
+        <v/>
+      </c>
+      <c r="E41" s="7">
+        <f>E34+E35+E40</f>
+        <v/>
+      </c>
+      <c r="F41" s="7">
+        <f>F34+F35+F40</f>
+        <v/>
+      </c>
+      <c r="G41" s="7">
+        <f>G34+G35+G40</f>
+        <v/>
+      </c>
+      <c r="H41" s="7">
+        <f>H34+H35+H40</f>
+        <v/>
+      </c>
+      <c r="I41" s="7">
+        <f>I34+I35+I40</f>
+        <v/>
+      </c>
+      <c r="J41" s="7">
+        <f>J34+J35+J40</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 18:57:45
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -10,6 +10,9 @@
     <sheet name="ANNL P&amp;L" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="BALANCE SHEET" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="CASH FLOW" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="IS DRIVERS" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="BS DRIVERS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CF DRIVERS" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,11 +21,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;--&quot;"/>
     <numFmt numFmtId="165" formatCode="$#,##0_);($#,##0);&quot;$--&quot;_)"/>
+    <numFmt numFmtId="166" formatCode="0.0%;(0.0%);&quot;--&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.0;(0.0);&quot;--&quot;"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +42,13 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +65,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
         <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAEAEA"/>
+        <bgColor rgb="00EAEAEA"/>
       </patternFill>
     </fill>
   </fills>
@@ -75,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -86,6 +102,13 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3312,4 +3335,968 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>FY2025E</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Revenue Growth %</t>
+        </is>
+      </c>
+      <c r="C2" s="8">
+        <f>IFERROR(('ANNL P&amp;L'!C2-'ANNL P&amp;L'!B2)/'ANNL P&amp;L'!B2,0)</f>
+        <v/>
+      </c>
+      <c r="D2" s="8">
+        <f>IFERROR(('ANNL P&amp;L'!D2-'ANNL P&amp;L'!C2)/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="E2" s="8">
+        <f>IFERROR(('ANNL P&amp;L'!E2-'ANNL P&amp;L'!D2)/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="F2" s="9" t="n"/>
+      <c r="G2" s="9" t="n"/>
+      <c r="H2" s="9" t="n"/>
+      <c r="I2" s="9" t="n"/>
+      <c r="J2" s="9" t="n"/>
+      <c r="K2" s="9" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>COGS % of Revenue</t>
+        </is>
+      </c>
+      <c r="B3" s="8">
+        <f>IFERROR('ANNL P&amp;L'!B3/'ANNL P&amp;L'!B2,0)</f>
+        <v/>
+      </c>
+      <c r="C3" s="8">
+        <f>IFERROR('ANNL P&amp;L'!C3/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D3" s="8">
+        <f>IFERROR('ANNL P&amp;L'!D3/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E3" s="8">
+        <f>IFERROR('ANNL P&amp;L'!E3/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F3" s="9" t="n"/>
+      <c r="G3" s="9" t="n"/>
+      <c r="H3" s="9" t="n"/>
+      <c r="I3" s="9" t="n"/>
+      <c r="J3" s="9" t="n"/>
+      <c r="K3" s="9" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>SG&amp;A % of Revenue</t>
+        </is>
+      </c>
+      <c r="B4" s="8">
+        <f>IFERROR('ANNL P&amp;L'!B5/'ANNL P&amp;L'!B2,0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="8">
+        <f>IFERROR('ANNL P&amp;L'!C5/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D4" s="8">
+        <f>IFERROR('ANNL P&amp;L'!D5/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E4" s="8">
+        <f>IFERROR('ANNL P&amp;L'!E5/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="9" t="n"/>
+      <c r="H4" s="9" t="n"/>
+      <c r="I4" s="9" t="n"/>
+      <c r="J4" s="9" t="n"/>
+      <c r="K4" s="9" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Interest Income (Expense) $</t>
+        </is>
+      </c>
+      <c r="B5" s="4">
+        <f>'ANNL P&amp;L'!B7</f>
+        <v/>
+      </c>
+      <c r="C5" s="4">
+        <f>'ANNL P&amp;L'!C7</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>'ANNL P&amp;L'!D7</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>'ANNL P&amp;L'!E7</f>
+        <v/>
+      </c>
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="10" t="n"/>
+      <c r="H5" s="10" t="n"/>
+      <c r="I5" s="10" t="n"/>
+      <c r="J5" s="10" t="n"/>
+      <c r="K5" s="10" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>FX / Other Income $</t>
+        </is>
+      </c>
+      <c r="B6" s="4">
+        <f>'ANNL P&amp;L'!B8+'ANNL P&amp;L'!B9</f>
+        <v/>
+      </c>
+      <c r="C6" s="4">
+        <f>'ANNL P&amp;L'!C8+'ANNL P&amp;L'!C9</f>
+        <v/>
+      </c>
+      <c r="D6" s="4">
+        <f>'ANNL P&amp;L'!D8+'ANNL P&amp;L'!D9</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>'ANNL P&amp;L'!E8+'ANNL P&amp;L'!E9</f>
+        <v/>
+      </c>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="10" t="n"/>
+      <c r="H6" s="10" t="n"/>
+      <c r="I6" s="10" t="n"/>
+      <c r="J6" s="10" t="n"/>
+      <c r="K6" s="10" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Effective Tax Rate %</t>
+        </is>
+      </c>
+      <c r="B7" s="8">
+        <f>IFERROR('ANNL P&amp;L'!B11/'ANNL P&amp;L'!B10,0)</f>
+        <v/>
+      </c>
+      <c r="C7" s="8">
+        <f>IFERROR('ANNL P&amp;L'!C11/'ANNL P&amp;L'!C10,0)</f>
+        <v/>
+      </c>
+      <c r="D7" s="8">
+        <f>IFERROR('ANNL P&amp;L'!D11/'ANNL P&amp;L'!D10,0)</f>
+        <v/>
+      </c>
+      <c r="E7" s="8">
+        <f>IFERROR('ANNL P&amp;L'!E11/'ANNL P&amp;L'!E10,0)</f>
+        <v/>
+      </c>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="9" t="n"/>
+      <c r="J7" s="9" t="n"/>
+      <c r="K7" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>FY2025E</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Current Assets</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="n"/>
+      <c r="C2" s="12" t="n"/>
+      <c r="D2" s="12" t="n"/>
+      <c r="E2" s="12" t="n"/>
+      <c r="F2" s="12" t="n"/>
+      <c r="G2" s="12" t="n"/>
+      <c r="H2" s="12" t="n"/>
+      <c r="I2" s="12" t="n"/>
+      <c r="J2" s="12" t="n"/>
+      <c r="K2" s="12" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>DSO (days)</t>
+        </is>
+      </c>
+      <c r="C3" s="13">
+        <f>IFERROR('BALANCE SHEET'!B4/'ANNL P&amp;L'!C2*365,0)</f>
+        <v/>
+      </c>
+      <c r="D3" s="13">
+        <f>IFERROR('BALANCE SHEET'!C4/'ANNL P&amp;L'!D2*365,0)</f>
+        <v/>
+      </c>
+      <c r="E3" s="13">
+        <f>IFERROR('BALANCE SHEET'!D4/'ANNL P&amp;L'!E2*365,0)</f>
+        <v/>
+      </c>
+      <c r="F3" s="14" t="n"/>
+      <c r="G3" s="14" t="n"/>
+      <c r="H3" s="14" t="n"/>
+      <c r="I3" s="14" t="n"/>
+      <c r="J3" s="14" t="n"/>
+      <c r="K3" s="14" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>DIO (days)</t>
+        </is>
+      </c>
+      <c r="C4" s="13">
+        <f>IFERROR('BALANCE SHEET'!B6/'ANNL P&amp;L'!C3*365,0)</f>
+        <v/>
+      </c>
+      <c r="D4" s="13">
+        <f>IFERROR('BALANCE SHEET'!C6/'ANNL P&amp;L'!D3*365,0)</f>
+        <v/>
+      </c>
+      <c r="E4" s="13">
+        <f>IFERROR('BALANCE SHEET'!D6/'ANNL P&amp;L'!E3*365,0)</f>
+        <v/>
+      </c>
+      <c r="F4" s="14" t="n"/>
+      <c r="G4" s="14" t="n"/>
+      <c r="H4" s="14" t="n"/>
+      <c r="I4" s="14" t="n"/>
+      <c r="J4" s="14" t="n"/>
+      <c r="K4" s="14" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Note Receivable - Current % of Rev</t>
+        </is>
+      </c>
+      <c r="C5" s="8">
+        <f>IFERROR('BALANCE SHEET'!B5/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D5" s="8">
+        <f>IFERROR('BALANCE SHEET'!C5/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E5" s="8">
+        <f>IFERROR('BALANCE SHEET'!D5/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9" t="n"/>
+      <c r="I5" s="9" t="n"/>
+      <c r="J5" s="9" t="n"/>
+      <c r="K5" s="9" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Deferred Other Costs - Current % of Rev</t>
+        </is>
+      </c>
+      <c r="C6" s="8">
+        <f>IFERROR('BALANCE SHEET'!B7/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D6" s="8">
+        <f>IFERROR('BALANCE SHEET'!C7/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E6" s="8">
+        <f>IFERROR('BALANCE SHEET'!D7/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="9" t="n"/>
+      <c r="J6" s="9" t="n"/>
+      <c r="K6" s="9" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Prepaid Expenses % of Rev</t>
+        </is>
+      </c>
+      <c r="C7" s="8">
+        <f>IFERROR('BALANCE SHEET'!B8/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D7" s="8">
+        <f>IFERROR('BALANCE SHEET'!C8/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E7" s="8">
+        <f>IFERROR('BALANCE SHEET'!D8/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="9" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="9" t="n"/>
+      <c r="J7" s="9" t="n"/>
+      <c r="K7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="12" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="12" t="n"/>
+      <c r="K8" s="12" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>DPO (days)</t>
+        </is>
+      </c>
+      <c r="C9" s="13">
+        <f>IFERROR('BALANCE SHEET'!B20/'ANNL P&amp;L'!C3*365,0)</f>
+        <v/>
+      </c>
+      <c r="D9" s="13">
+        <f>IFERROR('BALANCE SHEET'!C20/'ANNL P&amp;L'!D3*365,0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="13">
+        <f>IFERROR('BALANCE SHEET'!D20/'ANNL P&amp;L'!E3*365,0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="14" t="n"/>
+      <c r="G9" s="14" t="n"/>
+      <c r="H9" s="14" t="n"/>
+      <c r="I9" s="14" t="n"/>
+      <c r="J9" s="14" t="n"/>
+      <c r="K9" s="14" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Accrued Expenses % of Rev</t>
+        </is>
+      </c>
+      <c r="C10" s="8">
+        <f>IFERROR('BALANCE SHEET'!B21/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D10" s="8">
+        <f>IFERROR('BALANCE SHEET'!C21/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="8">
+        <f>IFERROR('BALANCE SHEET'!D21/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F10" s="9" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="9" t="n"/>
+      <c r="I10" s="9" t="n"/>
+      <c r="J10" s="9" t="n"/>
+      <c r="K10" s="9" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Income Taxes Payable % of Rev</t>
+        </is>
+      </c>
+      <c r="C11" s="8">
+        <f>IFERROR('BALANCE SHEET'!B22/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D11" s="8">
+        <f>IFERROR('BALANCE SHEET'!C22/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="8">
+        <f>IFERROR('BALANCE SHEET'!D22/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="9" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="9" t="n"/>
+      <c r="I11" s="9" t="n"/>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="9" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Accrued Distributor Termination Fees % of Rev</t>
+        </is>
+      </c>
+      <c r="C12" s="8">
+        <f>IFERROR('BALANCE SHEET'!B23/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D12" s="8">
+        <f>IFERROR('BALANCE SHEET'!C23/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="8">
+        <f>IFERROR('BALANCE SHEET'!D23/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="9" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="9" t="n"/>
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="9" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Accrued Promotional Allowance % of Rev</t>
+        </is>
+      </c>
+      <c r="C13" s="8">
+        <f>IFERROR('BALANCE SHEET'!B24/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D13" s="8">
+        <f>IFERROR('BALANCE SHEET'!C24/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="8">
+        <f>IFERROR('BALANCE SHEET'!D24/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F13" s="9" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="9" t="n"/>
+      <c r="I13" s="9" t="n"/>
+      <c r="J13" s="9" t="n"/>
+      <c r="K13" s="9" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Lease Liability - Operating - Current % of Rev</t>
+        </is>
+      </c>
+      <c r="C14" s="8">
+        <f>IFERROR('BALANCE SHEET'!B25/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D14" s="8">
+        <f>IFERROR('BALANCE SHEET'!C25/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E14" s="8">
+        <f>IFERROR('BALANCE SHEET'!D25/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F14" s="9" t="n"/>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="9" t="n"/>
+      <c r="I14" s="9" t="n"/>
+      <c r="J14" s="9" t="n"/>
+      <c r="K14" s="9" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Lease Liability - Finance - Current % of Rev</t>
+        </is>
+      </c>
+      <c r="C15" s="8">
+        <f>IFERROR('BALANCE SHEET'!B26/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D15" s="8">
+        <f>IFERROR('BALANCE SHEET'!C26/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="8">
+        <f>IFERROR('BALANCE SHEET'!D26/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="9" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="9" t="n"/>
+      <c r="I15" s="9" t="n"/>
+      <c r="J15" s="9" t="n"/>
+      <c r="K15" s="9" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Deferred Revenue - Current % of Rev</t>
+        </is>
+      </c>
+      <c r="C16" s="8">
+        <f>IFERROR('BALANCE SHEET'!B27/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D16" s="8">
+        <f>IFERROR('BALANCE SHEET'!C27/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="8">
+        <f>IFERROR('BALANCE SHEET'!D27/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="9" t="n"/>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="9" t="n"/>
+      <c r="I16" s="9" t="n"/>
+      <c r="J16" s="9" t="n"/>
+      <c r="K16" s="9" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Other Current Liabilities % of Rev</t>
+        </is>
+      </c>
+      <c r="C17" s="8">
+        <f>IFERROR('BALANCE SHEET'!B28/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D17" s="8">
+        <f>IFERROR('BALANCE SHEET'!C28/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E17" s="8">
+        <f>IFERROR('BALANCE SHEET'!D28/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="9" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="9" t="n"/>
+      <c r="I17" s="9" t="n"/>
+      <c r="J17" s="9" t="n"/>
+      <c r="K17" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>FY2025E</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>D&amp;A $</t>
+        </is>
+      </c>
+      <c r="B2" s="4">
+        <f>'CASH FLOW'!B3</f>
+        <v/>
+      </c>
+      <c r="C2" s="4">
+        <f>'CASH FLOW'!C3</f>
+        <v/>
+      </c>
+      <c r="D2" s="4">
+        <f>'CASH FLOW'!D3</f>
+        <v/>
+      </c>
+      <c r="E2" s="4">
+        <f>'CASH FLOW'!E3</f>
+        <v/>
+      </c>
+      <c r="F2" s="10" t="n"/>
+      <c r="G2" s="10" t="n"/>
+      <c r="H2" s="10" t="n"/>
+      <c r="I2" s="10" t="n"/>
+      <c r="J2" s="10" t="n"/>
+      <c r="K2" s="10" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>SBC $</t>
+        </is>
+      </c>
+      <c r="B3" s="4">
+        <f>'CASH FLOW'!B9</f>
+        <v/>
+      </c>
+      <c r="C3" s="4">
+        <f>'CASH FLOW'!C9</f>
+        <v/>
+      </c>
+      <c r="D3" s="4">
+        <f>'CASH FLOW'!D9</f>
+        <v/>
+      </c>
+      <c r="E3" s="4">
+        <f>'CASH FLOW'!E9</f>
+        <v/>
+      </c>
+      <c r="F3" s="10" t="n"/>
+      <c r="G3" s="10" t="n"/>
+      <c r="H3" s="10" t="n"/>
+      <c r="I3" s="10" t="n"/>
+      <c r="J3" s="10" t="n"/>
+      <c r="K3" s="10" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>CapEx $</t>
+        </is>
+      </c>
+      <c r="B4" s="4">
+        <f>'CASH FLOW'!B28</f>
+        <v/>
+      </c>
+      <c r="C4" s="4">
+        <f>'CASH FLOW'!C28</f>
+        <v/>
+      </c>
+      <c r="D4" s="4">
+        <f>'CASH FLOW'!D28</f>
+        <v/>
+      </c>
+      <c r="E4" s="4">
+        <f>'CASH FLOW'!E28</f>
+        <v/>
+      </c>
+      <c r="F4" s="10" t="n"/>
+      <c r="G4" s="10" t="n"/>
+      <c r="H4" s="10" t="n"/>
+      <c r="I4" s="10" t="n"/>
+      <c r="J4" s="10" t="n"/>
+      <c r="K4" s="10" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Preferred Dividends $</t>
+        </is>
+      </c>
+      <c r="B5" s="4">
+        <f>'CASH FLOW'!B35</f>
+        <v/>
+      </c>
+      <c r="C5" s="4">
+        <f>'CASH FLOW'!C35</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>'CASH FLOW'!D35</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>'CASH FLOW'!E35</f>
+        <v/>
+      </c>
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="10" t="n"/>
+      <c r="H5" s="10" t="n"/>
+      <c r="I5" s="10" t="n"/>
+      <c r="J5" s="10" t="n"/>
+      <c r="K5" s="10" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Share Repurchases $</t>
+        </is>
+      </c>
+      <c r="B6" s="4">
+        <f>'CASH FLOW'!B37</f>
+        <v/>
+      </c>
+      <c r="C6" s="4">
+        <f>'CASH FLOW'!C37</f>
+        <v/>
+      </c>
+      <c r="D6" s="4">
+        <f>'CASH FLOW'!D37</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>'CASH FLOW'!E37</f>
+        <v/>
+      </c>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="10" t="n"/>
+      <c r="H6" s="10" t="n"/>
+      <c r="I6" s="10" t="n"/>
+      <c r="J6" s="10" t="n"/>
+      <c r="K6" s="10" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Net Debt $</t>
+        </is>
+      </c>
+      <c r="C7" s="4">
+        <f>('BALANCE SHEET'!B25+'BALANCE SHEET'!B26+'BALANCE SHEET'!B30+'BALANCE SHEET'!B31)-('BALANCE SHEET'!B2+'BALANCE SHEET'!B3)</f>
+        <v/>
+      </c>
+      <c r="D7" s="4">
+        <f>('BALANCE SHEET'!C25+'BALANCE SHEET'!C26+'BALANCE SHEET'!C30+'BALANCE SHEET'!C31)-('BALANCE SHEET'!C2+'BALANCE SHEET'!C3)</f>
+        <v/>
+      </c>
+      <c r="E7" s="4">
+        <f>('BALANCE SHEET'!D25+'BALANCE SHEET'!D26+'BALANCE SHEET'!D30+'BALANCE SHEET'!D31)-('BALANCE SHEET'!D2+'BALANCE SHEET'!D3)</f>
+        <v/>
+      </c>
+      <c r="F7" s="10" t="n"/>
+      <c r="G7" s="10" t="n"/>
+      <c r="H7" s="10" t="n"/>
+      <c r="I7" s="10" t="n"/>
+      <c r="J7" s="10" t="n"/>
+      <c r="K7" s="10" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-04-23 19:07:59
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -3113,7 +3113,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Dividends Paid</t>
+          <t>Dividends</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
@@ -4216,7 +4216,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Preferred Dividends $</t>
+          <t>Dividends $</t>
         </is>
       </c>
       <c r="B5" s="4">

</xml_diff>

<commit_message>
vault backup: 2026-04-23 19:23:20
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -909,7 +909,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Dividends</t>
+          <t>Preferred Dividends</t>
         </is>
       </c>
       <c r="B13" s="4" t="n">
@@ -3113,7 +3113,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>Dividends</t>
+          <t>Preferred Dividends</t>
         </is>
       </c>
       <c r="B35" s="4" t="n">
@@ -4057,7 +4057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -4216,77 +4216,61 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Dividends $</t>
-        </is>
-      </c>
-      <c r="B5" s="4">
-        <f>'CASH FLOW'!B35</f>
-        <v/>
-      </c>
-      <c r="C5" s="4">
-        <f>'CASH FLOW'!C35</f>
-        <v/>
-      </c>
-      <c r="D5" s="4">
-        <f>'CASH FLOW'!D35</f>
-        <v/>
-      </c>
-      <c r="E5" s="4">
-        <f>'CASH FLOW'!E35</f>
-        <v/>
-      </c>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="10" t="n"/>
-      <c r="I5" s="10" t="n"/>
-      <c r="J5" s="10" t="n"/>
-      <c r="K5" s="10" t="n"/>
+          <t>Preferred Dividends % of Preferred Balance</t>
+        </is>
+      </c>
+      <c r="C5" s="8">
+        <f>IFERROR('CASH FLOW'!C35/'BALANCE SHEET'!B35,0)</f>
+        <v/>
+      </c>
+      <c r="D5" s="8">
+        <f>IFERROR('CASH FLOW'!D35/'BALANCE SHEET'!C35,0)</f>
+        <v/>
+      </c>
+      <c r="E5" s="8">
+        <f>IFERROR('CASH FLOW'!E35/'BALANCE SHEET'!D35,0)</f>
+        <v/>
+      </c>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9" t="n"/>
+      <c r="I5" s="9" t="n"/>
+      <c r="J5" s="9" t="n"/>
+      <c r="K5" s="9" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Share Repurchases $</t>
-        </is>
-      </c>
-      <c r="B6" s="4">
-        <f>'CASH FLOW'!B37</f>
-        <v/>
-      </c>
-      <c r="C6" s="4">
-        <f>'CASH FLOW'!C37</f>
-        <v/>
-      </c>
-      <c r="D6" s="4">
-        <f>'CASH FLOW'!D37</f>
-        <v/>
-      </c>
-      <c r="E6" s="4">
-        <f>'CASH FLOW'!E37</f>
-        <v/>
-      </c>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
-      <c r="H6" s="10" t="n"/>
-      <c r="I6" s="10" t="n"/>
-      <c r="J6" s="10" t="n"/>
-      <c r="K6" s="10" t="n"/>
+          <t>Common Dividends % of Net Income</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="9" t="n"/>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="9" t="n"/>
+      <c r="J6" s="9" t="n"/>
+      <c r="K6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Net Debt $</t>
-        </is>
+          <t>Share Repurchases $</t>
+        </is>
+      </c>
+      <c r="B7" s="4">
+        <f>'CASH FLOW'!B37</f>
+        <v/>
       </c>
       <c r="C7" s="4">
-        <f>('BALANCE SHEET'!B25+'BALANCE SHEET'!B26+'BALANCE SHEET'!B30+'BALANCE SHEET'!B31)-('BALANCE SHEET'!B2+'BALANCE SHEET'!B3)</f>
+        <f>'CASH FLOW'!C37</f>
         <v/>
       </c>
       <c r="D7" s="4">
-        <f>('BALANCE SHEET'!C25+'BALANCE SHEET'!C26+'BALANCE SHEET'!C30+'BALANCE SHEET'!C31)-('BALANCE SHEET'!C2+'BALANCE SHEET'!C3)</f>
+        <f>'CASH FLOW'!D37</f>
         <v/>
       </c>
       <c r="E7" s="4">
-        <f>('BALANCE SHEET'!D25+'BALANCE SHEET'!D26+'BALANCE SHEET'!D30+'BALANCE SHEET'!D31)-('BALANCE SHEET'!D2+'BALANCE SHEET'!D3)</f>
+        <f>'CASH FLOW'!E37</f>
         <v/>
       </c>
       <c r="F7" s="10" t="n"/>
@@ -4296,6 +4280,31 @@
       <c r="J7" s="10" t="n"/>
       <c r="K7" s="10" t="n"/>
     </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Net Debt $</t>
+        </is>
+      </c>
+      <c r="C8" s="4">
+        <f>('BALANCE SHEET'!B25+'BALANCE SHEET'!B26+'BALANCE SHEET'!B30+'BALANCE SHEET'!B31)-('BALANCE SHEET'!B2+'BALANCE SHEET'!B3)</f>
+        <v/>
+      </c>
+      <c r="D8" s="4">
+        <f>('BALANCE SHEET'!C25+'BALANCE SHEET'!C26+'BALANCE SHEET'!C30+'BALANCE SHEET'!C31)-('BALANCE SHEET'!C2+'BALANCE SHEET'!C3)</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>('BALANCE SHEET'!D25+'BALANCE SHEET'!D26+'BALANCE SHEET'!D30+'BALANCE SHEET'!D31)-('BALANCE SHEET'!D2+'BALANCE SHEET'!D3)</f>
+        <v/>
+      </c>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="10" t="n"/>
+      <c r="H8" s="10" t="n"/>
+      <c r="I8" s="10" t="n"/>
+      <c r="J8" s="10" t="n"/>
+      <c r="K8" s="10" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 19:38:39
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -7,12 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ANNL P&amp;L" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="BALANCE SHEET" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="CASH FLOW" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="IS DRIVERS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="BS DRIVERS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="CF DRIVERS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ASSUMPTIONS" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ANNL P&amp;L" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BALANCE SHEET" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CASH FLOW" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="IS DRIVERS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="BS DRIVERS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CF DRIVERS" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -48,7 +49,7 @@
       <color rgb="00595959"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -65,6 +66,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F2F2F2"/>
         <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -91,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -102,11 +109,14 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -474,6 +484,72 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Assumption</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Days in Year</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="n">
+        <v>365</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Used in DSO, DIO, DPO formulas</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Share Repurchases $</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Per-period repurchase assumption for projection</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1086,7 +1162,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2166,7 +2242,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3337,721 +3413,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr"/>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>FY2021</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>FY2022</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>FY2023</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>FY2024</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>FY2025E</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>FY2026E</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>FY2027E</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>FY2028E</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>FY2029E</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>FY2030E</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Revenue Growth %</t>
-        </is>
-      </c>
-      <c r="C2" s="8">
-        <f>IFERROR(('ANNL P&amp;L'!C2-'ANNL P&amp;L'!B2)/'ANNL P&amp;L'!B2,0)</f>
-        <v/>
-      </c>
-      <c r="D2" s="8">
-        <f>IFERROR(('ANNL P&amp;L'!D2-'ANNL P&amp;L'!C2)/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="E2" s="8">
-        <f>IFERROR(('ANNL P&amp;L'!E2-'ANNL P&amp;L'!D2)/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="F2" s="9" t="n"/>
-      <c r="G2" s="9" t="n"/>
-      <c r="H2" s="9" t="n"/>
-      <c r="I2" s="9" t="n"/>
-      <c r="J2" s="9" t="n"/>
-      <c r="K2" s="9" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>COGS % of Revenue</t>
-        </is>
-      </c>
-      <c r="B3" s="8">
-        <f>IFERROR('ANNL P&amp;L'!B3/'ANNL P&amp;L'!B2,0)</f>
-        <v/>
-      </c>
-      <c r="C3" s="8">
-        <f>IFERROR('ANNL P&amp;L'!C3/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="D3" s="8">
-        <f>IFERROR('ANNL P&amp;L'!D3/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="E3" s="8">
-        <f>IFERROR('ANNL P&amp;L'!E3/'ANNL P&amp;L'!E2,0)</f>
-        <v/>
-      </c>
-      <c r="F3" s="9" t="n"/>
-      <c r="G3" s="9" t="n"/>
-      <c r="H3" s="9" t="n"/>
-      <c r="I3" s="9" t="n"/>
-      <c r="J3" s="9" t="n"/>
-      <c r="K3" s="9" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>SG&amp;A % of Revenue</t>
-        </is>
-      </c>
-      <c r="B4" s="8">
-        <f>IFERROR('ANNL P&amp;L'!B5/'ANNL P&amp;L'!B2,0)</f>
-        <v/>
-      </c>
-      <c r="C4" s="8">
-        <f>IFERROR('ANNL P&amp;L'!C5/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="D4" s="8">
-        <f>IFERROR('ANNL P&amp;L'!D5/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="E4" s="8">
-        <f>IFERROR('ANNL P&amp;L'!E5/'ANNL P&amp;L'!E2,0)</f>
-        <v/>
-      </c>
-      <c r="F4" s="9" t="n"/>
-      <c r="G4" s="9" t="n"/>
-      <c r="H4" s="9" t="n"/>
-      <c r="I4" s="9" t="n"/>
-      <c r="J4" s="9" t="n"/>
-      <c r="K4" s="9" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Interest Income (Expense) $</t>
-        </is>
-      </c>
-      <c r="B5" s="4">
-        <f>'ANNL P&amp;L'!B7</f>
-        <v/>
-      </c>
-      <c r="C5" s="4">
-        <f>'ANNL P&amp;L'!C7</f>
-        <v/>
-      </c>
-      <c r="D5" s="4">
-        <f>'ANNL P&amp;L'!D7</f>
-        <v/>
-      </c>
-      <c r="E5" s="4">
-        <f>'ANNL P&amp;L'!E7</f>
-        <v/>
-      </c>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="10" t="n"/>
-      <c r="I5" s="10" t="n"/>
-      <c r="J5" s="10" t="n"/>
-      <c r="K5" s="10" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>FX / Other Income $</t>
-        </is>
-      </c>
-      <c r="B6" s="4">
-        <f>'ANNL P&amp;L'!B8+'ANNL P&amp;L'!B9</f>
-        <v/>
-      </c>
-      <c r="C6" s="4">
-        <f>'ANNL P&amp;L'!C8+'ANNL P&amp;L'!C9</f>
-        <v/>
-      </c>
-      <c r="D6" s="4">
-        <f>'ANNL P&amp;L'!D8+'ANNL P&amp;L'!D9</f>
-        <v/>
-      </c>
-      <c r="E6" s="4">
-        <f>'ANNL P&amp;L'!E8+'ANNL P&amp;L'!E9</f>
-        <v/>
-      </c>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
-      <c r="H6" s="10" t="n"/>
-      <c r="I6" s="10" t="n"/>
-      <c r="J6" s="10" t="n"/>
-      <c r="K6" s="10" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Effective Tax Rate %</t>
-        </is>
-      </c>
-      <c r="B7" s="8">
-        <f>IFERROR('ANNL P&amp;L'!B11/'ANNL P&amp;L'!B10,0)</f>
-        <v/>
-      </c>
-      <c r="C7" s="8">
-        <f>IFERROR('ANNL P&amp;L'!C11/'ANNL P&amp;L'!C10,0)</f>
-        <v/>
-      </c>
-      <c r="D7" s="8">
-        <f>IFERROR('ANNL P&amp;L'!D11/'ANNL P&amp;L'!D10,0)</f>
-        <v/>
-      </c>
-      <c r="E7" s="8">
-        <f>IFERROR('ANNL P&amp;L'!E11/'ANNL P&amp;L'!E10,0)</f>
-        <v/>
-      </c>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="9" t="n"/>
-      <c r="I7" s="9" t="n"/>
-      <c r="J7" s="9" t="n"/>
-      <c r="K7" s="9" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr"/>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>FY2021</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>FY2022</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>FY2023</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>FY2024</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>FY2025E</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>FY2026E</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>FY2027E</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>FY2028E</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>FY2029E</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>FY2030E</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="11" t="inlineStr">
-        <is>
-          <t>Current Assets</t>
-        </is>
-      </c>
-      <c r="B2" s="12" t="n"/>
-      <c r="C2" s="12" t="n"/>
-      <c r="D2" s="12" t="n"/>
-      <c r="E2" s="12" t="n"/>
-      <c r="F2" s="12" t="n"/>
-      <c r="G2" s="12" t="n"/>
-      <c r="H2" s="12" t="n"/>
-      <c r="I2" s="12" t="n"/>
-      <c r="J2" s="12" t="n"/>
-      <c r="K2" s="12" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>DSO (days)</t>
-        </is>
-      </c>
-      <c r="C3" s="13">
-        <f>IFERROR('BALANCE SHEET'!B4/'ANNL P&amp;L'!C2*365,0)</f>
-        <v/>
-      </c>
-      <c r="D3" s="13">
-        <f>IFERROR('BALANCE SHEET'!C4/'ANNL P&amp;L'!D2*365,0)</f>
-        <v/>
-      </c>
-      <c r="E3" s="13">
-        <f>IFERROR('BALANCE SHEET'!D4/'ANNL P&amp;L'!E2*365,0)</f>
-        <v/>
-      </c>
-      <c r="F3" s="14" t="n"/>
-      <c r="G3" s="14" t="n"/>
-      <c r="H3" s="14" t="n"/>
-      <c r="I3" s="14" t="n"/>
-      <c r="J3" s="14" t="n"/>
-      <c r="K3" s="14" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>DIO (days)</t>
-        </is>
-      </c>
-      <c r="C4" s="13">
-        <f>IFERROR('BALANCE SHEET'!B6/'ANNL P&amp;L'!C3*365,0)</f>
-        <v/>
-      </c>
-      <c r="D4" s="13">
-        <f>IFERROR('BALANCE SHEET'!C6/'ANNL P&amp;L'!D3*365,0)</f>
-        <v/>
-      </c>
-      <c r="E4" s="13">
-        <f>IFERROR('BALANCE SHEET'!D6/'ANNL P&amp;L'!E3*365,0)</f>
-        <v/>
-      </c>
-      <c r="F4" s="14" t="n"/>
-      <c r="G4" s="14" t="n"/>
-      <c r="H4" s="14" t="n"/>
-      <c r="I4" s="14" t="n"/>
-      <c r="J4" s="14" t="n"/>
-      <c r="K4" s="14" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>Note Receivable - Current % of Rev</t>
-        </is>
-      </c>
-      <c r="C5" s="8">
-        <f>IFERROR('BALANCE SHEET'!B5/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="D5" s="8">
-        <f>IFERROR('BALANCE SHEET'!C5/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="E5" s="8">
-        <f>IFERROR('BALANCE SHEET'!D5/'ANNL P&amp;L'!E2,0)</f>
-        <v/>
-      </c>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="9" t="n"/>
-      <c r="I5" s="9" t="n"/>
-      <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Deferred Other Costs - Current % of Rev</t>
-        </is>
-      </c>
-      <c r="C6" s="8">
-        <f>IFERROR('BALANCE SHEET'!B7/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="D6" s="8">
-        <f>IFERROR('BALANCE SHEET'!C7/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="E6" s="8">
-        <f>IFERROR('BALANCE SHEET'!D7/'ANNL P&amp;L'!E2,0)</f>
-        <v/>
-      </c>
-      <c r="F6" s="9" t="n"/>
-      <c r="G6" s="9" t="n"/>
-      <c r="H6" s="9" t="n"/>
-      <c r="I6" s="9" t="n"/>
-      <c r="J6" s="9" t="n"/>
-      <c r="K6" s="9" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Prepaid Expenses % of Rev</t>
-        </is>
-      </c>
-      <c r="C7" s="8">
-        <f>IFERROR('BALANCE SHEET'!B8/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="D7" s="8">
-        <f>IFERROR('BALANCE SHEET'!C8/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="E7" s="8">
-        <f>IFERROR('BALANCE SHEET'!D8/'ANNL P&amp;L'!E2,0)</f>
-        <v/>
-      </c>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="9" t="n"/>
-      <c r="I7" s="9" t="n"/>
-      <c r="J7" s="9" t="n"/>
-      <c r="K7" s="9" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>Current Liabilities</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="n"/>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="12" t="n"/>
-      <c r="E8" s="12" t="n"/>
-      <c r="F8" s="12" t="n"/>
-      <c r="G8" s="12" t="n"/>
-      <c r="H8" s="12" t="n"/>
-      <c r="I8" s="12" t="n"/>
-      <c r="J8" s="12" t="n"/>
-      <c r="K8" s="12" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>DPO (days)</t>
-        </is>
-      </c>
-      <c r="C9" s="13">
-        <f>IFERROR('BALANCE SHEET'!B20/'ANNL P&amp;L'!C3*365,0)</f>
-        <v/>
-      </c>
-      <c r="D9" s="13">
-        <f>IFERROR('BALANCE SHEET'!C20/'ANNL P&amp;L'!D3*365,0)</f>
-        <v/>
-      </c>
-      <c r="E9" s="13">
-        <f>IFERROR('BALANCE SHEET'!D20/'ANNL P&amp;L'!E3*365,0)</f>
-        <v/>
-      </c>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="14" t="n"/>
-      <c r="I9" s="14" t="n"/>
-      <c r="J9" s="14" t="n"/>
-      <c r="K9" s="14" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Accrued Expenses % of Rev</t>
-        </is>
-      </c>
-      <c r="C10" s="8">
-        <f>IFERROR('BALANCE SHEET'!B21/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="D10" s="8">
-        <f>IFERROR('BALANCE SHEET'!C21/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="E10" s="8">
-        <f>IFERROR('BALANCE SHEET'!D21/'ANNL P&amp;L'!E2,0)</f>
-        <v/>
-      </c>
-      <c r="F10" s="9" t="n"/>
-      <c r="G10" s="9" t="n"/>
-      <c r="H10" s="9" t="n"/>
-      <c r="I10" s="9" t="n"/>
-      <c r="J10" s="9" t="n"/>
-      <c r="K10" s="9" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Income Taxes Payable % of Rev</t>
-        </is>
-      </c>
-      <c r="C11" s="8">
-        <f>IFERROR('BALANCE SHEET'!B22/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="D11" s="8">
-        <f>IFERROR('BALANCE SHEET'!C22/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="E11" s="8">
-        <f>IFERROR('BALANCE SHEET'!D22/'ANNL P&amp;L'!E2,0)</f>
-        <v/>
-      </c>
-      <c r="F11" s="9" t="n"/>
-      <c r="G11" s="9" t="n"/>
-      <c r="H11" s="9" t="n"/>
-      <c r="I11" s="9" t="n"/>
-      <c r="J11" s="9" t="n"/>
-      <c r="K11" s="9" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>Accrued Distributor Termination Fees % of Rev</t>
-        </is>
-      </c>
-      <c r="C12" s="8">
-        <f>IFERROR('BALANCE SHEET'!B23/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="D12" s="8">
-        <f>IFERROR('BALANCE SHEET'!C23/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="E12" s="8">
-        <f>IFERROR('BALANCE SHEET'!D23/'ANNL P&amp;L'!E2,0)</f>
-        <v/>
-      </c>
-      <c r="F12" s="9" t="n"/>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="9" t="n"/>
-      <c r="I12" s="9" t="n"/>
-      <c r="J12" s="9" t="n"/>
-      <c r="K12" s="9" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Accrued Promotional Allowance % of Rev</t>
-        </is>
-      </c>
-      <c r="C13" s="8">
-        <f>IFERROR('BALANCE SHEET'!B24/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="D13" s="8">
-        <f>IFERROR('BALANCE SHEET'!C24/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="E13" s="8">
-        <f>IFERROR('BALANCE SHEET'!D24/'ANNL P&amp;L'!E2,0)</f>
-        <v/>
-      </c>
-      <c r="F13" s="9" t="n"/>
-      <c r="G13" s="9" t="n"/>
-      <c r="H13" s="9" t="n"/>
-      <c r="I13" s="9" t="n"/>
-      <c r="J13" s="9" t="n"/>
-      <c r="K13" s="9" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Lease Liability - Operating - Current % of Rev</t>
-        </is>
-      </c>
-      <c r="C14" s="8">
-        <f>IFERROR('BALANCE SHEET'!B25/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="D14" s="8">
-        <f>IFERROR('BALANCE SHEET'!C25/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="E14" s="8">
-        <f>IFERROR('BALANCE SHEET'!D25/'ANNL P&amp;L'!E2,0)</f>
-        <v/>
-      </c>
-      <c r="F14" s="9" t="n"/>
-      <c r="G14" s="9" t="n"/>
-      <c r="H14" s="9" t="n"/>
-      <c r="I14" s="9" t="n"/>
-      <c r="J14" s="9" t="n"/>
-      <c r="K14" s="9" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>Lease Liability - Finance - Current % of Rev</t>
-        </is>
-      </c>
-      <c r="C15" s="8">
-        <f>IFERROR('BALANCE SHEET'!B26/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="D15" s="8">
-        <f>IFERROR('BALANCE SHEET'!C26/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="E15" s="8">
-        <f>IFERROR('BALANCE SHEET'!D26/'ANNL P&amp;L'!E2,0)</f>
-        <v/>
-      </c>
-      <c r="F15" s="9" t="n"/>
-      <c r="G15" s="9" t="n"/>
-      <c r="H15" s="9" t="n"/>
-      <c r="I15" s="9" t="n"/>
-      <c r="J15" s="9" t="n"/>
-      <c r="K15" s="9" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Deferred Revenue - Current % of Rev</t>
-        </is>
-      </c>
-      <c r="C16" s="8">
-        <f>IFERROR('BALANCE SHEET'!B27/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="D16" s="8">
-        <f>IFERROR('BALANCE SHEET'!C27/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="E16" s="8">
-        <f>IFERROR('BALANCE SHEET'!D27/'ANNL P&amp;L'!E2,0)</f>
-        <v/>
-      </c>
-      <c r="F16" s="9" t="n"/>
-      <c r="G16" s="9" t="n"/>
-      <c r="H16" s="9" t="n"/>
-      <c r="I16" s="9" t="n"/>
-      <c r="J16" s="9" t="n"/>
-      <c r="K16" s="9" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Other Current Liabilities % of Rev</t>
-        </is>
-      </c>
-      <c r="C17" s="8">
-        <f>IFERROR('BALANCE SHEET'!B28/'ANNL P&amp;L'!C2,0)</f>
-        <v/>
-      </c>
-      <c r="D17" s="8">
-        <f>IFERROR('BALANCE SHEET'!C28/'ANNL P&amp;L'!D2,0)</f>
-        <v/>
-      </c>
-      <c r="E17" s="8">
-        <f>IFERROR('BALANCE SHEET'!D28/'ANNL P&amp;L'!E2,0)</f>
-        <v/>
-      </c>
-      <c r="F17" s="9" t="n"/>
-      <c r="G17" s="9" t="n"/>
-      <c r="H17" s="9" t="n"/>
-      <c r="I17" s="9" t="n"/>
-      <c r="J17" s="9" t="n"/>
-      <c r="K17" s="9" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4129,35 +3491,1208 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>D&amp;A $</t>
-        </is>
-      </c>
-      <c r="B2" s="4">
-        <f>'CASH FLOW'!B3</f>
-        <v/>
-      </c>
-      <c r="C2" s="4">
-        <f>'CASH FLOW'!C3</f>
-        <v/>
-      </c>
-      <c r="D2" s="4">
-        <f>'CASH FLOW'!D3</f>
-        <v/>
-      </c>
-      <c r="E2" s="4">
-        <f>'CASH FLOW'!E3</f>
-        <v/>
-      </c>
-      <c r="F2" s="10" t="n"/>
-      <c r="G2" s="10" t="n"/>
-      <c r="H2" s="10" t="n"/>
-      <c r="I2" s="10" t="n"/>
-      <c r="J2" s="10" t="n"/>
-      <c r="K2" s="10" t="n"/>
+          <t>Revenue Growth %</t>
+        </is>
+      </c>
+      <c r="C2" s="10">
+        <f>IFERROR(('ANNL P&amp;L'!C2-'ANNL P&amp;L'!B2)/'ANNL P&amp;L'!B2,0)</f>
+        <v/>
+      </c>
+      <c r="D2" s="10">
+        <f>IFERROR(('ANNL P&amp;L'!D2-'ANNL P&amp;L'!C2)/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="E2" s="10">
+        <f>IFERROR(('ANNL P&amp;L'!E2-'ANNL P&amp;L'!D2)/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="F2" s="11" t="n"/>
+      <c r="G2" s="11" t="n"/>
+      <c r="H2" s="11" t="n"/>
+      <c r="I2" s="11" t="n"/>
+      <c r="J2" s="11" t="n"/>
+      <c r="K2" s="11" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
+          <t>COGS % of Revenue</t>
+        </is>
+      </c>
+      <c r="B3" s="10">
+        <f>IFERROR('ANNL P&amp;L'!B3/'ANNL P&amp;L'!B2,0)</f>
+        <v/>
+      </c>
+      <c r="C3" s="10">
+        <f>IFERROR('ANNL P&amp;L'!C3/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D3" s="10">
+        <f>IFERROR('ANNL P&amp;L'!D3/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E3" s="10">
+        <f>IFERROR('ANNL P&amp;L'!E3/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F3" s="12">
+        <f>E3</f>
+        <v/>
+      </c>
+      <c r="G3" s="12">
+        <f>F3</f>
+        <v/>
+      </c>
+      <c r="H3" s="12">
+        <f>G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="12">
+        <f>H3</f>
+        <v/>
+      </c>
+      <c r="J3" s="12">
+        <f>I3</f>
+        <v/>
+      </c>
+      <c r="K3" s="12">
+        <f>J3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>SG&amp;A % of Revenue</t>
+        </is>
+      </c>
+      <c r="B4" s="10">
+        <f>IFERROR('ANNL P&amp;L'!B5/'ANNL P&amp;L'!B2,0)</f>
+        <v/>
+      </c>
+      <c r="C4" s="10">
+        <f>IFERROR('ANNL P&amp;L'!C5/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D4" s="10">
+        <f>IFERROR('ANNL P&amp;L'!D5/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E4" s="10">
+        <f>IFERROR('ANNL P&amp;L'!E5/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F4" s="12">
+        <f>E4</f>
+        <v/>
+      </c>
+      <c r="G4" s="12">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="H4" s="12">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="12">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="J4" s="12">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="K4" s="12">
+        <f>J4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Interest Income (Expense) $</t>
+        </is>
+      </c>
+      <c r="B5" s="4">
+        <f>'ANNL P&amp;L'!B7</f>
+        <v/>
+      </c>
+      <c r="C5" s="4">
+        <f>'ANNL P&amp;L'!C7</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>'ANNL P&amp;L'!D7</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>'ANNL P&amp;L'!E7</f>
+        <v/>
+      </c>
+      <c r="F5" s="13">
+        <f>E5</f>
+        <v/>
+      </c>
+      <c r="G5" s="13">
+        <f>F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="13">
+        <f>G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="13">
+        <f>H5</f>
+        <v/>
+      </c>
+      <c r="J5" s="13">
+        <f>I5</f>
+        <v/>
+      </c>
+      <c r="K5" s="13">
+        <f>J5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Foreign Currency Gain (Loss) $</t>
+        </is>
+      </c>
+      <c r="B6" s="4">
+        <f>'ANNL P&amp;L'!B8</f>
+        <v/>
+      </c>
+      <c r="C6" s="4">
+        <f>'ANNL P&amp;L'!C8</f>
+        <v/>
+      </c>
+      <c r="D6" s="4">
+        <f>'ANNL P&amp;L'!D8</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>'ANNL P&amp;L'!E8</f>
+        <v/>
+      </c>
+      <c r="F6" s="13">
+        <f>E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="13">
+        <f>F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="13">
+        <f>G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="13">
+        <f>H6</f>
+        <v/>
+      </c>
+      <c r="J6" s="13">
+        <f>I6</f>
+        <v/>
+      </c>
+      <c r="K6" s="13">
+        <f>J6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Other Income (Expense) $</t>
+        </is>
+      </c>
+      <c r="B7" s="4">
+        <f>'ANNL P&amp;L'!B9</f>
+        <v/>
+      </c>
+      <c r="C7" s="4">
+        <f>'ANNL P&amp;L'!C9</f>
+        <v/>
+      </c>
+      <c r="D7" s="4">
+        <f>'ANNL P&amp;L'!D9</f>
+        <v/>
+      </c>
+      <c r="E7" s="4">
+        <f>'ANNL P&amp;L'!E9</f>
+        <v/>
+      </c>
+      <c r="F7" s="13">
+        <f>E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="13">
+        <f>F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="13">
+        <f>G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="13">
+        <f>H7</f>
+        <v/>
+      </c>
+      <c r="J7" s="13">
+        <f>I7</f>
+        <v/>
+      </c>
+      <c r="K7" s="13">
+        <f>J7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Effective Tax Rate %</t>
+        </is>
+      </c>
+      <c r="B8" s="10">
+        <f>IFERROR('ANNL P&amp;L'!B11/'ANNL P&amp;L'!B10,0)</f>
+        <v/>
+      </c>
+      <c r="C8" s="10">
+        <f>IFERROR('ANNL P&amp;L'!C11/'ANNL P&amp;L'!C10,0)</f>
+        <v/>
+      </c>
+      <c r="D8" s="10">
+        <f>IFERROR('ANNL P&amp;L'!D11/'ANNL P&amp;L'!D10,0)</f>
+        <v/>
+      </c>
+      <c r="E8" s="10">
+        <f>IFERROR('ANNL P&amp;L'!E11/'ANNL P&amp;L'!E10,0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="12">
+        <f>E8</f>
+        <v/>
+      </c>
+      <c r="G8" s="12">
+        <f>F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="12">
+        <f>G8</f>
+        <v/>
+      </c>
+      <c r="I8" s="12">
+        <f>H8</f>
+        <v/>
+      </c>
+      <c r="J8" s="12">
+        <f>I8</f>
+        <v/>
+      </c>
+      <c r="K8" s="12">
+        <f>J8</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>FY2025E</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Current Assets</t>
+        </is>
+      </c>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="15" t="n"/>
+      <c r="G2" s="15" t="n"/>
+      <c r="H2" s="15" t="n"/>
+      <c r="I2" s="15" t="n"/>
+      <c r="J2" s="15" t="n"/>
+      <c r="K2" s="15" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>DSO (days)</t>
+        </is>
+      </c>
+      <c r="C3" s="16">
+        <f>IFERROR('BALANCE SHEET'!B4/'ANNL P&amp;L'!C2*ASSUMPTIONS!$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="D3" s="16">
+        <f>IFERROR('BALANCE SHEET'!C4/'ANNL P&amp;L'!D2*ASSUMPTIONS!$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="E3" s="16">
+        <f>IFERROR('BALANCE SHEET'!D4/'ANNL P&amp;L'!E2*ASSUMPTIONS!$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="F3" s="17">
+        <f>E3</f>
+        <v/>
+      </c>
+      <c r="G3" s="17">
+        <f>F3</f>
+        <v/>
+      </c>
+      <c r="H3" s="17">
+        <f>G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="17">
+        <f>H3</f>
+        <v/>
+      </c>
+      <c r="J3" s="17">
+        <f>I3</f>
+        <v/>
+      </c>
+      <c r="K3" s="17">
+        <f>J3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>DIO (days)</t>
+        </is>
+      </c>
+      <c r="C4" s="16">
+        <f>IFERROR('BALANCE SHEET'!B6/'ANNL P&amp;L'!C3*ASSUMPTIONS!$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="D4" s="16">
+        <f>IFERROR('BALANCE SHEET'!C6/'ANNL P&amp;L'!D3*ASSUMPTIONS!$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="E4" s="16">
+        <f>IFERROR('BALANCE SHEET'!D6/'ANNL P&amp;L'!E3*ASSUMPTIONS!$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="F4" s="17">
+        <f>E4</f>
+        <v/>
+      </c>
+      <c r="G4" s="17">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="H4" s="17">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="17">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="J4" s="17">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="K4" s="17">
+        <f>J4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Note Receivable - Current % of Rev</t>
+        </is>
+      </c>
+      <c r="C5" s="10">
+        <f>IFERROR('BALANCE SHEET'!B5/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D5" s="10">
+        <f>IFERROR('BALANCE SHEET'!C5/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E5" s="10">
+        <f>IFERROR('BALANCE SHEET'!D5/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F5" s="12">
+        <f>E5</f>
+        <v/>
+      </c>
+      <c r="G5" s="12">
+        <f>F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="12">
+        <f>G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="12">
+        <f>H5</f>
+        <v/>
+      </c>
+      <c r="J5" s="12">
+        <f>I5</f>
+        <v/>
+      </c>
+      <c r="K5" s="12">
+        <f>J5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Deferred Other Costs - Current % of Rev</t>
+        </is>
+      </c>
+      <c r="C6" s="10">
+        <f>IFERROR('BALANCE SHEET'!B7/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D6" s="10">
+        <f>IFERROR('BALANCE SHEET'!C7/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E6" s="10">
+        <f>IFERROR('BALANCE SHEET'!D7/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F6" s="12">
+        <f>E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="12">
+        <f>F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="12">
+        <f>H6</f>
+        <v/>
+      </c>
+      <c r="J6" s="12">
+        <f>I6</f>
+        <v/>
+      </c>
+      <c r="K6" s="12">
+        <f>J6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Prepaid Expenses % of Rev</t>
+        </is>
+      </c>
+      <c r="C7" s="10">
+        <f>IFERROR('BALANCE SHEET'!B8/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D7" s="10">
+        <f>IFERROR('BALANCE SHEET'!C8/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E7" s="10">
+        <f>IFERROR('BALANCE SHEET'!D8/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F7" s="12">
+        <f>E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="12">
+        <f>F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="12">
+        <f>G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="12">
+        <f>H7</f>
+        <v/>
+      </c>
+      <c r="J7" s="12">
+        <f>I7</f>
+        <v/>
+      </c>
+      <c r="K7" s="12">
+        <f>J7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Non-Current Assets</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n"/>
+      <c r="C8" s="15" t="n"/>
+      <c r="D8" s="15" t="n"/>
+      <c r="E8" s="15" t="n"/>
+      <c r="F8" s="15" t="n"/>
+      <c r="G8" s="15" t="n"/>
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="15" t="n"/>
+      <c r="J8" s="15" t="n"/>
+      <c r="K8" s="15" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Other Non-Current Assets % of Rev</t>
+        </is>
+      </c>
+      <c r="C9" s="10">
+        <f>IFERROR('BALANCE SHEET'!B18/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D9" s="10">
+        <f>IFERROR('BALANCE SHEET'!C18/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="10">
+        <f>IFERROR('BALANCE SHEET'!D18/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="12">
+        <f>E9</f>
+        <v/>
+      </c>
+      <c r="G9" s="12">
+        <f>F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="12">
+        <f>G9</f>
+        <v/>
+      </c>
+      <c r="I9" s="12">
+        <f>H9</f>
+        <v/>
+      </c>
+      <c r="J9" s="12">
+        <f>I9</f>
+        <v/>
+      </c>
+      <c r="K9" s="12">
+        <f>J9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Current Liabilities</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="15" t="n"/>
+      <c r="I10" s="15" t="n"/>
+      <c r="J10" s="15" t="n"/>
+      <c r="K10" s="15" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>DPO (days)</t>
+        </is>
+      </c>
+      <c r="C11" s="16">
+        <f>IFERROR('BALANCE SHEET'!B20/'ANNL P&amp;L'!C3*ASSUMPTIONS!$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="D11" s="16">
+        <f>IFERROR('BALANCE SHEET'!C20/'ANNL P&amp;L'!D3*ASSUMPTIONS!$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="16">
+        <f>IFERROR('BALANCE SHEET'!D20/'ANNL P&amp;L'!E3*ASSUMPTIONS!$B$2,0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="17">
+        <f>E11</f>
+        <v/>
+      </c>
+      <c r="G11" s="17">
+        <f>F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="17">
+        <f>G11</f>
+        <v/>
+      </c>
+      <c r="I11" s="17">
+        <f>H11</f>
+        <v/>
+      </c>
+      <c r="J11" s="17">
+        <f>I11</f>
+        <v/>
+      </c>
+      <c r="K11" s="17">
+        <f>J11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Accrued Expenses % of Rev</t>
+        </is>
+      </c>
+      <c r="C12" s="10">
+        <f>IFERROR('BALANCE SHEET'!B21/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D12" s="10">
+        <f>IFERROR('BALANCE SHEET'!C21/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="10">
+        <f>IFERROR('BALANCE SHEET'!D21/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="12">
+        <f>E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="12">
+        <f>F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="12">
+        <f>G12</f>
+        <v/>
+      </c>
+      <c r="I12" s="12">
+        <f>H12</f>
+        <v/>
+      </c>
+      <c r="J12" s="12">
+        <f>I12</f>
+        <v/>
+      </c>
+      <c r="K12" s="12">
+        <f>J12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Income Taxes Payable % of Rev</t>
+        </is>
+      </c>
+      <c r="C13" s="10">
+        <f>IFERROR('BALANCE SHEET'!B22/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D13" s="10">
+        <f>IFERROR('BALANCE SHEET'!C22/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="10">
+        <f>IFERROR('BALANCE SHEET'!D22/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F13" s="12">
+        <f>E13</f>
+        <v/>
+      </c>
+      <c r="G13" s="12">
+        <f>F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="12">
+        <f>G13</f>
+        <v/>
+      </c>
+      <c r="I13" s="12">
+        <f>H13</f>
+        <v/>
+      </c>
+      <c r="J13" s="12">
+        <f>I13</f>
+        <v/>
+      </c>
+      <c r="K13" s="12">
+        <f>J13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Accrued Distributor Termination Fees % of Rev</t>
+        </is>
+      </c>
+      <c r="C14" s="10">
+        <f>IFERROR('BALANCE SHEET'!B23/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D14" s="10">
+        <f>IFERROR('BALANCE SHEET'!C23/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E14" s="10">
+        <f>IFERROR('BALANCE SHEET'!D23/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F14" s="12">
+        <f>E14</f>
+        <v/>
+      </c>
+      <c r="G14" s="12">
+        <f>F14</f>
+        <v/>
+      </c>
+      <c r="H14" s="12">
+        <f>G14</f>
+        <v/>
+      </c>
+      <c r="I14" s="12">
+        <f>H14</f>
+        <v/>
+      </c>
+      <c r="J14" s="12">
+        <f>I14</f>
+        <v/>
+      </c>
+      <c r="K14" s="12">
+        <f>J14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Accrued Promotional Allowance % of Rev</t>
+        </is>
+      </c>
+      <c r="C15" s="10">
+        <f>IFERROR('BALANCE SHEET'!B24/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D15" s="10">
+        <f>IFERROR('BALANCE SHEET'!C24/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="10">
+        <f>IFERROR('BALANCE SHEET'!D24/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="12">
+        <f>E15</f>
+        <v/>
+      </c>
+      <c r="G15" s="12">
+        <f>F15</f>
+        <v/>
+      </c>
+      <c r="H15" s="12">
+        <f>G15</f>
+        <v/>
+      </c>
+      <c r="I15" s="12">
+        <f>H15</f>
+        <v/>
+      </c>
+      <c r="J15" s="12">
+        <f>I15</f>
+        <v/>
+      </c>
+      <c r="K15" s="12">
+        <f>J15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Lease Liability - Operating - Current % of Rev</t>
+        </is>
+      </c>
+      <c r="C16" s="10">
+        <f>IFERROR('BALANCE SHEET'!B25/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D16" s="10">
+        <f>IFERROR('BALANCE SHEET'!C25/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="10">
+        <f>IFERROR('BALANCE SHEET'!D25/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="12">
+        <f>E16</f>
+        <v/>
+      </c>
+      <c r="G16" s="12">
+        <f>F16</f>
+        <v/>
+      </c>
+      <c r="H16" s="12">
+        <f>G16</f>
+        <v/>
+      </c>
+      <c r="I16" s="12">
+        <f>H16</f>
+        <v/>
+      </c>
+      <c r="J16" s="12">
+        <f>I16</f>
+        <v/>
+      </c>
+      <c r="K16" s="12">
+        <f>J16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Lease Liability - Finance - Current % of Rev</t>
+        </is>
+      </c>
+      <c r="C17" s="10">
+        <f>IFERROR('BALANCE SHEET'!B26/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D17" s="10">
+        <f>IFERROR('BALANCE SHEET'!C26/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E17" s="10">
+        <f>IFERROR('BALANCE SHEET'!D26/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="12">
+        <f>E17</f>
+        <v/>
+      </c>
+      <c r="G17" s="12">
+        <f>F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="12">
+        <f>G17</f>
+        <v/>
+      </c>
+      <c r="I17" s="12">
+        <f>H17</f>
+        <v/>
+      </c>
+      <c r="J17" s="12">
+        <f>I17</f>
+        <v/>
+      </c>
+      <c r="K17" s="12">
+        <f>J17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Deferred Revenue - Current % of Rev</t>
+        </is>
+      </c>
+      <c r="C18" s="10">
+        <f>IFERROR('BALANCE SHEET'!B27/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D18" s="10">
+        <f>IFERROR('BALANCE SHEET'!C27/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E18" s="10">
+        <f>IFERROR('BALANCE SHEET'!D27/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="12">
+        <f>E18</f>
+        <v/>
+      </c>
+      <c r="G18" s="12">
+        <f>F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="12">
+        <f>G18</f>
+        <v/>
+      </c>
+      <c r="I18" s="12">
+        <f>H18</f>
+        <v/>
+      </c>
+      <c r="J18" s="12">
+        <f>I18</f>
+        <v/>
+      </c>
+      <c r="K18" s="12">
+        <f>J18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Other Current Liabilities % of Rev</t>
+        </is>
+      </c>
+      <c r="C19" s="10">
+        <f>IFERROR('BALANCE SHEET'!B28/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
+      </c>
+      <c r="D19" s="10">
+        <f>IFERROR('BALANCE SHEET'!C28/'ANNL P&amp;L'!D2,0)</f>
+        <v/>
+      </c>
+      <c r="E19" s="10">
+        <f>IFERROR('BALANCE SHEET'!D28/'ANNL P&amp;L'!E2,0)</f>
+        <v/>
+      </c>
+      <c r="F19" s="12">
+        <f>E19</f>
+        <v/>
+      </c>
+      <c r="G19" s="12">
+        <f>F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="12">
+        <f>G19</f>
+        <v/>
+      </c>
+      <c r="I19" s="12">
+        <f>H19</f>
+        <v/>
+      </c>
+      <c r="J19" s="12">
+        <f>I19</f>
+        <v/>
+      </c>
+      <c r="K19" s="12">
+        <f>J19</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr"/>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>FY2025E</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>FY2026E</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>FY2027E</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>FY2028E</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>FY2029E</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>FY2030E</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>D&amp;A % of PP&amp;E</t>
+        </is>
+      </c>
+      <c r="D2" s="10">
+        <f>IFERROR('CASH FLOW'!D3/'BALANCE SHEET'!B11,0)</f>
+        <v/>
+      </c>
+      <c r="E2" s="10">
+        <f>IFERROR('CASH FLOW'!E3/'BALANCE SHEET'!C11,0)</f>
+        <v/>
+      </c>
+      <c r="F2" s="12">
+        <f>E2</f>
+        <v/>
+      </c>
+      <c r="G2" s="12">
+        <f>F2</f>
+        <v/>
+      </c>
+      <c r="H2" s="12">
+        <f>G2</f>
+        <v/>
+      </c>
+      <c r="I2" s="12">
+        <f>H2</f>
+        <v/>
+      </c>
+      <c r="J2" s="12">
+        <f>I2</f>
+        <v/>
+      </c>
+      <c r="K2" s="12">
+        <f>J2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
           <t>SBC $</t>
         </is>
       </c>
@@ -4177,41 +4712,69 @@
         <f>'CASH FLOW'!E9</f>
         <v/>
       </c>
-      <c r="F3" s="10" t="n"/>
-      <c r="G3" s="10" t="n"/>
-      <c r="H3" s="10" t="n"/>
-      <c r="I3" s="10" t="n"/>
-      <c r="J3" s="10" t="n"/>
-      <c r="K3" s="10" t="n"/>
+      <c r="F3" s="13">
+        <f>E3</f>
+        <v/>
+      </c>
+      <c r="G3" s="13">
+        <f>F3</f>
+        <v/>
+      </c>
+      <c r="H3" s="13">
+        <f>G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="13">
+        <f>H3</f>
+        <v/>
+      </c>
+      <c r="J3" s="13">
+        <f>I3</f>
+        <v/>
+      </c>
+      <c r="K3" s="13">
+        <f>J3</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>CapEx $</t>
-        </is>
-      </c>
-      <c r="B4" s="4">
-        <f>'CASH FLOW'!B28</f>
-        <v/>
-      </c>
-      <c r="C4" s="4">
-        <f>'CASH FLOW'!C28</f>
-        <v/>
-      </c>
-      <c r="D4" s="4">
-        <f>'CASH FLOW'!D28</f>
-        <v/>
-      </c>
-      <c r="E4" s="4">
-        <f>'CASH FLOW'!E28</f>
-        <v/>
-      </c>
-      <c r="F4" s="10" t="n"/>
-      <c r="G4" s="10" t="n"/>
-      <c r="H4" s="10" t="n"/>
-      <c r="I4" s="10" t="n"/>
-      <c r="J4" s="10" t="n"/>
-      <c r="K4" s="10" t="n"/>
+          <t>CapEx % of PP&amp;E</t>
+        </is>
+      </c>
+      <c r="D4" s="10">
+        <f>IFERROR('CASH FLOW'!D28/'BALANCE SHEET'!B11,0)</f>
+        <v/>
+      </c>
+      <c r="E4" s="10">
+        <f>IFERROR('CASH FLOW'!E28/'BALANCE SHEET'!C11,0)</f>
+        <v/>
+      </c>
+      <c r="F4" s="12">
+        <f>E4</f>
+        <v/>
+      </c>
+      <c r="G4" s="12">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="H4" s="12">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="12">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="J4" s="12">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="K4" s="12">
+        <f>J4</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -4219,24 +4782,42 @@
           <t>Preferred Dividends % of Preferred Balance</t>
         </is>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="10">
         <f>IFERROR('CASH FLOW'!C35/'BALANCE SHEET'!B35,0)</f>
         <v/>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="10">
         <f>IFERROR('CASH FLOW'!D35/'BALANCE SHEET'!C35,0)</f>
         <v/>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="10">
         <f>IFERROR('CASH FLOW'!E35/'BALANCE SHEET'!D35,0)</f>
         <v/>
       </c>
-      <c r="F5" s="9" t="n"/>
-      <c r="G5" s="9" t="n"/>
-      <c r="H5" s="9" t="n"/>
-      <c r="I5" s="9" t="n"/>
-      <c r="J5" s="9" t="n"/>
-      <c r="K5" s="9" t="n"/>
+      <c r="F5" s="12">
+        <f>E5</f>
+        <v/>
+      </c>
+      <c r="G5" s="12">
+        <f>F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="12">
+        <f>G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="12">
+        <f>H5</f>
+        <v/>
+      </c>
+      <c r="J5" s="12">
+        <f>I5</f>
+        <v/>
+      </c>
+      <c r="K5" s="12">
+        <f>J5</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -4244,12 +4825,30 @@
           <t>Common Dividends % of Net Income</t>
         </is>
       </c>
-      <c r="F6" s="9" t="n"/>
-      <c r="G6" s="9" t="n"/>
-      <c r="H6" s="9" t="n"/>
-      <c r="I6" s="9" t="n"/>
-      <c r="J6" s="9" t="n"/>
-      <c r="K6" s="9" t="n"/>
+      <c r="F6" s="12">
+        <f>E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="12">
+        <f>F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="12">
+        <f>G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="12">
+        <f>H6</f>
+        <v/>
+      </c>
+      <c r="J6" s="12">
+        <f>I6</f>
+        <v/>
+      </c>
+      <c r="K6" s="12">
+        <f>J6</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -4273,12 +4872,30 @@
         <f>'CASH FLOW'!E37</f>
         <v/>
       </c>
-      <c r="F7" s="10" t="n"/>
-      <c r="G7" s="10" t="n"/>
-      <c r="H7" s="10" t="n"/>
-      <c r="I7" s="10" t="n"/>
-      <c r="J7" s="10" t="n"/>
-      <c r="K7" s="10" t="n"/>
+      <c r="F7" s="13">
+        <f>ASSUMPTIONS!$B$3</f>
+        <v/>
+      </c>
+      <c r="G7" s="13">
+        <f>ASSUMPTIONS!$B$3</f>
+        <v/>
+      </c>
+      <c r="H7" s="13">
+        <f>ASSUMPTIONS!$B$3</f>
+        <v/>
+      </c>
+      <c r="I7" s="13">
+        <f>ASSUMPTIONS!$B$3</f>
+        <v/>
+      </c>
+      <c r="J7" s="13">
+        <f>ASSUMPTIONS!$B$3</f>
+        <v/>
+      </c>
+      <c r="K7" s="13">
+        <f>ASSUMPTIONS!$B$3</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -4298,12 +4915,30 @@
         <f>('BALANCE SHEET'!D25+'BALANCE SHEET'!D26+'BALANCE SHEET'!D30+'BALANCE SHEET'!D31)-('BALANCE SHEET'!D2+'BALANCE SHEET'!D3)</f>
         <v/>
       </c>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-      <c r="H8" s="10" t="n"/>
-      <c r="I8" s="10" t="n"/>
-      <c r="J8" s="10" t="n"/>
-      <c r="K8" s="10" t="n"/>
+      <c r="F8" s="13">
+        <f>('BALANCE SHEET'!E25+'BALANCE SHEET'!E26+'BALANCE SHEET'!E30+'BALANCE SHEET'!E31)-('BALANCE SHEET'!E2+'BALANCE SHEET'!E3)</f>
+        <v/>
+      </c>
+      <c r="G8" s="13">
+        <f>('BALANCE SHEET'!F25+'BALANCE SHEET'!F26+'BALANCE SHEET'!F30+'BALANCE SHEET'!F31)-('BALANCE SHEET'!F2+'BALANCE SHEET'!F3)</f>
+        <v/>
+      </c>
+      <c r="H8" s="13">
+        <f>('BALANCE SHEET'!G25+'BALANCE SHEET'!G26+'BALANCE SHEET'!G30+'BALANCE SHEET'!G31)-('BALANCE SHEET'!G2+'BALANCE SHEET'!G3)</f>
+        <v/>
+      </c>
+      <c r="I8" s="13">
+        <f>('BALANCE SHEET'!H25+'BALANCE SHEET'!H26+'BALANCE SHEET'!H30+'BALANCE SHEET'!H31)-('BALANCE SHEET'!H2+'BALANCE SHEET'!H3)</f>
+        <v/>
+      </c>
+      <c r="J8" s="13">
+        <f>('BALANCE SHEET'!I25+'BALANCE SHEET'!I26+'BALANCE SHEET'!I30+'BALANCE SHEET'!I31)-('BALANCE SHEET'!I2+'BALANCE SHEET'!I3)</f>
+        <v/>
+      </c>
+      <c r="K8" s="13">
+        <f>('BALANCE SHEET'!J25+'BALANCE SHEET'!J26+'BALANCE SHEET'!J30+'BALANCE SHEET'!J31)-('BALANCE SHEET'!J2+'BALANCE SHEET'!J3)</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 19:43:49
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -637,12 +637,30 @@
       <c r="E2" s="4" t="n">
         <v>1355630</v>
       </c>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="n"/>
-      <c r="J2" s="5" t="n"/>
-      <c r="K2" s="5" t="n"/>
+      <c r="F2" s="5">
+        <f>E2*(1+'IS DRIVERS'!F2)</f>
+        <v/>
+      </c>
+      <c r="G2" s="5">
+        <f>F2*(1+'IS DRIVERS'!G2)</f>
+        <v/>
+      </c>
+      <c r="H2" s="5">
+        <f>G2*(1+'IS DRIVERS'!H2)</f>
+        <v/>
+      </c>
+      <c r="I2" s="5">
+        <f>H2*(1+'IS DRIVERS'!I2)</f>
+        <v/>
+      </c>
+      <c r="J2" s="5">
+        <f>I2*(1+'IS DRIVERS'!J2)</f>
+        <v/>
+      </c>
+      <c r="K2" s="5">
+        <f>J2*(1+'IS DRIVERS'!K2)</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -662,12 +680,30 @@
       <c r="E3" s="4" t="n">
         <v>675423</v>
       </c>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="n"/>
+      <c r="F3" s="5">
+        <f>'IS DRIVERS'!F3*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G3" s="5">
+        <f>'IS DRIVERS'!G3*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H3" s="5">
+        <f>'IS DRIVERS'!H3*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I3" s="5">
+        <f>'IS DRIVERS'!I3*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J3" s="5">
+        <f>'IS DRIVERS'!J3*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
+      <c r="K3" s="5">
+        <f>'IS DRIVERS'!K3*'ANNL P&amp;L'!K2</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -734,12 +770,30 @@
       <c r="E5" s="4" t="n">
         <v>524479</v>
       </c>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
+      <c r="F5" s="5">
+        <f>'IS DRIVERS'!F4*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G5" s="5">
+        <f>'IS DRIVERS'!G4*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H5" s="5">
+        <f>'IS DRIVERS'!H4*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I5" s="5">
+        <f>'IS DRIVERS'!I4*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J5" s="5">
+        <f>'IS DRIVERS'!J4*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
+      <c r="K5" s="5">
+        <f>'IS DRIVERS'!K4*'ANNL P&amp;L'!K2</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -806,12 +860,30 @@
       <c r="E7" s="4" t="n">
         <v>-39263</v>
       </c>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
+      <c r="F7" s="5">
+        <f>'IS DRIVERS'!F5</f>
+        <v/>
+      </c>
+      <c r="G7" s="5">
+        <f>'IS DRIVERS'!G5</f>
+        <v/>
+      </c>
+      <c r="H7" s="5">
+        <f>'IS DRIVERS'!H5</f>
+        <v/>
+      </c>
+      <c r="I7" s="5">
+        <f>'IS DRIVERS'!I5</f>
+        <v/>
+      </c>
+      <c r="J7" s="5">
+        <f>'IS DRIVERS'!J5</f>
+        <v/>
+      </c>
+      <c r="K7" s="5">
+        <f>'IS DRIVERS'!K5</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -831,12 +903,30 @@
       <c r="E8" s="4" t="n">
         <v>1734</v>
       </c>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
+      <c r="F8" s="5">
+        <f>'IS DRIVERS'!F6</f>
+        <v/>
+      </c>
+      <c r="G8" s="5">
+        <f>'IS DRIVERS'!G6</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>'IS DRIVERS'!H6</f>
+        <v/>
+      </c>
+      <c r="I8" s="5">
+        <f>'IS DRIVERS'!I6</f>
+        <v/>
+      </c>
+      <c r="J8" s="5">
+        <f>'IS DRIVERS'!J6</f>
+        <v/>
+      </c>
+      <c r="K8" s="5">
+        <f>'IS DRIVERS'!K6</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -856,12 +946,30 @@
       <c r="E9" s="4" t="n">
         <v>-1793</v>
       </c>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
+      <c r="F9" s="5">
+        <f>'IS DRIVERS'!F7</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>'IS DRIVERS'!G7</f>
+        <v/>
+      </c>
+      <c r="H9" s="5">
+        <f>'IS DRIVERS'!H7</f>
+        <v/>
+      </c>
+      <c r="I9" s="5">
+        <f>'IS DRIVERS'!I7</f>
+        <v/>
+      </c>
+      <c r="J9" s="5">
+        <f>'IS DRIVERS'!J7</f>
+        <v/>
+      </c>
+      <c r="K9" s="5">
+        <f>'IS DRIVERS'!K7</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -928,12 +1036,30 @@
       <c r="E11" s="4" t="n">
         <v>49976</v>
       </c>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
+      <c r="F11" s="5">
+        <f>'ANNL P&amp;L'!F10*'IS DRIVERS'!F8</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>'ANNL P&amp;L'!G10*'IS DRIVERS'!G8</f>
+        <v/>
+      </c>
+      <c r="H11" s="5">
+        <f>'ANNL P&amp;L'!H10*'IS DRIVERS'!H8</f>
+        <v/>
+      </c>
+      <c r="I11" s="5">
+        <f>'ANNL P&amp;L'!I10*'IS DRIVERS'!I8</f>
+        <v/>
+      </c>
+      <c r="J11" s="5">
+        <f>'ANNL P&amp;L'!J10*'IS DRIVERS'!J8</f>
+        <v/>
+      </c>
+      <c r="K11" s="5">
+        <f>'ANNL P&amp;L'!K10*'IS DRIVERS'!K8</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1000,12 +1126,30 @@
       <c r="E13" s="4" t="n">
         <v>-27500</v>
       </c>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
+      <c r="F13" s="5">
+        <f>'CASH FLOW'!F35</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>'CASH FLOW'!G35</f>
+        <v/>
+      </c>
+      <c r="H13" s="5">
+        <f>'CASH FLOW'!H35</f>
+        <v/>
+      </c>
+      <c r="I13" s="5">
+        <f>'CASH FLOW'!I35</f>
+        <v/>
+      </c>
+      <c r="J13" s="5">
+        <f>'CASH FLOW'!J35</f>
+        <v/>
+      </c>
+      <c r="K13" s="5">
+        <f>'CASH FLOW'!K35</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1025,12 +1169,30 @@
       <c r="E14" s="4" t="n">
         <v>-10117</v>
       </c>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
-      <c r="K14" s="5" t="n"/>
+      <c r="F14" s="5">
+        <f>E14</f>
+        <v/>
+      </c>
+      <c r="G14" s="5">
+        <f>F14</f>
+        <v/>
+      </c>
+      <c r="H14" s="5">
+        <f>G14</f>
+        <v/>
+      </c>
+      <c r="I14" s="5">
+        <f>H14</f>
+        <v/>
+      </c>
+      <c r="J14" s="5">
+        <f>I14</f>
+        <v/>
+      </c>
+      <c r="K14" s="5">
+        <f>J14</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1050,12 +1212,30 @@
       <c r="E15" s="4" t="n">
         <v>107457</v>
       </c>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
-      <c r="K15" s="5" t="n"/>
+      <c r="F15" s="5">
+        <f>'ANNL P&amp;L'!F12+'ANNL P&amp;L'!F13+'ANNL P&amp;L'!F14</f>
+        <v/>
+      </c>
+      <c r="G15" s="5">
+        <f>'ANNL P&amp;L'!G12+'ANNL P&amp;L'!G13+'ANNL P&amp;L'!G14</f>
+        <v/>
+      </c>
+      <c r="H15" s="5">
+        <f>'ANNL P&amp;L'!H12+'ANNL P&amp;L'!H13+'ANNL P&amp;L'!H14</f>
+        <v/>
+      </c>
+      <c r="I15" s="5">
+        <f>'ANNL P&amp;L'!I12+'ANNL P&amp;L'!I13+'ANNL P&amp;L'!I14</f>
+        <v/>
+      </c>
+      <c r="J15" s="5">
+        <f>'ANNL P&amp;L'!J12+'ANNL P&amp;L'!J13+'ANNL P&amp;L'!J14</f>
+        <v/>
+      </c>
+      <c r="K15" s="5">
+        <f>'ANNL P&amp;L'!K12+'ANNL P&amp;L'!K13+'ANNL P&amp;L'!K14</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1125,12 +1305,30 @@
       <c r="E18" s="4" t="n">
         <v>233667</v>
       </c>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="5" t="n"/>
-      <c r="K18" s="5" t="n"/>
+      <c r="F18" s="5">
+        <f>E18</f>
+        <v/>
+      </c>
+      <c r="G18" s="5">
+        <f>F18</f>
+        <v/>
+      </c>
+      <c r="H18" s="5">
+        <f>G18</f>
+        <v/>
+      </c>
+      <c r="I18" s="5">
+        <f>H18</f>
+        <v/>
+      </c>
+      <c r="J18" s="5">
+        <f>I18</f>
+        <v/>
+      </c>
+      <c r="K18" s="5">
+        <f>J18</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1150,12 +1348,30 @@
       <c r="E19" s="4" t="n">
         <v>237404</v>
       </c>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="n"/>
-      <c r="I19" s="5" t="n"/>
-      <c r="J19" s="5" t="n"/>
-      <c r="K19" s="5" t="n"/>
+      <c r="F19" s="5">
+        <f>E19</f>
+        <v/>
+      </c>
+      <c r="G19" s="5">
+        <f>F19</f>
+        <v/>
+      </c>
+      <c r="H19" s="5">
+        <f>G19</f>
+        <v/>
+      </c>
+      <c r="I19" s="5">
+        <f>H19</f>
+        <v/>
+      </c>
+      <c r="J19" s="5">
+        <f>I19</f>
+        <v/>
+      </c>
+      <c r="K19" s="5">
+        <f>J19</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1246,12 +1462,30 @@
       <c r="D2" s="4" t="n">
         <v>890190</v>
       </c>
-      <c r="E2" s="5" t="n"/>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="n"/>
-      <c r="J2" s="5" t="n"/>
+      <c r="E2" s="5">
+        <f>D2+'CASH FLOW'!E40</f>
+        <v/>
+      </c>
+      <c r="F2" s="5">
+        <f>E2+'CASH FLOW'!F40</f>
+        <v/>
+      </c>
+      <c r="G2" s="5">
+        <f>F2+'CASH FLOW'!G40</f>
+        <v/>
+      </c>
+      <c r="H2" s="5">
+        <f>G2+'CASH FLOW'!H40</f>
+        <v/>
+      </c>
+      <c r="I2" s="5">
+        <f>H2+'CASH FLOW'!I40</f>
+        <v/>
+      </c>
+      <c r="J2" s="5">
+        <f>I2+'CASH FLOW'!J40</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1268,12 +1502,30 @@
       <c r="D3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
+      <c r="E3" s="5">
+        <f>D3</f>
+        <v/>
+      </c>
+      <c r="F3" s="5">
+        <f>E3</f>
+        <v/>
+      </c>
+      <c r="G3" s="5">
+        <f>F3</f>
+        <v/>
+      </c>
+      <c r="H3" s="5">
+        <f>G3</f>
+        <v/>
+      </c>
+      <c r="I3" s="5">
+        <f>H3</f>
+        <v/>
+      </c>
+      <c r="J3" s="5">
+        <f>I3</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1290,12 +1542,30 @@
       <c r="D4" s="4" t="n">
         <v>270342</v>
       </c>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
+      <c r="E4" s="5">
+        <f>'BS DRIVERS'!E3*'ANNL P&amp;L'!E2/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="F4" s="5">
+        <f>'BS DRIVERS'!F3*'ANNL P&amp;L'!F2/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="G4" s="5">
+        <f>'BS DRIVERS'!G3*'ANNL P&amp;L'!G2/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="H4" s="5">
+        <f>'BS DRIVERS'!H3*'ANNL P&amp;L'!H2/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="I4" s="5">
+        <f>'BS DRIVERS'!I3*'ANNL P&amp;L'!I2/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="J4" s="5">
+        <f>'BS DRIVERS'!J3*'ANNL P&amp;L'!J2/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1312,12 +1582,30 @@
       <c r="D5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
+      <c r="E5" s="5">
+        <f>'BS DRIVERS'!E5*'ANNL P&amp;L'!E2</f>
+        <v/>
+      </c>
+      <c r="F5" s="5">
+        <f>'BS DRIVERS'!F5*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G5" s="5">
+        <f>'BS DRIVERS'!G5*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H5" s="5">
+        <f>'BS DRIVERS'!H5*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I5" s="5">
+        <f>'BS DRIVERS'!I5*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J5" s="5">
+        <f>'BS DRIVERS'!J5*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -1334,12 +1622,30 @@
       <c r="D6" s="4" t="n">
         <v>131165</v>
       </c>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
+      <c r="E6" s="5">
+        <f>'BS DRIVERS'!E4*'ANNL P&amp;L'!E3/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="F6" s="5">
+        <f>'BS DRIVERS'!F4*'ANNL P&amp;L'!F3/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="G6" s="5">
+        <f>'BS DRIVERS'!G4*'ANNL P&amp;L'!G3/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="H6" s="5">
+        <f>'BS DRIVERS'!H4*'ANNL P&amp;L'!H3/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="I6" s="5">
+        <f>'BS DRIVERS'!I4*'ANNL P&amp;L'!I3/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="J6" s="5">
+        <f>'BS DRIVERS'!J4*'ANNL P&amp;L'!J3/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1356,12 +1662,30 @@
       <c r="D7" s="4" t="n">
         <v>14124</v>
       </c>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
+      <c r="E7" s="5">
+        <f>'BS DRIVERS'!E6*'ANNL P&amp;L'!E2</f>
+        <v/>
+      </c>
+      <c r="F7" s="5">
+        <f>'BS DRIVERS'!F6*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G7" s="5">
+        <f>'BS DRIVERS'!G6*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H7" s="5">
+        <f>'BS DRIVERS'!H6*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I7" s="5">
+        <f>'BS DRIVERS'!I6*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J7" s="5">
+        <f>'BS DRIVERS'!J6*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -1378,12 +1702,30 @@
       <c r="D8" s="4" t="n">
         <v>18759</v>
       </c>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
+      <c r="E8" s="5">
+        <f>'BS DRIVERS'!E7*'ANNL P&amp;L'!E2</f>
+        <v/>
+      </c>
+      <c r="F8" s="5">
+        <f>'BS DRIVERS'!F7*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G8" s="5">
+        <f>'BS DRIVERS'!G7*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>'BS DRIVERS'!H7*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I8" s="5">
+        <f>'BS DRIVERS'!I7*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J8" s="5">
+        <f>'BS DRIVERS'!J7*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1443,12 +1785,30 @@
       <c r="D10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
+      <c r="E10" s="5">
+        <f>D10</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>E10</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="5">
+        <f>G10</f>
+        <v/>
+      </c>
+      <c r="I10" s="5">
+        <f>H10</f>
+        <v/>
+      </c>
+      <c r="J10" s="5">
+        <f>I10</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1465,12 +1825,30 @@
       <c r="D11" s="4" t="n">
         <v>55602</v>
       </c>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
+      <c r="E11" s="5">
+        <f>D11-'CASH FLOW'!E28-'CASH FLOW'!E3</f>
+        <v/>
+      </c>
+      <c r="F11" s="5">
+        <f>E11-'CASH FLOW'!F28-'CASH FLOW'!F3</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>F11-'CASH FLOW'!G28-'CASH FLOW'!G3</f>
+        <v/>
+      </c>
+      <c r="H11" s="5">
+        <f>G11-'CASH FLOW'!H28-'CASH FLOW'!H3</f>
+        <v/>
+      </c>
+      <c r="I11" s="5">
+        <f>H11-'CASH FLOW'!I28-'CASH FLOW'!I3</f>
+        <v/>
+      </c>
+      <c r="J11" s="5">
+        <f>I11-'CASH FLOW'!J28-'CASH FLOW'!J3</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -1487,12 +1865,30 @@
       <c r="D12" s="4" t="n">
         <v>21606</v>
       </c>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
+      <c r="E12" s="5">
+        <f>D12</f>
+        <v/>
+      </c>
+      <c r="F12" s="5">
+        <f>E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="5">
+        <f>G12</f>
+        <v/>
+      </c>
+      <c r="I12" s="5">
+        <f>H12</f>
+        <v/>
+      </c>
+      <c r="J12" s="5">
+        <f>I12</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1509,12 +1905,30 @@
       <c r="D13" s="4" t="n">
         <v>230</v>
       </c>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
+      <c r="E13" s="5">
+        <f>D13</f>
+        <v/>
+      </c>
+      <c r="F13" s="5">
+        <f>E13</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="5">
+        <f>G13</f>
+        <v/>
+      </c>
+      <c r="I13" s="5">
+        <f>H13</f>
+        <v/>
+      </c>
+      <c r="J13" s="5">
+        <f>I13</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1531,12 +1945,30 @@
       <c r="D14" s="4" t="n">
         <v>12213</v>
       </c>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
+      <c r="E14" s="5">
+        <f>D14</f>
+        <v/>
+      </c>
+      <c r="F14" s="5">
+        <f>E14</f>
+        <v/>
+      </c>
+      <c r="G14" s="5">
+        <f>F14</f>
+        <v/>
+      </c>
+      <c r="H14" s="5">
+        <f>G14</f>
+        <v/>
+      </c>
+      <c r="I14" s="5">
+        <f>H14</f>
+        <v/>
+      </c>
+      <c r="J14" s="5">
+        <f>I14</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1553,12 +1985,30 @@
       <c r="D15" s="4" t="n">
         <v>71582</v>
       </c>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
+      <c r="E15" s="5">
+        <f>D15</f>
+        <v/>
+      </c>
+      <c r="F15" s="5">
+        <f>E15</f>
+        <v/>
+      </c>
+      <c r="G15" s="5">
+        <f>F15</f>
+        <v/>
+      </c>
+      <c r="H15" s="5">
+        <f>G15</f>
+        <v/>
+      </c>
+      <c r="I15" s="5">
+        <f>H15</f>
+        <v/>
+      </c>
+      <c r="J15" s="5">
+        <f>I15</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -1575,12 +2025,30 @@
       <c r="D16" s="4" t="n">
         <v>234215</v>
       </c>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
+      <c r="E16" s="5">
+        <f>D16-'CASH FLOW'!E6</f>
+        <v/>
+      </c>
+      <c r="F16" s="5">
+        <f>E16-'CASH FLOW'!F6</f>
+        <v/>
+      </c>
+      <c r="G16" s="5">
+        <f>F16-'CASH FLOW'!G6</f>
+        <v/>
+      </c>
+      <c r="H16" s="5">
+        <f>G16-'CASH FLOW'!H6</f>
+        <v/>
+      </c>
+      <c r="I16" s="5">
+        <f>H16-'CASH FLOW'!I6</f>
+        <v/>
+      </c>
+      <c r="J16" s="5">
+        <f>I16-'CASH FLOW'!J6</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1597,12 +2065,30 @@
       <c r="D17" s="4" t="n">
         <v>38699</v>
       </c>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
+      <c r="E17" s="5">
+        <f>D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="5">
+        <f>E17</f>
+        <v/>
+      </c>
+      <c r="G17" s="5">
+        <f>F17</f>
+        <v/>
+      </c>
+      <c r="H17" s="5">
+        <f>G17</f>
+        <v/>
+      </c>
+      <c r="I17" s="5">
+        <f>H17</f>
+        <v/>
+      </c>
+      <c r="J17" s="5">
+        <f>I17</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1619,12 +2105,30 @@
       <c r="D18" s="4" t="n">
         <v>8154</v>
       </c>
-      <c r="E18" s="5" t="n"/>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="5" t="n"/>
+      <c r="E18" s="5">
+        <f>'BS DRIVERS'!E9*'ANNL P&amp;L'!E2</f>
+        <v/>
+      </c>
+      <c r="F18" s="5">
+        <f>'BS DRIVERS'!F9*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G18" s="5">
+        <f>'BS DRIVERS'!G9*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H18" s="5">
+        <f>'BS DRIVERS'!H9*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I18" s="5">
+        <f>'BS DRIVERS'!I9*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J18" s="5">
+        <f>'BS DRIVERS'!J9*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1684,12 +2188,30 @@
       <c r="D20" s="4" t="n">
         <v>41287</v>
       </c>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="n"/>
-      <c r="I20" s="5" t="n"/>
-      <c r="J20" s="5" t="n"/>
+      <c r="E20" s="5">
+        <f>'BS DRIVERS'!E11*'ANNL P&amp;L'!E3/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="F20" s="5">
+        <f>'BS DRIVERS'!F11*'ANNL P&amp;L'!F3/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="G20" s="5">
+        <f>'BS DRIVERS'!G11*'ANNL P&amp;L'!G3/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="H20" s="5">
+        <f>'BS DRIVERS'!H11*'ANNL P&amp;L'!H3/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="I20" s="5">
+        <f>'BS DRIVERS'!I11*'ANNL P&amp;L'!I3/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
+      <c r="J20" s="5">
+        <f>'BS DRIVERS'!J11*'ANNL P&amp;L'!J3/ASSUMPTIONS!$B$2</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -1706,12 +2228,30 @@
       <c r="D21" s="4" t="n">
         <v>148780</v>
       </c>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="n"/>
-      <c r="I21" s="5" t="n"/>
-      <c r="J21" s="5" t="n"/>
+      <c r="E21" s="5">
+        <f>'BS DRIVERS'!E12*'ANNL P&amp;L'!E2</f>
+        <v/>
+      </c>
+      <c r="F21" s="5">
+        <f>'BS DRIVERS'!F12*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G21" s="5">
+        <f>'BS DRIVERS'!G12*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H21" s="5">
+        <f>'BS DRIVERS'!H12*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I21" s="5">
+        <f>'BS DRIVERS'!I12*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J21" s="5">
+        <f>'BS DRIVERS'!J12*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1728,12 +2268,30 @@
       <c r="D22" s="4" t="n">
         <v>10834</v>
       </c>
-      <c r="E22" s="5" t="n"/>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="5" t="n"/>
-      <c r="H22" s="5" t="n"/>
-      <c r="I22" s="5" t="n"/>
-      <c r="J22" s="5" t="n"/>
+      <c r="E22" s="5">
+        <f>'BS DRIVERS'!E13*'ANNL P&amp;L'!E2</f>
+        <v/>
+      </c>
+      <c r="F22" s="5">
+        <f>'BS DRIVERS'!F13*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G22" s="5">
+        <f>'BS DRIVERS'!G13*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H22" s="5">
+        <f>'BS DRIVERS'!H13*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I22" s="5">
+        <f>'BS DRIVERS'!I13*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J22" s="5">
+        <f>'BS DRIVERS'!J13*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1750,12 +2308,30 @@
       <c r="D23" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="5" t="n"/>
-      <c r="I23" s="5" t="n"/>
-      <c r="J23" s="5" t="n"/>
+      <c r="E23" s="5">
+        <f>'BS DRIVERS'!E14*'ANNL P&amp;L'!E2</f>
+        <v/>
+      </c>
+      <c r="F23" s="5">
+        <f>'BS DRIVERS'!F14*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G23" s="5">
+        <f>'BS DRIVERS'!G14*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H23" s="5">
+        <f>'BS DRIVERS'!H14*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I23" s="5">
+        <f>'BS DRIVERS'!I14*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J23" s="5">
+        <f>'BS DRIVERS'!J14*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1772,12 +2348,30 @@
       <c r="D24" s="4" t="n">
         <v>135948</v>
       </c>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="5" t="n"/>
-      <c r="I24" s="5" t="n"/>
-      <c r="J24" s="5" t="n"/>
+      <c r="E24" s="5">
+        <f>'BS DRIVERS'!E15*'ANNL P&amp;L'!E2</f>
+        <v/>
+      </c>
+      <c r="F24" s="5">
+        <f>'BS DRIVERS'!F15*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G24" s="5">
+        <f>'BS DRIVERS'!G15*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H24" s="5">
+        <f>'BS DRIVERS'!H15*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I24" s="5">
+        <f>'BS DRIVERS'!I15*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J24" s="5">
+        <f>'BS DRIVERS'!J15*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -1794,12 +2388,30 @@
       <c r="D25" s="4" t="n">
         <v>3265</v>
       </c>
-      <c r="E25" s="5" t="n"/>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="5" t="n"/>
-      <c r="I25" s="5" t="n"/>
-      <c r="J25" s="5" t="n"/>
+      <c r="E25" s="5">
+        <f>'BS DRIVERS'!E16*'ANNL P&amp;L'!E2</f>
+        <v/>
+      </c>
+      <c r="F25" s="5">
+        <f>'BS DRIVERS'!F16*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G25" s="5">
+        <f>'BS DRIVERS'!G16*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H25" s="5">
+        <f>'BS DRIVERS'!H16*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I25" s="5">
+        <f>'BS DRIVERS'!I16*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J25" s="5">
+        <f>'BS DRIVERS'!J16*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -1816,12 +2428,30 @@
       <c r="D26" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="E26" s="5" t="n"/>
-      <c r="F26" s="5" t="n"/>
-      <c r="G26" s="5" t="n"/>
-      <c r="H26" s="5" t="n"/>
-      <c r="I26" s="5" t="n"/>
-      <c r="J26" s="5" t="n"/>
+      <c r="E26" s="5">
+        <f>'BS DRIVERS'!E17*'ANNL P&amp;L'!E2</f>
+        <v/>
+      </c>
+      <c r="F26" s="5">
+        <f>'BS DRIVERS'!F17*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G26" s="5">
+        <f>'BS DRIVERS'!G17*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H26" s="5">
+        <f>'BS DRIVERS'!H17*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I26" s="5">
+        <f>'BS DRIVERS'!I17*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J26" s="5">
+        <f>'BS DRIVERS'!J17*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1838,12 +2468,30 @@
       <c r="D27" s="4" t="n">
         <v>9513</v>
       </c>
-      <c r="E27" s="5" t="n"/>
-      <c r="F27" s="5" t="n"/>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="5" t="n"/>
-      <c r="I27" s="5" t="n"/>
-      <c r="J27" s="5" t="n"/>
+      <c r="E27" s="5">
+        <f>'BS DRIVERS'!E18*'ANNL P&amp;L'!E2</f>
+        <v/>
+      </c>
+      <c r="F27" s="5">
+        <f>'BS DRIVERS'!F18*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G27" s="5">
+        <f>'BS DRIVERS'!G18*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H27" s="5">
+        <f>'BS DRIVERS'!H18*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I27" s="5">
+        <f>'BS DRIVERS'!I18*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J27" s="5">
+        <f>'BS DRIVERS'!J18*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -1860,12 +2508,30 @@
       <c r="D28" s="4" t="n">
         <v>15808</v>
       </c>
-      <c r="E28" s="5" t="n"/>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="n"/>
-      <c r="I28" s="5" t="n"/>
-      <c r="J28" s="5" t="n"/>
+      <c r="E28" s="5">
+        <f>'BS DRIVERS'!E19*'ANNL P&amp;L'!E2</f>
+        <v/>
+      </c>
+      <c r="F28" s="5">
+        <f>'BS DRIVERS'!F19*'ANNL P&amp;L'!F2</f>
+        <v/>
+      </c>
+      <c r="G28" s="5">
+        <f>'BS DRIVERS'!G19*'ANNL P&amp;L'!G2</f>
+        <v/>
+      </c>
+      <c r="H28" s="5">
+        <f>'BS DRIVERS'!H19*'ANNL P&amp;L'!H2</f>
+        <v/>
+      </c>
+      <c r="I28" s="5">
+        <f>'BS DRIVERS'!I19*'ANNL P&amp;L'!I2</f>
+        <v/>
+      </c>
+      <c r="J28" s="5">
+        <f>'BS DRIVERS'!J19*'ANNL P&amp;L'!J2</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -1925,12 +2591,30 @@
       <c r="D30" s="4" t="n">
         <v>16674</v>
       </c>
-      <c r="E30" s="5" t="n"/>
-      <c r="F30" s="5" t="n"/>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="5" t="n"/>
-      <c r="I30" s="5" t="n"/>
-      <c r="J30" s="5" t="n"/>
+      <c r="E30" s="5">
+        <f>D30</f>
+        <v/>
+      </c>
+      <c r="F30" s="5">
+        <f>E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="5">
+        <f>F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="5">
+        <f>G30</f>
+        <v/>
+      </c>
+      <c r="I30" s="5">
+        <f>H30</f>
+        <v/>
+      </c>
+      <c r="J30" s="5">
+        <f>I30</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -1947,12 +2631,30 @@
       <c r="D31" s="4" t="n">
         <v>211</v>
       </c>
-      <c r="E31" s="5" t="n"/>
-      <c r="F31" s="5" t="n"/>
-      <c r="G31" s="5" t="n"/>
-      <c r="H31" s="5" t="n"/>
-      <c r="I31" s="5" t="n"/>
-      <c r="J31" s="5" t="n"/>
+      <c r="E31" s="5">
+        <f>D31</f>
+        <v/>
+      </c>
+      <c r="F31" s="5">
+        <f>E31</f>
+        <v/>
+      </c>
+      <c r="G31" s="5">
+        <f>F31</f>
+        <v/>
+      </c>
+      <c r="H31" s="5">
+        <f>G31</f>
+        <v/>
+      </c>
+      <c r="I31" s="5">
+        <f>H31</f>
+        <v/>
+      </c>
+      <c r="J31" s="5">
+        <f>I31</f>
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -1969,12 +2671,30 @@
       <c r="D32" s="4" t="n">
         <v>2330</v>
       </c>
-      <c r="E32" s="5" t="n"/>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="5" t="n"/>
-      <c r="H32" s="5" t="n"/>
-      <c r="I32" s="5" t="n"/>
-      <c r="J32" s="5" t="n"/>
+      <c r="E32" s="5">
+        <f>D32</f>
+        <v/>
+      </c>
+      <c r="F32" s="5">
+        <f>E32</f>
+        <v/>
+      </c>
+      <c r="G32" s="5">
+        <f>F32</f>
+        <v/>
+      </c>
+      <c r="H32" s="5">
+        <f>G32</f>
+        <v/>
+      </c>
+      <c r="I32" s="5">
+        <f>H32</f>
+        <v/>
+      </c>
+      <c r="J32" s="5">
+        <f>I32</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -1991,12 +2711,30 @@
       <c r="D33" s="4" t="n">
         <v>157714</v>
       </c>
-      <c r="E33" s="5" t="n"/>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="5" t="n"/>
-      <c r="I33" s="5" t="n"/>
-      <c r="J33" s="5" t="n"/>
+      <c r="E33" s="5">
+        <f>D33</f>
+        <v/>
+      </c>
+      <c r="F33" s="5">
+        <f>E33</f>
+        <v/>
+      </c>
+      <c r="G33" s="5">
+        <f>F33</f>
+        <v/>
+      </c>
+      <c r="H33" s="5">
+        <f>G33</f>
+        <v/>
+      </c>
+      <c r="I33" s="5">
+        <f>H33</f>
+        <v/>
+      </c>
+      <c r="J33" s="5">
+        <f>I33</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -2056,12 +2794,30 @@
       <c r="D35" s="4" t="n">
         <v>824488</v>
       </c>
-      <c r="E35" s="5" t="n"/>
-      <c r="F35" s="5" t="n"/>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="5" t="n"/>
-      <c r="I35" s="5" t="n"/>
-      <c r="J35" s="5" t="n"/>
+      <c r="E35" s="5">
+        <f>D35</f>
+        <v/>
+      </c>
+      <c r="F35" s="5">
+        <f>E35</f>
+        <v/>
+      </c>
+      <c r="G35" s="5">
+        <f>F35</f>
+        <v/>
+      </c>
+      <c r="H35" s="5">
+        <f>G35</f>
+        <v/>
+      </c>
+      <c r="I35" s="5">
+        <f>H35</f>
+        <v/>
+      </c>
+      <c r="J35" s="5">
+        <f>I35</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -2078,12 +2834,30 @@
       <c r="D36" s="4" t="n">
         <v>79</v>
       </c>
-      <c r="E36" s="5" t="n"/>
-      <c r="F36" s="5" t="n"/>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="5" t="n"/>
-      <c r="I36" s="5" t="n"/>
-      <c r="J36" s="5" t="n"/>
+      <c r="E36" s="5">
+        <f>D36</f>
+        <v/>
+      </c>
+      <c r="F36" s="5">
+        <f>E36</f>
+        <v/>
+      </c>
+      <c r="G36" s="5">
+        <f>F36</f>
+        <v/>
+      </c>
+      <c r="H36" s="5">
+        <f>G36</f>
+        <v/>
+      </c>
+      <c r="I36" s="5">
+        <f>H36</f>
+        <v/>
+      </c>
+      <c r="J36" s="5">
+        <f>I36</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -2100,12 +2874,30 @@
       <c r="D37" s="4" t="n">
         <v>297579</v>
       </c>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="5" t="n"/>
-      <c r="I37" s="5" t="n"/>
-      <c r="J37" s="5" t="n"/>
+      <c r="E37" s="5">
+        <f>D37+'CASH FLOW'!E9</f>
+        <v/>
+      </c>
+      <c r="F37" s="5">
+        <f>E37+'CASH FLOW'!F9</f>
+        <v/>
+      </c>
+      <c r="G37" s="5">
+        <f>F37+'CASH FLOW'!G9</f>
+        <v/>
+      </c>
+      <c r="H37" s="5">
+        <f>G37+'CASH FLOW'!H9</f>
+        <v/>
+      </c>
+      <c r="I37" s="5">
+        <f>H37+'CASH FLOW'!I9</f>
+        <v/>
+      </c>
+      <c r="J37" s="5">
+        <f>I37+'CASH FLOW'!J9</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -2122,12 +2914,30 @@
       <c r="D38" s="4" t="n">
         <v>-3250</v>
       </c>
-      <c r="E38" s="5" t="n"/>
-      <c r="F38" s="5" t="n"/>
-      <c r="G38" s="5" t="n"/>
-      <c r="H38" s="5" t="n"/>
-      <c r="I38" s="5" t="n"/>
-      <c r="J38" s="5" t="n"/>
+      <c r="E38" s="5">
+        <f>D38</f>
+        <v/>
+      </c>
+      <c r="F38" s="5">
+        <f>E38</f>
+        <v/>
+      </c>
+      <c r="G38" s="5">
+        <f>F38</f>
+        <v/>
+      </c>
+      <c r="H38" s="5">
+        <f>G38</f>
+        <v/>
+      </c>
+      <c r="I38" s="5">
+        <f>H38</f>
+        <v/>
+      </c>
+      <c r="J38" s="5">
+        <f>I38</f>
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
@@ -2144,12 +2954,30 @@
       <c r="D39" s="4" t="n">
         <v>105521</v>
       </c>
-      <c r="E39" s="5" t="n"/>
-      <c r="F39" s="5" t="n"/>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="5" t="n"/>
-      <c r="I39" s="5" t="n"/>
-      <c r="J39" s="5" t="n"/>
+      <c r="E39" s="5">
+        <f>D39+'ANNL P&amp;L'!E12+'CASH FLOW'!E35</f>
+        <v/>
+      </c>
+      <c r="F39" s="5">
+        <f>E39+'ANNL P&amp;L'!F12+'CASH FLOW'!F35</f>
+        <v/>
+      </c>
+      <c r="G39" s="5">
+        <f>F39+'ANNL P&amp;L'!G12+'CASH FLOW'!G35</f>
+        <v/>
+      </c>
+      <c r="H39" s="5">
+        <f>G39+'ANNL P&amp;L'!H12+'CASH FLOW'!H35</f>
+        <v/>
+      </c>
+      <c r="I39" s="5">
+        <f>H39+'ANNL P&amp;L'!I12+'CASH FLOW'!I35</f>
+        <v/>
+      </c>
+      <c r="J39" s="5">
+        <f>I39+'ANNL P&amp;L'!J12+'CASH FLOW'!J35</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -2335,12 +3163,30 @@
       <c r="E2" s="4" t="n">
         <v>145074</v>
       </c>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="n"/>
-      <c r="J2" s="5" t="n"/>
-      <c r="K2" s="5" t="n"/>
+      <c r="F2" s="5">
+        <f>'ANNL P&amp;L'!F12</f>
+        <v/>
+      </c>
+      <c r="G2" s="5">
+        <f>'ANNL P&amp;L'!G12</f>
+        <v/>
+      </c>
+      <c r="H2" s="5">
+        <f>'ANNL P&amp;L'!H12</f>
+        <v/>
+      </c>
+      <c r="I2" s="5">
+        <f>'ANNL P&amp;L'!I12</f>
+        <v/>
+      </c>
+      <c r="J2" s="5">
+        <f>'ANNL P&amp;L'!J12</f>
+        <v/>
+      </c>
+      <c r="K2" s="5">
+        <f>'ANNL P&amp;L'!K12</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -2360,12 +3206,30 @@
       <c r="E3" s="4" t="n">
         <v>7274</v>
       </c>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="n"/>
-      <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="n"/>
+      <c r="F3" s="5">
+        <f>'CF DRIVERS'!F2*'BALANCE SHEET'!D11</f>
+        <v/>
+      </c>
+      <c r="G3" s="5">
+        <f>'CF DRIVERS'!G2*'BALANCE SHEET'!E11</f>
+        <v/>
+      </c>
+      <c r="H3" s="5">
+        <f>'CF DRIVERS'!H2*'BALANCE SHEET'!F11</f>
+        <v/>
+      </c>
+      <c r="I3" s="5">
+        <f>'CF DRIVERS'!I2*'BALANCE SHEET'!G11</f>
+        <v/>
+      </c>
+      <c r="J3" s="5">
+        <f>'CF DRIVERS'!J2*'BALANCE SHEET'!H11</f>
+        <v/>
+      </c>
+      <c r="K3" s="5">
+        <f>'CF DRIVERS'!K2*'BALANCE SHEET'!I11</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -2385,12 +3249,30 @@
       <c r="E4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-      <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
+      <c r="F4" s="5">
+        <f>E4</f>
+        <v/>
+      </c>
+      <c r="G4" s="5">
+        <f>F4</f>
+        <v/>
+      </c>
+      <c r="H4" s="5">
+        <f>G4</f>
+        <v/>
+      </c>
+      <c r="I4" s="5">
+        <f>H4</f>
+        <v/>
+      </c>
+      <c r="J4" s="5">
+        <f>I4</f>
+        <v/>
+      </c>
+      <c r="K4" s="5">
+        <f>J4</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -2410,12 +3292,30 @@
       <c r="E5" s="4" t="n">
         <v>3294</v>
       </c>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="n"/>
-      <c r="J5" s="5" t="n"/>
-      <c r="K5" s="5" t="n"/>
+      <c r="F5" s="5">
+        <f>E5</f>
+        <v/>
+      </c>
+      <c r="G5" s="5">
+        <f>F5</f>
+        <v/>
+      </c>
+      <c r="H5" s="5">
+        <f>G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="5">
+        <f>H5</f>
+        <v/>
+      </c>
+      <c r="J5" s="5">
+        <f>I5</f>
+        <v/>
+      </c>
+      <c r="K5" s="5">
+        <f>J5</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -2435,12 +3335,30 @@
       <c r="E6" s="4" t="n">
         <v>14124</v>
       </c>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="n"/>
+      <c r="F6" s="5">
+        <f>E6</f>
+        <v/>
+      </c>
+      <c r="G6" s="5">
+        <f>F6</f>
+        <v/>
+      </c>
+      <c r="H6" s="5">
+        <f>G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="5">
+        <f>H6</f>
+        <v/>
+      </c>
+      <c r="J6" s="5">
+        <f>I6</f>
+        <v/>
+      </c>
+      <c r="K6" s="5">
+        <f>J6</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -2460,12 +3378,30 @@
       <c r="E7" s="4" t="n">
         <v>19086</v>
       </c>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
+      <c r="F7" s="5">
+        <f>E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="5">
+        <f>F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="5">
+        <f>G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="5">
+        <f>H7</f>
+        <v/>
+      </c>
+      <c r="J7" s="5">
+        <f>I7</f>
+        <v/>
+      </c>
+      <c r="K7" s="5">
+        <f>J7</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -2485,12 +3421,30 @@
       <c r="E8" s="4" t="n">
         <v>173</v>
       </c>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="n"/>
-      <c r="J8" s="5" t="n"/>
-      <c r="K8" s="5" t="n"/>
+      <c r="F8" s="5">
+        <f>E8</f>
+        <v/>
+      </c>
+      <c r="G8" s="5">
+        <f>F8</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>G8</f>
+        <v/>
+      </c>
+      <c r="I8" s="5">
+        <f>H8</f>
+        <v/>
+      </c>
+      <c r="J8" s="5">
+        <f>I8</f>
+        <v/>
+      </c>
+      <c r="K8" s="5">
+        <f>J8</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -2510,12 +3464,30 @@
       <c r="E9" s="4" t="n">
         <v>19591</v>
       </c>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
+      <c r="F9" s="5">
+        <f>'CF DRIVERS'!F3</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>'CF DRIVERS'!G3</f>
+        <v/>
+      </c>
+      <c r="H9" s="5">
+        <f>'CF DRIVERS'!H3</f>
+        <v/>
+      </c>
+      <c r="I9" s="5">
+        <f>'CF DRIVERS'!I3</f>
+        <v/>
+      </c>
+      <c r="J9" s="5">
+        <f>'CF DRIVERS'!J3</f>
+        <v/>
+      </c>
+      <c r="K9" s="5">
+        <f>'CF DRIVERS'!K3</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -2535,12 +3507,30 @@
       <c r="E10" s="4" t="n">
         <v>-9730</v>
       </c>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
+      <c r="F10" s="5">
+        <f>E10</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>F10</f>
+        <v/>
+      </c>
+      <c r="H10" s="5">
+        <f>G10</f>
+        <v/>
+      </c>
+      <c r="I10" s="5">
+        <f>H10</f>
+        <v/>
+      </c>
+      <c r="J10" s="5">
+        <f>I10</f>
+        <v/>
+      </c>
+      <c r="K10" s="5">
+        <f>J10</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -2560,12 +3550,30 @@
       <c r="E11" s="4" t="n">
         <v>1734</v>
       </c>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
+      <c r="F11" s="5">
+        <f>E11</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>F11</f>
+        <v/>
+      </c>
+      <c r="H11" s="5">
+        <f>G11</f>
+        <v/>
+      </c>
+      <c r="I11" s="5">
+        <f>H11</f>
+        <v/>
+      </c>
+      <c r="J11" s="5">
+        <f>I11</f>
+        <v/>
+      </c>
+      <c r="K11" s="5">
+        <f>J11</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -2585,12 +3593,30 @@
       <c r="E12" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
-      <c r="K12" s="5" t="n"/>
+      <c r="F12" s="5">
+        <f>E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>F12</f>
+        <v/>
+      </c>
+      <c r="H12" s="5">
+        <f>G12</f>
+        <v/>
+      </c>
+      <c r="I12" s="5">
+        <f>H12</f>
+        <v/>
+      </c>
+      <c r="J12" s="5">
+        <f>I12</f>
+        <v/>
+      </c>
+      <c r="K12" s="5">
+        <f>J12</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -2610,12 +3636,30 @@
       <c r="E13" s="4" t="n">
         <v>-324</v>
       </c>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
+      <c r="F13" s="5">
+        <f>E13</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>F13</f>
+        <v/>
+      </c>
+      <c r="H13" s="5">
+        <f>G13</f>
+        <v/>
+      </c>
+      <c r="I13" s="5">
+        <f>H13</f>
+        <v/>
+      </c>
+      <c r="J13" s="5">
+        <f>I13</f>
+        <v/>
+      </c>
+      <c r="K13" s="5">
+        <f>J13</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -2635,12 +3679,30 @@
       <c r="E14" s="4" t="n">
         <v>-89665</v>
       </c>
-      <c r="F14" s="5" t="n"/>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="5" t="n"/>
-      <c r="J14" s="5" t="n"/>
-      <c r="K14" s="5" t="n"/>
+      <c r="F14" s="5">
+        <f>-('BALANCE SHEET'!E4-'BALANCE SHEET'!D4)</f>
+        <v/>
+      </c>
+      <c r="G14" s="5">
+        <f>-('BALANCE SHEET'!F4-'BALANCE SHEET'!E4)</f>
+        <v/>
+      </c>
+      <c r="H14" s="5">
+        <f>-('BALANCE SHEET'!G4-'BALANCE SHEET'!F4)</f>
+        <v/>
+      </c>
+      <c r="I14" s="5">
+        <f>-('BALANCE SHEET'!H4-'BALANCE SHEET'!G4)</f>
+        <v/>
+      </c>
+      <c r="J14" s="5">
+        <f>-('BALANCE SHEET'!I4-'BALANCE SHEET'!H4)</f>
+        <v/>
+      </c>
+      <c r="K14" s="5">
+        <f>-('BALANCE SHEET'!J4-'BALANCE SHEET'!I4)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -2660,12 +3722,30 @@
       <c r="E15" s="4" t="n">
         <v>2318</v>
       </c>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
-      <c r="K15" s="5" t="n"/>
+      <c r="F15" s="5">
+        <f>-('BALANCE SHEET'!E5-'BALANCE SHEET'!D5)</f>
+        <v/>
+      </c>
+      <c r="G15" s="5">
+        <f>-('BALANCE SHEET'!F5-'BALANCE SHEET'!E5)</f>
+        <v/>
+      </c>
+      <c r="H15" s="5">
+        <f>-('BALANCE SHEET'!G5-'BALANCE SHEET'!F5)</f>
+        <v/>
+      </c>
+      <c r="I15" s="5">
+        <f>-('BALANCE SHEET'!H5-'BALANCE SHEET'!G5)</f>
+        <v/>
+      </c>
+      <c r="J15" s="5">
+        <f>-('BALANCE SHEET'!I5-'BALANCE SHEET'!H5)</f>
+        <v/>
+      </c>
+      <c r="K15" s="5">
+        <f>-('BALANCE SHEET'!J5-'BALANCE SHEET'!I5)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -2685,12 +3765,30 @@
       <c r="E16" s="4" t="n">
         <v>77190</v>
       </c>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
-      <c r="K16" s="5" t="n"/>
+      <c r="F16" s="5">
+        <f>-('BALANCE SHEET'!E6-'BALANCE SHEET'!D6)</f>
+        <v/>
+      </c>
+      <c r="G16" s="5">
+        <f>-('BALANCE SHEET'!F6-'BALANCE SHEET'!E6)</f>
+        <v/>
+      </c>
+      <c r="H16" s="5">
+        <f>-('BALANCE SHEET'!G6-'BALANCE SHEET'!F6)</f>
+        <v/>
+      </c>
+      <c r="I16" s="5">
+        <f>-('BALANCE SHEET'!H6-'BALANCE SHEET'!G6)</f>
+        <v/>
+      </c>
+      <c r="J16" s="5">
+        <f>-('BALANCE SHEET'!I6-'BALANCE SHEET'!H6)</f>
+        <v/>
+      </c>
+      <c r="K16" s="5">
+        <f>-('BALANCE SHEET'!J6-'BALANCE SHEET'!I6)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -2710,12 +3808,30 @@
       <c r="E17" s="4" t="n">
         <v>1074</v>
       </c>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="n"/>
+      <c r="F17" s="5">
+        <f>-('BALANCE SHEET'!E8-'BALANCE SHEET'!D8)</f>
+        <v/>
+      </c>
+      <c r="G17" s="5">
+        <f>-('BALANCE SHEET'!F8-'BALANCE SHEET'!E8)</f>
+        <v/>
+      </c>
+      <c r="H17" s="5">
+        <f>-('BALANCE SHEET'!G8-'BALANCE SHEET'!F8)</f>
+        <v/>
+      </c>
+      <c r="I17" s="5">
+        <f>-('BALANCE SHEET'!H8-'BALANCE SHEET'!G8)</f>
+        <v/>
+      </c>
+      <c r="J17" s="5">
+        <f>-('BALANCE SHEET'!I8-'BALANCE SHEET'!H8)</f>
+        <v/>
+      </c>
+      <c r="K17" s="5">
+        <f>-('BALANCE SHEET'!J8-'BALANCE SHEET'!I8)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -2735,12 +3851,30 @@
       <c r="E18" s="4" t="n">
         <v>-1170</v>
       </c>
-      <c r="F18" s="5" t="n"/>
-      <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="n"/>
-      <c r="I18" s="5" t="n"/>
-      <c r="J18" s="5" t="n"/>
-      <c r="K18" s="5" t="n"/>
+      <c r="F18" s="5">
+        <f>('BALANCE SHEET'!E20-'BALANCE SHEET'!D20)</f>
+        <v/>
+      </c>
+      <c r="G18" s="5">
+        <f>('BALANCE SHEET'!F20-'BALANCE SHEET'!E20)</f>
+        <v/>
+      </c>
+      <c r="H18" s="5">
+        <f>('BALANCE SHEET'!G20-'BALANCE SHEET'!F20)</f>
+        <v/>
+      </c>
+      <c r="I18" s="5">
+        <f>('BALANCE SHEET'!H20-'BALANCE SHEET'!G20)</f>
+        <v/>
+      </c>
+      <c r="J18" s="5">
+        <f>('BALANCE SHEET'!I20-'BALANCE SHEET'!H20)</f>
+        <v/>
+      </c>
+      <c r="K18" s="5">
+        <f>('BALANCE SHEET'!J20-'BALANCE SHEET'!I20)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -2760,12 +3894,30 @@
       <c r="E19" s="4" t="n">
         <v>85398</v>
       </c>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="n"/>
-      <c r="I19" s="5" t="n"/>
-      <c r="J19" s="5" t="n"/>
-      <c r="K19" s="5" t="n"/>
+      <c r="F19" s="5">
+        <f>('BALANCE SHEET'!E21-'BALANCE SHEET'!D21)</f>
+        <v/>
+      </c>
+      <c r="G19" s="5">
+        <f>('BALANCE SHEET'!F21-'BALANCE SHEET'!E21)</f>
+        <v/>
+      </c>
+      <c r="H19" s="5">
+        <f>('BALANCE SHEET'!G21-'BALANCE SHEET'!F21)</f>
+        <v/>
+      </c>
+      <c r="I19" s="5">
+        <f>('BALANCE SHEET'!H21-'BALANCE SHEET'!G21)</f>
+        <v/>
+      </c>
+      <c r="J19" s="5">
+        <f>('BALANCE SHEET'!I21-'BALANCE SHEET'!H21)</f>
+        <v/>
+      </c>
+      <c r="K19" s="5">
+        <f>('BALANCE SHEET'!J21-'BALANCE SHEET'!I21)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -2785,12 +3937,30 @@
       <c r="E20" s="4" t="n">
         <v>-34616</v>
       </c>
-      <c r="F20" s="5" t="n"/>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="n"/>
-      <c r="I20" s="5" t="n"/>
-      <c r="J20" s="5" t="n"/>
-      <c r="K20" s="5" t="n"/>
+      <c r="F20" s="5">
+        <f>('BALANCE SHEET'!E28-'BALANCE SHEET'!D28)</f>
+        <v/>
+      </c>
+      <c r="G20" s="5">
+        <f>('BALANCE SHEET'!F28-'BALANCE SHEET'!E28)</f>
+        <v/>
+      </c>
+      <c r="H20" s="5">
+        <f>('BALANCE SHEET'!G28-'BALANCE SHEET'!F28)</f>
+        <v/>
+      </c>
+      <c r="I20" s="5">
+        <f>('BALANCE SHEET'!H28-'BALANCE SHEET'!G28)</f>
+        <v/>
+      </c>
+      <c r="J20" s="5">
+        <f>('BALANCE SHEET'!I28-'BALANCE SHEET'!H28)</f>
+        <v/>
+      </c>
+      <c r="K20" s="5">
+        <f>('BALANCE SHEET'!J28-'BALANCE SHEET'!I28)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -2810,12 +3980,30 @@
       <c r="E21" s="4" t="n">
         <v>36161</v>
       </c>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="n"/>
-      <c r="I21" s="5" t="n"/>
-      <c r="J21" s="5" t="n"/>
-      <c r="K21" s="5" t="n"/>
+      <c r="F21" s="5">
+        <f>('BALANCE SHEET'!E24-'BALANCE SHEET'!D24)</f>
+        <v/>
+      </c>
+      <c r="G21" s="5">
+        <f>('BALANCE SHEET'!F24-'BALANCE SHEET'!E24)</f>
+        <v/>
+      </c>
+      <c r="H21" s="5">
+        <f>('BALANCE SHEET'!G24-'BALANCE SHEET'!F24)</f>
+        <v/>
+      </c>
+      <c r="I21" s="5">
+        <f>('BALANCE SHEET'!H24-'BALANCE SHEET'!G24)</f>
+        <v/>
+      </c>
+      <c r="J21" s="5">
+        <f>('BALANCE SHEET'!I24-'BALANCE SHEET'!H24)</f>
+        <v/>
+      </c>
+      <c r="K21" s="5">
+        <f>('BALANCE SHEET'!J24-'BALANCE SHEET'!I24)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -2835,12 +4023,30 @@
       <c r="E22" s="4" t="n">
         <v>-248</v>
       </c>
-      <c r="F22" s="5" t="n"/>
-      <c r="G22" s="5" t="n"/>
-      <c r="H22" s="5" t="n"/>
-      <c r="I22" s="5" t="n"/>
-      <c r="J22" s="5" t="n"/>
-      <c r="K22" s="5" t="n"/>
+      <c r="F22" s="5">
+        <f>('BALANCE SHEET'!E23-'BALANCE SHEET'!D23)</f>
+        <v/>
+      </c>
+      <c r="G22" s="5">
+        <f>('BALANCE SHEET'!F23-'BALANCE SHEET'!E23)</f>
+        <v/>
+      </c>
+      <c r="H22" s="5">
+        <f>('BALANCE SHEET'!G23-'BALANCE SHEET'!F23)</f>
+        <v/>
+      </c>
+      <c r="I22" s="5">
+        <f>('BALANCE SHEET'!H23-'BALANCE SHEET'!G23)</f>
+        <v/>
+      </c>
+      <c r="J22" s="5">
+        <f>('BALANCE SHEET'!I23-'BALANCE SHEET'!H23)</f>
+        <v/>
+      </c>
+      <c r="K22" s="5">
+        <f>('BALANCE SHEET'!J23-'BALANCE SHEET'!I23)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -2860,12 +4066,30 @@
       <c r="E23" s="4" t="n">
         <v>535</v>
       </c>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="5" t="n"/>
-      <c r="I23" s="5" t="n"/>
-      <c r="J23" s="5" t="n"/>
-      <c r="K23" s="5" t="n"/>
+      <c r="F23" s="5">
+        <f>E23</f>
+        <v/>
+      </c>
+      <c r="G23" s="5">
+        <f>F23</f>
+        <v/>
+      </c>
+      <c r="H23" s="5">
+        <f>G23</f>
+        <v/>
+      </c>
+      <c r="I23" s="5">
+        <f>H23</f>
+        <v/>
+      </c>
+      <c r="J23" s="5">
+        <f>I23</f>
+        <v/>
+      </c>
+      <c r="K23" s="5">
+        <f>J23</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -2885,12 +4109,30 @@
       <c r="E24" s="4" t="n">
         <v>-9513</v>
       </c>
-      <c r="F24" s="5" t="n"/>
-      <c r="G24" s="5" t="n"/>
-      <c r="H24" s="5" t="n"/>
-      <c r="I24" s="5" t="n"/>
-      <c r="J24" s="5" t="n"/>
-      <c r="K24" s="5" t="n"/>
+      <c r="F24" s="5">
+        <f>(('BALANCE SHEET'!E27+'BALANCE SHEET'!E33)-('BALANCE SHEET'!D27+'BALANCE SHEET'!D33))</f>
+        <v/>
+      </c>
+      <c r="G24" s="5">
+        <f>(('BALANCE SHEET'!F27+'BALANCE SHEET'!F33)-('BALANCE SHEET'!E27+'BALANCE SHEET'!E33))</f>
+        <v/>
+      </c>
+      <c r="H24" s="5">
+        <f>(('BALANCE SHEET'!G27+'BALANCE SHEET'!G33)-('BALANCE SHEET'!F27+'BALANCE SHEET'!F33))</f>
+        <v/>
+      </c>
+      <c r="I24" s="5">
+        <f>(('BALANCE SHEET'!H27+'BALANCE SHEET'!H33)-('BALANCE SHEET'!G27+'BALANCE SHEET'!G33))</f>
+        <v/>
+      </c>
+      <c r="J24" s="5">
+        <f>(('BALANCE SHEET'!I27+'BALANCE SHEET'!I33)-('BALANCE SHEET'!H27+'BALANCE SHEET'!H33))</f>
+        <v/>
+      </c>
+      <c r="K24" s="5">
+        <f>(('BALANCE SHEET'!J27+'BALANCE SHEET'!J33)-('BALANCE SHEET'!I27+'BALANCE SHEET'!I33))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -2910,12 +4152,30 @@
       <c r="E25" s="4" t="n">
         <v>-4862</v>
       </c>
-      <c r="F25" s="5" t="n"/>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="5" t="n"/>
-      <c r="I25" s="5" t="n"/>
-      <c r="J25" s="5" t="n"/>
-      <c r="K25" s="5" t="n"/>
+      <c r="F25" s="5">
+        <f>-('BALANCE SHEET'!E18-'BALANCE SHEET'!D18)</f>
+        <v/>
+      </c>
+      <c r="G25" s="5">
+        <f>-('BALANCE SHEET'!F18-'BALANCE SHEET'!E18)</f>
+        <v/>
+      </c>
+      <c r="H25" s="5">
+        <f>-('BALANCE SHEET'!G18-'BALANCE SHEET'!F18)</f>
+        <v/>
+      </c>
+      <c r="I25" s="5">
+        <f>-('BALANCE SHEET'!H18-'BALANCE SHEET'!G18)</f>
+        <v/>
+      </c>
+      <c r="J25" s="5">
+        <f>-('BALANCE SHEET'!I18-'BALANCE SHEET'!H18)</f>
+        <v/>
+      </c>
+      <c r="K25" s="5">
+        <f>-('BALANCE SHEET'!J18-'BALANCE SHEET'!I18)</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
@@ -2982,12 +4242,30 @@
       <c r="E27" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F27" s="5" t="n"/>
-      <c r="G27" s="5" t="n"/>
-      <c r="H27" s="5" t="n"/>
-      <c r="I27" s="5" t="n"/>
-      <c r="J27" s="5" t="n"/>
-      <c r="K27" s="5" t="n"/>
+      <c r="F27" s="5">
+        <f>E27</f>
+        <v/>
+      </c>
+      <c r="G27" s="5">
+        <f>F27</f>
+        <v/>
+      </c>
+      <c r="H27" s="5">
+        <f>G27</f>
+        <v/>
+      </c>
+      <c r="I27" s="5">
+        <f>H27</f>
+        <v/>
+      </c>
+      <c r="J27" s="5">
+        <f>I27</f>
+        <v/>
+      </c>
+      <c r="K27" s="5">
+        <f>J27</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -3007,12 +4285,30 @@
       <c r="E28" s="4" t="n">
         <v>-23390</v>
       </c>
-      <c r="F28" s="5" t="n"/>
-      <c r="G28" s="5" t="n"/>
-      <c r="H28" s="5" t="n"/>
-      <c r="I28" s="5" t="n"/>
-      <c r="J28" s="5" t="n"/>
-      <c r="K28" s="5" t="n"/>
+      <c r="F28" s="5">
+        <f>'CF DRIVERS'!F4*'BALANCE SHEET'!D11</f>
+        <v/>
+      </c>
+      <c r="G28" s="5">
+        <f>'CF DRIVERS'!G4*'BALANCE SHEET'!E11</f>
+        <v/>
+      </c>
+      <c r="H28" s="5">
+        <f>'CF DRIVERS'!H4*'BALANCE SHEET'!F11</f>
+        <v/>
+      </c>
+      <c r="I28" s="5">
+        <f>'CF DRIVERS'!I4*'BALANCE SHEET'!G11</f>
+        <v/>
+      </c>
+      <c r="J28" s="5">
+        <f>'CF DRIVERS'!J4*'BALANCE SHEET'!H11</f>
+        <v/>
+      </c>
+      <c r="K28" s="5">
+        <f>'CF DRIVERS'!K4*'BALANCE SHEET'!I11</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -3032,12 +4328,30 @@
       <c r="E29" s="4" t="n">
         <v>-3000</v>
       </c>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="5" t="n"/>
-      <c r="I29" s="5" t="n"/>
-      <c r="J29" s="5" t="n"/>
-      <c r="K29" s="5" t="n"/>
+      <c r="F29" s="5">
+        <f>E29</f>
+        <v/>
+      </c>
+      <c r="G29" s="5">
+        <f>F29</f>
+        <v/>
+      </c>
+      <c r="H29" s="5">
+        <f>G29</f>
+        <v/>
+      </c>
+      <c r="I29" s="5">
+        <f>H29</f>
+        <v/>
+      </c>
+      <c r="J29" s="5">
+        <f>I29</f>
+        <v/>
+      </c>
+      <c r="K29" s="5">
+        <f>J29</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -3057,12 +4371,30 @@
       <c r="E30" s="4" t="n">
         <v>-75336</v>
       </c>
-      <c r="F30" s="5" t="n"/>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="5" t="n"/>
-      <c r="I30" s="5" t="n"/>
-      <c r="J30" s="5" t="n"/>
-      <c r="K30" s="5" t="n"/>
+      <c r="F30" s="5">
+        <f>E30</f>
+        <v/>
+      </c>
+      <c r="G30" s="5">
+        <f>F30</f>
+        <v/>
+      </c>
+      <c r="H30" s="5">
+        <f>G30</f>
+        <v/>
+      </c>
+      <c r="I30" s="5">
+        <f>H30</f>
+        <v/>
+      </c>
+      <c r="J30" s="5">
+        <f>I30</f>
+        <v/>
+      </c>
+      <c r="K30" s="5">
+        <f>J30</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -3129,12 +4461,30 @@
       <c r="E32" s="4" t="n">
         <v>-61</v>
       </c>
-      <c r="F32" s="5" t="n"/>
-      <c r="G32" s="5" t="n"/>
-      <c r="H32" s="5" t="n"/>
-      <c r="I32" s="5" t="n"/>
-      <c r="J32" s="5" t="n"/>
-      <c r="K32" s="5" t="n"/>
+      <c r="F32" s="5">
+        <f>E32</f>
+        <v/>
+      </c>
+      <c r="G32" s="5">
+        <f>F32</f>
+        <v/>
+      </c>
+      <c r="H32" s="5">
+        <f>G32</f>
+        <v/>
+      </c>
+      <c r="I32" s="5">
+        <f>H32</f>
+        <v/>
+      </c>
+      <c r="J32" s="5">
+        <f>I32</f>
+        <v/>
+      </c>
+      <c r="K32" s="5">
+        <f>J32</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
@@ -3154,12 +4504,30 @@
       <c r="E33" s="4" t="n">
         <v>3856</v>
       </c>
-      <c r="F33" s="5" t="n"/>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="5" t="n"/>
-      <c r="I33" s="5" t="n"/>
-      <c r="J33" s="5" t="n"/>
-      <c r="K33" s="5" t="n"/>
+      <c r="F33" s="5">
+        <f>E33</f>
+        <v/>
+      </c>
+      <c r="G33" s="5">
+        <f>F33</f>
+        <v/>
+      </c>
+      <c r="H33" s="5">
+        <f>G33</f>
+        <v/>
+      </c>
+      <c r="I33" s="5">
+        <f>H33</f>
+        <v/>
+      </c>
+      <c r="J33" s="5">
+        <f>I33</f>
+        <v/>
+      </c>
+      <c r="K33" s="5">
+        <f>J33</f>
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
@@ -3179,12 +4547,30 @@
       <c r="E34" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F34" s="5" t="n"/>
-      <c r="G34" s="5" t="n"/>
-      <c r="H34" s="5" t="n"/>
-      <c r="I34" s="5" t="n"/>
-      <c r="J34" s="5" t="n"/>
-      <c r="K34" s="5" t="n"/>
+      <c r="F34" s="5">
+        <f>E34</f>
+        <v/>
+      </c>
+      <c r="G34" s="5">
+        <f>F34</f>
+        <v/>
+      </c>
+      <c r="H34" s="5">
+        <f>G34</f>
+        <v/>
+      </c>
+      <c r="I34" s="5">
+        <f>H34</f>
+        <v/>
+      </c>
+      <c r="J34" s="5">
+        <f>I34</f>
+        <v/>
+      </c>
+      <c r="K34" s="5">
+        <f>J34</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -3204,12 +4590,30 @@
       <c r="E35" s="4" t="n">
         <v>-27500</v>
       </c>
-      <c r="F35" s="5" t="n"/>
-      <c r="G35" s="5" t="n"/>
-      <c r="H35" s="5" t="n"/>
-      <c r="I35" s="5" t="n"/>
-      <c r="J35" s="5" t="n"/>
-      <c r="K35" s="5" t="n"/>
+      <c r="F35" s="5">
+        <f>'CF DRIVERS'!F5*'BALANCE SHEET'!E35</f>
+        <v/>
+      </c>
+      <c r="G35" s="5">
+        <f>'CF DRIVERS'!G5*'BALANCE SHEET'!F35</f>
+        <v/>
+      </c>
+      <c r="H35" s="5">
+        <f>'CF DRIVERS'!H5*'BALANCE SHEET'!G35</f>
+        <v/>
+      </c>
+      <c r="I35" s="5">
+        <f>'CF DRIVERS'!I5*'BALANCE SHEET'!H35</f>
+        <v/>
+      </c>
+      <c r="J35" s="5">
+        <f>'CF DRIVERS'!J5*'BALANCE SHEET'!I35</f>
+        <v/>
+      </c>
+      <c r="K35" s="5">
+        <f>'CF DRIVERS'!K5*'BALANCE SHEET'!J35</f>
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
@@ -3229,12 +4633,30 @@
       <c r="E36" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F36" s="5" t="n"/>
-      <c r="G36" s="5" t="n"/>
-      <c r="H36" s="5" t="n"/>
-      <c r="I36" s="5" t="n"/>
-      <c r="J36" s="5" t="n"/>
-      <c r="K36" s="5" t="n"/>
+      <c r="F36" s="5">
+        <f>E36</f>
+        <v/>
+      </c>
+      <c r="G36" s="5">
+        <f>F36</f>
+        <v/>
+      </c>
+      <c r="H36" s="5">
+        <f>G36</f>
+        <v/>
+      </c>
+      <c r="I36" s="5">
+        <f>H36</f>
+        <v/>
+      </c>
+      <c r="J36" s="5">
+        <f>I36</f>
+        <v/>
+      </c>
+      <c r="K36" s="5">
+        <f>J36</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
@@ -3254,12 +4676,30 @@
       <c r="E37" s="4" t="n">
         <v>-2261</v>
       </c>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="5" t="n"/>
-      <c r="I37" s="5" t="n"/>
-      <c r="J37" s="5" t="n"/>
-      <c r="K37" s="5" t="n"/>
+      <c r="F37" s="5">
+        <f>'CF DRIVERS'!F7</f>
+        <v/>
+      </c>
+      <c r="G37" s="5">
+        <f>'CF DRIVERS'!G7</f>
+        <v/>
+      </c>
+      <c r="H37" s="5">
+        <f>'CF DRIVERS'!H7</f>
+        <v/>
+      </c>
+      <c r="I37" s="5">
+        <f>'CF DRIVERS'!I7</f>
+        <v/>
+      </c>
+      <c r="J37" s="5">
+        <f>'CF DRIVERS'!J7</f>
+        <v/>
+      </c>
+      <c r="K37" s="5">
+        <f>'CF DRIVERS'!K7</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -3326,12 +4766,30 @@
       <c r="E39" s="4" t="n">
         <v>-997</v>
       </c>
-      <c r="F39" s="5" t="n"/>
-      <c r="G39" s="5" t="n"/>
-      <c r="H39" s="5" t="n"/>
-      <c r="I39" s="5" t="n"/>
-      <c r="J39" s="5" t="n"/>
-      <c r="K39" s="5" t="n"/>
+      <c r="F39" s="5">
+        <f>E39</f>
+        <v/>
+      </c>
+      <c r="G39" s="5">
+        <f>F39</f>
+        <v/>
+      </c>
+      <c r="H39" s="5">
+        <f>G39</f>
+        <v/>
+      </c>
+      <c r="I39" s="5">
+        <f>H39</f>
+        <v/>
+      </c>
+      <c r="J39" s="5">
+        <f>I39</f>
+        <v/>
+      </c>
+      <c r="K39" s="5">
+        <f>J39</f>
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -3351,12 +4809,30 @@
       <c r="E40" s="4" t="n">
         <v>134209</v>
       </c>
-      <c r="F40" s="5" t="n"/>
-      <c r="G40" s="5" t="n"/>
-      <c r="H40" s="5" t="n"/>
-      <c r="I40" s="5" t="n"/>
-      <c r="J40" s="5" t="n"/>
-      <c r="K40" s="5" t="n"/>
+      <c r="F40" s="5">
+        <f>'CASH FLOW'!F26+'CASH FLOW'!F31+'CASH FLOW'!F38+'CASH FLOW'!F39</f>
+        <v/>
+      </c>
+      <c r="G40" s="5">
+        <f>'CASH FLOW'!G26+'CASH FLOW'!G31+'CASH FLOW'!G38+'CASH FLOW'!G39</f>
+        <v/>
+      </c>
+      <c r="H40" s="5">
+        <f>'CASH FLOW'!H26+'CASH FLOW'!H31+'CASH FLOW'!H38+'CASH FLOW'!H39</f>
+        <v/>
+      </c>
+      <c r="I40" s="5">
+        <f>'CASH FLOW'!I26+'CASH FLOW'!I31+'CASH FLOW'!I38+'CASH FLOW'!I39</f>
+        <v/>
+      </c>
+      <c r="J40" s="5">
+        <f>'CASH FLOW'!J26+'CASH FLOW'!J31+'CASH FLOW'!J38+'CASH FLOW'!J39</f>
+        <v/>
+      </c>
+      <c r="K40" s="5">
+        <f>'CASH FLOW'!K26+'CASH FLOW'!K31+'CASH FLOW'!K38+'CASH FLOW'!K39</f>
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -3376,12 +4852,30 @@
       <c r="E41" s="4" t="n">
         <v>755981</v>
       </c>
-      <c r="F41" s="5" t="n"/>
-      <c r="G41" s="5" t="n"/>
-      <c r="H41" s="5" t="n"/>
-      <c r="I41" s="5" t="n"/>
-      <c r="J41" s="5" t="n"/>
-      <c r="K41" s="5" t="n"/>
+      <c r="F41" s="5">
+        <f>'CASH FLOW'!E42</f>
+        <v/>
+      </c>
+      <c r="G41" s="5">
+        <f>'CASH FLOW'!F42</f>
+        <v/>
+      </c>
+      <c r="H41" s="5">
+        <f>'CASH FLOW'!G42</f>
+        <v/>
+      </c>
+      <c r="I41" s="5">
+        <f>'CASH FLOW'!H42</f>
+        <v/>
+      </c>
+      <c r="J41" s="5">
+        <f>'CASH FLOW'!I42</f>
+        <v/>
+      </c>
+      <c r="K41" s="5">
+        <f>'CASH FLOW'!J42</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
@@ -3401,12 +4895,30 @@
       <c r="E42" s="4" t="n">
         <v>890190</v>
       </c>
-      <c r="F42" s="5" t="n"/>
-      <c r="G42" s="5" t="n"/>
-      <c r="H42" s="5" t="n"/>
-      <c r="I42" s="5" t="n"/>
-      <c r="J42" s="5" t="n"/>
-      <c r="K42" s="5" t="n"/>
+      <c r="F42" s="5">
+        <f>'CASH FLOW'!F41+'CASH FLOW'!F40</f>
+        <v/>
+      </c>
+      <c r="G42" s="5">
+        <f>'CASH FLOW'!G41+'CASH FLOW'!G40</f>
+        <v/>
+      </c>
+      <c r="H42" s="5">
+        <f>'CASH FLOW'!H41+'CASH FLOW'!H40</f>
+        <v/>
+      </c>
+      <c r="I42" s="5">
+        <f>'CASH FLOW'!I41+'CASH FLOW'!I40</f>
+        <v/>
+      </c>
+      <c r="J42" s="5">
+        <f>'CASH FLOW'!J41+'CASH FLOW'!J40</f>
+        <v/>
+      </c>
+      <c r="K42" s="5">
+        <f>'CASH FLOW'!K41+'CASH FLOW'!K40</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
vault backup: 2026-04-23 19:49:25
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -4328,30 +4328,12 @@
       <c r="E29" s="4" t="n">
         <v>-3000</v>
       </c>
-      <c r="F29" s="5">
-        <f>E29</f>
-        <v/>
-      </c>
-      <c r="G29" s="5">
-        <f>F29</f>
-        <v/>
-      </c>
-      <c r="H29" s="5">
-        <f>G29</f>
-        <v/>
-      </c>
-      <c r="I29" s="5">
-        <f>H29</f>
-        <v/>
-      </c>
-      <c r="J29" s="5">
-        <f>I29</f>
-        <v/>
-      </c>
-      <c r="K29" s="5">
-        <f>J29</f>
-        <v/>
-      </c>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+      <c r="H29" s="5" t="n"/>
+      <c r="I29" s="5" t="n"/>
+      <c r="J29" s="5" t="n"/>
+      <c r="K29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -4371,30 +4353,12 @@
       <c r="E30" s="4" t="n">
         <v>-75336</v>
       </c>
-      <c r="F30" s="5">
-        <f>E30</f>
-        <v/>
-      </c>
-      <c r="G30" s="5">
-        <f>F30</f>
-        <v/>
-      </c>
-      <c r="H30" s="5">
-        <f>G30</f>
-        <v/>
-      </c>
-      <c r="I30" s="5">
-        <f>H30</f>
-        <v/>
-      </c>
-      <c r="J30" s="5">
-        <f>I30</f>
-        <v/>
-      </c>
-      <c r="K30" s="5">
-        <f>J30</f>
-        <v/>
-      </c>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+      <c r="H30" s="5" t="n"/>
+      <c r="I30" s="5" t="n"/>
+      <c r="J30" s="5" t="n"/>
+      <c r="K30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">

</xml_diff>

<commit_message>
vault backup: 2026-04-23 19:58:14
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -638,27 +638,27 @@
         <v>1355630</v>
       </c>
       <c r="F2" s="5">
-        <f>E2*(1+'IS DRIVERS'!F2)</f>
+        <f>'ANNL P&amp;L'!E2*(1+'IS DRIVERS'!F2)</f>
         <v/>
       </c>
       <c r="G2" s="5">
-        <f>F2*(1+'IS DRIVERS'!G2)</f>
+        <f>'ANNL P&amp;L'!F2*(1+'IS DRIVERS'!G2)</f>
         <v/>
       </c>
       <c r="H2" s="5">
-        <f>G2*(1+'IS DRIVERS'!H2)</f>
+        <f>'ANNL P&amp;L'!G2*(1+'IS DRIVERS'!H2)</f>
         <v/>
       </c>
       <c r="I2" s="5">
-        <f>H2*(1+'IS DRIVERS'!I2)</f>
+        <f>'ANNL P&amp;L'!H2*(1+'IS DRIVERS'!I2)</f>
         <v/>
       </c>
       <c r="J2" s="5">
-        <f>I2*(1+'IS DRIVERS'!J2)</f>
+        <f>'ANNL P&amp;L'!I2*(1+'IS DRIVERS'!J2)</f>
         <v/>
       </c>
       <c r="K2" s="5">
-        <f>J2*(1+'IS DRIVERS'!K2)</f>
+        <f>'ANNL P&amp;L'!J2*(1+'IS DRIVERS'!K2)</f>
         <v/>
       </c>
     </row>
@@ -1463,27 +1463,27 @@
         <v>890190</v>
       </c>
       <c r="E2" s="5">
-        <f>D2+'CASH FLOW'!E40</f>
+        <f>D2+'CASH FLOW'!F40</f>
         <v/>
       </c>
       <c r="F2" s="5">
-        <f>E2+'CASH FLOW'!F40</f>
+        <f>E2+'CASH FLOW'!G40</f>
         <v/>
       </c>
       <c r="G2" s="5">
-        <f>F2+'CASH FLOW'!G40</f>
+        <f>F2+'CASH FLOW'!H40</f>
         <v/>
       </c>
       <c r="H2" s="5">
-        <f>G2+'CASH FLOW'!H40</f>
+        <f>G2+'CASH FLOW'!I40</f>
         <v/>
       </c>
       <c r="I2" s="5">
-        <f>H2+'CASH FLOW'!I40</f>
+        <f>H2+'CASH FLOW'!J40</f>
         <v/>
       </c>
       <c r="J2" s="5">
-        <f>I2+'CASH FLOW'!J40</f>
+        <f>I2+'CASH FLOW'!K40</f>
         <v/>
       </c>
     </row>
@@ -1543,27 +1543,27 @@
         <v>270342</v>
       </c>
       <c r="E4" s="5">
-        <f>'BS DRIVERS'!E3*'ANNL P&amp;L'!E2/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!F3*'ANNL P&amp;L'!F2/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="F4" s="5">
-        <f>'BS DRIVERS'!F3*'ANNL P&amp;L'!F2/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!G3*'ANNL P&amp;L'!G2/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="G4" s="5">
-        <f>'BS DRIVERS'!G3*'ANNL P&amp;L'!G2/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!H3*'ANNL P&amp;L'!H2/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="H4" s="5">
-        <f>'BS DRIVERS'!H3*'ANNL P&amp;L'!H2/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!I3*'ANNL P&amp;L'!I2/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="I4" s="5">
-        <f>'BS DRIVERS'!I3*'ANNL P&amp;L'!I2/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!J3*'ANNL P&amp;L'!J2/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="J4" s="5">
-        <f>'BS DRIVERS'!J3*'ANNL P&amp;L'!J2/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!K3*'ANNL P&amp;L'!K2/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
     </row>
@@ -1583,27 +1583,27 @@
         <v>0</v>
       </c>
       <c r="E5" s="5">
-        <f>'BS DRIVERS'!E5*'ANNL P&amp;L'!E2</f>
+        <f>'BS DRIVERS'!F5*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
       <c r="F5" s="5">
-        <f>'BS DRIVERS'!F5*'ANNL P&amp;L'!F2</f>
+        <f>'BS DRIVERS'!G5*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
       <c r="G5" s="5">
-        <f>'BS DRIVERS'!G5*'ANNL P&amp;L'!G2</f>
+        <f>'BS DRIVERS'!H5*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
       <c r="H5" s="5">
-        <f>'BS DRIVERS'!H5*'ANNL P&amp;L'!H2</f>
+        <f>'BS DRIVERS'!I5*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
       <c r="I5" s="5">
-        <f>'BS DRIVERS'!I5*'ANNL P&amp;L'!I2</f>
+        <f>'BS DRIVERS'!J5*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
       <c r="J5" s="5">
-        <f>'BS DRIVERS'!J5*'ANNL P&amp;L'!J2</f>
+        <f>'BS DRIVERS'!K5*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
     </row>
@@ -1623,27 +1623,27 @@
         <v>131165</v>
       </c>
       <c r="E6" s="5">
-        <f>'BS DRIVERS'!E4*'ANNL P&amp;L'!E3/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!F4*'ANNL P&amp;L'!F3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="F6" s="5">
-        <f>'BS DRIVERS'!F4*'ANNL P&amp;L'!F3/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!G4*'ANNL P&amp;L'!G3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="G6" s="5">
-        <f>'BS DRIVERS'!G4*'ANNL P&amp;L'!G3/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!H4*'ANNL P&amp;L'!H3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="H6" s="5">
-        <f>'BS DRIVERS'!H4*'ANNL P&amp;L'!H3/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!I4*'ANNL P&amp;L'!I3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="I6" s="5">
-        <f>'BS DRIVERS'!I4*'ANNL P&amp;L'!I3/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!J4*'ANNL P&amp;L'!J3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="J6" s="5">
-        <f>'BS DRIVERS'!J4*'ANNL P&amp;L'!J3/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!K4*'ANNL P&amp;L'!K3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
     </row>
@@ -1663,27 +1663,27 @@
         <v>14124</v>
       </c>
       <c r="E7" s="5">
-        <f>'BS DRIVERS'!E6*'ANNL P&amp;L'!E2</f>
+        <f>'BS DRIVERS'!F6*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
       <c r="F7" s="5">
-        <f>'BS DRIVERS'!F6*'ANNL P&amp;L'!F2</f>
+        <f>'BS DRIVERS'!G6*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
       <c r="G7" s="5">
-        <f>'BS DRIVERS'!G6*'ANNL P&amp;L'!G2</f>
+        <f>'BS DRIVERS'!H6*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
       <c r="H7" s="5">
-        <f>'BS DRIVERS'!H6*'ANNL P&amp;L'!H2</f>
+        <f>'BS DRIVERS'!I6*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
       <c r="I7" s="5">
-        <f>'BS DRIVERS'!I6*'ANNL P&amp;L'!I2</f>
+        <f>'BS DRIVERS'!J6*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
       <c r="J7" s="5">
-        <f>'BS DRIVERS'!J6*'ANNL P&amp;L'!J2</f>
+        <f>'BS DRIVERS'!K6*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
     </row>
@@ -1703,27 +1703,27 @@
         <v>18759</v>
       </c>
       <c r="E8" s="5">
-        <f>'BS DRIVERS'!E7*'ANNL P&amp;L'!E2</f>
+        <f>'BS DRIVERS'!F7*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
       <c r="F8" s="5">
-        <f>'BS DRIVERS'!F7*'ANNL P&amp;L'!F2</f>
+        <f>'BS DRIVERS'!G7*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
       <c r="G8" s="5">
-        <f>'BS DRIVERS'!G7*'ANNL P&amp;L'!G2</f>
+        <f>'BS DRIVERS'!H7*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
       <c r="H8" s="5">
-        <f>'BS DRIVERS'!H7*'ANNL P&amp;L'!H2</f>
+        <f>'BS DRIVERS'!I7*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
       <c r="I8" s="5">
-        <f>'BS DRIVERS'!I7*'ANNL P&amp;L'!I2</f>
+        <f>'BS DRIVERS'!J7*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
       <c r="J8" s="5">
-        <f>'BS DRIVERS'!J7*'ANNL P&amp;L'!J2</f>
+        <f>'BS DRIVERS'!K7*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
     </row>
@@ -1826,27 +1826,27 @@
         <v>55602</v>
       </c>
       <c r="E11" s="5">
-        <f>D11-'CASH FLOW'!E28-'CASH FLOW'!E3</f>
+        <f>D11-'CASH FLOW'!F28-'CASH FLOW'!F3</f>
         <v/>
       </c>
       <c r="F11" s="5">
-        <f>E11-'CASH FLOW'!F28-'CASH FLOW'!F3</f>
+        <f>E11-'CASH FLOW'!G28-'CASH FLOW'!G3</f>
         <v/>
       </c>
       <c r="G11" s="5">
-        <f>F11-'CASH FLOW'!G28-'CASH FLOW'!G3</f>
+        <f>F11-'CASH FLOW'!H28-'CASH FLOW'!H3</f>
         <v/>
       </c>
       <c r="H11" s="5">
-        <f>G11-'CASH FLOW'!H28-'CASH FLOW'!H3</f>
+        <f>G11-'CASH FLOW'!I28-'CASH FLOW'!I3</f>
         <v/>
       </c>
       <c r="I11" s="5">
-        <f>H11-'CASH FLOW'!I28-'CASH FLOW'!I3</f>
+        <f>H11-'CASH FLOW'!J28-'CASH FLOW'!J3</f>
         <v/>
       </c>
       <c r="J11" s="5">
-        <f>I11-'CASH FLOW'!J28-'CASH FLOW'!J3</f>
+        <f>I11-'CASH FLOW'!K28-'CASH FLOW'!K3</f>
         <v/>
       </c>
     </row>
@@ -2026,27 +2026,27 @@
         <v>234215</v>
       </c>
       <c r="E16" s="5">
-        <f>D16-'CASH FLOW'!E6</f>
+        <f>D16-'CASH FLOW'!F6</f>
         <v/>
       </c>
       <c r="F16" s="5">
-        <f>E16-'CASH FLOW'!F6</f>
+        <f>E16-'CASH FLOW'!G6</f>
         <v/>
       </c>
       <c r="G16" s="5">
-        <f>F16-'CASH FLOW'!G6</f>
+        <f>F16-'CASH FLOW'!H6</f>
         <v/>
       </c>
       <c r="H16" s="5">
-        <f>G16-'CASH FLOW'!H6</f>
+        <f>G16-'CASH FLOW'!I6</f>
         <v/>
       </c>
       <c r="I16" s="5">
-        <f>H16-'CASH FLOW'!I6</f>
+        <f>H16-'CASH FLOW'!J6</f>
         <v/>
       </c>
       <c r="J16" s="5">
-        <f>I16-'CASH FLOW'!J6</f>
+        <f>I16-'CASH FLOW'!K6</f>
         <v/>
       </c>
     </row>
@@ -2106,27 +2106,27 @@
         <v>8154</v>
       </c>
       <c r="E18" s="5">
-        <f>'BS DRIVERS'!E9*'ANNL P&amp;L'!E2</f>
+        <f>'BS DRIVERS'!F9*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
       <c r="F18" s="5">
-        <f>'BS DRIVERS'!F9*'ANNL P&amp;L'!F2</f>
+        <f>'BS DRIVERS'!G9*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
       <c r="G18" s="5">
-        <f>'BS DRIVERS'!G9*'ANNL P&amp;L'!G2</f>
+        <f>'BS DRIVERS'!H9*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
       <c r="H18" s="5">
-        <f>'BS DRIVERS'!H9*'ANNL P&amp;L'!H2</f>
+        <f>'BS DRIVERS'!I9*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
       <c r="I18" s="5">
-        <f>'BS DRIVERS'!I9*'ANNL P&amp;L'!I2</f>
+        <f>'BS DRIVERS'!J9*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
       <c r="J18" s="5">
-        <f>'BS DRIVERS'!J9*'ANNL P&amp;L'!J2</f>
+        <f>'BS DRIVERS'!K9*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
     </row>
@@ -2189,27 +2189,27 @@
         <v>41287</v>
       </c>
       <c r="E20" s="5">
-        <f>'BS DRIVERS'!E11*'ANNL P&amp;L'!E3/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!F11*'ANNL P&amp;L'!F3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="F20" s="5">
-        <f>'BS DRIVERS'!F11*'ANNL P&amp;L'!F3/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!G11*'ANNL P&amp;L'!G3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="G20" s="5">
-        <f>'BS DRIVERS'!G11*'ANNL P&amp;L'!G3/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!H11*'ANNL P&amp;L'!H3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="H20" s="5">
-        <f>'BS DRIVERS'!H11*'ANNL P&amp;L'!H3/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!I11*'ANNL P&amp;L'!I3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="I20" s="5">
-        <f>'BS DRIVERS'!I11*'ANNL P&amp;L'!I3/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!J11*'ANNL P&amp;L'!J3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
       <c r="J20" s="5">
-        <f>'BS DRIVERS'!J11*'ANNL P&amp;L'!J3/ASSUMPTIONS!$B$2</f>
+        <f>'BS DRIVERS'!K11*'ANNL P&amp;L'!K3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
     </row>
@@ -2229,27 +2229,27 @@
         <v>148780</v>
       </c>
       <c r="E21" s="5">
-        <f>'BS DRIVERS'!E12*'ANNL P&amp;L'!E2</f>
+        <f>'BS DRIVERS'!F12*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
       <c r="F21" s="5">
-        <f>'BS DRIVERS'!F12*'ANNL P&amp;L'!F2</f>
+        <f>'BS DRIVERS'!G12*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
       <c r="G21" s="5">
-        <f>'BS DRIVERS'!G12*'ANNL P&amp;L'!G2</f>
+        <f>'BS DRIVERS'!H12*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
       <c r="H21" s="5">
-        <f>'BS DRIVERS'!H12*'ANNL P&amp;L'!H2</f>
+        <f>'BS DRIVERS'!I12*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
       <c r="I21" s="5">
-        <f>'BS DRIVERS'!I12*'ANNL P&amp;L'!I2</f>
+        <f>'BS DRIVERS'!J12*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
       <c r="J21" s="5">
-        <f>'BS DRIVERS'!J12*'ANNL P&amp;L'!J2</f>
+        <f>'BS DRIVERS'!K12*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
     </row>
@@ -2269,27 +2269,27 @@
         <v>10834</v>
       </c>
       <c r="E22" s="5">
-        <f>'BS DRIVERS'!E13*'ANNL P&amp;L'!E2</f>
+        <f>'BS DRIVERS'!F13*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
       <c r="F22" s="5">
-        <f>'BS DRIVERS'!F13*'ANNL P&amp;L'!F2</f>
+        <f>'BS DRIVERS'!G13*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
       <c r="G22" s="5">
-        <f>'BS DRIVERS'!G13*'ANNL P&amp;L'!G2</f>
+        <f>'BS DRIVERS'!H13*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
       <c r="H22" s="5">
-        <f>'BS DRIVERS'!H13*'ANNL P&amp;L'!H2</f>
+        <f>'BS DRIVERS'!I13*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
       <c r="I22" s="5">
-        <f>'BS DRIVERS'!I13*'ANNL P&amp;L'!I2</f>
+        <f>'BS DRIVERS'!J13*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
       <c r="J22" s="5">
-        <f>'BS DRIVERS'!J13*'ANNL P&amp;L'!J2</f>
+        <f>'BS DRIVERS'!K13*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
     </row>
@@ -2309,27 +2309,27 @@
         <v>0</v>
       </c>
       <c r="E23" s="5">
-        <f>'BS DRIVERS'!E14*'ANNL P&amp;L'!E2</f>
+        <f>'BS DRIVERS'!F14*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
       <c r="F23" s="5">
-        <f>'BS DRIVERS'!F14*'ANNL P&amp;L'!F2</f>
+        <f>'BS DRIVERS'!G14*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
       <c r="G23" s="5">
-        <f>'BS DRIVERS'!G14*'ANNL P&amp;L'!G2</f>
+        <f>'BS DRIVERS'!H14*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
       <c r="H23" s="5">
-        <f>'BS DRIVERS'!H14*'ANNL P&amp;L'!H2</f>
+        <f>'BS DRIVERS'!I14*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
       <c r="I23" s="5">
-        <f>'BS DRIVERS'!I14*'ANNL P&amp;L'!I2</f>
+        <f>'BS DRIVERS'!J14*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
       <c r="J23" s="5">
-        <f>'BS DRIVERS'!J14*'ANNL P&amp;L'!J2</f>
+        <f>'BS DRIVERS'!K14*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
     </row>
@@ -2349,27 +2349,27 @@
         <v>135948</v>
       </c>
       <c r="E24" s="5">
-        <f>'BS DRIVERS'!E15*'ANNL P&amp;L'!E2</f>
+        <f>'BS DRIVERS'!F15*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
       <c r="F24" s="5">
-        <f>'BS DRIVERS'!F15*'ANNL P&amp;L'!F2</f>
+        <f>'BS DRIVERS'!G15*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
       <c r="G24" s="5">
-        <f>'BS DRIVERS'!G15*'ANNL P&amp;L'!G2</f>
+        <f>'BS DRIVERS'!H15*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
       <c r="H24" s="5">
-        <f>'BS DRIVERS'!H15*'ANNL P&amp;L'!H2</f>
+        <f>'BS DRIVERS'!I15*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
       <c r="I24" s="5">
-        <f>'BS DRIVERS'!I15*'ANNL P&amp;L'!I2</f>
+        <f>'BS DRIVERS'!J15*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
       <c r="J24" s="5">
-        <f>'BS DRIVERS'!J15*'ANNL P&amp;L'!J2</f>
+        <f>'BS DRIVERS'!K15*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
     </row>
@@ -2389,27 +2389,27 @@
         <v>3265</v>
       </c>
       <c r="E25" s="5">
-        <f>'BS DRIVERS'!E16*'ANNL P&amp;L'!E2</f>
+        <f>'BS DRIVERS'!F16*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
       <c r="F25" s="5">
-        <f>'BS DRIVERS'!F16*'ANNL P&amp;L'!F2</f>
+        <f>'BS DRIVERS'!G16*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
       <c r="G25" s="5">
-        <f>'BS DRIVERS'!G16*'ANNL P&amp;L'!G2</f>
+        <f>'BS DRIVERS'!H16*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
       <c r="H25" s="5">
-        <f>'BS DRIVERS'!H16*'ANNL P&amp;L'!H2</f>
+        <f>'BS DRIVERS'!I16*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
       <c r="I25" s="5">
-        <f>'BS DRIVERS'!I16*'ANNL P&amp;L'!I2</f>
+        <f>'BS DRIVERS'!J16*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
       <c r="J25" s="5">
-        <f>'BS DRIVERS'!J16*'ANNL P&amp;L'!J2</f>
+        <f>'BS DRIVERS'!K16*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
     </row>
@@ -2429,27 +2429,27 @@
         <v>100</v>
       </c>
       <c r="E26" s="5">
-        <f>'BS DRIVERS'!E17*'ANNL P&amp;L'!E2</f>
+        <f>'BS DRIVERS'!F17*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
       <c r="F26" s="5">
-        <f>'BS DRIVERS'!F17*'ANNL P&amp;L'!F2</f>
+        <f>'BS DRIVERS'!G17*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
       <c r="G26" s="5">
-        <f>'BS DRIVERS'!G17*'ANNL P&amp;L'!G2</f>
+        <f>'BS DRIVERS'!H17*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
       <c r="H26" s="5">
-        <f>'BS DRIVERS'!H17*'ANNL P&amp;L'!H2</f>
+        <f>'BS DRIVERS'!I17*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
       <c r="I26" s="5">
-        <f>'BS DRIVERS'!I17*'ANNL P&amp;L'!I2</f>
+        <f>'BS DRIVERS'!J17*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
       <c r="J26" s="5">
-        <f>'BS DRIVERS'!J17*'ANNL P&amp;L'!J2</f>
+        <f>'BS DRIVERS'!K17*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
     </row>
@@ -2469,27 +2469,27 @@
         <v>9513</v>
       </c>
       <c r="E27" s="5">
-        <f>'BS DRIVERS'!E18*'ANNL P&amp;L'!E2</f>
+        <f>'BS DRIVERS'!F18*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
       <c r="F27" s="5">
-        <f>'BS DRIVERS'!F18*'ANNL P&amp;L'!F2</f>
+        <f>'BS DRIVERS'!G18*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
       <c r="G27" s="5">
-        <f>'BS DRIVERS'!G18*'ANNL P&amp;L'!G2</f>
+        <f>'BS DRIVERS'!H18*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
       <c r="H27" s="5">
-        <f>'BS DRIVERS'!H18*'ANNL P&amp;L'!H2</f>
+        <f>'BS DRIVERS'!I18*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
       <c r="I27" s="5">
-        <f>'BS DRIVERS'!I18*'ANNL P&amp;L'!I2</f>
+        <f>'BS DRIVERS'!J18*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
       <c r="J27" s="5">
-        <f>'BS DRIVERS'!J18*'ANNL P&amp;L'!J2</f>
+        <f>'BS DRIVERS'!K18*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
     </row>
@@ -2509,27 +2509,27 @@
         <v>15808</v>
       </c>
       <c r="E28" s="5">
-        <f>'BS DRIVERS'!E19*'ANNL P&amp;L'!E2</f>
+        <f>'BS DRIVERS'!F19*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
       <c r="F28" s="5">
-        <f>'BS DRIVERS'!F19*'ANNL P&amp;L'!F2</f>
+        <f>'BS DRIVERS'!G19*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
       <c r="G28" s="5">
-        <f>'BS DRIVERS'!G19*'ANNL P&amp;L'!G2</f>
+        <f>'BS DRIVERS'!H19*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
       <c r="H28" s="5">
-        <f>'BS DRIVERS'!H19*'ANNL P&amp;L'!H2</f>
+        <f>'BS DRIVERS'!I19*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
       <c r="I28" s="5">
-        <f>'BS DRIVERS'!I19*'ANNL P&amp;L'!I2</f>
+        <f>'BS DRIVERS'!J19*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
       <c r="J28" s="5">
-        <f>'BS DRIVERS'!J19*'ANNL P&amp;L'!J2</f>
+        <f>'BS DRIVERS'!K19*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
     </row>
@@ -2875,27 +2875,27 @@
         <v>297579</v>
       </c>
       <c r="E37" s="5">
-        <f>D37+'CASH FLOW'!E9</f>
+        <f>D37+'CASH FLOW'!F9+'CASH FLOW'!F33</f>
         <v/>
       </c>
       <c r="F37" s="5">
-        <f>E37+'CASH FLOW'!F9</f>
+        <f>E37+'CASH FLOW'!G9+'CASH FLOW'!G33</f>
         <v/>
       </c>
       <c r="G37" s="5">
-        <f>F37+'CASH FLOW'!G9</f>
+        <f>F37+'CASH FLOW'!H9+'CASH FLOW'!H33</f>
         <v/>
       </c>
       <c r="H37" s="5">
-        <f>G37+'CASH FLOW'!H9</f>
+        <f>G37+'CASH FLOW'!I9+'CASH FLOW'!I33</f>
         <v/>
       </c>
       <c r="I37" s="5">
-        <f>H37+'CASH FLOW'!I9</f>
+        <f>H37+'CASH FLOW'!J9+'CASH FLOW'!J33</f>
         <v/>
       </c>
       <c r="J37" s="5">
-        <f>I37+'CASH FLOW'!J9</f>
+        <f>I37+'CASH FLOW'!K9+'CASH FLOW'!K33</f>
         <v/>
       </c>
     </row>
@@ -2955,27 +2955,27 @@
         <v>105521</v>
       </c>
       <c r="E39" s="5">
-        <f>D39+'ANNL P&amp;L'!E12+'CASH FLOW'!E35</f>
+        <f>D39+'ANNL P&amp;L'!F12+'CASH FLOW'!F35</f>
         <v/>
       </c>
       <c r="F39" s="5">
-        <f>E39+'ANNL P&amp;L'!F12+'CASH FLOW'!F35</f>
+        <f>E39+'ANNL P&amp;L'!G12+'CASH FLOW'!G35</f>
         <v/>
       </c>
       <c r="G39" s="5">
-        <f>F39+'ANNL P&amp;L'!G12+'CASH FLOW'!G35</f>
+        <f>F39+'ANNL P&amp;L'!H12+'CASH FLOW'!H35</f>
         <v/>
       </c>
       <c r="H39" s="5">
-        <f>G39+'ANNL P&amp;L'!H12+'CASH FLOW'!H35</f>
+        <f>G39+'ANNL P&amp;L'!I12+'CASH FLOW'!I35</f>
         <v/>
       </c>
       <c r="I39" s="5">
-        <f>H39+'ANNL P&amp;L'!I12+'CASH FLOW'!I35</f>
+        <f>H39+'ANNL P&amp;L'!J12+'CASH FLOW'!J35</f>
         <v/>
       </c>
       <c r="J39" s="5">
-        <f>I39+'ANNL P&amp;L'!J12+'CASH FLOW'!J35</f>
+        <f>I39+'ANNL P&amp;L'!K12+'CASH FLOW'!K35</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-04-24 09:57:05
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -904,27 +904,27 @@
         <v>1734</v>
       </c>
       <c r="F8" s="5">
-        <f>'IS DRIVERS'!F6</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="G8" s="5">
-        <f>'IS DRIVERS'!G6</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="H8" s="5">
-        <f>'IS DRIVERS'!H6</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="I8" s="5">
-        <f>'IS DRIVERS'!I6</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="J8" s="5">
-        <f>'IS DRIVERS'!J6</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="K8" s="5">
-        <f>'IS DRIVERS'!K6</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -2915,27 +2915,27 @@
         <v>-3250</v>
       </c>
       <c r="E38" s="5">
-        <f>D38</f>
+        <f>D38+'CASH FLOW'!F39</f>
         <v/>
       </c>
       <c r="F38" s="5">
-        <f>E38</f>
+        <f>E38+'CASH FLOW'!G39</f>
         <v/>
       </c>
       <c r="G38" s="5">
-        <f>F38</f>
+        <f>F38+'CASH FLOW'!H39</f>
         <v/>
       </c>
       <c r="H38" s="5">
-        <f>G38</f>
+        <f>G38+'CASH FLOW'!I39</f>
         <v/>
       </c>
       <c r="I38" s="5">
-        <f>H38</f>
+        <f>H38+'CASH FLOW'!J39</f>
         <v/>
       </c>
       <c r="J38" s="5">
-        <f>I38</f>
+        <f>I38+'CASH FLOW'!K39</f>
         <v/>
       </c>
     </row>
@@ -3293,27 +3293,27 @@
         <v>3294</v>
       </c>
       <c r="F5" s="5">
-        <f>E5</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="G5" s="5">
-        <f>F5</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="H5" s="5">
-        <f>G5</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="I5" s="5">
-        <f>H5</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="J5" s="5">
-        <f>I5</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="K5" s="5">
-        <f>J5</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -3379,27 +3379,27 @@
         <v>19086</v>
       </c>
       <c r="F7" s="5">
-        <f>E7</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="G7" s="5">
-        <f>F7</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="H7" s="5">
-        <f>G7</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="I7" s="5">
-        <f>H7</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="J7" s="5">
-        <f>I7</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="K7" s="5">
-        <f>J7</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -3422,27 +3422,27 @@
         <v>173</v>
       </c>
       <c r="F8" s="5">
-        <f>E8</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="G8" s="5">
-        <f>F8</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="H8" s="5">
-        <f>G8</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="I8" s="5">
-        <f>H8</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="J8" s="5">
-        <f>I8</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="K8" s="5">
-        <f>J8</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -3508,27 +3508,27 @@
         <v>-9730</v>
       </c>
       <c r="F10" s="5">
-        <f>E10</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="G10" s="5">
-        <f>F10</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="H10" s="5">
-        <f>G10</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="I10" s="5">
-        <f>H10</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="J10" s="5">
-        <f>I10</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="K10" s="5">
-        <f>J10</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -3551,27 +3551,27 @@
         <v>1734</v>
       </c>
       <c r="F11" s="5">
-        <f>E11</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="G11" s="5">
-        <f>F11</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="H11" s="5">
-        <f>G11</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="I11" s="5">
-        <f>H11</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="J11" s="5">
-        <f>I11</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="K11" s="5">
-        <f>J11</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -3594,27 +3594,27 @@
         <v>0</v>
       </c>
       <c r="F12" s="5">
-        <f>E12</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="G12" s="5">
-        <f>F12</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="H12" s="5">
-        <f>G12</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="I12" s="5">
-        <f>H12</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="J12" s="5">
-        <f>I12</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="K12" s="5">
-        <f>J12</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -3637,27 +3637,27 @@
         <v>-324</v>
       </c>
       <c r="F13" s="5">
-        <f>E13</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="G13" s="5">
-        <f>F13</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="H13" s="5">
-        <f>G13</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="I13" s="5">
-        <f>H13</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="J13" s="5">
-        <f>I13</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="K13" s="5">
-        <f>J13</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -4067,27 +4067,27 @@
         <v>535</v>
       </c>
       <c r="F23" s="5">
-        <f>E23</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="G23" s="5">
-        <f>F23</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="H23" s="5">
-        <f>G23</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="I23" s="5">
-        <f>H23</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="J23" s="5">
-        <f>I23</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="K23" s="5">
-        <f>J23</f>
+        <f>0</f>
         <v/>
       </c>
     </row>
@@ -4426,27 +4426,27 @@
         <v>-61</v>
       </c>
       <c r="F32" s="5">
-        <f>E32</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="G32" s="5">
-        <f>F32</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="H32" s="5">
-        <f>G32</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="I32" s="5">
-        <f>H32</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="J32" s="5">
-        <f>I32</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="K32" s="5">
-        <f>J32</f>
+        <f>0</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-04-24 10:02:14
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -111,10 +111,10 @@
     <xf numFmtId="165" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -637,27 +637,27 @@
       <c r="E2" s="4" t="n">
         <v>1355630</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="10">
         <f>'ANNL P&amp;L'!E2*(1+'IS DRIVERS'!F2)</f>
         <v/>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="10">
         <f>'ANNL P&amp;L'!F2*(1+'IS DRIVERS'!G2)</f>
         <v/>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="10">
         <f>'ANNL P&amp;L'!G2*(1+'IS DRIVERS'!H2)</f>
         <v/>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="10">
         <f>'ANNL P&amp;L'!H2*(1+'IS DRIVERS'!I2)</f>
         <v/>
       </c>
-      <c r="J2" s="5">
+      <c r="J2" s="10">
         <f>'ANNL P&amp;L'!I2*(1+'IS DRIVERS'!J2)</f>
         <v/>
       </c>
-      <c r="K2" s="5">
+      <c r="K2" s="10">
         <f>'ANNL P&amp;L'!J2*(1+'IS DRIVERS'!K2)</f>
         <v/>
       </c>
@@ -680,27 +680,27 @@
       <c r="E3" s="4" t="n">
         <v>675423</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="10">
         <f>'IS DRIVERS'!F3*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="10">
         <f>'IS DRIVERS'!G3*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="10">
         <f>'IS DRIVERS'!H3*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="10">
         <f>'IS DRIVERS'!I3*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="J3" s="5">
+      <c r="J3" s="10">
         <f>'IS DRIVERS'!J3*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="K3" s="5">
+      <c r="K3" s="10">
         <f>'IS DRIVERS'!K3*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -770,27 +770,27 @@
       <c r="E5" s="4" t="n">
         <v>524479</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="10">
         <f>'IS DRIVERS'!F4*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="10">
         <f>'IS DRIVERS'!G4*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="10">
         <f>'IS DRIVERS'!H4*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="10">
         <f>'IS DRIVERS'!I4*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="10">
         <f>'IS DRIVERS'!J4*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="10">
         <f>'IS DRIVERS'!K4*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -860,27 +860,27 @@
       <c r="E7" s="4" t="n">
         <v>-39263</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="10">
         <f>'IS DRIVERS'!F5</f>
         <v/>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="10">
         <f>'IS DRIVERS'!G5</f>
         <v/>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="10">
         <f>'IS DRIVERS'!H5</f>
         <v/>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="10">
         <f>'IS DRIVERS'!I5</f>
         <v/>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="10">
         <f>'IS DRIVERS'!J5</f>
         <v/>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="10">
         <f>'IS DRIVERS'!K5</f>
         <v/>
       </c>
@@ -903,27 +903,27 @@
       <c r="E8" s="4" t="n">
         <v>1734</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="10">
         <f>0</f>
         <v/>
       </c>
@@ -946,27 +946,27 @@
       <c r="E9" s="4" t="n">
         <v>-1793</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="10">
         <f>'IS DRIVERS'!F7</f>
         <v/>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="10">
         <f>'IS DRIVERS'!G7</f>
         <v/>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="10">
         <f>'IS DRIVERS'!H7</f>
         <v/>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="10">
         <f>'IS DRIVERS'!I7</f>
         <v/>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="10">
         <f>'IS DRIVERS'!J7</f>
         <v/>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="10">
         <f>'IS DRIVERS'!K7</f>
         <v/>
       </c>
@@ -1036,27 +1036,27 @@
       <c r="E11" s="4" t="n">
         <v>49976</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="10">
         <f>'ANNL P&amp;L'!F10*'IS DRIVERS'!F8</f>
         <v/>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="10">
         <f>'ANNL P&amp;L'!G10*'IS DRIVERS'!G8</f>
         <v/>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="10">
         <f>'ANNL P&amp;L'!H10*'IS DRIVERS'!H8</f>
         <v/>
       </c>
-      <c r="I11" s="5">
+      <c r="I11" s="10">
         <f>'ANNL P&amp;L'!I10*'IS DRIVERS'!I8</f>
         <v/>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="10">
         <f>'ANNL P&amp;L'!J10*'IS DRIVERS'!J8</f>
         <v/>
       </c>
-      <c r="K11" s="5">
+      <c r="K11" s="10">
         <f>'ANNL P&amp;L'!K10*'IS DRIVERS'!K8</f>
         <v/>
       </c>
@@ -1126,27 +1126,27 @@
       <c r="E13" s="4" t="n">
         <v>-27500</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="10">
         <f>'CASH FLOW'!F35</f>
         <v/>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="10">
         <f>'CASH FLOW'!G35</f>
         <v/>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="10">
         <f>'CASH FLOW'!H35</f>
         <v/>
       </c>
-      <c r="I13" s="5">
+      <c r="I13" s="10">
         <f>'CASH FLOW'!I35</f>
         <v/>
       </c>
-      <c r="J13" s="5">
+      <c r="J13" s="10">
         <f>'CASH FLOW'!J35</f>
         <v/>
       </c>
-      <c r="K13" s="5">
+      <c r="K13" s="10">
         <f>'CASH FLOW'!K35</f>
         <v/>
       </c>
@@ -1169,27 +1169,27 @@
       <c r="E14" s="4" t="n">
         <v>-10117</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="10">
         <f>E14</f>
         <v/>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="10">
         <f>F14</f>
         <v/>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="10">
         <f>G14</f>
         <v/>
       </c>
-      <c r="I14" s="5">
+      <c r="I14" s="10">
         <f>H14</f>
         <v/>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="10">
         <f>I14</f>
         <v/>
       </c>
-      <c r="K14" s="5">
+      <c r="K14" s="10">
         <f>J14</f>
         <v/>
       </c>
@@ -1212,27 +1212,27 @@
       <c r="E15" s="4" t="n">
         <v>107457</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="10">
         <f>'ANNL P&amp;L'!F12+'ANNL P&amp;L'!F13+'ANNL P&amp;L'!F14</f>
         <v/>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="10">
         <f>'ANNL P&amp;L'!G12+'ANNL P&amp;L'!G13+'ANNL P&amp;L'!G14</f>
         <v/>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="10">
         <f>'ANNL P&amp;L'!H12+'ANNL P&amp;L'!H13+'ANNL P&amp;L'!H14</f>
         <v/>
       </c>
-      <c r="I15" s="5">
+      <c r="I15" s="10">
         <f>'ANNL P&amp;L'!I12+'ANNL P&amp;L'!I13+'ANNL P&amp;L'!I14</f>
         <v/>
       </c>
-      <c r="J15" s="5">
+      <c r="J15" s="10">
         <f>'ANNL P&amp;L'!J12+'ANNL P&amp;L'!J13+'ANNL P&amp;L'!J14</f>
         <v/>
       </c>
-      <c r="K15" s="5">
+      <c r="K15" s="10">
         <f>'ANNL P&amp;L'!K12+'ANNL P&amp;L'!K13+'ANNL P&amp;L'!K14</f>
         <v/>
       </c>
@@ -1255,12 +1255,12 @@
       <c r="E16" s="4" t="n">
         <v>0.46</v>
       </c>
-      <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="n"/>
-      <c r="J16" s="5" t="n"/>
-      <c r="K16" s="5" t="n"/>
+      <c r="F16" s="10" t="n"/>
+      <c r="G16" s="10" t="n"/>
+      <c r="H16" s="10" t="n"/>
+      <c r="I16" s="10" t="n"/>
+      <c r="J16" s="10" t="n"/>
+      <c r="K16" s="10" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1280,12 +1280,12 @@
       <c r="E17" s="4" t="n">
         <v>0.45</v>
       </c>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
+      <c r="H17" s="10" t="n"/>
+      <c r="I17" s="10" t="n"/>
+      <c r="J17" s="10" t="n"/>
+      <c r="K17" s="10" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
@@ -1305,27 +1305,27 @@
       <c r="E18" s="4" t="n">
         <v>233667</v>
       </c>
-      <c r="F18" s="5">
+      <c r="F18" s="10">
         <f>E18</f>
         <v/>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="10">
         <f>F18</f>
         <v/>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="10">
         <f>G18</f>
         <v/>
       </c>
-      <c r="I18" s="5">
+      <c r="I18" s="10">
         <f>H18</f>
         <v/>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="10">
         <f>I18</f>
         <v/>
       </c>
-      <c r="K18" s="5">
+      <c r="K18" s="10">
         <f>J18</f>
         <v/>
       </c>
@@ -1348,27 +1348,27 @@
       <c r="E19" s="4" t="n">
         <v>237404</v>
       </c>
-      <c r="F19" s="5">
+      <c r="F19" s="10">
         <f>E19</f>
         <v/>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="10">
         <f>F19</f>
         <v/>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="10">
         <f>G19</f>
         <v/>
       </c>
-      <c r="I19" s="5">
+      <c r="I19" s="10">
         <f>H19</f>
         <v/>
       </c>
-      <c r="J19" s="5">
+      <c r="J19" s="10">
         <f>I19</f>
         <v/>
       </c>
-      <c r="K19" s="5">
+      <c r="K19" s="10">
         <f>J19</f>
         <v/>
       </c>
@@ -1462,27 +1462,27 @@
       <c r="D2" s="4" t="n">
         <v>890190</v>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="10">
         <f>D2+'CASH FLOW'!F40</f>
         <v/>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="10">
         <f>E2+'CASH FLOW'!G40</f>
         <v/>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="10">
         <f>F2+'CASH FLOW'!H40</f>
         <v/>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="10">
         <f>G2+'CASH FLOW'!I40</f>
         <v/>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="10">
         <f>H2+'CASH FLOW'!J40</f>
         <v/>
       </c>
-      <c r="J2" s="5">
+      <c r="J2" s="10">
         <f>I2+'CASH FLOW'!K40</f>
         <v/>
       </c>
@@ -1502,27 +1502,27 @@
       <c r="D3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="5">
+      <c r="E3" s="10">
         <f>D3</f>
         <v/>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="10">
         <f>E3</f>
         <v/>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="10">
         <f>F3</f>
         <v/>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="10">
         <f>G3</f>
         <v/>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="10">
         <f>H3</f>
         <v/>
       </c>
-      <c r="J3" s="5">
+      <c r="J3" s="10">
         <f>I3</f>
         <v/>
       </c>
@@ -1542,27 +1542,27 @@
       <c r="D4" s="4" t="n">
         <v>270342</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="10">
         <f>'BS DRIVERS'!F3*'ANNL P&amp;L'!F2/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="10">
         <f>'BS DRIVERS'!G3*'ANNL P&amp;L'!G2/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="10">
         <f>'BS DRIVERS'!H3*'ANNL P&amp;L'!H2/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="10">
         <f>'BS DRIVERS'!I3*'ANNL P&amp;L'!I2/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="10">
         <f>'BS DRIVERS'!J3*'ANNL P&amp;L'!J2/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="10">
         <f>'BS DRIVERS'!K3*'ANNL P&amp;L'!K2/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
@@ -1582,27 +1582,27 @@
       <c r="D5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="10">
         <f>'BS DRIVERS'!F5*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="10">
         <f>'BS DRIVERS'!G5*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="10">
         <f>'BS DRIVERS'!H5*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="10">
         <f>'BS DRIVERS'!I5*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="10">
         <f>'BS DRIVERS'!J5*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="10">
         <f>'BS DRIVERS'!K5*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -1622,27 +1622,27 @@
       <c r="D6" s="4" t="n">
         <v>131165</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="10">
         <f>'BS DRIVERS'!F4*'ANNL P&amp;L'!F3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="10">
         <f>'BS DRIVERS'!G4*'ANNL P&amp;L'!G3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="10">
         <f>'BS DRIVERS'!H4*'ANNL P&amp;L'!H3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="10">
         <f>'BS DRIVERS'!I4*'ANNL P&amp;L'!I3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="10">
         <f>'BS DRIVERS'!J4*'ANNL P&amp;L'!J3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="10">
         <f>'BS DRIVERS'!K4*'ANNL P&amp;L'!K3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
@@ -1662,27 +1662,27 @@
       <c r="D7" s="4" t="n">
         <v>14124</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="10">
         <f>'BS DRIVERS'!F6*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="10">
         <f>'BS DRIVERS'!G6*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="10">
         <f>'BS DRIVERS'!H6*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="10">
         <f>'BS DRIVERS'!I6*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="10">
         <f>'BS DRIVERS'!J6*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="10">
         <f>'BS DRIVERS'!K6*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -1702,27 +1702,27 @@
       <c r="D8" s="4" t="n">
         <v>18759</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="10">
         <f>'BS DRIVERS'!F7*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="10">
         <f>'BS DRIVERS'!G7*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="10">
         <f>'BS DRIVERS'!H7*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="10">
         <f>'BS DRIVERS'!I7*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="10">
         <f>'BS DRIVERS'!J7*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="10">
         <f>'BS DRIVERS'!K7*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -1785,27 +1785,27 @@
       <c r="D10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="10">
         <f>D10</f>
         <v/>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="10">
         <f>E10</f>
         <v/>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="10">
         <f>F10</f>
         <v/>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="10">
         <f>G10</f>
         <v/>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="10">
         <f>H10</f>
         <v/>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="10">
         <f>I10</f>
         <v/>
       </c>
@@ -1825,27 +1825,27 @@
       <c r="D11" s="4" t="n">
         <v>55602</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="10">
         <f>D11-'CASH FLOW'!F28-'CASH FLOW'!F3</f>
         <v/>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="10">
         <f>E11-'CASH FLOW'!G28-'CASH FLOW'!G3</f>
         <v/>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="10">
         <f>F11-'CASH FLOW'!H28-'CASH FLOW'!H3</f>
         <v/>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="10">
         <f>G11-'CASH FLOW'!I28-'CASH FLOW'!I3</f>
         <v/>
       </c>
-      <c r="I11" s="5">
+      <c r="I11" s="10">
         <f>H11-'CASH FLOW'!J28-'CASH FLOW'!J3</f>
         <v/>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="10">
         <f>I11-'CASH FLOW'!K28-'CASH FLOW'!K3</f>
         <v/>
       </c>
@@ -1865,27 +1865,27 @@
       <c r="D12" s="4" t="n">
         <v>21606</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="10">
         <f>D12</f>
         <v/>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="10">
         <f>E12</f>
         <v/>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="10">
         <f>F12</f>
         <v/>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="10">
         <f>G12</f>
         <v/>
       </c>
-      <c r="I12" s="5">
+      <c r="I12" s="10">
         <f>H12</f>
         <v/>
       </c>
-      <c r="J12" s="5">
+      <c r="J12" s="10">
         <f>I12</f>
         <v/>
       </c>
@@ -1905,27 +1905,27 @@
       <c r="D13" s="4" t="n">
         <v>230</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="10">
         <f>D13</f>
         <v/>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="10">
         <f>E13</f>
         <v/>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="10">
         <f>F13</f>
         <v/>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="10">
         <f>G13</f>
         <v/>
       </c>
-      <c r="I13" s="5">
+      <c r="I13" s="10">
         <f>H13</f>
         <v/>
       </c>
-      <c r="J13" s="5">
+      <c r="J13" s="10">
         <f>I13</f>
         <v/>
       </c>
@@ -1945,27 +1945,27 @@
       <c r="D14" s="4" t="n">
         <v>12213</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="10">
         <f>D14</f>
         <v/>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="10">
         <f>E14</f>
         <v/>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="10">
         <f>F14</f>
         <v/>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="10">
         <f>G14</f>
         <v/>
       </c>
-      <c r="I14" s="5">
+      <c r="I14" s="10">
         <f>H14</f>
         <v/>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="10">
         <f>I14</f>
         <v/>
       </c>
@@ -1985,27 +1985,27 @@
       <c r="D15" s="4" t="n">
         <v>71582</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="10">
         <f>D15</f>
         <v/>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="10">
         <f>E15</f>
         <v/>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="10">
         <f>F15</f>
         <v/>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="10">
         <f>G15</f>
         <v/>
       </c>
-      <c r="I15" s="5">
+      <c r="I15" s="10">
         <f>H15</f>
         <v/>
       </c>
-      <c r="J15" s="5">
+      <c r="J15" s="10">
         <f>I15</f>
         <v/>
       </c>
@@ -2025,27 +2025,27 @@
       <c r="D16" s="4" t="n">
         <v>234215</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="10">
         <f>D16-'CASH FLOW'!F6</f>
         <v/>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="10">
         <f>E16-'CASH FLOW'!G6</f>
         <v/>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="10">
         <f>F16-'CASH FLOW'!H6</f>
         <v/>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="10">
         <f>G16-'CASH FLOW'!I6</f>
         <v/>
       </c>
-      <c r="I16" s="5">
+      <c r="I16" s="10">
         <f>H16-'CASH FLOW'!J6</f>
         <v/>
       </c>
-      <c r="J16" s="5">
+      <c r="J16" s="10">
         <f>I16-'CASH FLOW'!K6</f>
         <v/>
       </c>
@@ -2065,27 +2065,27 @@
       <c r="D17" s="4" t="n">
         <v>38699</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="10">
         <f>D17</f>
         <v/>
       </c>
-      <c r="F17" s="5">
+      <c r="F17" s="10">
         <f>E17</f>
         <v/>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="10">
         <f>F17</f>
         <v/>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="10">
         <f>G17</f>
         <v/>
       </c>
-      <c r="I17" s="5">
+      <c r="I17" s="10">
         <f>H17</f>
         <v/>
       </c>
-      <c r="J17" s="5">
+      <c r="J17" s="10">
         <f>I17</f>
         <v/>
       </c>
@@ -2105,27 +2105,27 @@
       <c r="D18" s="4" t="n">
         <v>8154</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="10">
         <f>'BS DRIVERS'!F9*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="F18" s="5">
+      <c r="F18" s="10">
         <f>'BS DRIVERS'!G9*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="10">
         <f>'BS DRIVERS'!H9*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="10">
         <f>'BS DRIVERS'!I9*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="I18" s="5">
+      <c r="I18" s="10">
         <f>'BS DRIVERS'!J9*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="10">
         <f>'BS DRIVERS'!K9*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -2188,27 +2188,27 @@
       <c r="D20" s="4" t="n">
         <v>41287</v>
       </c>
-      <c r="E20" s="5">
+      <c r="E20" s="10">
         <f>'BS DRIVERS'!F11*'ANNL P&amp;L'!F3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="F20" s="5">
+      <c r="F20" s="10">
         <f>'BS DRIVERS'!G11*'ANNL P&amp;L'!G3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="10">
         <f>'BS DRIVERS'!H11*'ANNL P&amp;L'!H3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="10">
         <f>'BS DRIVERS'!I11*'ANNL P&amp;L'!I3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="I20" s="5">
+      <c r="I20" s="10">
         <f>'BS DRIVERS'!J11*'ANNL P&amp;L'!J3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
-      <c r="J20" s="5">
+      <c r="J20" s="10">
         <f>'BS DRIVERS'!K11*'ANNL P&amp;L'!K3/ASSUMPTIONS!$B$2</f>
         <v/>
       </c>
@@ -2228,27 +2228,27 @@
       <c r="D21" s="4" t="n">
         <v>148780</v>
       </c>
-      <c r="E21" s="5">
+      <c r="E21" s="10">
         <f>'BS DRIVERS'!F12*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="F21" s="5">
+      <c r="F21" s="10">
         <f>'BS DRIVERS'!G12*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="10">
         <f>'BS DRIVERS'!H12*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="10">
         <f>'BS DRIVERS'!I12*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="I21" s="5">
+      <c r="I21" s="10">
         <f>'BS DRIVERS'!J12*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="J21" s="5">
+      <c r="J21" s="10">
         <f>'BS DRIVERS'!K12*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -2268,27 +2268,27 @@
       <c r="D22" s="4" t="n">
         <v>10834</v>
       </c>
-      <c r="E22" s="5">
+      <c r="E22" s="10">
         <f>'BS DRIVERS'!F13*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="F22" s="5">
+      <c r="F22" s="10">
         <f>'BS DRIVERS'!G13*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="G22" s="5">
+      <c r="G22" s="10">
         <f>'BS DRIVERS'!H13*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="H22" s="5">
+      <c r="H22" s="10">
         <f>'BS DRIVERS'!I13*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="I22" s="5">
+      <c r="I22" s="10">
         <f>'BS DRIVERS'!J13*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="J22" s="5">
+      <c r="J22" s="10">
         <f>'BS DRIVERS'!K13*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -2308,27 +2308,27 @@
       <c r="D23" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="5">
+      <c r="E23" s="10">
         <f>'BS DRIVERS'!F14*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="F23" s="5">
+      <c r="F23" s="10">
         <f>'BS DRIVERS'!G14*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="10">
         <f>'BS DRIVERS'!H14*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="H23" s="5">
+      <c r="H23" s="10">
         <f>'BS DRIVERS'!I14*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="I23" s="5">
+      <c r="I23" s="10">
         <f>'BS DRIVERS'!J14*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="J23" s="5">
+      <c r="J23" s="10">
         <f>'BS DRIVERS'!K14*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -2348,27 +2348,27 @@
       <c r="D24" s="4" t="n">
         <v>135948</v>
       </c>
-      <c r="E24" s="5">
+      <c r="E24" s="10">
         <f>'BS DRIVERS'!F15*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="F24" s="5">
+      <c r="F24" s="10">
         <f>'BS DRIVERS'!G15*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="G24" s="5">
+      <c r="G24" s="10">
         <f>'BS DRIVERS'!H15*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="H24" s="5">
+      <c r="H24" s="10">
         <f>'BS DRIVERS'!I15*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="I24" s="5">
+      <c r="I24" s="10">
         <f>'BS DRIVERS'!J15*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="J24" s="5">
+      <c r="J24" s="10">
         <f>'BS DRIVERS'!K15*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -2388,27 +2388,27 @@
       <c r="D25" s="4" t="n">
         <v>3265</v>
       </c>
-      <c r="E25" s="5">
+      <c r="E25" s="10">
         <f>'BS DRIVERS'!F16*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="F25" s="5">
+      <c r="F25" s="10">
         <f>'BS DRIVERS'!G16*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="G25" s="5">
+      <c r="G25" s="10">
         <f>'BS DRIVERS'!H16*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="H25" s="5">
+      <c r="H25" s="10">
         <f>'BS DRIVERS'!I16*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="I25" s="5">
+      <c r="I25" s="10">
         <f>'BS DRIVERS'!J16*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="J25" s="5">
+      <c r="J25" s="10">
         <f>'BS DRIVERS'!K16*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -2428,27 +2428,27 @@
       <c r="D26" s="4" t="n">
         <v>100</v>
       </c>
-      <c r="E26" s="5">
+      <c r="E26" s="10">
         <f>'BS DRIVERS'!F17*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="F26" s="5">
+      <c r="F26" s="10">
         <f>'BS DRIVERS'!G17*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="G26" s="5">
+      <c r="G26" s="10">
         <f>'BS DRIVERS'!H17*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="H26" s="5">
+      <c r="H26" s="10">
         <f>'BS DRIVERS'!I17*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="I26" s="5">
+      <c r="I26" s="10">
         <f>'BS DRIVERS'!J17*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="J26" s="5">
+      <c r="J26" s="10">
         <f>'BS DRIVERS'!K17*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -2468,27 +2468,27 @@
       <c r="D27" s="4" t="n">
         <v>9513</v>
       </c>
-      <c r="E27" s="5">
+      <c r="E27" s="10">
         <f>'BS DRIVERS'!F18*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="F27" s="5">
+      <c r="F27" s="10">
         <f>'BS DRIVERS'!G18*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="G27" s="5">
+      <c r="G27" s="10">
         <f>'BS DRIVERS'!H18*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="H27" s="5">
+      <c r="H27" s="10">
         <f>'BS DRIVERS'!I18*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="I27" s="5">
+      <c r="I27" s="10">
         <f>'BS DRIVERS'!J18*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="J27" s="5">
+      <c r="J27" s="10">
         <f>'BS DRIVERS'!K18*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -2508,27 +2508,27 @@
       <c r="D28" s="4" t="n">
         <v>15808</v>
       </c>
-      <c r="E28" s="5">
+      <c r="E28" s="10">
         <f>'BS DRIVERS'!F19*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
-      <c r="F28" s="5">
+      <c r="F28" s="10">
         <f>'BS DRIVERS'!G19*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
-      <c r="G28" s="5">
+      <c r="G28" s="10">
         <f>'BS DRIVERS'!H19*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
-      <c r="H28" s="5">
+      <c r="H28" s="10">
         <f>'BS DRIVERS'!I19*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
-      <c r="I28" s="5">
+      <c r="I28" s="10">
         <f>'BS DRIVERS'!J19*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
-      <c r="J28" s="5">
+      <c r="J28" s="10">
         <f>'BS DRIVERS'!K19*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
@@ -2591,27 +2591,27 @@
       <c r="D30" s="4" t="n">
         <v>16674</v>
       </c>
-      <c r="E30" s="5">
+      <c r="E30" s="10">
         <f>D30</f>
         <v/>
       </c>
-      <c r="F30" s="5">
+      <c r="F30" s="10">
         <f>E30</f>
         <v/>
       </c>
-      <c r="G30" s="5">
+      <c r="G30" s="10">
         <f>F30</f>
         <v/>
       </c>
-      <c r="H30" s="5">
+      <c r="H30" s="10">
         <f>G30</f>
         <v/>
       </c>
-      <c r="I30" s="5">
+      <c r="I30" s="10">
         <f>H30</f>
         <v/>
       </c>
-      <c r="J30" s="5">
+      <c r="J30" s="10">
         <f>I30</f>
         <v/>
       </c>
@@ -2631,27 +2631,27 @@
       <c r="D31" s="4" t="n">
         <v>211</v>
       </c>
-      <c r="E31" s="5">
+      <c r="E31" s="10">
         <f>D31</f>
         <v/>
       </c>
-      <c r="F31" s="5">
+      <c r="F31" s="10">
         <f>E31</f>
         <v/>
       </c>
-      <c r="G31" s="5">
+      <c r="G31" s="10">
         <f>F31</f>
         <v/>
       </c>
-      <c r="H31" s="5">
+      <c r="H31" s="10">
         <f>G31</f>
         <v/>
       </c>
-      <c r="I31" s="5">
+      <c r="I31" s="10">
         <f>H31</f>
         <v/>
       </c>
-      <c r="J31" s="5">
+      <c r="J31" s="10">
         <f>I31</f>
         <v/>
       </c>
@@ -2671,27 +2671,27 @@
       <c r="D32" s="4" t="n">
         <v>2330</v>
       </c>
-      <c r="E32" s="5">
+      <c r="E32" s="10">
         <f>D32</f>
         <v/>
       </c>
-      <c r="F32" s="5">
+      <c r="F32" s="10">
         <f>E32</f>
         <v/>
       </c>
-      <c r="G32" s="5">
+      <c r="G32" s="10">
         <f>F32</f>
         <v/>
       </c>
-      <c r="H32" s="5">
+      <c r="H32" s="10">
         <f>G32</f>
         <v/>
       </c>
-      <c r="I32" s="5">
+      <c r="I32" s="10">
         <f>H32</f>
         <v/>
       </c>
-      <c r="J32" s="5">
+      <c r="J32" s="10">
         <f>I32</f>
         <v/>
       </c>
@@ -2711,27 +2711,27 @@
       <c r="D33" s="4" t="n">
         <v>157714</v>
       </c>
-      <c r="E33" s="5">
+      <c r="E33" s="10">
         <f>D33</f>
         <v/>
       </c>
-      <c r="F33" s="5">
+      <c r="F33" s="10">
         <f>E33</f>
         <v/>
       </c>
-      <c r="G33" s="5">
+      <c r="G33" s="10">
         <f>F33</f>
         <v/>
       </c>
-      <c r="H33" s="5">
+      <c r="H33" s="10">
         <f>G33</f>
         <v/>
       </c>
-      <c r="I33" s="5">
+      <c r="I33" s="10">
         <f>H33</f>
         <v/>
       </c>
-      <c r="J33" s="5">
+      <c r="J33" s="10">
         <f>I33</f>
         <v/>
       </c>
@@ -2794,27 +2794,27 @@
       <c r="D35" s="4" t="n">
         <v>824488</v>
       </c>
-      <c r="E35" s="5">
+      <c r="E35" s="10">
         <f>D35</f>
         <v/>
       </c>
-      <c r="F35" s="5">
+      <c r="F35" s="10">
         <f>E35</f>
         <v/>
       </c>
-      <c r="G35" s="5">
+      <c r="G35" s="10">
         <f>F35</f>
         <v/>
       </c>
-      <c r="H35" s="5">
+      <c r="H35" s="10">
         <f>G35</f>
         <v/>
       </c>
-      <c r="I35" s="5">
+      <c r="I35" s="10">
         <f>H35</f>
         <v/>
       </c>
-      <c r="J35" s="5">
+      <c r="J35" s="10">
         <f>I35</f>
         <v/>
       </c>
@@ -2834,27 +2834,27 @@
       <c r="D36" s="4" t="n">
         <v>79</v>
       </c>
-      <c r="E36" s="5">
+      <c r="E36" s="10">
         <f>D36</f>
         <v/>
       </c>
-      <c r="F36" s="5">
+      <c r="F36" s="10">
         <f>E36</f>
         <v/>
       </c>
-      <c r="G36" s="5">
+      <c r="G36" s="10">
         <f>F36</f>
         <v/>
       </c>
-      <c r="H36" s="5">
+      <c r="H36" s="10">
         <f>G36</f>
         <v/>
       </c>
-      <c r="I36" s="5">
+      <c r="I36" s="10">
         <f>H36</f>
         <v/>
       </c>
-      <c r="J36" s="5">
+      <c r="J36" s="10">
         <f>I36</f>
         <v/>
       </c>
@@ -2874,27 +2874,27 @@
       <c r="D37" s="4" t="n">
         <v>297579</v>
       </c>
-      <c r="E37" s="5">
+      <c r="E37" s="10">
         <f>D37+'CASH FLOW'!F9+'CASH FLOW'!F33</f>
         <v/>
       </c>
-      <c r="F37" s="5">
+      <c r="F37" s="10">
         <f>E37+'CASH FLOW'!G9+'CASH FLOW'!G33</f>
         <v/>
       </c>
-      <c r="G37" s="5">
+      <c r="G37" s="10">
         <f>F37+'CASH FLOW'!H9+'CASH FLOW'!H33</f>
         <v/>
       </c>
-      <c r="H37" s="5">
+      <c r="H37" s="10">
         <f>G37+'CASH FLOW'!I9+'CASH FLOW'!I33</f>
         <v/>
       </c>
-      <c r="I37" s="5">
+      <c r="I37" s="10">
         <f>H37+'CASH FLOW'!J9+'CASH FLOW'!J33</f>
         <v/>
       </c>
-      <c r="J37" s="5">
+      <c r="J37" s="10">
         <f>I37+'CASH FLOW'!K9+'CASH FLOW'!K33</f>
         <v/>
       </c>
@@ -2914,27 +2914,27 @@
       <c r="D38" s="4" t="n">
         <v>-3250</v>
       </c>
-      <c r="E38" s="5">
+      <c r="E38" s="10">
         <f>D38+'CASH FLOW'!F39</f>
         <v/>
       </c>
-      <c r="F38" s="5">
+      <c r="F38" s="10">
         <f>E38+'CASH FLOW'!G39</f>
         <v/>
       </c>
-      <c r="G38" s="5">
+      <c r="G38" s="10">
         <f>F38+'CASH FLOW'!H39</f>
         <v/>
       </c>
-      <c r="H38" s="5">
+      <c r="H38" s="10">
         <f>G38+'CASH FLOW'!I39</f>
         <v/>
       </c>
-      <c r="I38" s="5">
+      <c r="I38" s="10">
         <f>H38+'CASH FLOW'!J39</f>
         <v/>
       </c>
-      <c r="J38" s="5">
+      <c r="J38" s="10">
         <f>I38+'CASH FLOW'!K39</f>
         <v/>
       </c>
@@ -2954,27 +2954,27 @@
       <c r="D39" s="4" t="n">
         <v>105521</v>
       </c>
-      <c r="E39" s="5">
+      <c r="E39" s="10">
         <f>D39+'ANNL P&amp;L'!F12+'CASH FLOW'!F35</f>
         <v/>
       </c>
-      <c r="F39" s="5">
+      <c r="F39" s="10">
         <f>E39+'ANNL P&amp;L'!G12+'CASH FLOW'!G35</f>
         <v/>
       </c>
-      <c r="G39" s="5">
+      <c r="G39" s="10">
         <f>F39+'ANNL P&amp;L'!H12+'CASH FLOW'!H35</f>
         <v/>
       </c>
-      <c r="H39" s="5">
+      <c r="H39" s="10">
         <f>G39+'ANNL P&amp;L'!I12+'CASH FLOW'!I35</f>
         <v/>
       </c>
-      <c r="I39" s="5">
+      <c r="I39" s="10">
         <f>H39+'ANNL P&amp;L'!J12+'CASH FLOW'!J35</f>
         <v/>
       </c>
-      <c r="J39" s="5">
+      <c r="J39" s="10">
         <f>I39+'ANNL P&amp;L'!K12+'CASH FLOW'!K35</f>
         <v/>
       </c>
@@ -3163,27 +3163,27 @@
       <c r="E2" s="4" t="n">
         <v>145074</v>
       </c>
-      <c r="F2" s="5">
+      <c r="F2" s="10">
         <f>'ANNL P&amp;L'!F12</f>
         <v/>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="10">
         <f>'ANNL P&amp;L'!G12</f>
         <v/>
       </c>
-      <c r="H2" s="5">
+      <c r="H2" s="10">
         <f>'ANNL P&amp;L'!H12</f>
         <v/>
       </c>
-      <c r="I2" s="5">
+      <c r="I2" s="10">
         <f>'ANNL P&amp;L'!I12</f>
         <v/>
       </c>
-      <c r="J2" s="5">
+      <c r="J2" s="10">
         <f>'ANNL P&amp;L'!J12</f>
         <v/>
       </c>
-      <c r="K2" s="5">
+      <c r="K2" s="10">
         <f>'ANNL P&amp;L'!K12</f>
         <v/>
       </c>
@@ -3206,27 +3206,27 @@
       <c r="E3" s="4" t="n">
         <v>7274</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="10">
         <f>'CF DRIVERS'!F2*'BALANCE SHEET'!D11</f>
         <v/>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="10">
         <f>'CF DRIVERS'!G2*'BALANCE SHEET'!E11</f>
         <v/>
       </c>
-      <c r="H3" s="5">
+      <c r="H3" s="10">
         <f>'CF DRIVERS'!H2*'BALANCE SHEET'!F11</f>
         <v/>
       </c>
-      <c r="I3" s="5">
+      <c r="I3" s="10">
         <f>'CF DRIVERS'!I2*'BALANCE SHEET'!G11</f>
         <v/>
       </c>
-      <c r="J3" s="5">
+      <c r="J3" s="10">
         <f>'CF DRIVERS'!J2*'BALANCE SHEET'!H11</f>
         <v/>
       </c>
-      <c r="K3" s="5">
+      <c r="K3" s="10">
         <f>'CF DRIVERS'!K2*'BALANCE SHEET'!I11</f>
         <v/>
       </c>
@@ -3249,27 +3249,27 @@
       <c r="E4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="10">
         <f>E4</f>
         <v/>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="10">
         <f>F4</f>
         <v/>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="10">
         <f>G4</f>
         <v/>
       </c>
-      <c r="I4" s="5">
+      <c r="I4" s="10">
         <f>H4</f>
         <v/>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="10">
         <f>I4</f>
         <v/>
       </c>
-      <c r="K4" s="5">
+      <c r="K4" s="10">
         <f>J4</f>
         <v/>
       </c>
@@ -3292,27 +3292,27 @@
       <c r="E5" s="4" t="n">
         <v>3294</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="G5" s="5">
+      <c r="G5" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="H5" s="5">
+      <c r="H5" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="I5" s="5">
+      <c r="I5" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="K5" s="5">
+      <c r="K5" s="10">
         <f>0</f>
         <v/>
       </c>
@@ -3335,27 +3335,27 @@
       <c r="E6" s="4" t="n">
         <v>14124</v>
       </c>
-      <c r="F6" s="5">
+      <c r="F6" s="10">
         <f>E6</f>
         <v/>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="10">
         <f>F6</f>
         <v/>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="10">
         <f>G6</f>
         <v/>
       </c>
-      <c r="I6" s="5">
+      <c r="I6" s="10">
         <f>H6</f>
         <v/>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="10">
         <f>I6</f>
         <v/>
       </c>
-      <c r="K6" s="5">
+      <c r="K6" s="10">
         <f>J6</f>
         <v/>
       </c>
@@ -3378,27 +3378,27 @@
       <c r="E7" s="4" t="n">
         <v>19086</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="H7" s="5">
+      <c r="H7" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="I7" s="5">
+      <c r="I7" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="K7" s="5">
+      <c r="K7" s="10">
         <f>0</f>
         <v/>
       </c>
@@ -3421,27 +3421,27 @@
       <c r="E8" s="4" t="n">
         <v>173</v>
       </c>
-      <c r="F8" s="5">
+      <c r="F8" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="H8" s="5">
+      <c r="H8" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="I8" s="5">
+      <c r="I8" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="K8" s="5">
+      <c r="K8" s="10">
         <f>0</f>
         <v/>
       </c>
@@ -3464,27 +3464,27 @@
       <c r="E9" s="4" t="n">
         <v>19591</v>
       </c>
-      <c r="F9" s="5">
+      <c r="F9" s="10">
         <f>'CF DRIVERS'!F3</f>
         <v/>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="10">
         <f>'CF DRIVERS'!G3</f>
         <v/>
       </c>
-      <c r="H9" s="5">
+      <c r="H9" s="10">
         <f>'CF DRIVERS'!H3</f>
         <v/>
       </c>
-      <c r="I9" s="5">
+      <c r="I9" s="10">
         <f>'CF DRIVERS'!I3</f>
         <v/>
       </c>
-      <c r="J9" s="5">
+      <c r="J9" s="10">
         <f>'CF DRIVERS'!J3</f>
         <v/>
       </c>
-      <c r="K9" s="5">
+      <c r="K9" s="10">
         <f>'CF DRIVERS'!K3</f>
         <v/>
       </c>
@@ -3507,27 +3507,27 @@
       <c r="E10" s="4" t="n">
         <v>-9730</v>
       </c>
-      <c r="F10" s="5">
+      <c r="F10" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="G10" s="5">
+      <c r="G10" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="H10" s="5">
+      <c r="H10" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="I10" s="5">
+      <c r="I10" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="J10" s="5">
+      <c r="J10" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="K10" s="5">
+      <c r="K10" s="10">
         <f>0</f>
         <v/>
       </c>
@@ -3550,27 +3550,27 @@
       <c r="E11" s="4" t="n">
         <v>1734</v>
       </c>
-      <c r="F11" s="5">
+      <c r="F11" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="I11" s="5">
+      <c r="I11" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="J11" s="5">
+      <c r="J11" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="K11" s="5">
+      <c r="K11" s="10">
         <f>0</f>
         <v/>
       </c>
@@ -3593,27 +3593,27 @@
       <c r="E12" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="5">
+      <c r="F12" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="I12" s="5">
+      <c r="I12" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="J12" s="5">
+      <c r="J12" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="K12" s="5">
+      <c r="K12" s="10">
         <f>0</f>
         <v/>
       </c>
@@ -3636,27 +3636,27 @@
       <c r="E13" s="4" t="n">
         <v>-324</v>
       </c>
-      <c r="F13" s="5">
+      <c r="F13" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="I13" s="5">
+      <c r="I13" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="J13" s="5">
+      <c r="J13" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="K13" s="5">
+      <c r="K13" s="10">
         <f>0</f>
         <v/>
       </c>
@@ -3679,27 +3679,27 @@
       <c r="E14" s="4" t="n">
         <v>-89665</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="10">
         <f>-('BALANCE SHEET'!E4-'BALANCE SHEET'!D4)</f>
         <v/>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="10">
         <f>-('BALANCE SHEET'!F4-'BALANCE SHEET'!E4)</f>
         <v/>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="10">
         <f>-('BALANCE SHEET'!G4-'BALANCE SHEET'!F4)</f>
         <v/>
       </c>
-      <c r="I14" s="5">
+      <c r="I14" s="10">
         <f>-('BALANCE SHEET'!H4-'BALANCE SHEET'!G4)</f>
         <v/>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="10">
         <f>-('BALANCE SHEET'!I4-'BALANCE SHEET'!H4)</f>
         <v/>
       </c>
-      <c r="K14" s="5">
+      <c r="K14" s="10">
         <f>-('BALANCE SHEET'!J4-'BALANCE SHEET'!I4)</f>
         <v/>
       </c>
@@ -3722,27 +3722,27 @@
       <c r="E15" s="4" t="n">
         <v>2318</v>
       </c>
-      <c r="F15" s="5">
+      <c r="F15" s="10">
         <f>-('BALANCE SHEET'!E5-'BALANCE SHEET'!D5)</f>
         <v/>
       </c>
-      <c r="G15" s="5">
+      <c r="G15" s="10">
         <f>-('BALANCE SHEET'!F5-'BALANCE SHEET'!E5)</f>
         <v/>
       </c>
-      <c r="H15" s="5">
+      <c r="H15" s="10">
         <f>-('BALANCE SHEET'!G5-'BALANCE SHEET'!F5)</f>
         <v/>
       </c>
-      <c r="I15" s="5">
+      <c r="I15" s="10">
         <f>-('BALANCE SHEET'!H5-'BALANCE SHEET'!G5)</f>
         <v/>
       </c>
-      <c r="J15" s="5">
+      <c r="J15" s="10">
         <f>-('BALANCE SHEET'!I5-'BALANCE SHEET'!H5)</f>
         <v/>
       </c>
-      <c r="K15" s="5">
+      <c r="K15" s="10">
         <f>-('BALANCE SHEET'!J5-'BALANCE SHEET'!I5)</f>
         <v/>
       </c>
@@ -3765,27 +3765,27 @@
       <c r="E16" s="4" t="n">
         <v>77190</v>
       </c>
-      <c r="F16" s="5">
+      <c r="F16" s="10">
         <f>-('BALANCE SHEET'!E6-'BALANCE SHEET'!D6)</f>
         <v/>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="10">
         <f>-('BALANCE SHEET'!F6-'BALANCE SHEET'!E6)</f>
         <v/>
       </c>
-      <c r="H16" s="5">
+      <c r="H16" s="10">
         <f>-('BALANCE SHEET'!G6-'BALANCE SHEET'!F6)</f>
         <v/>
       </c>
-      <c r="I16" s="5">
+      <c r="I16" s="10">
         <f>-('BALANCE SHEET'!H6-'BALANCE SHEET'!G6)</f>
         <v/>
       </c>
-      <c r="J16" s="5">
+      <c r="J16" s="10">
         <f>-('BALANCE SHEET'!I6-'BALANCE SHEET'!H6)</f>
         <v/>
       </c>
-      <c r="K16" s="5">
+      <c r="K16" s="10">
         <f>-('BALANCE SHEET'!J6-'BALANCE SHEET'!I6)</f>
         <v/>
       </c>
@@ -3808,27 +3808,27 @@
       <c r="E17" s="4" t="n">
         <v>1074</v>
       </c>
-      <c r="F17" s="5">
+      <c r="F17" s="10">
         <f>-('BALANCE SHEET'!E8-'BALANCE SHEET'!D8)</f>
         <v/>
       </c>
-      <c r="G17" s="5">
+      <c r="G17" s="10">
         <f>-('BALANCE SHEET'!F8-'BALANCE SHEET'!E8)</f>
         <v/>
       </c>
-      <c r="H17" s="5">
+      <c r="H17" s="10">
         <f>-('BALANCE SHEET'!G8-'BALANCE SHEET'!F8)</f>
         <v/>
       </c>
-      <c r="I17" s="5">
+      <c r="I17" s="10">
         <f>-('BALANCE SHEET'!H8-'BALANCE SHEET'!G8)</f>
         <v/>
       </c>
-      <c r="J17" s="5">
+      <c r="J17" s="10">
         <f>-('BALANCE SHEET'!I8-'BALANCE SHEET'!H8)</f>
         <v/>
       </c>
-      <c r="K17" s="5">
+      <c r="K17" s="10">
         <f>-('BALANCE SHEET'!J8-'BALANCE SHEET'!I8)</f>
         <v/>
       </c>
@@ -3851,27 +3851,27 @@
       <c r="E18" s="4" t="n">
         <v>-1170</v>
       </c>
-      <c r="F18" s="5">
+      <c r="F18" s="10">
         <f>('BALANCE SHEET'!E20-'BALANCE SHEET'!D20)</f>
         <v/>
       </c>
-      <c r="G18" s="5">
+      <c r="G18" s="10">
         <f>('BALANCE SHEET'!F20-'BALANCE SHEET'!E20)</f>
         <v/>
       </c>
-      <c r="H18" s="5">
+      <c r="H18" s="10">
         <f>('BALANCE SHEET'!G20-'BALANCE SHEET'!F20)</f>
         <v/>
       </c>
-      <c r="I18" s="5">
+      <c r="I18" s="10">
         <f>('BALANCE SHEET'!H20-'BALANCE SHEET'!G20)</f>
         <v/>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="10">
         <f>('BALANCE SHEET'!I20-'BALANCE SHEET'!H20)</f>
         <v/>
       </c>
-      <c r="K18" s="5">
+      <c r="K18" s="10">
         <f>('BALANCE SHEET'!J20-'BALANCE SHEET'!I20)</f>
         <v/>
       </c>
@@ -3894,27 +3894,27 @@
       <c r="E19" s="4" t="n">
         <v>85398</v>
       </c>
-      <c r="F19" s="5">
+      <c r="F19" s="10">
         <f>('BALANCE SHEET'!E21-'BALANCE SHEET'!D21)</f>
         <v/>
       </c>
-      <c r="G19" s="5">
+      <c r="G19" s="10">
         <f>('BALANCE SHEET'!F21-'BALANCE SHEET'!E21)</f>
         <v/>
       </c>
-      <c r="H19" s="5">
+      <c r="H19" s="10">
         <f>('BALANCE SHEET'!G21-'BALANCE SHEET'!F21)</f>
         <v/>
       </c>
-      <c r="I19" s="5">
+      <c r="I19" s="10">
         <f>('BALANCE SHEET'!H21-'BALANCE SHEET'!G21)</f>
         <v/>
       </c>
-      <c r="J19" s="5">
+      <c r="J19" s="10">
         <f>('BALANCE SHEET'!I21-'BALANCE SHEET'!H21)</f>
         <v/>
       </c>
-      <c r="K19" s="5">
+      <c r="K19" s="10">
         <f>('BALANCE SHEET'!J21-'BALANCE SHEET'!I21)</f>
         <v/>
       </c>
@@ -3937,27 +3937,27 @@
       <c r="E20" s="4" t="n">
         <v>-34616</v>
       </c>
-      <c r="F20" s="5">
+      <c r="F20" s="10">
         <f>('BALANCE SHEET'!E28-'BALANCE SHEET'!D28)</f>
         <v/>
       </c>
-      <c r="G20" s="5">
+      <c r="G20" s="10">
         <f>('BALANCE SHEET'!F28-'BALANCE SHEET'!E28)</f>
         <v/>
       </c>
-      <c r="H20" s="5">
+      <c r="H20" s="10">
         <f>('BALANCE SHEET'!G28-'BALANCE SHEET'!F28)</f>
         <v/>
       </c>
-      <c r="I20" s="5">
+      <c r="I20" s="10">
         <f>('BALANCE SHEET'!H28-'BALANCE SHEET'!G28)</f>
         <v/>
       </c>
-      <c r="J20" s="5">
+      <c r="J20" s="10">
         <f>('BALANCE SHEET'!I28-'BALANCE SHEET'!H28)</f>
         <v/>
       </c>
-      <c r="K20" s="5">
+      <c r="K20" s="10">
         <f>('BALANCE SHEET'!J28-'BALANCE SHEET'!I28)</f>
         <v/>
       </c>
@@ -3980,27 +3980,27 @@
       <c r="E21" s="4" t="n">
         <v>36161</v>
       </c>
-      <c r="F21" s="5">
+      <c r="F21" s="10">
         <f>('BALANCE SHEET'!E24-'BALANCE SHEET'!D24)</f>
         <v/>
       </c>
-      <c r="G21" s="5">
+      <c r="G21" s="10">
         <f>('BALANCE SHEET'!F24-'BALANCE SHEET'!E24)</f>
         <v/>
       </c>
-      <c r="H21" s="5">
+      <c r="H21" s="10">
         <f>('BALANCE SHEET'!G24-'BALANCE SHEET'!F24)</f>
         <v/>
       </c>
-      <c r="I21" s="5">
+      <c r="I21" s="10">
         <f>('BALANCE SHEET'!H24-'BALANCE SHEET'!G24)</f>
         <v/>
       </c>
-      <c r="J21" s="5">
+      <c r="J21" s="10">
         <f>('BALANCE SHEET'!I24-'BALANCE SHEET'!H24)</f>
         <v/>
       </c>
-      <c r="K21" s="5">
+      <c r="K21" s="10">
         <f>('BALANCE SHEET'!J24-'BALANCE SHEET'!I24)</f>
         <v/>
       </c>
@@ -4023,27 +4023,27 @@
       <c r="E22" s="4" t="n">
         <v>-248</v>
       </c>
-      <c r="F22" s="5">
+      <c r="F22" s="10">
         <f>('BALANCE SHEET'!E23-'BALANCE SHEET'!D23)</f>
         <v/>
       </c>
-      <c r="G22" s="5">
+      <c r="G22" s="10">
         <f>('BALANCE SHEET'!F23-'BALANCE SHEET'!E23)</f>
         <v/>
       </c>
-      <c r="H22" s="5">
+      <c r="H22" s="10">
         <f>('BALANCE SHEET'!G23-'BALANCE SHEET'!F23)</f>
         <v/>
       </c>
-      <c r="I22" s="5">
+      <c r="I22" s="10">
         <f>('BALANCE SHEET'!H23-'BALANCE SHEET'!G23)</f>
         <v/>
       </c>
-      <c r="J22" s="5">
+      <c r="J22" s="10">
         <f>('BALANCE SHEET'!I23-'BALANCE SHEET'!H23)</f>
         <v/>
       </c>
-      <c r="K22" s="5">
+      <c r="K22" s="10">
         <f>('BALANCE SHEET'!J23-'BALANCE SHEET'!I23)</f>
         <v/>
       </c>
@@ -4066,27 +4066,27 @@
       <c r="E23" s="4" t="n">
         <v>535</v>
       </c>
-      <c r="F23" s="5">
+      <c r="F23" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="H23" s="5">
+      <c r="H23" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="I23" s="5">
+      <c r="I23" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="J23" s="5">
+      <c r="J23" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="K23" s="5">
+      <c r="K23" s="10">
         <f>0</f>
         <v/>
       </c>
@@ -4109,27 +4109,27 @@
       <c r="E24" s="4" t="n">
         <v>-9513</v>
       </c>
-      <c r="F24" s="5">
+      <c r="F24" s="10">
         <f>(('BALANCE SHEET'!E27+'BALANCE SHEET'!E33)-('BALANCE SHEET'!D27+'BALANCE SHEET'!D33))</f>
         <v/>
       </c>
-      <c r="G24" s="5">
+      <c r="G24" s="10">
         <f>(('BALANCE SHEET'!F27+'BALANCE SHEET'!F33)-('BALANCE SHEET'!E27+'BALANCE SHEET'!E33))</f>
         <v/>
       </c>
-      <c r="H24" s="5">
+      <c r="H24" s="10">
         <f>(('BALANCE SHEET'!G27+'BALANCE SHEET'!G33)-('BALANCE SHEET'!F27+'BALANCE SHEET'!F33))</f>
         <v/>
       </c>
-      <c r="I24" s="5">
+      <c r="I24" s="10">
         <f>(('BALANCE SHEET'!H27+'BALANCE SHEET'!H33)-('BALANCE SHEET'!G27+'BALANCE SHEET'!G33))</f>
         <v/>
       </c>
-      <c r="J24" s="5">
+      <c r="J24" s="10">
         <f>(('BALANCE SHEET'!I27+'BALANCE SHEET'!I33)-('BALANCE SHEET'!H27+'BALANCE SHEET'!H33))</f>
         <v/>
       </c>
-      <c r="K24" s="5">
+      <c r="K24" s="10">
         <f>(('BALANCE SHEET'!J27+'BALANCE SHEET'!J33)-('BALANCE SHEET'!I27+'BALANCE SHEET'!I33))</f>
         <v/>
       </c>
@@ -4152,27 +4152,27 @@
       <c r="E25" s="4" t="n">
         <v>-4862</v>
       </c>
-      <c r="F25" s="5">
+      <c r="F25" s="10">
         <f>-('BALANCE SHEET'!E18-'BALANCE SHEET'!D18)</f>
         <v/>
       </c>
-      <c r="G25" s="5">
+      <c r="G25" s="10">
         <f>-('BALANCE SHEET'!F18-'BALANCE SHEET'!E18)</f>
         <v/>
       </c>
-      <c r="H25" s="5">
+      <c r="H25" s="10">
         <f>-('BALANCE SHEET'!G18-'BALANCE SHEET'!F18)</f>
         <v/>
       </c>
-      <c r="I25" s="5">
+      <c r="I25" s="10">
         <f>-('BALANCE SHEET'!H18-'BALANCE SHEET'!G18)</f>
         <v/>
       </c>
-      <c r="J25" s="5">
+      <c r="J25" s="10">
         <f>-('BALANCE SHEET'!I18-'BALANCE SHEET'!H18)</f>
         <v/>
       </c>
-      <c r="K25" s="5">
+      <c r="K25" s="10">
         <f>-('BALANCE SHEET'!J18-'BALANCE SHEET'!I18)</f>
         <v/>
       </c>
@@ -4242,27 +4242,27 @@
       <c r="E27" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F27" s="5">
+      <c r="F27" s="10">
         <f>E27</f>
         <v/>
       </c>
-      <c r="G27" s="5">
+      <c r="G27" s="10">
         <f>F27</f>
         <v/>
       </c>
-      <c r="H27" s="5">
+      <c r="H27" s="10">
         <f>G27</f>
         <v/>
       </c>
-      <c r="I27" s="5">
+      <c r="I27" s="10">
         <f>H27</f>
         <v/>
       </c>
-      <c r="J27" s="5">
+      <c r="J27" s="10">
         <f>I27</f>
         <v/>
       </c>
-      <c r="K27" s="5">
+      <c r="K27" s="10">
         <f>J27</f>
         <v/>
       </c>
@@ -4285,27 +4285,27 @@
       <c r="E28" s="4" t="n">
         <v>-23390</v>
       </c>
-      <c r="F28" s="5">
+      <c r="F28" s="10">
         <f>'CF DRIVERS'!F4*'BALANCE SHEET'!D11</f>
         <v/>
       </c>
-      <c r="G28" s="5">
+      <c r="G28" s="10">
         <f>'CF DRIVERS'!G4*'BALANCE SHEET'!E11</f>
         <v/>
       </c>
-      <c r="H28" s="5">
+      <c r="H28" s="10">
         <f>'CF DRIVERS'!H4*'BALANCE SHEET'!F11</f>
         <v/>
       </c>
-      <c r="I28" s="5">
+      <c r="I28" s="10">
         <f>'CF DRIVERS'!I4*'BALANCE SHEET'!G11</f>
         <v/>
       </c>
-      <c r="J28" s="5">
+      <c r="J28" s="10">
         <f>'CF DRIVERS'!J4*'BALANCE SHEET'!H11</f>
         <v/>
       </c>
-      <c r="K28" s="5">
+      <c r="K28" s="10">
         <f>'CF DRIVERS'!K4*'BALANCE SHEET'!I11</f>
         <v/>
       </c>
@@ -4328,12 +4328,12 @@
       <c r="E29" s="4" t="n">
         <v>-3000</v>
       </c>
-      <c r="F29" s="5" t="n"/>
-      <c r="G29" s="5" t="n"/>
-      <c r="H29" s="5" t="n"/>
-      <c r="I29" s="5" t="n"/>
-      <c r="J29" s="5" t="n"/>
-      <c r="K29" s="5" t="n"/>
+      <c r="F29" s="10" t="n"/>
+      <c r="G29" s="10" t="n"/>
+      <c r="H29" s="10" t="n"/>
+      <c r="I29" s="10" t="n"/>
+      <c r="J29" s="10" t="n"/>
+      <c r="K29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
@@ -4353,12 +4353,12 @@
       <c r="E30" s="4" t="n">
         <v>-75336</v>
       </c>
-      <c r="F30" s="5" t="n"/>
-      <c r="G30" s="5" t="n"/>
-      <c r="H30" s="5" t="n"/>
-      <c r="I30" s="5" t="n"/>
-      <c r="J30" s="5" t="n"/>
-      <c r="K30" s="5" t="n"/>
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="10" t="n"/>
+      <c r="H30" s="10" t="n"/>
+      <c r="I30" s="10" t="n"/>
+      <c r="J30" s="10" t="n"/>
+      <c r="K30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -4425,27 +4425,27 @@
       <c r="E32" s="4" t="n">
         <v>-61</v>
       </c>
-      <c r="F32" s="5">
+      <c r="F32" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="G32" s="5">
+      <c r="G32" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="H32" s="5">
+      <c r="H32" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="I32" s="5">
+      <c r="I32" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="J32" s="5">
+      <c r="J32" s="10">
         <f>0</f>
         <v/>
       </c>
-      <c r="K32" s="5">
+      <c r="K32" s="10">
         <f>0</f>
         <v/>
       </c>
@@ -4468,27 +4468,27 @@
       <c r="E33" s="4" t="n">
         <v>3856</v>
       </c>
-      <c r="F33" s="5">
+      <c r="F33" s="10">
         <f>E33</f>
         <v/>
       </c>
-      <c r="G33" s="5">
+      <c r="G33" s="10">
         <f>F33</f>
         <v/>
       </c>
-      <c r="H33" s="5">
+      <c r="H33" s="10">
         <f>G33</f>
         <v/>
       </c>
-      <c r="I33" s="5">
+      <c r="I33" s="10">
         <f>H33</f>
         <v/>
       </c>
-      <c r="J33" s="5">
+      <c r="J33" s="10">
         <f>I33</f>
         <v/>
       </c>
-      <c r="K33" s="5">
+      <c r="K33" s="10">
         <f>J33</f>
         <v/>
       </c>
@@ -4511,27 +4511,27 @@
       <c r="E34" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F34" s="5">
+      <c r="F34" s="10">
         <f>E34</f>
         <v/>
       </c>
-      <c r="G34" s="5">
+      <c r="G34" s="10">
         <f>F34</f>
         <v/>
       </c>
-      <c r="H34" s="5">
+      <c r="H34" s="10">
         <f>G34</f>
         <v/>
       </c>
-      <c r="I34" s="5">
+      <c r="I34" s="10">
         <f>H34</f>
         <v/>
       </c>
-      <c r="J34" s="5">
+      <c r="J34" s="10">
         <f>I34</f>
         <v/>
       </c>
-      <c r="K34" s="5">
+      <c r="K34" s="10">
         <f>J34</f>
         <v/>
       </c>
@@ -4554,27 +4554,27 @@
       <c r="E35" s="4" t="n">
         <v>-27500</v>
       </c>
-      <c r="F35" s="5">
+      <c r="F35" s="10">
         <f>'CF DRIVERS'!F5*'BALANCE SHEET'!E35</f>
         <v/>
       </c>
-      <c r="G35" s="5">
+      <c r="G35" s="10">
         <f>'CF DRIVERS'!G5*'BALANCE SHEET'!F35</f>
         <v/>
       </c>
-      <c r="H35" s="5">
+      <c r="H35" s="10">
         <f>'CF DRIVERS'!H5*'BALANCE SHEET'!G35</f>
         <v/>
       </c>
-      <c r="I35" s="5">
+      <c r="I35" s="10">
         <f>'CF DRIVERS'!I5*'BALANCE SHEET'!H35</f>
         <v/>
       </c>
-      <c r="J35" s="5">
+      <c r="J35" s="10">
         <f>'CF DRIVERS'!J5*'BALANCE SHEET'!I35</f>
         <v/>
       </c>
-      <c r="K35" s="5">
+      <c r="K35" s="10">
         <f>'CF DRIVERS'!K5*'BALANCE SHEET'!J35</f>
         <v/>
       </c>
@@ -4597,27 +4597,27 @@
       <c r="E36" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F36" s="5">
+      <c r="F36" s="10">
         <f>E36</f>
         <v/>
       </c>
-      <c r="G36" s="5">
+      <c r="G36" s="10">
         <f>F36</f>
         <v/>
       </c>
-      <c r="H36" s="5">
+      <c r="H36" s="10">
         <f>G36</f>
         <v/>
       </c>
-      <c r="I36" s="5">
+      <c r="I36" s="10">
         <f>H36</f>
         <v/>
       </c>
-      <c r="J36" s="5">
+      <c r="J36" s="10">
         <f>I36</f>
         <v/>
       </c>
-      <c r="K36" s="5">
+      <c r="K36" s="10">
         <f>J36</f>
         <v/>
       </c>
@@ -4640,27 +4640,27 @@
       <c r="E37" s="4" t="n">
         <v>-2261</v>
       </c>
-      <c r="F37" s="5">
+      <c r="F37" s="10">
         <f>'CF DRIVERS'!F7</f>
         <v/>
       </c>
-      <c r="G37" s="5">
+      <c r="G37" s="10">
         <f>'CF DRIVERS'!G7</f>
         <v/>
       </c>
-      <c r="H37" s="5">
+      <c r="H37" s="10">
         <f>'CF DRIVERS'!H7</f>
         <v/>
       </c>
-      <c r="I37" s="5">
+      <c r="I37" s="10">
         <f>'CF DRIVERS'!I7</f>
         <v/>
       </c>
-      <c r="J37" s="5">
+      <c r="J37" s="10">
         <f>'CF DRIVERS'!J7</f>
         <v/>
       </c>
-      <c r="K37" s="5">
+      <c r="K37" s="10">
         <f>'CF DRIVERS'!K7</f>
         <v/>
       </c>
@@ -4730,27 +4730,27 @@
       <c r="E39" s="4" t="n">
         <v>-997</v>
       </c>
-      <c r="F39" s="5">
+      <c r="F39" s="10">
         <f>E39</f>
         <v/>
       </c>
-      <c r="G39" s="5">
+      <c r="G39" s="10">
         <f>F39</f>
         <v/>
       </c>
-      <c r="H39" s="5">
+      <c r="H39" s="10">
         <f>G39</f>
         <v/>
       </c>
-      <c r="I39" s="5">
+      <c r="I39" s="10">
         <f>H39</f>
         <v/>
       </c>
-      <c r="J39" s="5">
+      <c r="J39" s="10">
         <f>I39</f>
         <v/>
       </c>
-      <c r="K39" s="5">
+      <c r="K39" s="10">
         <f>J39</f>
         <v/>
       </c>
@@ -4773,27 +4773,27 @@
       <c r="E40" s="4" t="n">
         <v>134209</v>
       </c>
-      <c r="F40" s="5">
+      <c r="F40" s="10">
         <f>'CASH FLOW'!F26+'CASH FLOW'!F31+'CASH FLOW'!F38+'CASH FLOW'!F39</f>
         <v/>
       </c>
-      <c r="G40" s="5">
+      <c r="G40" s="10">
         <f>'CASH FLOW'!G26+'CASH FLOW'!G31+'CASH FLOW'!G38+'CASH FLOW'!G39</f>
         <v/>
       </c>
-      <c r="H40" s="5">
+      <c r="H40" s="10">
         <f>'CASH FLOW'!H26+'CASH FLOW'!H31+'CASH FLOW'!H38+'CASH FLOW'!H39</f>
         <v/>
       </c>
-      <c r="I40" s="5">
+      <c r="I40" s="10">
         <f>'CASH FLOW'!I26+'CASH FLOW'!I31+'CASH FLOW'!I38+'CASH FLOW'!I39</f>
         <v/>
       </c>
-      <c r="J40" s="5">
+      <c r="J40" s="10">
         <f>'CASH FLOW'!J26+'CASH FLOW'!J31+'CASH FLOW'!J38+'CASH FLOW'!J39</f>
         <v/>
       </c>
-      <c r="K40" s="5">
+      <c r="K40" s="10">
         <f>'CASH FLOW'!K26+'CASH FLOW'!K31+'CASH FLOW'!K38+'CASH FLOW'!K39</f>
         <v/>
       </c>
@@ -4816,27 +4816,27 @@
       <c r="E41" s="4" t="n">
         <v>755981</v>
       </c>
-      <c r="F41" s="5">
+      <c r="F41" s="10">
         <f>'CASH FLOW'!E42</f>
         <v/>
       </c>
-      <c r="G41" s="5">
+      <c r="G41" s="10">
         <f>'CASH FLOW'!F42</f>
         <v/>
       </c>
-      <c r="H41" s="5">
+      <c r="H41" s="10">
         <f>'CASH FLOW'!G42</f>
         <v/>
       </c>
-      <c r="I41" s="5">
+      <c r="I41" s="10">
         <f>'CASH FLOW'!H42</f>
         <v/>
       </c>
-      <c r="J41" s="5">
+      <c r="J41" s="10">
         <f>'CASH FLOW'!I42</f>
         <v/>
       </c>
-      <c r="K41" s="5">
+      <c r="K41" s="10">
         <f>'CASH FLOW'!J42</f>
         <v/>
       </c>
@@ -4859,27 +4859,27 @@
       <c r="E42" s="4" t="n">
         <v>890190</v>
       </c>
-      <c r="F42" s="5">
+      <c r="F42" s="10">
         <f>'CASH FLOW'!F41+'CASH FLOW'!F40</f>
         <v/>
       </c>
-      <c r="G42" s="5">
+      <c r="G42" s="10">
         <f>'CASH FLOW'!G41+'CASH FLOW'!G40</f>
         <v/>
       </c>
-      <c r="H42" s="5">
+      <c r="H42" s="10">
         <f>'CASH FLOW'!H41+'CASH FLOW'!H40</f>
         <v/>
       </c>
-      <c r="I42" s="5">
+      <c r="I42" s="10">
         <f>'CASH FLOW'!I41+'CASH FLOW'!I40</f>
         <v/>
       </c>
-      <c r="J42" s="5">
+      <c r="J42" s="10">
         <f>'CASH FLOW'!J41+'CASH FLOW'!J40</f>
         <v/>
       </c>
-      <c r="K42" s="5">
+      <c r="K42" s="10">
         <f>'CASH FLOW'!K41+'CASH FLOW'!K40</f>
         <v/>
       </c>
@@ -4970,24 +4970,24 @@
           <t>Revenue Growth %</t>
         </is>
       </c>
-      <c r="C2" s="10">
+      <c r="C2" s="11">
         <f>IFERROR(('ANNL P&amp;L'!C2-'ANNL P&amp;L'!B2)/'ANNL P&amp;L'!B2,0)</f>
         <v/>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="11">
         <f>IFERROR(('ANNL P&amp;L'!D2-'ANNL P&amp;L'!C2)/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="E2" s="10">
+      <c r="E2" s="11">
         <f>IFERROR(('ANNL P&amp;L'!E2-'ANNL P&amp;L'!D2)/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="F2" s="11" t="n"/>
-      <c r="G2" s="11" t="n"/>
-      <c r="H2" s="11" t="n"/>
-      <c r="I2" s="11" t="n"/>
-      <c r="J2" s="11" t="n"/>
-      <c r="K2" s="11" t="n"/>
+      <c r="F2" s="12" t="n"/>
+      <c r="G2" s="12" t="n"/>
+      <c r="H2" s="12" t="n"/>
+      <c r="I2" s="12" t="n"/>
+      <c r="J2" s="12" t="n"/>
+      <c r="K2" s="12" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -4995,43 +4995,43 @@
           <t>COGS % of Revenue</t>
         </is>
       </c>
-      <c r="B3" s="10">
+      <c r="B3" s="11">
         <f>IFERROR('ANNL P&amp;L'!B3/'ANNL P&amp;L'!B2,0)</f>
         <v/>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="11">
         <f>IFERROR('ANNL P&amp;L'!C3/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D3" s="10">
+      <c r="D3" s="11">
         <f>IFERROR('ANNL P&amp;L'!D3/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E3" s="10">
+      <c r="E3" s="11">
         <f>IFERROR('ANNL P&amp;L'!E3/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F3" s="12">
+      <c r="F3" s="13">
         <f>E3</f>
         <v/>
       </c>
-      <c r="G3" s="12">
+      <c r="G3" s="13">
         <f>F3</f>
         <v/>
       </c>
-      <c r="H3" s="12">
+      <c r="H3" s="13">
         <f>G3</f>
         <v/>
       </c>
-      <c r="I3" s="12">
+      <c r="I3" s="13">
         <f>H3</f>
         <v/>
       </c>
-      <c r="J3" s="12">
+      <c r="J3" s="13">
         <f>I3</f>
         <v/>
       </c>
-      <c r="K3" s="12">
+      <c r="K3" s="13">
         <f>J3</f>
         <v/>
       </c>
@@ -5042,43 +5042,43 @@
           <t>SG&amp;A % of Revenue</t>
         </is>
       </c>
-      <c r="B4" s="10">
+      <c r="B4" s="11">
         <f>IFERROR('ANNL P&amp;L'!B5/'ANNL P&amp;L'!B2,0)</f>
         <v/>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="11">
         <f>IFERROR('ANNL P&amp;L'!C5/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="11">
         <f>IFERROR('ANNL P&amp;L'!D5/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="11">
         <f>IFERROR('ANNL P&amp;L'!E5/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="13">
         <f>E4</f>
         <v/>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="13">
         <f>F4</f>
         <v/>
       </c>
-      <c r="H4" s="12">
+      <c r="H4" s="13">
         <f>G4</f>
         <v/>
       </c>
-      <c r="I4" s="12">
+      <c r="I4" s="13">
         <f>H4</f>
         <v/>
       </c>
-      <c r="J4" s="12">
+      <c r="J4" s="13">
         <f>I4</f>
         <v/>
       </c>
-      <c r="K4" s="12">
+      <c r="K4" s="13">
         <f>J4</f>
         <v/>
       </c>
@@ -5105,27 +5105,27 @@
         <f>'ANNL P&amp;L'!E7</f>
         <v/>
       </c>
-      <c r="F5" s="13">
+      <c r="F5" s="10">
         <f>E5</f>
         <v/>
       </c>
-      <c r="G5" s="13">
+      <c r="G5" s="10">
         <f>F5</f>
         <v/>
       </c>
-      <c r="H5" s="13">
+      <c r="H5" s="10">
         <f>G5</f>
         <v/>
       </c>
-      <c r="I5" s="13">
+      <c r="I5" s="10">
         <f>H5</f>
         <v/>
       </c>
-      <c r="J5" s="13">
+      <c r="J5" s="10">
         <f>I5</f>
         <v/>
       </c>
-      <c r="K5" s="13">
+      <c r="K5" s="10">
         <f>J5</f>
         <v/>
       </c>
@@ -5152,27 +5152,27 @@
         <f>'ANNL P&amp;L'!E8</f>
         <v/>
       </c>
-      <c r="F6" s="13">
+      <c r="F6" s="10">
         <f>E6</f>
         <v/>
       </c>
-      <c r="G6" s="13">
+      <c r="G6" s="10">
         <f>F6</f>
         <v/>
       </c>
-      <c r="H6" s="13">
+      <c r="H6" s="10">
         <f>G6</f>
         <v/>
       </c>
-      <c r="I6" s="13">
+      <c r="I6" s="10">
         <f>H6</f>
         <v/>
       </c>
-      <c r="J6" s="13">
+      <c r="J6" s="10">
         <f>I6</f>
         <v/>
       </c>
-      <c r="K6" s="13">
+      <c r="K6" s="10">
         <f>J6</f>
         <v/>
       </c>
@@ -5199,27 +5199,27 @@
         <f>'ANNL P&amp;L'!E9</f>
         <v/>
       </c>
-      <c r="F7" s="13">
+      <c r="F7" s="10">
         <f>E7</f>
         <v/>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="10">
         <f>F7</f>
         <v/>
       </c>
-      <c r="H7" s="13">
+      <c r="H7" s="10">
         <f>G7</f>
         <v/>
       </c>
-      <c r="I7" s="13">
+      <c r="I7" s="10">
         <f>H7</f>
         <v/>
       </c>
-      <c r="J7" s="13">
+      <c r="J7" s="10">
         <f>I7</f>
         <v/>
       </c>
-      <c r="K7" s="13">
+      <c r="K7" s="10">
         <f>J7</f>
         <v/>
       </c>
@@ -5230,43 +5230,43 @@
           <t>Effective Tax Rate %</t>
         </is>
       </c>
-      <c r="B8" s="10">
+      <c r="B8" s="11">
         <f>IFERROR('ANNL P&amp;L'!B11/'ANNL P&amp;L'!B10,0)</f>
         <v/>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="11">
         <f>IFERROR('ANNL P&amp;L'!C11/'ANNL P&amp;L'!C10,0)</f>
         <v/>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="11">
         <f>IFERROR('ANNL P&amp;L'!D11/'ANNL P&amp;L'!D10,0)</f>
         <v/>
       </c>
-      <c r="E8" s="10">
+      <c r="E8" s="11">
         <f>IFERROR('ANNL P&amp;L'!E11/'ANNL P&amp;L'!E10,0)</f>
         <v/>
       </c>
-      <c r="F8" s="12">
+      <c r="F8" s="13">
         <f>E8</f>
         <v/>
       </c>
-      <c r="G8" s="12">
+      <c r="G8" s="13">
         <f>F8</f>
         <v/>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="13">
         <f>G8</f>
         <v/>
       </c>
-      <c r="I8" s="12">
+      <c r="I8" s="13">
         <f>H8</f>
         <v/>
       </c>
-      <c r="J8" s="12">
+      <c r="J8" s="13">
         <f>I8</f>
         <v/>
       </c>
-      <c r="K8" s="12">
+      <c r="K8" s="13">
         <f>J8</f>
         <v/>
       </c>
@@ -5460,39 +5460,39 @@
           <t>Note Receivable - Current % of Rev</t>
         </is>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="11">
         <f>IFERROR('BALANCE SHEET'!B5/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="11">
         <f>IFERROR('BALANCE SHEET'!C5/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="11">
         <f>IFERROR('BALANCE SHEET'!D5/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="13">
         <f>E5</f>
         <v/>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="13">
         <f>F5</f>
         <v/>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="13">
         <f>G5</f>
         <v/>
       </c>
-      <c r="I5" s="12">
+      <c r="I5" s="13">
         <f>H5</f>
         <v/>
       </c>
-      <c r="J5" s="12">
+      <c r="J5" s="13">
         <f>I5</f>
         <v/>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="13">
         <f>J5</f>
         <v/>
       </c>
@@ -5503,39 +5503,39 @@
           <t>Deferred Other Costs - Current % of Rev</t>
         </is>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="11">
         <f>IFERROR('BALANCE SHEET'!B7/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="11">
         <f>IFERROR('BALANCE SHEET'!C7/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="11">
         <f>IFERROR('BALANCE SHEET'!D7/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="13">
         <f>E6</f>
         <v/>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="13">
         <f>F6</f>
         <v/>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="13">
         <f>G6</f>
         <v/>
       </c>
-      <c r="I6" s="12">
+      <c r="I6" s="13">
         <f>H6</f>
         <v/>
       </c>
-      <c r="J6" s="12">
+      <c r="J6" s="13">
         <f>I6</f>
         <v/>
       </c>
-      <c r="K6" s="12">
+      <c r="K6" s="13">
         <f>J6</f>
         <v/>
       </c>
@@ -5546,39 +5546,39 @@
           <t>Prepaid Expenses % of Rev</t>
         </is>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="11">
         <f>IFERROR('BALANCE SHEET'!B8/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="11">
         <f>IFERROR('BALANCE SHEET'!C8/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E7" s="10">
+      <c r="E7" s="11">
         <f>IFERROR('BALANCE SHEET'!D8/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="13">
         <f>E7</f>
         <v/>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="13">
         <f>F7</f>
         <v/>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="13">
         <f>G7</f>
         <v/>
       </c>
-      <c r="I7" s="12">
+      <c r="I7" s="13">
         <f>H7</f>
         <v/>
       </c>
-      <c r="J7" s="12">
+      <c r="J7" s="13">
         <f>I7</f>
         <v/>
       </c>
-      <c r="K7" s="12">
+      <c r="K7" s="13">
         <f>J7</f>
         <v/>
       </c>
@@ -5606,39 +5606,39 @@
           <t>Other Non-Current Assets % of Rev</t>
         </is>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="11">
         <f>IFERROR('BALANCE SHEET'!B18/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="11">
         <f>IFERROR('BALANCE SHEET'!C18/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E9" s="10">
+      <c r="E9" s="11">
         <f>IFERROR('BALANCE SHEET'!D18/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F9" s="12">
+      <c r="F9" s="13">
         <f>E9</f>
         <v/>
       </c>
-      <c r="G9" s="12">
+      <c r="G9" s="13">
         <f>F9</f>
         <v/>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="13">
         <f>G9</f>
         <v/>
       </c>
-      <c r="I9" s="12">
+      <c r="I9" s="13">
         <f>H9</f>
         <v/>
       </c>
-      <c r="J9" s="12">
+      <c r="J9" s="13">
         <f>I9</f>
         <v/>
       </c>
-      <c r="K9" s="12">
+      <c r="K9" s="13">
         <f>J9</f>
         <v/>
       </c>
@@ -5709,39 +5709,39 @@
           <t>Accrued Expenses % of Rev</t>
         </is>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="11">
         <f>IFERROR('BALANCE SHEET'!B21/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D12" s="10">
+      <c r="D12" s="11">
         <f>IFERROR('BALANCE SHEET'!C21/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="11">
         <f>IFERROR('BALANCE SHEET'!D21/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="13">
         <f>E12</f>
         <v/>
       </c>
-      <c r="G12" s="12">
+      <c r="G12" s="13">
         <f>F12</f>
         <v/>
       </c>
-      <c r="H12" s="12">
+      <c r="H12" s="13">
         <f>G12</f>
         <v/>
       </c>
-      <c r="I12" s="12">
+      <c r="I12" s="13">
         <f>H12</f>
         <v/>
       </c>
-      <c r="J12" s="12">
+      <c r="J12" s="13">
         <f>I12</f>
         <v/>
       </c>
-      <c r="K12" s="12">
+      <c r="K12" s="13">
         <f>J12</f>
         <v/>
       </c>
@@ -5752,39 +5752,39 @@
           <t>Income Taxes Payable % of Rev</t>
         </is>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="11">
         <f>IFERROR('BALANCE SHEET'!B22/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D13" s="10">
+      <c r="D13" s="11">
         <f>IFERROR('BALANCE SHEET'!C22/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E13" s="10">
+      <c r="E13" s="11">
         <f>IFERROR('BALANCE SHEET'!D22/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="13">
         <f>E13</f>
         <v/>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="13">
         <f>F13</f>
         <v/>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="13">
         <f>G13</f>
         <v/>
       </c>
-      <c r="I13" s="12">
+      <c r="I13" s="13">
         <f>H13</f>
         <v/>
       </c>
-      <c r="J13" s="12">
+      <c r="J13" s="13">
         <f>I13</f>
         <v/>
       </c>
-      <c r="K13" s="12">
+      <c r="K13" s="13">
         <f>J13</f>
         <v/>
       </c>
@@ -5795,39 +5795,39 @@
           <t>Accrued Distributor Termination Fees % of Rev</t>
         </is>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="11">
         <f>IFERROR('BALANCE SHEET'!B23/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D14" s="10">
+      <c r="D14" s="11">
         <f>IFERROR('BALANCE SHEET'!C23/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E14" s="10">
+      <c r="E14" s="11">
         <f>IFERROR('BALANCE SHEET'!D23/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F14" s="12">
+      <c r="F14" s="13">
         <f>E14</f>
         <v/>
       </c>
-      <c r="G14" s="12">
+      <c r="G14" s="13">
         <f>F14</f>
         <v/>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="13">
         <f>G14</f>
         <v/>
       </c>
-      <c r="I14" s="12">
+      <c r="I14" s="13">
         <f>H14</f>
         <v/>
       </c>
-      <c r="J14" s="12">
+      <c r="J14" s="13">
         <f>I14</f>
         <v/>
       </c>
-      <c r="K14" s="12">
+      <c r="K14" s="13">
         <f>J14</f>
         <v/>
       </c>
@@ -5838,39 +5838,39 @@
           <t>Accrued Promotional Allowance % of Rev</t>
         </is>
       </c>
-      <c r="C15" s="10">
+      <c r="C15" s="11">
         <f>IFERROR('BALANCE SHEET'!B24/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D15" s="10">
+      <c r="D15" s="11">
         <f>IFERROR('BALANCE SHEET'!C24/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E15" s="10">
+      <c r="E15" s="11">
         <f>IFERROR('BALANCE SHEET'!D24/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F15" s="12">
+      <c r="F15" s="13">
         <f>E15</f>
         <v/>
       </c>
-      <c r="G15" s="12">
+      <c r="G15" s="13">
         <f>F15</f>
         <v/>
       </c>
-      <c r="H15" s="12">
+      <c r="H15" s="13">
         <f>G15</f>
         <v/>
       </c>
-      <c r="I15" s="12">
+      <c r="I15" s="13">
         <f>H15</f>
         <v/>
       </c>
-      <c r="J15" s="12">
+      <c r="J15" s="13">
         <f>I15</f>
         <v/>
       </c>
-      <c r="K15" s="12">
+      <c r="K15" s="13">
         <f>J15</f>
         <v/>
       </c>
@@ -5881,39 +5881,39 @@
           <t>Lease Liability - Operating - Current % of Rev</t>
         </is>
       </c>
-      <c r="C16" s="10">
+      <c r="C16" s="11">
         <f>IFERROR('BALANCE SHEET'!B25/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D16" s="10">
+      <c r="D16" s="11">
         <f>IFERROR('BALANCE SHEET'!C25/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E16" s="10">
+      <c r="E16" s="11">
         <f>IFERROR('BALANCE SHEET'!D25/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F16" s="12">
+      <c r="F16" s="13">
         <f>E16</f>
         <v/>
       </c>
-      <c r="G16" s="12">
+      <c r="G16" s="13">
         <f>F16</f>
         <v/>
       </c>
-      <c r="H16" s="12">
+      <c r="H16" s="13">
         <f>G16</f>
         <v/>
       </c>
-      <c r="I16" s="12">
+      <c r="I16" s="13">
         <f>H16</f>
         <v/>
       </c>
-      <c r="J16" s="12">
+      <c r="J16" s="13">
         <f>I16</f>
         <v/>
       </c>
-      <c r="K16" s="12">
+      <c r="K16" s="13">
         <f>J16</f>
         <v/>
       </c>
@@ -5924,39 +5924,39 @@
           <t>Lease Liability - Finance - Current % of Rev</t>
         </is>
       </c>
-      <c r="C17" s="10">
+      <c r="C17" s="11">
         <f>IFERROR('BALANCE SHEET'!B26/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D17" s="10">
+      <c r="D17" s="11">
         <f>IFERROR('BALANCE SHEET'!C26/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E17" s="10">
+      <c r="E17" s="11">
         <f>IFERROR('BALANCE SHEET'!D26/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F17" s="12">
+      <c r="F17" s="13">
         <f>E17</f>
         <v/>
       </c>
-      <c r="G17" s="12">
+      <c r="G17" s="13">
         <f>F17</f>
         <v/>
       </c>
-      <c r="H17" s="12">
+      <c r="H17" s="13">
         <f>G17</f>
         <v/>
       </c>
-      <c r="I17" s="12">
+      <c r="I17" s="13">
         <f>H17</f>
         <v/>
       </c>
-      <c r="J17" s="12">
+      <c r="J17" s="13">
         <f>I17</f>
         <v/>
       </c>
-      <c r="K17" s="12">
+      <c r="K17" s="13">
         <f>J17</f>
         <v/>
       </c>
@@ -5967,39 +5967,39 @@
           <t>Deferred Revenue - Current % of Rev</t>
         </is>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="11">
         <f>IFERROR('BALANCE SHEET'!B27/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="11">
         <f>IFERROR('BALANCE SHEET'!C27/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E18" s="10">
+      <c r="E18" s="11">
         <f>IFERROR('BALANCE SHEET'!D27/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F18" s="12">
+      <c r="F18" s="13">
         <f>E18</f>
         <v/>
       </c>
-      <c r="G18" s="12">
+      <c r="G18" s="13">
         <f>F18</f>
         <v/>
       </c>
-      <c r="H18" s="12">
+      <c r="H18" s="13">
         <f>G18</f>
         <v/>
       </c>
-      <c r="I18" s="12">
+      <c r="I18" s="13">
         <f>H18</f>
         <v/>
       </c>
-      <c r="J18" s="12">
+      <c r="J18" s="13">
         <f>I18</f>
         <v/>
       </c>
-      <c r="K18" s="12">
+      <c r="K18" s="13">
         <f>J18</f>
         <v/>
       </c>
@@ -6010,39 +6010,39 @@
           <t>Other Current Liabilities % of Rev</t>
         </is>
       </c>
-      <c r="C19" s="10">
+      <c r="C19" s="11">
         <f>IFERROR('BALANCE SHEET'!B28/'ANNL P&amp;L'!C2,0)</f>
         <v/>
       </c>
-      <c r="D19" s="10">
+      <c r="D19" s="11">
         <f>IFERROR('BALANCE SHEET'!C28/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
-      <c r="E19" s="10">
+      <c r="E19" s="11">
         <f>IFERROR('BALANCE SHEET'!D28/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
-      <c r="F19" s="12">
+      <c r="F19" s="13">
         <f>E19</f>
         <v/>
       </c>
-      <c r="G19" s="12">
+      <c r="G19" s="13">
         <f>F19</f>
         <v/>
       </c>
-      <c r="H19" s="12">
+      <c r="H19" s="13">
         <f>G19</f>
         <v/>
       </c>
-      <c r="I19" s="12">
+      <c r="I19" s="13">
         <f>H19</f>
         <v/>
       </c>
-      <c r="J19" s="12">
+      <c r="J19" s="13">
         <f>I19</f>
         <v/>
       </c>
-      <c r="K19" s="12">
+      <c r="K19" s="13">
         <f>J19</f>
         <v/>
       </c>
@@ -6133,35 +6133,35 @@
           <t>D&amp;A % of PP&amp;E</t>
         </is>
       </c>
-      <c r="D2" s="10">
+      <c r="D2" s="11">
         <f>IFERROR('CASH FLOW'!D3/'BALANCE SHEET'!B11,0)</f>
         <v/>
       </c>
-      <c r="E2" s="10">
+      <c r="E2" s="11">
         <f>IFERROR('CASH FLOW'!E3/'BALANCE SHEET'!C11,0)</f>
         <v/>
       </c>
-      <c r="F2" s="12">
+      <c r="F2" s="13">
         <f>E2</f>
         <v/>
       </c>
-      <c r="G2" s="12">
+      <c r="G2" s="13">
         <f>F2</f>
         <v/>
       </c>
-      <c r="H2" s="12">
+      <c r="H2" s="13">
         <f>G2</f>
         <v/>
       </c>
-      <c r="I2" s="12">
+      <c r="I2" s="13">
         <f>H2</f>
         <v/>
       </c>
-      <c r="J2" s="12">
+      <c r="J2" s="13">
         <f>I2</f>
         <v/>
       </c>
-      <c r="K2" s="12">
+      <c r="K2" s="13">
         <f>J2</f>
         <v/>
       </c>
@@ -6188,27 +6188,27 @@
         <f>'CASH FLOW'!E9</f>
         <v/>
       </c>
-      <c r="F3" s="13">
+      <c r="F3" s="10">
         <f>E3</f>
         <v/>
       </c>
-      <c r="G3" s="13">
+      <c r="G3" s="10">
         <f>F3</f>
         <v/>
       </c>
-      <c r="H3" s="13">
+      <c r="H3" s="10">
         <f>G3</f>
         <v/>
       </c>
-      <c r="I3" s="13">
+      <c r="I3" s="10">
         <f>H3</f>
         <v/>
       </c>
-      <c r="J3" s="13">
+      <c r="J3" s="10">
         <f>I3</f>
         <v/>
       </c>
-      <c r="K3" s="13">
+      <c r="K3" s="10">
         <f>J3</f>
         <v/>
       </c>
@@ -6219,35 +6219,35 @@
           <t>CapEx % of PP&amp;E</t>
         </is>
       </c>
-      <c r="D4" s="10">
+      <c r="D4" s="11">
         <f>IFERROR('CASH FLOW'!D28/'BALANCE SHEET'!B11,0)</f>
         <v/>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="11">
         <f>IFERROR('CASH FLOW'!E28/'BALANCE SHEET'!C11,0)</f>
         <v/>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="13">
         <f>E4</f>
         <v/>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="13">
         <f>F4</f>
         <v/>
       </c>
-      <c r="H4" s="12">
+      <c r="H4" s="13">
         <f>G4</f>
         <v/>
       </c>
-      <c r="I4" s="12">
+      <c r="I4" s="13">
         <f>H4</f>
         <v/>
       </c>
-      <c r="J4" s="12">
+      <c r="J4" s="13">
         <f>I4</f>
         <v/>
       </c>
-      <c r="K4" s="12">
+      <c r="K4" s="13">
         <f>J4</f>
         <v/>
       </c>
@@ -6258,39 +6258,39 @@
           <t>Preferred Dividends % of Preferred Balance</t>
         </is>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="11">
         <f>IFERROR('CASH FLOW'!C35/'BALANCE SHEET'!B35,0)</f>
         <v/>
       </c>
-      <c r="D5" s="10">
+      <c r="D5" s="11">
         <f>IFERROR('CASH FLOW'!D35/'BALANCE SHEET'!C35,0)</f>
         <v/>
       </c>
-      <c r="E5" s="10">
+      <c r="E5" s="11">
         <f>IFERROR('CASH FLOW'!E35/'BALANCE SHEET'!D35,0)</f>
         <v/>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="13">
         <f>E5</f>
         <v/>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="13">
         <f>F5</f>
         <v/>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="13">
         <f>G5</f>
         <v/>
       </c>
-      <c r="I5" s="12">
+      <c r="I5" s="13">
         <f>H5</f>
         <v/>
       </c>
-      <c r="J5" s="12">
+      <c r="J5" s="13">
         <f>I5</f>
         <v/>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="13">
         <f>J5</f>
         <v/>
       </c>
@@ -6301,27 +6301,27 @@
           <t>Common Dividends % of Net Income</t>
         </is>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="13">
         <f>E6</f>
         <v/>
       </c>
-      <c r="G6" s="12">
+      <c r="G6" s="13">
         <f>F6</f>
         <v/>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="13">
         <f>G6</f>
         <v/>
       </c>
-      <c r="I6" s="12">
+      <c r="I6" s="13">
         <f>H6</f>
         <v/>
       </c>
-      <c r="J6" s="12">
+      <c r="J6" s="13">
         <f>I6</f>
         <v/>
       </c>
-      <c r="K6" s="12">
+      <c r="K6" s="13">
         <f>J6</f>
         <v/>
       </c>
@@ -6348,27 +6348,27 @@
         <f>'CASH FLOW'!E37</f>
         <v/>
       </c>
-      <c r="F7" s="13">
+      <c r="F7" s="10">
         <f>ASSUMPTIONS!$B$3</f>
         <v/>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="10">
         <f>ASSUMPTIONS!$B$3</f>
         <v/>
       </c>
-      <c r="H7" s="13">
+      <c r="H7" s="10">
         <f>ASSUMPTIONS!$B$3</f>
         <v/>
       </c>
-      <c r="I7" s="13">
+      <c r="I7" s="10">
         <f>ASSUMPTIONS!$B$3</f>
         <v/>
       </c>
-      <c r="J7" s="13">
+      <c r="J7" s="10">
         <f>ASSUMPTIONS!$B$3</f>
         <v/>
       </c>
-      <c r="K7" s="13">
+      <c r="K7" s="10">
         <f>ASSUMPTIONS!$B$3</f>
         <v/>
       </c>
@@ -6391,27 +6391,27 @@
         <f>('BALANCE SHEET'!D25+'BALANCE SHEET'!D26+'BALANCE SHEET'!D30+'BALANCE SHEET'!D31)-('BALANCE SHEET'!D2+'BALANCE SHEET'!D3)</f>
         <v/>
       </c>
-      <c r="F8" s="13">
+      <c r="F8" s="10">
         <f>('BALANCE SHEET'!E25+'BALANCE SHEET'!E26+'BALANCE SHEET'!E30+'BALANCE SHEET'!E31)-('BALANCE SHEET'!E2+'BALANCE SHEET'!E3)</f>
         <v/>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="10">
         <f>('BALANCE SHEET'!F25+'BALANCE SHEET'!F26+'BALANCE SHEET'!F30+'BALANCE SHEET'!F31)-('BALANCE SHEET'!F2+'BALANCE SHEET'!F3)</f>
         <v/>
       </c>
-      <c r="H8" s="13">
+      <c r="H8" s="10">
         <f>('BALANCE SHEET'!G25+'BALANCE SHEET'!G26+'BALANCE SHEET'!G30+'BALANCE SHEET'!G31)-('BALANCE SHEET'!G2+'BALANCE SHEET'!G3)</f>
         <v/>
       </c>
-      <c r="I8" s="13">
+      <c r="I8" s="10">
         <f>('BALANCE SHEET'!H25+'BALANCE SHEET'!H26+'BALANCE SHEET'!H30+'BALANCE SHEET'!H31)-('BALANCE SHEET'!H2+'BALANCE SHEET'!H3)</f>
         <v/>
       </c>
-      <c r="J8" s="13">
+      <c r="J8" s="10">
         <f>('BALANCE SHEET'!I25+'BALANCE SHEET'!I26+'BALANCE SHEET'!I30+'BALANCE SHEET'!I31)-('BALANCE SHEET'!I2+'BALANCE SHEET'!I3)</f>
         <v/>
       </c>
-      <c r="K8" s="13">
+      <c r="K8" s="10">
         <f>('BALANCE SHEET'!J25+'BALANCE SHEET'!J26+'BALANCE SHEET'!J30+'BALANCE SHEET'!J31)-('BALANCE SHEET'!J2+'BALANCE SHEET'!J3)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
vault backup: 2026-04-24 10:12:33
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -3207,27 +3207,27 @@
         <v>7274</v>
       </c>
       <c r="F3" s="10">
-        <f>'CF DRIVERS'!F2*'BALANCE SHEET'!D11</f>
+        <f>'CF DRIVERS'!F3*'BALANCE SHEET'!D11</f>
         <v/>
       </c>
       <c r="G3" s="10">
-        <f>'CF DRIVERS'!G2*'BALANCE SHEET'!E11</f>
+        <f>'CF DRIVERS'!G3*'BALANCE SHEET'!E11</f>
         <v/>
       </c>
       <c r="H3" s="10">
-        <f>'CF DRIVERS'!H2*'BALANCE SHEET'!F11</f>
+        <f>'CF DRIVERS'!H3*'BALANCE SHEET'!F11</f>
         <v/>
       </c>
       <c r="I3" s="10">
-        <f>'CF DRIVERS'!I2*'BALANCE SHEET'!G11</f>
+        <f>'CF DRIVERS'!I3*'BALANCE SHEET'!G11</f>
         <v/>
       </c>
       <c r="J3" s="10">
-        <f>'CF DRIVERS'!J2*'BALANCE SHEET'!H11</f>
+        <f>'CF DRIVERS'!J3*'BALANCE SHEET'!H11</f>
         <v/>
       </c>
       <c r="K3" s="10">
-        <f>'CF DRIVERS'!K2*'BALANCE SHEET'!I11</f>
+        <f>'CF DRIVERS'!K3*'BALANCE SHEET'!I11</f>
         <v/>
       </c>
     </row>
@@ -3293,27 +3293,27 @@
         <v>3294</v>
       </c>
       <c r="F5" s="10">
-        <f>0</f>
+        <f>'CF DRIVERS'!F2*'ANNL P&amp;L'!F2</f>
         <v/>
       </c>
       <c r="G5" s="10">
-        <f>0</f>
+        <f>'CF DRIVERS'!G2*'ANNL P&amp;L'!G2</f>
         <v/>
       </c>
       <c r="H5" s="10">
-        <f>0</f>
+        <f>'CF DRIVERS'!H2*'ANNL P&amp;L'!H2</f>
         <v/>
       </c>
       <c r="I5" s="10">
-        <f>0</f>
+        <f>'CF DRIVERS'!I2*'ANNL P&amp;L'!I2</f>
         <v/>
       </c>
       <c r="J5" s="10">
-        <f>0</f>
+        <f>'CF DRIVERS'!J2*'ANNL P&amp;L'!J2</f>
         <v/>
       </c>
       <c r="K5" s="10">
-        <f>0</f>
+        <f>'CF DRIVERS'!K2*'ANNL P&amp;L'!K2</f>
         <v/>
       </c>
     </row>
@@ -3465,27 +3465,27 @@
         <v>19591</v>
       </c>
       <c r="F9" s="10">
-        <f>'CF DRIVERS'!F3</f>
+        <f>'CF DRIVERS'!F4</f>
         <v/>
       </c>
       <c r="G9" s="10">
-        <f>'CF DRIVERS'!G3</f>
+        <f>'CF DRIVERS'!G4</f>
         <v/>
       </c>
       <c r="H9" s="10">
-        <f>'CF DRIVERS'!H3</f>
+        <f>'CF DRIVERS'!H4</f>
         <v/>
       </c>
       <c r="I9" s="10">
-        <f>'CF DRIVERS'!I3</f>
+        <f>'CF DRIVERS'!I4</f>
         <v/>
       </c>
       <c r="J9" s="10">
-        <f>'CF DRIVERS'!J3</f>
+        <f>'CF DRIVERS'!J4</f>
         <v/>
       </c>
       <c r="K9" s="10">
-        <f>'CF DRIVERS'!K3</f>
+        <f>'CF DRIVERS'!K4</f>
         <v/>
       </c>
     </row>
@@ -4286,27 +4286,27 @@
         <v>-23390</v>
       </c>
       <c r="F28" s="10">
-        <f>'CF DRIVERS'!F4*'BALANCE SHEET'!D11</f>
+        <f>'CF DRIVERS'!F5*'BALANCE SHEET'!D11</f>
         <v/>
       </c>
       <c r="G28" s="10">
-        <f>'CF DRIVERS'!G4*'BALANCE SHEET'!E11</f>
+        <f>'CF DRIVERS'!G5*'BALANCE SHEET'!E11</f>
         <v/>
       </c>
       <c r="H28" s="10">
-        <f>'CF DRIVERS'!H4*'BALANCE SHEET'!F11</f>
+        <f>'CF DRIVERS'!H5*'BALANCE SHEET'!F11</f>
         <v/>
       </c>
       <c r="I28" s="10">
-        <f>'CF DRIVERS'!I4*'BALANCE SHEET'!G11</f>
+        <f>'CF DRIVERS'!I5*'BALANCE SHEET'!G11</f>
         <v/>
       </c>
       <c r="J28" s="10">
-        <f>'CF DRIVERS'!J4*'BALANCE SHEET'!H11</f>
+        <f>'CF DRIVERS'!J5*'BALANCE SHEET'!H11</f>
         <v/>
       </c>
       <c r="K28" s="10">
-        <f>'CF DRIVERS'!K4*'BALANCE SHEET'!I11</f>
+        <f>'CF DRIVERS'!K5*'BALANCE SHEET'!I11</f>
         <v/>
       </c>
     </row>
@@ -4555,27 +4555,27 @@
         <v>-27500</v>
       </c>
       <c r="F35" s="10">
-        <f>'CF DRIVERS'!F5*'BALANCE SHEET'!E35</f>
+        <f>'CF DRIVERS'!F6*'BALANCE SHEET'!E35</f>
         <v/>
       </c>
       <c r="G35" s="10">
-        <f>'CF DRIVERS'!G5*'BALANCE SHEET'!F35</f>
+        <f>'CF DRIVERS'!G6*'BALANCE SHEET'!F35</f>
         <v/>
       </c>
       <c r="H35" s="10">
-        <f>'CF DRIVERS'!H5*'BALANCE SHEET'!G35</f>
+        <f>'CF DRIVERS'!H6*'BALANCE SHEET'!G35</f>
         <v/>
       </c>
       <c r="I35" s="10">
-        <f>'CF DRIVERS'!I5*'BALANCE SHEET'!H35</f>
+        <f>'CF DRIVERS'!I6*'BALANCE SHEET'!H35</f>
         <v/>
       </c>
       <c r="J35" s="10">
-        <f>'CF DRIVERS'!J5*'BALANCE SHEET'!I35</f>
+        <f>'CF DRIVERS'!J6*'BALANCE SHEET'!I35</f>
         <v/>
       </c>
       <c r="K35" s="10">
-        <f>'CF DRIVERS'!K5*'BALANCE SHEET'!J35</f>
+        <f>'CF DRIVERS'!K6*'BALANCE SHEET'!J35</f>
         <v/>
       </c>
     </row>
@@ -4641,27 +4641,27 @@
         <v>-2261</v>
       </c>
       <c r="F37" s="10">
-        <f>'CF DRIVERS'!F7</f>
+        <f>'CF DRIVERS'!F8</f>
         <v/>
       </c>
       <c r="G37" s="10">
-        <f>'CF DRIVERS'!G7</f>
+        <f>'CF DRIVERS'!G8</f>
         <v/>
       </c>
       <c r="H37" s="10">
-        <f>'CF DRIVERS'!H7</f>
+        <f>'CF DRIVERS'!H8</f>
         <v/>
       </c>
       <c r="I37" s="10">
-        <f>'CF DRIVERS'!I7</f>
+        <f>'CF DRIVERS'!I8</f>
         <v/>
       </c>
       <c r="J37" s="10">
-        <f>'CF DRIVERS'!J7</f>
+        <f>'CF DRIVERS'!J8</f>
         <v/>
       </c>
       <c r="K37" s="10">
-        <f>'CF DRIVERS'!K7</f>
+        <f>'CF DRIVERS'!K8</f>
         <v/>
       </c>
     </row>
@@ -6058,7 +6058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -6130,15 +6130,23 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>D&amp;A % of PP&amp;E</t>
-        </is>
+          <t>Allowance for Credit Losses % of Revenue</t>
+        </is>
+      </c>
+      <c r="B2" s="11">
+        <f>IFERROR('CASH FLOW'!B5/'ANNL P&amp;L'!B2,0)</f>
+        <v/>
+      </c>
+      <c r="C2" s="11">
+        <f>IFERROR('CASH FLOW'!C5/'ANNL P&amp;L'!C2,0)</f>
+        <v/>
       </c>
       <c r="D2" s="11">
-        <f>IFERROR('CASH FLOW'!D3/'BALANCE SHEET'!B11,0)</f>
+        <f>IFERROR('CASH FLOW'!D5/'ANNL P&amp;L'!D2,0)</f>
         <v/>
       </c>
       <c r="E2" s="11">
-        <f>IFERROR('CASH FLOW'!E3/'BALANCE SHEET'!C11,0)</f>
+        <f>IFERROR('CASH FLOW'!E5/'ANNL P&amp;L'!E2,0)</f>
         <v/>
       </c>
       <c r="F2" s="13">
@@ -6169,46 +6177,38 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>SBC $</t>
-        </is>
-      </c>
-      <c r="B3" s="4">
-        <f>'CASH FLOW'!B9</f>
-        <v/>
-      </c>
-      <c r="C3" s="4">
-        <f>'CASH FLOW'!C9</f>
-        <v/>
-      </c>
-      <c r="D3" s="4">
-        <f>'CASH FLOW'!D9</f>
-        <v/>
-      </c>
-      <c r="E3" s="4">
-        <f>'CASH FLOW'!E9</f>
-        <v/>
-      </c>
-      <c r="F3" s="10">
+          <t>D&amp;A % of PP&amp;E</t>
+        </is>
+      </c>
+      <c r="D3" s="11">
+        <f>IFERROR('CASH FLOW'!D3/'BALANCE SHEET'!B11,0)</f>
+        <v/>
+      </c>
+      <c r="E3" s="11">
+        <f>IFERROR('CASH FLOW'!E3/'BALANCE SHEET'!C11,0)</f>
+        <v/>
+      </c>
+      <c r="F3" s="13">
         <f>E3</f>
         <v/>
       </c>
-      <c r="G3" s="10">
+      <c r="G3" s="13">
         <f>F3</f>
         <v/>
       </c>
-      <c r="H3" s="10">
+      <c r="H3" s="13">
         <f>G3</f>
         <v/>
       </c>
-      <c r="I3" s="10">
+      <c r="I3" s="13">
         <f>H3</f>
         <v/>
       </c>
-      <c r="J3" s="10">
+      <c r="J3" s="13">
         <f>I3</f>
         <v/>
       </c>
-      <c r="K3" s="10">
+      <c r="K3" s="13">
         <f>J3</f>
         <v/>
       </c>
@@ -6216,38 +6216,46 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>CapEx % of PP&amp;E</t>
-        </is>
-      </c>
-      <c r="D4" s="11">
-        <f>IFERROR('CASH FLOW'!D28/'BALANCE SHEET'!B11,0)</f>
-        <v/>
-      </c>
-      <c r="E4" s="11">
-        <f>IFERROR('CASH FLOW'!E28/'BALANCE SHEET'!C11,0)</f>
-        <v/>
-      </c>
-      <c r="F4" s="13">
+          <t>SBC $</t>
+        </is>
+      </c>
+      <c r="B4" s="4">
+        <f>'CASH FLOW'!B9</f>
+        <v/>
+      </c>
+      <c r="C4" s="4">
+        <f>'CASH FLOW'!C9</f>
+        <v/>
+      </c>
+      <c r="D4" s="4">
+        <f>'CASH FLOW'!D9</f>
+        <v/>
+      </c>
+      <c r="E4" s="4">
+        <f>'CASH FLOW'!E9</f>
+        <v/>
+      </c>
+      <c r="F4" s="10">
         <f>E4</f>
         <v/>
       </c>
-      <c r="G4" s="13">
+      <c r="G4" s="10">
         <f>F4</f>
         <v/>
       </c>
-      <c r="H4" s="13">
+      <c r="H4" s="10">
         <f>G4</f>
         <v/>
       </c>
-      <c r="I4" s="13">
+      <c r="I4" s="10">
         <f>H4</f>
         <v/>
       </c>
-      <c r="J4" s="13">
+      <c r="J4" s="10">
         <f>I4</f>
         <v/>
       </c>
-      <c r="K4" s="13">
+      <c r="K4" s="10">
         <f>J4</f>
         <v/>
       </c>
@@ -6255,19 +6263,15 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Preferred Dividends % of Preferred Balance</t>
-        </is>
-      </c>
-      <c r="C5" s="11">
-        <f>IFERROR('CASH FLOW'!C35/'BALANCE SHEET'!B35,0)</f>
-        <v/>
+          <t>CapEx % of PP&amp;E</t>
+        </is>
       </c>
       <c r="D5" s="11">
-        <f>IFERROR('CASH FLOW'!D35/'BALANCE SHEET'!C35,0)</f>
+        <f>IFERROR('CASH FLOW'!D28/'BALANCE SHEET'!B11,0)</f>
         <v/>
       </c>
       <c r="E5" s="11">
-        <f>IFERROR('CASH FLOW'!E35/'BALANCE SHEET'!D35,0)</f>
+        <f>IFERROR('CASH FLOW'!E28/'BALANCE SHEET'!C11,0)</f>
         <v/>
       </c>
       <c r="F5" s="13">
@@ -6298,8 +6302,20 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Common Dividends % of Net Income</t>
-        </is>
+          <t>Preferred Dividends % of Preferred Balance</t>
+        </is>
+      </c>
+      <c r="C6" s="11">
+        <f>IFERROR('CASH FLOW'!C35/'BALANCE SHEET'!B35,0)</f>
+        <v/>
+      </c>
+      <c r="D6" s="11">
+        <f>IFERROR('CASH FLOW'!D35/'BALANCE SHEET'!C35,0)</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>IFERROR('CASH FLOW'!E35/'BALANCE SHEET'!D35,0)</f>
+        <v/>
       </c>
       <c r="F6" s="13">
         <f>E6</f>
@@ -6329,89 +6345,120 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Share Repurchases $</t>
-        </is>
-      </c>
-      <c r="B7" s="4">
-        <f>'CASH FLOW'!B37</f>
-        <v/>
-      </c>
-      <c r="C7" s="4">
-        <f>'CASH FLOW'!C37</f>
-        <v/>
-      </c>
-      <c r="D7" s="4">
-        <f>'CASH FLOW'!D37</f>
-        <v/>
-      </c>
-      <c r="E7" s="4">
-        <f>'CASH FLOW'!E37</f>
-        <v/>
-      </c>
-      <c r="F7" s="10">
-        <f>ASSUMPTIONS!$B$3</f>
-        <v/>
-      </c>
-      <c r="G7" s="10">
-        <f>ASSUMPTIONS!$B$3</f>
-        <v/>
-      </c>
-      <c r="H7" s="10">
-        <f>ASSUMPTIONS!$B$3</f>
-        <v/>
-      </c>
-      <c r="I7" s="10">
-        <f>ASSUMPTIONS!$B$3</f>
-        <v/>
-      </c>
-      <c r="J7" s="10">
-        <f>ASSUMPTIONS!$B$3</f>
-        <v/>
-      </c>
-      <c r="K7" s="10">
-        <f>ASSUMPTIONS!$B$3</f>
+          <t>Common Dividends % of Net Income</t>
+        </is>
+      </c>
+      <c r="F7" s="13">
+        <f>E7</f>
+        <v/>
+      </c>
+      <c r="G7" s="13">
+        <f>F7</f>
+        <v/>
+      </c>
+      <c r="H7" s="13">
+        <f>G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="13">
+        <f>H7</f>
+        <v/>
+      </c>
+      <c r="J7" s="13">
+        <f>I7</f>
+        <v/>
+      </c>
+      <c r="K7" s="13">
+        <f>J7</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>Share Repurchases $</t>
+        </is>
+      </c>
+      <c r="B8" s="4">
+        <f>'CASH FLOW'!B37</f>
+        <v/>
+      </c>
+      <c r="C8" s="4">
+        <f>'CASH FLOW'!C37</f>
+        <v/>
+      </c>
+      <c r="D8" s="4">
+        <f>'CASH FLOW'!D37</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>'CASH FLOW'!E37</f>
+        <v/>
+      </c>
+      <c r="F8" s="10">
+        <f>ASSUMPTIONS!$B$3</f>
+        <v/>
+      </c>
+      <c r="G8" s="10">
+        <f>ASSUMPTIONS!$B$3</f>
+        <v/>
+      </c>
+      <c r="H8" s="10">
+        <f>ASSUMPTIONS!$B$3</f>
+        <v/>
+      </c>
+      <c r="I8" s="10">
+        <f>ASSUMPTIONS!$B$3</f>
+        <v/>
+      </c>
+      <c r="J8" s="10">
+        <f>ASSUMPTIONS!$B$3</f>
+        <v/>
+      </c>
+      <c r="K8" s="10">
+        <f>ASSUMPTIONS!$B$3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
           <t>Net Debt $</t>
         </is>
       </c>
-      <c r="C8" s="4">
+      <c r="C9" s="4">
         <f>('BALANCE SHEET'!B25+'BALANCE SHEET'!B26+'BALANCE SHEET'!B30+'BALANCE SHEET'!B31)-('BALANCE SHEET'!B2+'BALANCE SHEET'!B3)</f>
         <v/>
       </c>
-      <c r="D8" s="4">
+      <c r="D9" s="4">
         <f>('BALANCE SHEET'!C25+'BALANCE SHEET'!C26+'BALANCE SHEET'!C30+'BALANCE SHEET'!C31)-('BALANCE SHEET'!C2+'BALANCE SHEET'!C3)</f>
         <v/>
       </c>
-      <c r="E8" s="4">
+      <c r="E9" s="4">
         <f>('BALANCE SHEET'!D25+'BALANCE SHEET'!D26+'BALANCE SHEET'!D30+'BALANCE SHEET'!D31)-('BALANCE SHEET'!D2+'BALANCE SHEET'!D3)</f>
         <v/>
       </c>
-      <c r="F8" s="10">
+      <c r="F9" s="10">
         <f>('BALANCE SHEET'!E25+'BALANCE SHEET'!E26+'BALANCE SHEET'!E30+'BALANCE SHEET'!E31)-('BALANCE SHEET'!E2+'BALANCE SHEET'!E3)</f>
         <v/>
       </c>
-      <c r="G8" s="10">
+      <c r="G9" s="10">
         <f>('BALANCE SHEET'!F25+'BALANCE SHEET'!F26+'BALANCE SHEET'!F30+'BALANCE SHEET'!F31)-('BALANCE SHEET'!F2+'BALANCE SHEET'!F3)</f>
         <v/>
       </c>
-      <c r="H8" s="10">
+      <c r="H9" s="10">
         <f>('BALANCE SHEET'!G25+'BALANCE SHEET'!G26+'BALANCE SHEET'!G30+'BALANCE SHEET'!G31)-('BALANCE SHEET'!G2+'BALANCE SHEET'!G3)</f>
         <v/>
       </c>
-      <c r="I8" s="10">
+      <c r="I9" s="10">
         <f>('BALANCE SHEET'!H25+'BALANCE SHEET'!H26+'BALANCE SHEET'!H30+'BALANCE SHEET'!H31)-('BALANCE SHEET'!H2+'BALANCE SHEET'!H3)</f>
         <v/>
       </c>
-      <c r="J8" s="10">
+      <c r="J9" s="10">
         <f>('BALANCE SHEET'!I25+'BALANCE SHEET'!I26+'BALANCE SHEET'!I30+'BALANCE SHEET'!I31)-('BALANCE SHEET'!I2+'BALANCE SHEET'!I3)</f>
         <v/>
       </c>
-      <c r="K8" s="10">
+      <c r="K9" s="10">
         <f>('BALANCE SHEET'!J25+'BALANCE SHEET'!J26+'BALANCE SHEET'!J30+'BALANCE SHEET'!J31)-('BALANCE SHEET'!J2+'BALANCE SHEET'!J3)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
vault backup: 2026-04-26 16:32:44
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -2294,43 +2294,43 @@
         </is>
       </c>
       <c r="B44" s="6">
-        <f>SUM(B39:B43)</f>
+        <f>SUM(B38:B43)</f>
         <v/>
       </c>
       <c r="C44" s="6">
-        <f>SUM(C39:C43)</f>
+        <f>SUM(C38:C43)</f>
         <v/>
       </c>
       <c r="D44" s="6">
-        <f>SUM(D39:D43)</f>
+        <f>SUM(D38:D43)</f>
         <v/>
       </c>
       <c r="E44" s="6">
-        <f>SUM(E39:E43)</f>
+        <f>SUM(E38:E43)</f>
         <v/>
       </c>
       <c r="F44" s="7">
-        <f>SUM(F39:F43)</f>
+        <f>SUM(F38:F43)</f>
         <v/>
       </c>
       <c r="G44" s="7">
-        <f>SUM(G39:G43)</f>
+        <f>SUM(G38:G43)</f>
         <v/>
       </c>
       <c r="H44" s="7">
-        <f>SUM(H39:H43)</f>
+        <f>SUM(H38:H43)</f>
         <v/>
       </c>
       <c r="I44" s="7">
-        <f>SUM(I39:I43)</f>
+        <f>SUM(I38:I43)</f>
         <v/>
       </c>
       <c r="J44" s="7">
-        <f>SUM(J39:J43)</f>
+        <f>SUM(J38:J43)</f>
         <v/>
       </c>
       <c r="K44" s="7">
-        <f>SUM(K39:K43)</f>
+        <f>SUM(K38:K43)</f>
         <v/>
       </c>
     </row>
@@ -2341,43 +2341,43 @@
         </is>
       </c>
       <c r="B45" s="6">
-        <f>B37+B38+B44</f>
+        <f>B37+B44</f>
         <v/>
       </c>
       <c r="C45" s="6">
-        <f>C37+C38+C44</f>
+        <f>C37+C44</f>
         <v/>
       </c>
       <c r="D45" s="6">
-        <f>D37+D38+D44</f>
+        <f>D37+D44</f>
         <v/>
       </c>
       <c r="E45" s="6">
-        <f>E37+E38+E44</f>
+        <f>E37+E44</f>
         <v/>
       </c>
       <c r="F45" s="7">
-        <f>F37+F38+F44</f>
+        <f>F37+F44</f>
         <v/>
       </c>
       <c r="G45" s="7">
-        <f>G37+G38+G44</f>
+        <f>G37+G44</f>
         <v/>
       </c>
       <c r="H45" s="7">
-        <f>H37+H38+H44</f>
+        <f>H37+H44</f>
         <v/>
       </c>
       <c r="I45" s="7">
-        <f>I37+I38+I44</f>
+        <f>I37+I44</f>
         <v/>
       </c>
       <c r="J45" s="7">
-        <f>J37+J38+J44</f>
+        <f>J37+J44</f>
         <v/>
       </c>
       <c r="K45" s="7">
-        <f>K37+K38+K44</f>
+        <f>K37+K44</f>
         <v/>
       </c>
     </row>
@@ -2392,7 +2392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3824,6 +3824,57 @@
       <c r="K47" s="5" t="n"/>
       <c r="L47" s="5" t="n"/>
     </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Net Change in Cash</t>
+        </is>
+      </c>
+      <c r="B48" s="6">
+        <f>B28+B35+B46+B47</f>
+        <v/>
+      </c>
+      <c r="C48" s="6">
+        <f>C28+C35+C46+C47</f>
+        <v/>
+      </c>
+      <c r="D48" s="6">
+        <f>D28+D35+D46+D47</f>
+        <v/>
+      </c>
+      <c r="E48" s="6">
+        <f>E28+E35+E46+E47</f>
+        <v/>
+      </c>
+      <c r="F48" s="6">
+        <f>F28+F35+F46+F47</f>
+        <v/>
+      </c>
+      <c r="G48" s="6">
+        <f>G28+G35+G46+G47</f>
+        <v/>
+      </c>
+      <c r="H48" s="6">
+        <f>H28+H35+H46+H47</f>
+        <v/>
+      </c>
+      <c r="I48" s="6">
+        <f>I28+I35+I46+I47</f>
+        <v/>
+      </c>
+      <c r="J48" s="6">
+        <f>J28+J35+J46+J47</f>
+        <v/>
+      </c>
+      <c r="K48" s="6">
+        <f>K28+K35+K46+K47</f>
+        <v/>
+      </c>
+      <c r="L48" s="6">
+        <f>L28+L35+L46+L47</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3835,7 +3886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3848,51 +3899,63 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
+          <t>Q2 FY2022</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
           <t>Q3 FY2022</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Q1 FY2023</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2023</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2023</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Q1 FY2024</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2024</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2024</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Q1 FY2025</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2025</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2025</t>
         </is>
@@ -3905,30 +3968,36 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
+        <v>287408</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>475640</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
+        <v>259939</v>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>585822</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="F2" s="4" t="n">
         <v>970579</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="G2" s="4" t="n">
         <v>355708</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="H2" s="4" t="n">
         <v>757685</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="I2" s="4" t="n">
         <v>1023433</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="J2" s="4" t="n">
         <v>329276</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>1068535</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>1793641</v>
       </c>
     </row>
@@ -3939,30 +4008,36 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
+        <v>-174195</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>-283778</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
+        <v>-146121</v>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>-313010</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="F3" s="4" t="n">
         <v>-503685</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="G3" s="4" t="n">
         <v>-173501</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="H3" s="4" t="n">
         <v>-366380</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="I3" s="4" t="n">
         <v>-509899</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="J3" s="4" t="n">
         <v>-156903</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="K3" s="4" t="n">
         <v>-515311</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="L3" s="4" t="n">
         <v>-868138</v>
       </c>
     </row>
@@ -4008,6 +4083,14 @@
         <f>J2+J3</f>
         <v/>
       </c>
+      <c r="K4" s="6">
+        <f>K2+K3</f>
+        <v/>
+      </c>
+      <c r="L4" s="6">
+        <f>L2+L3</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -4016,30 +4099,36 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
+        <v>-90667</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>-316917</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
+        <v>-68905</v>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>-163086</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>-259471</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="G5" s="4" t="n">
         <v>-99017</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>-213867</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="I5" s="4" t="n">
         <v>-339310</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="J5" s="4" t="n">
         <v>-120342</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="K5" s="4" t="n">
         <v>-358228</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="L5" s="4" t="n">
         <v>-563799</v>
       </c>
     </row>
@@ -4074,6 +4163,12 @@
         <v>0</v>
       </c>
       <c r="J6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4" t="n">
         <v>246707</v>
       </c>
     </row>
@@ -4119,6 +4214,14 @@
         <f>J4+SUM(J5:J6)</f>
         <v/>
       </c>
+      <c r="K7" s="6">
+        <f>K4+SUM(K5:K6)</f>
+        <v/>
+      </c>
+      <c r="L7" s="6">
+        <f>L4+SUM(L5:L6)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -4127,30 +4230,36 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
+        <v>129</v>
+      </c>
+      <c r="C8" s="4" t="n">
         <v>1579</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="D8" s="4" t="n">
+        <v>4969</v>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>10542</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="F8" s="4" t="n">
         <v>17767</v>
       </c>
-      <c r="E8" s="4" t="n">
-        <v>9612</v>
-      </c>
-      <c r="F8" s="4" t="n">
+      <c r="G8" s="4" t="n">
+        <v>9640</v>
+      </c>
+      <c r="H8" s="4" t="n">
         <v>20287</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="I8" s="4" t="n">
         <v>31399</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="J8" s="4" t="n">
         <v>7846</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="K8" s="4" t="n">
         <v>-6196</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="L8" s="4" t="n">
         <v>-19592</v>
       </c>
     </row>
@@ -4161,30 +4270,36 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
+        <v>-676</v>
+      </c>
+      <c r="C9" s="4" t="n">
         <v>-930</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="D9" s="4" t="n">
+        <v>-118</v>
+      </c>
+      <c r="E9" s="4" t="n">
         <v>-1049</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="F9" s="4" t="n">
         <v>-1226</v>
       </c>
-      <c r="E9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="4" t="n">
+      <c r="G9" s="4" t="n">
+        <v>-369</v>
+      </c>
+      <c r="H9" s="4" t="n">
         <v>-633</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="I9" s="4" t="n">
         <v>-356</v>
       </c>
-      <c r="H9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="J9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4204,7 +4319,7 @@
         <v>0</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>-341</v>
+        <v>0</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>0</v>
@@ -4213,12 +4328,18 @@
         <v>0</v>
       </c>
       <c r="H10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="4" t="n">
         <v>1116</v>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="K10" s="4" t="n">
         <v>1658</v>
       </c>
-      <c r="J10" s="4" t="n">
+      <c r="L10" s="4" t="n">
         <v>7022</v>
       </c>
     </row>
@@ -4264,6 +4385,14 @@
         <f>J7+SUM(J8:J10)</f>
         <v/>
       </c>
+      <c r="K11" s="6">
+        <f>K7+SUM(K8:K10)</f>
+        <v/>
+      </c>
+      <c r="L11" s="6">
+        <f>L7+SUM(L8:L10)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -4272,30 +4401,36 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
+        <v>-6161</v>
+      </c>
+      <c r="C12" s="4" t="n">
         <v>-41653</v>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="D12" s="4" t="n">
+        <v>-8537</v>
+      </c>
+      <c r="E12" s="4" t="n">
         <v>-26483</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="F12" s="4" t="n">
         <v>-47279</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="G12" s="4" t="n">
         <v>-14650</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>-39498</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="I12" s="4" t="n">
         <v>-41317</v>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="J12" s="4" t="n">
         <v>-16574</v>
       </c>
-      <c r="I12" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>-46184</v>
       </c>
-      <c r="J12" s="4" t="n">
+      <c r="L12" s="4" t="n">
         <v>-19167</v>
       </c>
     </row>
@@ -4341,6 +4476,14 @@
         <f>J11+J12</f>
         <v/>
       </c>
+      <c r="K13" s="6">
+        <f>K11+K12</f>
+        <v/>
+      </c>
+      <c r="L13" s="6">
+        <f>L11+L12</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -4349,30 +4492,36 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
+        <v>15838</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>-166059</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="D14" s="4" t="n">
+        <v>41227</v>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>92736</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>176685</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="G14" s="4" t="n">
         <v>77811</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>157594</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="I14" s="4" t="n">
         <v>163950</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="J14" s="4" t="n">
         <v>44419</v>
       </c>
-      <c r="I14" s="4" t="n">
+      <c r="K14" s="4" t="n">
         <v>144274</v>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="L14" s="4" t="n">
         <v>83260</v>
       </c>
     </row>
@@ -4383,30 +4532,36 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="4" t="n">
         <v>-4596</v>
       </c>
-      <c r="C15" s="4" t="n">
+      <c r="D15" s="4" t="n">
+        <v>-6781</v>
+      </c>
+      <c r="E15" s="4" t="n">
         <v>-13637</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="F15" s="4" t="n">
         <v>-20512</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="G15" s="4" t="n">
         <v>-6837</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="H15" s="4" t="n">
         <v>-13675</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="I15" s="4" t="n">
         <v>-20588</v>
       </c>
-      <c r="H15" s="4" t="n">
+      <c r="J15" s="4" t="n">
         <v>-6781</v>
       </c>
-      <c r="I15" s="4" t="n">
+      <c r="K15" s="4" t="n">
         <v>-13632</v>
       </c>
-      <c r="J15" s="4" t="n">
+      <c r="L15" s="4" t="n">
         <v>-23289</v>
       </c>
     </row>
@@ -4420,27 +4575,33 @@
         <v>0</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>6898</v>
+        <v>0</v>
       </c>
       <c r="D16" s="4" t="n">
+        <v>2934</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>6727</v>
+      </c>
+      <c r="F16" s="4" t="n">
         <v>13263</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="G16" s="4" t="n">
         <v>6128</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="H16" s="4" t="n">
         <v>12417</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="I16" s="4" t="n">
         <v>12357</v>
       </c>
-      <c r="H16" s="4" t="n">
+      <c r="J16" s="4" t="n">
         <v>3219</v>
       </c>
-      <c r="I16" s="4" t="n">
+      <c r="K16" s="4" t="n">
         <v>10703</v>
       </c>
-      <c r="J16" s="4" t="n">
+      <c r="L16" s="4" t="n">
         <v>5272</v>
       </c>
     </row>
@@ -4451,30 +4612,36 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
+        <v>15838</v>
+      </c>
+      <c r="C17" s="4" t="n">
         <v>-170655</v>
       </c>
-      <c r="C17" s="4" t="n">
-        <v>72201</v>
-      </c>
       <c r="D17" s="4" t="n">
+        <v>31512</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>72372</v>
+      </c>
+      <c r="F17" s="4" t="n">
         <v>142910</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="G17" s="4" t="n">
         <v>64846</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="H17" s="4" t="n">
         <v>131502</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="I17" s="4" t="n">
         <v>131005</v>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="J17" s="4" t="n">
         <v>34419</v>
       </c>
-      <c r="I17" s="4" t="n">
+      <c r="K17" s="4" t="n">
         <v>119939</v>
       </c>
-      <c r="J17" s="4" t="n">
+      <c r="L17" s="4" t="n">
         <v>54699</v>
       </c>
     </row>
@@ -4489,7 +4656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4502,6 +4669,8 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4513,40 +4682,50 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
+          <t>Q2 FY2023</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
           <t>Q3 FY2023</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Q4 FY2023</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Q1 FY2024</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2024</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2024</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Q4 FY2024</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Q1 FY2025</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2025</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2025</t>
         </is>
@@ -4562,27 +4741,33 @@
         <v>614159</v>
       </c>
       <c r="C2" s="4" t="n">
+        <v>681054</v>
+      </c>
+      <c r="D2" s="4" t="n">
         <v>760022</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="E2" s="4" t="n">
         <v>755981</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="F2" s="4" t="n">
+        <v>879498</v>
+      </c>
+      <c r="G2" s="4" t="n">
         <v>903210</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="H2" s="4" t="n">
         <v>903748</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="I2" s="4" t="n">
         <v>890190</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="J2" s="4" t="n">
         <v>977285</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>615233</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>805955</v>
       </c>
     </row>
@@ -4617,6 +4802,12 @@
         <v>0</v>
       </c>
       <c r="J3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4" t="n">
         <v>126508</v>
       </c>
     </row>
@@ -4630,27 +4821,33 @@
         <v>63311</v>
       </c>
       <c r="C4" s="4" t="n">
+        <v>197811</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>215243</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="E4" s="4" t="n">
         <v>183703</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="F4" s="4" t="n">
+        <v>200117</v>
+      </c>
+      <c r="G4" s="4" t="n">
         <v>262920</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="H4" s="4" t="n">
         <v>208774</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="I4" s="4" t="n">
         <v>270342</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>256424</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>490389</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>513682</v>
       </c>
     </row>
@@ -4664,27 +4861,33 @@
         <v>2979</v>
       </c>
       <c r="C5" s="4" t="n">
+        <v>3323</v>
+      </c>
+      <c r="D5" s="4" t="n">
         <v>3309</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="E5" s="4" t="n">
         <v>2318</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="F5" s="4" t="n">
+        <v>2259</v>
+      </c>
+      <c r="G5" s="4" t="n">
         <v>1166</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>1025</v>
       </c>
-      <c r="G5" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="I5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4698,27 +4901,33 @@
         <v>173289</v>
       </c>
       <c r="C6" s="4" t="n">
+        <v>152545</v>
+      </c>
+      <c r="D6" s="4" t="n">
         <v>198704</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="E6" s="4" t="n">
         <v>229275</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="F6" s="4" t="n">
+        <v>197504</v>
+      </c>
+      <c r="G6" s="4" t="n">
         <v>180669</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>197572</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>131165</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="J6" s="4" t="n">
         <v>141159</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="K6" s="4" t="n">
         <v>230046</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="L6" s="4" t="n">
         <v>282514</v>
       </c>
     </row>
@@ -4732,27 +4941,33 @@
         <v>11341</v>
       </c>
       <c r="C7" s="4" t="n">
+        <v>23398</v>
+      </c>
+      <c r="D7" s="4" t="n">
         <v>23747</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="E7" s="4" t="n">
         <v>19503</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="F7" s="4" t="n">
+        <v>21523</v>
+      </c>
+      <c r="G7" s="4" t="n">
         <v>22900</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="H7" s="4" t="n">
         <v>38227</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="I7" s="4" t="n">
         <v>18759</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="J7" s="4" t="n">
         <v>22464</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>41420</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="L7" s="4" t="n">
         <v>163395</v>
       </c>
     </row>
@@ -4787,6 +5002,12 @@
         <v>14124</v>
       </c>
       <c r="J8" s="4" t="n">
+        <v>14124</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>14124</v>
+      </c>
+      <c r="L8" s="4" t="n">
         <v>49520</v>
       </c>
     </row>
@@ -4832,6 +5053,14 @@
         <f>SUM(J2:J8)</f>
         <v/>
       </c>
+      <c r="K9" s="6">
+        <f>SUM(K2:K8)</f>
+        <v/>
+      </c>
+      <c r="L9" s="6">
+        <f>SUM(L2:L8)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -4866,6 +5095,12 @@
       <c r="J10" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="K10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -4877,27 +5112,33 @@
         <v>10185</v>
       </c>
       <c r="C11" s="4" t="n">
+        <v>15892</v>
+      </c>
+      <c r="D11" s="4" t="n">
         <v>21061</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="E11" s="4" t="n">
         <v>24868</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="F11" s="4" t="n">
+        <v>28350</v>
+      </c>
+      <c r="G11" s="4" t="n">
         <v>36282</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="H11" s="4" t="n">
         <v>38370</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="I11" s="4" t="n">
         <v>55602</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="J11" s="4" t="n">
         <v>58698</v>
       </c>
-      <c r="I11" s="4" t="n">
+      <c r="K11" s="4" t="n">
         <v>72516</v>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="L11" s="4" t="n">
         <v>80925</v>
       </c>
     </row>
@@ -4911,27 +5152,33 @@
         <v>972</v>
       </c>
       <c r="C12" s="4" t="n">
+        <v>756</v>
+      </c>
+      <c r="D12" s="4" t="n">
         <v>1152</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="E12" s="4" t="n">
         <v>1957</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="F12" s="4" t="n">
+        <v>1688</v>
+      </c>
+      <c r="G12" s="4" t="n">
         <v>1507</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>5506</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="I12" s="4" t="n">
         <v>21606</v>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="J12" s="4" t="n">
         <v>20866</v>
       </c>
-      <c r="I12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="4" t="n">
+      <c r="K12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4945,27 +5192,33 @@
         <v>12254</v>
       </c>
       <c r="C13" s="4" t="n">
+        <v>12211</v>
+      </c>
+      <c r="D13" s="4" t="n">
         <v>11772</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="E13" s="4" t="n">
         <v>12139</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="F13" s="4" t="n">
+        <v>11741</v>
+      </c>
+      <c r="G13" s="4" t="n">
         <v>11491</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="H13" s="4" t="n">
         <v>11877</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="I13" s="4" t="n">
         <v>12213</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="J13" s="4" t="n">
         <v>12444</v>
       </c>
-      <c r="I13" s="4" t="n">
+      <c r="K13" s="4" t="n">
         <v>1222115</v>
       </c>
-      <c r="J13" s="4" t="n">
+      <c r="L13" s="4" t="n">
         <v>1397819</v>
       </c>
     </row>
@@ -4979,27 +5232,33 @@
         <v>13679</v>
       </c>
       <c r="C14" s="4" t="n">
+        <v>13937</v>
+      </c>
+      <c r="D14" s="4" t="n">
         <v>13588</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E14" s="4" t="n">
         <v>14173</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
+        <v>13866</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>13730</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>14360</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="I14" s="4" t="n">
         <v>71582</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="J14" s="4" t="n">
         <v>72128</v>
       </c>
-      <c r="I14" s="4" t="n">
+      <c r="K14" s="4" t="n">
         <v>802234</v>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="L14" s="4" t="n">
         <v>914957</v>
       </c>
     </row>
@@ -5013,27 +5272,33 @@
         <v>262462</v>
       </c>
       <c r="C15" s="4" t="n">
+        <v>255400</v>
+      </c>
+      <c r="D15" s="4" t="n">
         <v>251869</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="E15" s="4" t="n">
         <v>248338</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="F15" s="4" t="n">
+        <v>244807</v>
+      </c>
+      <c r="G15" s="4" t="n">
         <v>241276</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="H15" s="4" t="n">
         <v>237746</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="I15" s="4" t="n">
         <v>234215</v>
       </c>
-      <c r="H15" s="4" t="n">
+      <c r="J15" s="4" t="n">
         <v>230684</v>
       </c>
-      <c r="I15" s="4" t="n">
+      <c r="K15" s="4" t="n">
         <v>227153</v>
       </c>
-      <c r="J15" s="4" t="n">
+      <c r="L15" s="4" t="n">
         <v>784214</v>
       </c>
     </row>
@@ -5047,27 +5312,33 @@
         <v>501</v>
       </c>
       <c r="C16" s="4" t="n">
+        <v>28373</v>
+      </c>
+      <c r="D16" s="4" t="n">
         <v>30614</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="E16" s="4" t="n">
         <v>29518</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="F16" s="4" t="n">
+        <v>22437</v>
+      </c>
+      <c r="G16" s="4" t="n">
         <v>22727</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="H16" s="4" t="n">
         <v>24186</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="I16" s="4" t="n">
         <v>38699</v>
       </c>
-      <c r="H16" s="4" t="n">
+      <c r="J16" s="4" t="n">
         <v>38525</v>
       </c>
-      <c r="I16" s="4" t="n">
+      <c r="K16" s="4" t="n">
         <v>43158</v>
       </c>
-      <c r="J16" s="4" t="n">
+      <c r="L16" s="4" t="n">
         <v>110410</v>
       </c>
     </row>
@@ -5081,27 +5352,33 @@
         <v>208</v>
       </c>
       <c r="C17" s="4" t="n">
+        <v>171</v>
+      </c>
+      <c r="D17" s="4" t="n">
         <v>148</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="E17" s="4" t="n">
         <v>208</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="F17" s="4" t="n">
+        <v>263</v>
+      </c>
+      <c r="G17" s="4" t="n">
         <v>233</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="H17" s="4" t="n">
         <v>214</v>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="I17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5115,27 +5392,33 @@
         <v>263</v>
       </c>
       <c r="C18" s="4" t="n">
+        <v>254</v>
+      </c>
+      <c r="D18" s="4" t="n">
         <v>265</v>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="E18" s="4" t="n">
         <v>291</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="F18" s="4" t="n">
+        <v>7963</v>
+      </c>
+      <c r="G18" s="4" t="n">
         <v>6653</v>
       </c>
-      <c r="F18" s="4" t="n">
+      <c r="H18" s="4" t="n">
         <v>8594</v>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="I18" s="4" t="n">
         <v>8384</v>
       </c>
-      <c r="H18" s="4" t="n">
+      <c r="J18" s="4" t="n">
         <v>14717</v>
       </c>
-      <c r="I18" s="4" t="n">
+      <c r="K18" s="4" t="n">
         <v>36755</v>
       </c>
-      <c r="J18" s="4" t="n">
+      <c r="L18" s="4" t="n">
         <v>35809</v>
       </c>
     </row>
@@ -5181,6 +5464,14 @@
         <f>J9+SUM(J10:J18)</f>
         <v/>
       </c>
+      <c r="K19" s="6">
+        <f>K9+SUM(K10:K18)</f>
+        <v/>
+      </c>
+      <c r="L19" s="6">
+        <f>L9+SUM(L10:L18)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -5192,27 +5483,33 @@
         <v>106147</v>
       </c>
       <c r="C20" s="4" t="n">
+        <v>94313</v>
+      </c>
+      <c r="D20" s="4" t="n">
         <v>121088</v>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="E20" s="4" t="n">
         <v>42840</v>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="F20" s="4" t="n">
+        <v>40196</v>
+      </c>
+      <c r="G20" s="4" t="n">
         <v>47423</v>
       </c>
-      <c r="F20" s="4" t="n">
+      <c r="H20" s="4" t="n">
         <v>30938</v>
       </c>
-      <c r="G20" s="4" t="n">
+      <c r="I20" s="4" t="n">
         <v>41287</v>
       </c>
-      <c r="H20" s="4" t="n">
+      <c r="J20" s="4" t="n">
         <v>61052</v>
       </c>
-      <c r="I20" s="4" t="n">
+      <c r="K20" s="4" t="n">
         <v>120962</v>
       </c>
-      <c r="J20" s="4" t="n">
+      <c r="L20" s="4" t="n">
         <v>97794</v>
       </c>
     </row>
@@ -5229,24 +5526,30 @@
         <v>0</v>
       </c>
       <c r="D21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="4" t="n">
         <v>62120</v>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="F21" s="4" t="n">
+        <v>63871</v>
+      </c>
+      <c r="G21" s="4" t="n">
         <v>79633</v>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="H21" s="4" t="n">
         <v>73024</v>
       </c>
-      <c r="G21" s="4" t="n">
+      <c r="I21" s="4" t="n">
         <v>148780</v>
       </c>
-      <c r="H21" s="4" t="n">
+      <c r="J21" s="4" t="n">
         <v>152046</v>
       </c>
-      <c r="I21" s="4" t="n">
+      <c r="K21" s="4" t="n">
         <v>225859</v>
       </c>
-      <c r="J21" s="4" t="n">
+      <c r="L21" s="4" t="n">
         <v>311768</v>
       </c>
     </row>
@@ -5260,27 +5563,33 @@
         <v>1193</v>
       </c>
       <c r="C22" s="4" t="n">
+        <v>58798</v>
+      </c>
+      <c r="D22" s="4" t="n">
         <v>58855</v>
       </c>
-      <c r="D22" s="4" t="n">
+      <c r="E22" s="4" t="n">
         <v>50424</v>
       </c>
-      <c r="E22" s="4" t="n">
+      <c r="F22" s="4" t="n">
+        <v>58619</v>
+      </c>
+      <c r="G22" s="4" t="n">
         <v>5374</v>
       </c>
-      <c r="F22" s="4" t="n">
+      <c r="H22" s="4" t="n">
         <v>739</v>
       </c>
-      <c r="G22" s="4" t="n">
+      <c r="I22" s="4" t="n">
         <v>10834</v>
       </c>
-      <c r="H22" s="4" t="n">
+      <c r="J22" s="4" t="n">
         <v>26206</v>
       </c>
-      <c r="I22" s="4" t="n">
+      <c r="K22" s="4" t="n">
         <v>21765</v>
       </c>
-      <c r="J22" s="4" t="n">
+      <c r="L22" s="4" t="n">
         <v>49590</v>
       </c>
     </row>
@@ -5315,6 +5624,12 @@
         <v>0</v>
       </c>
       <c r="J23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="4" t="n">
         <v>252953</v>
       </c>
     </row>
@@ -5328,27 +5643,33 @@
         <v>35977</v>
       </c>
       <c r="C24" s="4" t="n">
+        <v>98933</v>
+      </c>
+      <c r="D24" s="4" t="n">
         <v>136557</v>
       </c>
-      <c r="D24" s="4" t="n">
+      <c r="E24" s="4" t="n">
         <v>99787</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="F24" s="4" t="n">
+        <v>129201</v>
+      </c>
+      <c r="G24" s="4" t="n">
         <v>156479</v>
       </c>
-      <c r="F24" s="4" t="n">
+      <c r="H24" s="4" t="n">
         <v>158810</v>
       </c>
-      <c r="G24" s="4" t="n">
+      <c r="I24" s="4" t="n">
         <v>135948</v>
       </c>
-      <c r="H24" s="4" t="n">
+      <c r="J24" s="4" t="n">
         <v>151327</v>
       </c>
-      <c r="I24" s="4" t="n">
+      <c r="K24" s="4" t="n">
         <v>200169</v>
       </c>
-      <c r="J24" s="4" t="n">
+      <c r="L24" s="4" t="n">
         <v>234068</v>
       </c>
     </row>
@@ -5362,27 +5683,33 @@
         <v>661</v>
       </c>
       <c r="C25" s="4" t="n">
+        <v>505</v>
+      </c>
+      <c r="D25" s="4" t="n">
         <v>628</v>
       </c>
-      <c r="D25" s="4" t="n">
+      <c r="E25" s="4" t="n">
         <v>980</v>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="F25" s="4" t="n">
+        <v>821</v>
+      </c>
+      <c r="G25" s="4" t="n">
         <v>729</v>
       </c>
-      <c r="F25" s="4" t="n">
+      <c r="H25" s="4" t="n">
         <v>1358</v>
       </c>
-      <c r="G25" s="4" t="n">
+      <c r="I25" s="4" t="n">
         <v>3265</v>
       </c>
-      <c r="H25" s="4" t="n">
+      <c r="J25" s="4" t="n">
         <v>3550</v>
       </c>
-      <c r="I25" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="4" t="n">
+      <c r="K25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5396,27 +5723,33 @@
         <v>70</v>
       </c>
       <c r="C26" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="D26" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="D26" s="4" t="n">
+      <c r="E26" s="4" t="n">
         <v>59</v>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="F26" s="4" t="n">
         <v>61</v>
       </c>
-      <c r="F26" s="4" t="n">
+      <c r="G26" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="H26" s="4" t="n">
         <v>99</v>
       </c>
-      <c r="G26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="I26" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5448,9 +5781,15 @@
         <v>0</v>
       </c>
       <c r="I27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="4" t="n">
         <v>25000</v>
       </c>
-      <c r="J27" s="4" t="n">
+      <c r="L27" s="4" t="n">
         <v>25000</v>
       </c>
     </row>
@@ -5467,7 +5806,7 @@
         <v>9500</v>
       </c>
       <c r="D28" s="4" t="n">
-        <v>9513</v>
+        <v>9500</v>
       </c>
       <c r="E28" s="4" t="n">
         <v>9513</v>
@@ -5482,9 +5821,15 @@
         <v>9513</v>
       </c>
       <c r="I28" s="4" t="n">
+        <v>9513</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>9513</v>
+      </c>
+      <c r="K28" s="4" t="n">
         <v>16071</v>
       </c>
-      <c r="J28" s="4" t="n">
+      <c r="L28" s="4" t="n">
         <v>25557</v>
       </c>
     </row>
@@ -5498,27 +5843,33 @@
         <v>3586</v>
       </c>
       <c r="C29" s="4" t="n">
+        <v>7109</v>
+      </c>
+      <c r="D29" s="4" t="n">
         <v>8826</v>
       </c>
-      <c r="D29" s="4" t="n">
+      <c r="E29" s="4" t="n">
         <v>10890</v>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="F29" s="4" t="n">
+        <v>12987</v>
+      </c>
+      <c r="G29" s="4" t="n">
         <v>13772</v>
       </c>
-      <c r="F29" s="4" t="n">
+      <c r="H29" s="4" t="n">
         <v>14979</v>
       </c>
-      <c r="G29" s="4" t="n">
+      <c r="I29" s="4" t="n">
         <v>15908</v>
       </c>
-      <c r="H29" s="4" t="n">
+      <c r="J29" s="4" t="n">
         <v>14160</v>
       </c>
-      <c r="I29" s="4" t="n">
+      <c r="K29" s="4" t="n">
         <v>49949</v>
       </c>
-      <c r="J29" s="4" t="n">
+      <c r="L29" s="4" t="n">
         <v>32258</v>
       </c>
     </row>
@@ -5564,6 +5915,14 @@
         <f>SUM(J20:J29)</f>
         <v/>
       </c>
+      <c r="K30" s="6">
+        <f>SUM(K20:K29)</f>
+        <v/>
+      </c>
+      <c r="L30" s="6">
+        <f>SUM(L20:L29)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -5575,27 +5934,33 @@
         <v>326</v>
       </c>
       <c r="C31" s="4" t="n">
+        <v>249</v>
+      </c>
+      <c r="D31" s="4" t="n">
         <v>512</v>
       </c>
-      <c r="D31" s="4" t="n">
+      <c r="E31" s="4" t="n">
         <v>955</v>
       </c>
-      <c r="E31" s="4" t="n">
+      <c r="F31" s="4" t="n">
+        <v>850</v>
+      </c>
+      <c r="G31" s="4" t="n">
         <v>762</v>
       </c>
-      <c r="F31" s="4" t="n">
+      <c r="H31" s="4" t="n">
         <v>4193</v>
       </c>
-      <c r="G31" s="4" t="n">
+      <c r="I31" s="4" t="n">
         <v>16674</v>
       </c>
-      <c r="H31" s="4" t="n">
+      <c r="J31" s="4" t="n">
         <v>16152</v>
       </c>
-      <c r="I31" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" s="4" t="n">
+      <c r="K31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5609,27 +5974,33 @@
         <v>162</v>
       </c>
       <c r="C32" s="4" t="n">
+        <v>147</v>
+      </c>
+      <c r="D32" s="4" t="n">
         <v>135</v>
       </c>
-      <c r="D32" s="4" t="n">
+      <c r="E32" s="4" t="n">
         <v>193</v>
       </c>
-      <c r="E32" s="4" t="n">
+      <c r="F32" s="4" t="n">
+        <v>245</v>
+      </c>
+      <c r="G32" s="4" t="n">
         <v>228</v>
       </c>
-      <c r="F32" s="4" t="n">
+      <c r="H32" s="4" t="n">
         <v>189</v>
       </c>
-      <c r="G32" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="I32" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5643,27 +6014,33 @@
         <v>15919</v>
       </c>
       <c r="C33" s="4" t="n">
+        <v>2333</v>
+      </c>
+      <c r="D33" s="4" t="n">
         <v>2249</v>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="E33" s="4" t="n">
         <v>2880</v>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="F33" s="4" t="n">
+        <v>2248</v>
+      </c>
+      <c r="G33" s="4" t="n">
         <v>2201</v>
       </c>
-      <c r="F33" s="4" t="n">
+      <c r="H33" s="4" t="n">
         <v>2275</v>
       </c>
-      <c r="G33" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="I33" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5695,9 +6072,15 @@
         <v>0</v>
       </c>
       <c r="I34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="4" t="n">
         <v>862917</v>
       </c>
-      <c r="J34" s="4" t="n">
+      <c r="L34" s="4" t="n">
         <v>861472</v>
       </c>
     </row>
@@ -5711,27 +6094,33 @@
         <v>179788</v>
       </c>
       <c r="C35" s="4" t="n">
+        <v>171745</v>
+      </c>
+      <c r="D35" s="4" t="n">
         <v>169370</v>
       </c>
-      <c r="D35" s="4" t="n">
+      <c r="E35" s="4" t="n">
         <v>167227</v>
       </c>
-      <c r="E35" s="4" t="n">
+      <c r="F35" s="4" t="n">
+        <v>164849</v>
+      </c>
+      <c r="G35" s="4" t="n">
         <v>162471</v>
       </c>
-      <c r="F35" s="4" t="n">
+      <c r="H35" s="4" t="n">
         <v>160092</v>
       </c>
-      <c r="G35" s="4" t="n">
+      <c r="I35" s="4" t="n">
         <v>157714</v>
       </c>
-      <c r="H35" s="4" t="n">
+      <c r="J35" s="4" t="n">
         <v>155336</v>
       </c>
-      <c r="I35" s="4" t="n">
+      <c r="K35" s="4" t="n">
         <v>156135</v>
       </c>
-      <c r="J35" s="4" t="n">
+      <c r="L35" s="4" t="n">
         <v>387432</v>
       </c>
     </row>
@@ -5757,15 +6146,21 @@
         <v>0</v>
       </c>
       <c r="G36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="4" t="n">
         <v>2541</v>
       </c>
-      <c r="H36" s="4" t="n">
+      <c r="J36" s="4" t="n">
         <v>2574</v>
       </c>
-      <c r="I36" s="4" t="n">
+      <c r="K36" s="4" t="n">
         <v>25002</v>
       </c>
-      <c r="J36" s="4" t="n">
+      <c r="L36" s="4" t="n">
         <v>24431</v>
       </c>
     </row>
@@ -5811,6 +6206,14 @@
         <f>J30+SUM(J31:J36)</f>
         <v/>
       </c>
+      <c r="K37" s="6">
+        <f>K30+SUM(K31:K36)</f>
+        <v/>
+      </c>
+      <c r="L37" s="6">
+        <f>L30+SUM(L31:L36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -5843,6 +6246,12 @@
         <v>824488</v>
       </c>
       <c r="J38" s="4" t="n">
+        <v>824488</v>
+      </c>
+      <c r="K38" s="4" t="n">
+        <v>824488</v>
+      </c>
+      <c r="L38" s="4" t="n">
         <v>1760275</v>
       </c>
     </row>
@@ -5862,21 +6271,27 @@
         <v>77</v>
       </c>
       <c r="E39" s="4" t="n">
+        <v>77</v>
+      </c>
+      <c r="F39" s="4" t="n">
         <v>78</v>
       </c>
-      <c r="F39" s="4" t="n">
-        <v>79</v>
-      </c>
       <c r="G39" s="4" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H39" s="4" t="n">
         <v>79</v>
       </c>
       <c r="I39" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="J39" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="K39" s="4" t="n">
         <v>101</v>
       </c>
-      <c r="J39" s="4" t="n">
+      <c r="L39" s="4" t="n">
         <v>101</v>
       </c>
     </row>
@@ -5890,27 +6305,33 @@
         <v>280668</v>
       </c>
       <c r="C40" s="4" t="n">
+        <v>278980</v>
+      </c>
+      <c r="D40" s="4" t="n">
         <v>277980</v>
       </c>
-      <c r="D40" s="4" t="n">
+      <c r="E40" s="4" t="n">
         <v>276717</v>
       </c>
-      <c r="E40" s="4" t="n">
+      <c r="F40" s="4" t="n">
+        <v>281247</v>
+      </c>
+      <c r="G40" s="4" t="n">
         <v>286173</v>
       </c>
-      <c r="F40" s="4" t="n">
+      <c r="H40" s="4" t="n">
         <v>292576</v>
       </c>
-      <c r="G40" s="4" t="n">
+      <c r="I40" s="4" t="n">
         <v>297579</v>
       </c>
-      <c r="H40" s="4" t="n">
+      <c r="J40" s="4" t="n">
         <v>300877</v>
       </c>
-      <c r="I40" s="4" t="n">
+      <c r="K40" s="4" t="n">
         <v>1028384</v>
       </c>
-      <c r="J40" s="4" t="n">
+      <c r="L40" s="4" t="n">
         <v>1035021</v>
       </c>
     </row>
@@ -5924,27 +6345,33 @@
         <v>-1881</v>
       </c>
       <c r="C41" s="4" t="n">
+        <v>-1877</v>
+      </c>
+      <c r="D41" s="4" t="n">
         <v>-2541</v>
       </c>
-      <c r="D41" s="4" t="n">
+      <c r="E41" s="4" t="n">
         <v>-701</v>
       </c>
-      <c r="E41" s="4" t="n">
+      <c r="F41" s="4" t="n">
+        <v>-2055</v>
+      </c>
+      <c r="G41" s="4" t="n">
         <v>-2363</v>
       </c>
-      <c r="F41" s="4" t="n">
+      <c r="H41" s="4" t="n">
         <v>-338</v>
       </c>
-      <c r="G41" s="4" t="n">
+      <c r="I41" s="4" t="n">
         <v>-3250</v>
       </c>
-      <c r="H41" s="4" t="n">
+      <c r="J41" s="4" t="n">
         <v>-1001</v>
       </c>
-      <c r="I41" s="4" t="n">
+      <c r="K41" s="4" t="n">
         <v>2178</v>
       </c>
-      <c r="J41" s="4" t="n">
+      <c r="L41" s="4" t="n">
         <v>2508</v>
       </c>
     </row>
@@ -5958,27 +6385,33 @@
         <v>-238772</v>
       </c>
       <c r="C42" s="4" t="n">
+        <v>-146118</v>
+      </c>
+      <c r="D42" s="4" t="n">
         <v>-62169</v>
       </c>
-      <c r="D42" s="4" t="n">
+      <c r="E42" s="4" t="n">
         <v>-12053</v>
       </c>
-      <c r="E42" s="4" t="n">
+      <c r="F42" s="4" t="n">
+        <v>58921</v>
+      </c>
+      <c r="G42" s="4" t="n">
         <v>131866</v>
       </c>
-      <c r="F42" s="4" t="n">
+      <c r="H42" s="4" t="n">
         <v>131309</v>
       </c>
-      <c r="G42" s="4" t="n">
+      <c r="I42" s="4" t="n">
         <v>105521</v>
       </c>
-      <c r="H42" s="4" t="n">
+      <c r="J42" s="4" t="n">
         <v>143159</v>
       </c>
-      <c r="I42" s="4" t="n">
+      <c r="K42" s="4" t="n">
         <v>236163</v>
       </c>
-      <c r="J42" s="4" t="n">
+      <c r="L42" s="4" t="n">
         <v>165480</v>
       </c>
     </row>
@@ -5989,39 +6422,47 @@
         </is>
       </c>
       <c r="B43" s="6">
-        <f>SUM(B39:B42)</f>
+        <f>SUM(B38:B42)</f>
         <v/>
       </c>
       <c r="C43" s="6">
-        <f>SUM(C39:C42)</f>
+        <f>SUM(C38:C42)</f>
         <v/>
       </c>
       <c r="D43" s="6">
-        <f>SUM(D39:D42)</f>
+        <f>SUM(D38:D42)</f>
         <v/>
       </c>
       <c r="E43" s="6">
-        <f>SUM(E39:E42)</f>
+        <f>SUM(E38:E42)</f>
         <v/>
       </c>
       <c r="F43" s="6">
-        <f>SUM(F39:F42)</f>
+        <f>SUM(F38:F42)</f>
         <v/>
       </c>
       <c r="G43" s="6">
-        <f>SUM(G39:G42)</f>
+        <f>SUM(G38:G42)</f>
         <v/>
       </c>
       <c r="H43" s="6">
-        <f>SUM(H39:H42)</f>
+        <f>SUM(H38:H42)</f>
         <v/>
       </c>
       <c r="I43" s="6">
-        <f>SUM(I39:I42)</f>
+        <f>SUM(I38:I42)</f>
         <v/>
       </c>
       <c r="J43" s="6">
-        <f>SUM(J39:J42)</f>
+        <f>SUM(J38:J42)</f>
+        <v/>
+      </c>
+      <c r="K43" s="6">
+        <f>SUM(K38:K42)</f>
+        <v/>
+      </c>
+      <c r="L43" s="6">
+        <f>SUM(L38:L42)</f>
         <v/>
       </c>
     </row>
@@ -6032,39 +6473,47 @@
         </is>
       </c>
       <c r="B44" s="6">
-        <f>B37+B38+B43</f>
+        <f>B37+B43</f>
         <v/>
       </c>
       <c r="C44" s="6">
-        <f>C37+C38+C43</f>
+        <f>C37+C43</f>
         <v/>
       </c>
       <c r="D44" s="6">
-        <f>D37+D38+D43</f>
+        <f>D37+D43</f>
         <v/>
       </c>
       <c r="E44" s="6">
-        <f>E37+E38+E43</f>
+        <f>E37+E43</f>
         <v/>
       </c>
       <c r="F44" s="6">
-        <f>F37+F38+F43</f>
+        <f>F37+F43</f>
         <v/>
       </c>
       <c r="G44" s="6">
-        <f>G37+G38+G43</f>
+        <f>G37+G43</f>
         <v/>
       </c>
       <c r="H44" s="6">
-        <f>H37+H38+H43</f>
+        <f>H37+H43</f>
         <v/>
       </c>
       <c r="I44" s="6">
-        <f>I37+I38+I43</f>
+        <f>I37+I43</f>
         <v/>
       </c>
       <c r="J44" s="6">
-        <f>J37+J38+J43</f>
+        <f>J37+J43</f>
+        <v/>
+      </c>
+      <c r="K44" s="6">
+        <f>K37+K43</f>
+        <v/>
+      </c>
+      <c r="L44" s="6">
+        <f>L37+L43</f>
         <v/>
       </c>
     </row>
@@ -6079,7 +6528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6092,51 +6541,63 @@
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
+          <t>Q2 FY2022</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
           <t>Q3 FY2022</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Q1 FY2023</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2023</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2023</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Q1 FY2024</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2024</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2024</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Q1 FY2025</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2025</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2025</t>
         </is>
@@ -6149,30 +6610,36 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
+        <v>15838</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>-166059</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
+        <v>41227</v>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>92736</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="F2" s="4" t="n">
         <v>176685</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="G2" s="4" t="n">
         <v>77811</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="H2" s="4" t="n">
         <v>157594</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="I2" s="4" t="n">
         <v>163950</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="J2" s="4" t="n">
         <v>44419</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>144274</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>83260</v>
       </c>
     </row>
@@ -6183,20 +6650,20 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
+        <v>556</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>952</v>
       </c>
-      <c r="C3" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="D3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>953</v>
+      </c>
+      <c r="F3" s="4" t="n">
         <v>1676</v>
       </c>
-      <c r="E3" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="G3" s="4" t="n">
         <v>0</v>
       </c>
@@ -6207,6 +6674,12 @@
         <v>0</v>
       </c>
       <c r="J3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6217,20 +6690,20 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
+        <v>275</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>402</v>
       </c>
-      <c r="C4" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="D4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>294</v>
+      </c>
+      <c r="F4" s="4" t="n">
         <v>445</v>
       </c>
-      <c r="E4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="G4" s="4" t="n">
         <v>0</v>
       </c>
@@ -6241,6 +6714,12 @@
         <v>0</v>
       </c>
       <c r="J4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6251,11 +6730,11 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>2379</v>
       </c>
-      <c r="C5" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="D5" s="4" t="n">
         <v>0</v>
       </c>
@@ -6275,6 +6754,12 @@
         <v>0</v>
       </c>
       <c r="J5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6288,27 +6773,33 @@
         <v>0</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1247</v>
+        <v>0</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>0</v>
+        <v>549</v>
       </c>
       <c r="E6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="4" t="n">
         <v>1229</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>2648</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>4888</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="J6" s="4" t="n">
         <v>2611</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="K6" s="4" t="n">
         <v>11730</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="L6" s="4" t="n">
         <v>20516</v>
       </c>
     </row>
@@ -6319,30 +6810,36 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
+        <v>466</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>705</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
+        <v>837</v>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>1088</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="F7" s="4" t="n">
         <v>1880</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="G7" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="H7" s="4" t="n">
         <v>4072</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="I7" s="4" t="n">
         <v>4279</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="J7" s="4" t="n">
         <v>2077</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>5529</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="L7" s="4" t="n">
         <v>3226</v>
       </c>
     </row>
@@ -6353,30 +6850,36 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="4" t="n">
         <v>2354</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="D8" s="4" t="n">
+        <v>3531</v>
+      </c>
+      <c r="E8" s="4" t="n">
         <v>7062</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="F8" s="4" t="n">
         <v>10593</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="G8" s="4" t="n">
         <v>3531</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="H8" s="4" t="n">
         <v>7062</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="I8" s="4" t="n">
         <v>10593</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="J8" s="4" t="n">
         <v>3531</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="K8" s="4" t="n">
         <v>7062</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="L8" s="4" t="n">
         <v>13391</v>
       </c>
     </row>
@@ -6387,30 +6890,36 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="C9" s="4" t="n">
         <v>1078</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="D9" s="4" t="n">
+        <v>1672</v>
+      </c>
+      <c r="E9" s="4" t="n">
         <v>-3888</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="F9" s="4" t="n">
         <v>2677</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="G9" s="4" t="n">
         <v>2386</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="H9" s="4" t="n">
         <v>11554</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="I9" s="4" t="n">
         <v>17118</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="J9" s="4" t="n">
         <v>5337</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="K9" s="4" t="n">
         <v>15262</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="L9" s="4" t="n">
         <v>22313</v>
       </c>
     </row>
@@ -6424,27 +6933,33 @@
         <v>0</v>
       </c>
       <c r="C10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="4" t="n">
         <v>191</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="F10" s="4" t="n">
         <v>195</v>
       </c>
-      <c r="E10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="4" t="n">
+      <c r="G10" s="4" t="n">
+        <v>-8</v>
+      </c>
+      <c r="H10" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="I10" s="4" t="n">
         <v>126</v>
       </c>
-      <c r="H10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="J10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6455,30 +6970,36 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
+        <v>8517</v>
+      </c>
+      <c r="C11" s="4" t="n">
         <v>14780</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="D11" s="4" t="n">
+        <v>5507</v>
+      </c>
+      <c r="E11" s="4" t="n">
         <v>11242</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="F11" s="4" t="n">
         <v>16221</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="G11" s="4" t="n">
         <v>3563</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="H11" s="4" t="n">
         <v>8309</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="I11" s="4" t="n">
         <v>13685</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="J11" s="4" t="n">
         <v>5029</v>
       </c>
-      <c r="I11" s="4" t="n">
+      <c r="K11" s="4" t="n">
         <v>11463</v>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="L11" s="4" t="n">
         <v>18847</v>
       </c>
     </row>
@@ -6489,30 +7010,36 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
+        <v>1072</v>
+      </c>
+      <c r="C12" s="4" t="n">
         <v>31329</v>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="D12" s="4" t="n">
+        <v>2873</v>
+      </c>
+      <c r="E12" s="4" t="n">
         <v>-41044</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="F12" s="4" t="n">
         <v>-44303</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="G12" s="4" t="n">
         <v>6450</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>6112</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="I12" s="4" t="n">
         <v>4727</v>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="J12" s="4" t="n">
         <v>269</v>
       </c>
-      <c r="I12" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>-4161</v>
       </c>
-      <c r="J12" s="4" t="n">
+      <c r="L12" s="4" t="n">
         <v>-71408</v>
       </c>
     </row>
@@ -6523,30 +7050,36 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
+        <v>602</v>
+      </c>
+      <c r="C13" s="4" t="n">
         <v>1007</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="D13" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="E13" s="4" t="n">
         <v>206</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="F13" s="4" t="n">
         <v>258</v>
       </c>
-      <c r="E13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="4" t="n">
+      <c r="G13" s="4" t="n">
+        <v>369</v>
+      </c>
+      <c r="H13" s="4" t="n">
         <v>633</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="I13" s="4" t="n">
         <v>356</v>
       </c>
-      <c r="H13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="J13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6578,9 +7111,15 @@
         <v>0</v>
       </c>
       <c r="I14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="4" t="n">
         <v>13800</v>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="L14" s="4" t="n">
         <v>13800</v>
       </c>
     </row>
@@ -6591,30 +7130,36 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="C15" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="D15" s="4" t="n">
+        <v>-4</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="F15" s="4" t="n">
         <v>-2</v>
       </c>
-      <c r="E15" s="4" t="n">
-        <v>361</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="G15" s="4" t="n">
-        <v>0</v>
+        <v>-7672</v>
       </c>
       <c r="H15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="4" t="n">
         <v>-1014</v>
       </c>
-      <c r="I15" s="4" t="n">
+      <c r="K15" s="4" t="n">
         <v>-257</v>
       </c>
-      <c r="J15" s="4" t="n">
+      <c r="L15" s="4" t="n">
         <v>1964</v>
       </c>
     </row>
@@ -6625,30 +7170,36 @@
         </is>
       </c>
       <c r="B16" s="4" t="n">
+        <v>-27920</v>
+      </c>
+      <c r="C16" s="4" t="n">
         <v>-78967</v>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="D16" s="4" t="n">
+        <v>-109639</v>
+      </c>
+      <c r="E16" s="4" t="n">
         <v>-135600</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="F16" s="4" t="n">
         <v>-153271</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="G16" s="4" t="n">
         <v>-18664</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="H16" s="4" t="n">
         <v>-82213</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="I16" s="4" t="n">
         <v>-26529</v>
       </c>
-      <c r="H16" s="4" t="n">
+      <c r="J16" s="4" t="n">
         <v>11841</v>
       </c>
-      <c r="I16" s="4" t="n">
+      <c r="K16" s="4" t="n">
         <v>-143153</v>
       </c>
-      <c r="J16" s="4" t="n">
+      <c r="L16" s="4" t="n">
         <v>-164133</v>
       </c>
     </row>
@@ -6659,30 +7210,36 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
+        <v>28753</v>
+      </c>
+      <c r="C17" s="4" t="n">
         <v>36211</v>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="D17" s="4" t="n">
+        <v>17338</v>
+      </c>
+      <c r="E17" s="4" t="n">
         <v>24632</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="F17" s="4" t="n">
         <v>-28092</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="G17" s="4" t="n">
         <v>29386</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="H17" s="4" t="n">
         <v>37052</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="I17" s="4" t="n">
         <v>14585</v>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="J17" s="4" t="n">
         <v>4794</v>
       </c>
-      <c r="I17" s="4" t="n">
+      <c r="K17" s="4" t="n">
         <v>23039</v>
       </c>
-      <c r="J17" s="4" t="n">
+      <c r="L17" s="4" t="n">
         <v>31132</v>
       </c>
     </row>
@@ -6693,30 +7250,36 @@
         </is>
       </c>
       <c r="B18" s="4" t="n">
+        <v>1257</v>
+      </c>
+      <c r="C18" s="4" t="n">
         <v>1459</v>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="D18" s="4" t="n">
+        <v>-4166</v>
+      </c>
+      <c r="E18" s="4" t="n">
         <v>-12058</v>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="F18" s="4" t="n">
         <v>-12406</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="G18" s="4" t="n">
         <v>-2076</v>
       </c>
-      <c r="F18" s="4" t="n">
+      <c r="H18" s="4" t="n">
         <v>-3469</v>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="I18" s="4" t="n">
         <v>-20261</v>
       </c>
-      <c r="H18" s="4" t="n">
+      <c r="J18" s="4" t="n">
         <v>-3687</v>
       </c>
-      <c r="I18" s="4" t="n">
+      <c r="K18" s="4" t="n">
         <v>-20645</v>
       </c>
-      <c r="J18" s="4" t="n">
+      <c r="L18" s="4" t="n">
         <v>-142920</v>
       </c>
     </row>
@@ -6727,20 +7290,20 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
+        <v>-7176</v>
+      </c>
+      <c r="C19" s="4" t="n">
         <v>-3050</v>
       </c>
-      <c r="C19" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="D19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>-12491</v>
+      </c>
+      <c r="F19" s="4" t="n">
         <v>14652</v>
       </c>
-      <c r="E19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="G19" s="4" t="n">
         <v>0</v>
       </c>
@@ -6751,6 +7314,12 @@
         <v>0</v>
       </c>
       <c r="J19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6761,30 +7330,36 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>0</v>
+        <v>488</v>
       </c>
       <c r="C20" s="4" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="4" t="n">
-        <v>-7695</v>
+        <v>0</v>
       </c>
       <c r="F20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="4" t="n">
         <v>-6362</v>
       </c>
-      <c r="G20" s="4" t="n">
+      <c r="I20" s="4" t="n">
         <v>-5303</v>
       </c>
-      <c r="H20" s="4" t="n">
+      <c r="J20" s="4" t="n">
         <v>-1552</v>
       </c>
-      <c r="I20" s="4" t="n">
+      <c r="K20" s="4" t="n">
         <v>-468</v>
       </c>
-      <c r="J20" s="4" t="n">
+      <c r="L20" s="4" t="n">
         <v>-275</v>
       </c>
     </row>
@@ -6798,27 +7373,33 @@
         <v>0</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>-10209</v>
+        <v>0</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>0</v>
+        <v>-19712</v>
       </c>
       <c r="E21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="4" t="n">
         <v>-3013</v>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="H21" s="4" t="n">
         <v>3950</v>
       </c>
-      <c r="G21" s="4" t="n">
+      <c r="I21" s="4" t="n">
         <v>-12259</v>
       </c>
-      <c r="H21" s="4" t="n">
+      <c r="J21" s="4" t="n">
         <v>11679</v>
       </c>
-      <c r="I21" s="4" t="n">
+      <c r="K21" s="4" t="n">
         <v>20789</v>
       </c>
-      <c r="J21" s="4" t="n">
+      <c r="L21" s="4" t="n">
         <v>4081</v>
       </c>
     </row>
@@ -6832,27 +7413,33 @@
         <v>0</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>-2282</v>
+        <v>0</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>0</v>
+        <v>12643</v>
       </c>
       <c r="E22" s="4" t="n">
-        <v>1750</v>
+        <v>0</v>
       </c>
       <c r="F22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>1998</v>
+      </c>
+      <c r="H22" s="4" t="n">
         <v>17760</v>
       </c>
-      <c r="G22" s="4" t="n">
+      <c r="I22" s="4" t="n">
         <v>11151</v>
       </c>
-      <c r="H22" s="4" t="n">
+      <c r="J22" s="4" t="n">
         <v>-8673</v>
       </c>
-      <c r="I22" s="4" t="n">
+      <c r="K22" s="4" t="n">
         <v>-7013</v>
       </c>
-      <c r="J22" s="4" t="n">
+      <c r="L22" s="4" t="n">
         <v>32961</v>
       </c>
     </row>
@@ -6863,30 +7450,36 @@
         </is>
       </c>
       <c r="B23" s="4" t="n">
+        <v>1820</v>
+      </c>
+      <c r="C23" s="4" t="n">
         <v>32590</v>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="D23" s="4" t="n">
+        <v>8759</v>
+      </c>
+      <c r="E23" s="4" t="n">
         <v>61128</v>
       </c>
-      <c r="D23" s="4" t="n">
+      <c r="F23" s="4" t="n">
         <v>62901</v>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="G23" s="4" t="n">
         <v>10344</v>
       </c>
-      <c r="F23" s="4" t="n">
+      <c r="H23" s="4" t="n">
         <v>-42094</v>
       </c>
-      <c r="G23" s="4" t="n">
+      <c r="I23" s="4" t="n">
         <v>-45537</v>
       </c>
-      <c r="H23" s="4" t="n">
+      <c r="J23" s="4" t="n">
         <v>13705</v>
       </c>
-      <c r="I23" s="4" t="n">
+      <c r="K23" s="4" t="n">
         <v>12927</v>
       </c>
-      <c r="J23" s="4" t="n">
+      <c r="L23" s="4" t="n">
         <v>42433</v>
       </c>
     </row>
@@ -6897,30 +7490,36 @@
         </is>
       </c>
       <c r="B24" s="4" t="n">
+        <v>17512</v>
+      </c>
+      <c r="C24" s="4" t="n">
         <v>24213</v>
       </c>
-      <c r="C24" s="4" t="n">
+      <c r="D24" s="4" t="n">
+        <v>32248</v>
+      </c>
+      <c r="E24" s="4" t="n">
         <v>62995</v>
       </c>
-      <c r="D24" s="4" t="n">
+      <c r="F24" s="4" t="n">
         <v>100580</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="G24" s="4" t="n">
         <v>29414</v>
       </c>
-      <c r="F24" s="4" t="n">
+      <c r="H24" s="4" t="n">
         <v>56692</v>
       </c>
-      <c r="G24" s="4" t="n">
+      <c r="I24" s="4" t="n">
         <v>59023</v>
       </c>
-      <c r="H24" s="4" t="n">
+      <c r="J24" s="4" t="n">
         <v>15379</v>
       </c>
-      <c r="I24" s="4" t="n">
+      <c r="K24" s="4" t="n">
         <v>64221</v>
       </c>
-      <c r="J24" s="4" t="n">
+      <c r="L24" s="4" t="n">
         <v>83276</v>
       </c>
     </row>
@@ -6931,30 +7530,36 @@
         </is>
       </c>
       <c r="B25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="4" t="n">
         <v>115551</v>
       </c>
-      <c r="C25" s="4" t="n">
+      <c r="D25" s="4" t="n">
+        <v>-2923</v>
+      </c>
+      <c r="E25" s="4" t="n">
         <v>-3986</v>
       </c>
-      <c r="D25" s="4" t="n">
+      <c r="F25" s="4" t="n">
         <v>-3986</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="4" t="n">
-        <v>-248</v>
       </c>
       <c r="G25" s="4" t="n">
         <v>-248</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>0</v>
+        <v>-248</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>0</v>
+        <v>-248</v>
       </c>
       <c r="J25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="4" t="n">
         <v>252953</v>
       </c>
     </row>
@@ -6965,30 +7570,36 @@
         </is>
       </c>
       <c r="B26" s="4" t="n">
+        <v>-95</v>
+      </c>
+      <c r="C26" s="4" t="n">
         <v>-126</v>
       </c>
-      <c r="C26" s="4" t="n">
+      <c r="D26" s="4" t="n">
+        <v>-15</v>
+      </c>
+      <c r="E26" s="4" t="n">
         <v>-38</v>
       </c>
-      <c r="D26" s="4" t="n">
+      <c r="F26" s="4" t="n">
         <v>-64</v>
       </c>
-      <c r="E26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="4" t="n">
+      <c r="G26" s="4" t="n">
+        <v>-23</v>
+      </c>
+      <c r="H26" s="4" t="n">
         <v>-34</v>
       </c>
-      <c r="G26" s="4" t="n">
+      <c r="I26" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="H26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="J26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6999,30 +7610,36 @@
         </is>
       </c>
       <c r="B27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="4" t="n">
         <v>154103</v>
       </c>
-      <c r="C27" s="4" t="n">
+      <c r="D27" s="4" t="n">
+        <v>-4625</v>
+      </c>
+      <c r="E27" s="4" t="n">
         <v>-8219</v>
       </c>
-      <c r="D27" s="4" t="n">
+      <c r="F27" s="4" t="n">
         <v>-10593</v>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="G27" s="4" t="n">
         <v>-2378</v>
       </c>
-      <c r="F27" s="4" t="n">
+      <c r="H27" s="4" t="n">
         <v>-4757</v>
       </c>
-      <c r="G27" s="4" t="n">
+      <c r="I27" s="4" t="n">
         <v>-7135</v>
       </c>
-      <c r="H27" s="4" t="n">
+      <c r="J27" s="4" t="n">
         <v>-2378</v>
       </c>
-      <c r="I27" s="4" t="n">
+      <c r="K27" s="4" t="n">
         <v>-7320</v>
       </c>
-      <c r="J27" s="4" t="n">
+      <c r="L27" s="4" t="n">
         <v>233463</v>
       </c>
     </row>
@@ -7068,6 +7685,14 @@
         <f>SUM(J2:J27)</f>
         <v/>
       </c>
+      <c r="K28" s="6">
+        <f>SUM(K2:K27)</f>
+        <v/>
+      </c>
+      <c r="L28" s="6">
+        <f>SUM(L2:L27)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -7079,16 +7704,16 @@
         <v>2592</v>
       </c>
       <c r="C29" s="4" t="n">
-        <v>3233</v>
+        <v>2592</v>
       </c>
       <c r="D29" s="4" t="n">
         <v>3233</v>
       </c>
       <c r="E29" s="4" t="n">
-        <v>0</v>
+        <v>3233</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>0</v>
+        <v>3233</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>0</v>
@@ -7100,6 +7725,12 @@
         <v>0</v>
       </c>
       <c r="J29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7110,30 +7741,36 @@
         </is>
       </c>
       <c r="B30" s="4" t="n">
+        <v>-2456</v>
+      </c>
+      <c r="C30" s="4" t="n">
         <v>-3477</v>
       </c>
-      <c r="C30" s="4" t="n">
+      <c r="D30" s="4" t="n">
+        <v>-2253</v>
+      </c>
+      <c r="E30" s="4" t="n">
         <v>-6810</v>
       </c>
-      <c r="D30" s="4" t="n">
+      <c r="F30" s="4" t="n">
         <v>-12687</v>
       </c>
-      <c r="E30" s="4" t="n">
+      <c r="G30" s="4" t="n">
         <v>-4525</v>
       </c>
-      <c r="F30" s="4" t="n">
+      <c r="H30" s="4" t="n">
         <v>-13739</v>
       </c>
-      <c r="G30" s="4" t="n">
+      <c r="I30" s="4" t="n">
         <v>-17983</v>
       </c>
-      <c r="H30" s="4" t="n">
+      <c r="J30" s="4" t="n">
         <v>-6944</v>
       </c>
-      <c r="I30" s="4" t="n">
+      <c r="K30" s="4" t="n">
         <v>-15194</v>
       </c>
-      <c r="J30" s="4" t="n">
+      <c r="L30" s="4" t="n">
         <v>-25539</v>
       </c>
     </row>
@@ -7159,15 +7796,21 @@
         <v>0</v>
       </c>
       <c r="G31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="4" t="n">
         <v>-3000</v>
       </c>
-      <c r="H31" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I31" s="4" t="n">
+      <c r="J31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="4" t="n">
         <v>-5000</v>
       </c>
-      <c r="J31" s="4" t="n">
+      <c r="L31" s="4" t="n">
         <v>-5000</v>
       </c>
     </row>
@@ -7199,9 +7842,15 @@
         <v>0</v>
       </c>
       <c r="I32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="4" t="n">
         <v>-1256351</v>
       </c>
-      <c r="J32" s="4" t="n">
+      <c r="L32" s="4" t="n">
         <v>-1278769</v>
       </c>
     </row>
@@ -7236,6 +7885,12 @@
         <v>0</v>
       </c>
       <c r="J33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="4" t="n">
         <v>30617</v>
       </c>
     </row>
@@ -7281,6 +7936,14 @@
         <f>SUM(J29:J33)</f>
         <v/>
       </c>
+      <c r="K34" s="6">
+        <f>SUM(K29:K33)</f>
+        <v/>
+      </c>
+      <c r="L34" s="6">
+        <f>SUM(L29:L33)</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -7289,30 +7952,36 @@
         </is>
       </c>
       <c r="B35" s="4" t="n">
+        <v>-37</v>
+      </c>
+      <c r="C35" s="4" t="n">
         <v>-49</v>
       </c>
-      <c r="C35" s="4" t="n">
+      <c r="D35" s="4" t="n">
+        <v>-11</v>
+      </c>
+      <c r="E35" s="4" t="n">
         <v>-22</v>
       </c>
-      <c r="D35" s="4" t="n">
+      <c r="F35" s="4" t="n">
         <v>-33</v>
       </c>
-      <c r="E35" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="4" t="n">
+      <c r="G35" s="4" t="n">
+        <v>-15</v>
+      </c>
+      <c r="H35" s="4" t="n">
         <v>-30</v>
       </c>
-      <c r="G35" s="4" t="n">
+      <c r="I35" s="4" t="n">
         <v>-46</v>
       </c>
-      <c r="H35" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I35" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="J35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7323,30 +7992,36 @@
         </is>
       </c>
       <c r="B36" s="4" t="n">
+        <v>1260</v>
+      </c>
+      <c r="C36" s="4" t="n">
         <v>3104</v>
       </c>
-      <c r="C36" s="4" t="n">
+      <c r="D36" s="4" t="n">
+        <v>478</v>
+      </c>
+      <c r="E36" s="4" t="n">
         <v>707</v>
       </c>
-      <c r="D36" s="4" t="n">
+      <c r="F36" s="4" t="n">
         <v>1603</v>
       </c>
-      <c r="E36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" s="4" t="n">
+      <c r="G36" s="4" t="n">
+        <v>967</v>
+      </c>
+      <c r="H36" s="4" t="n">
         <v>1147</v>
       </c>
-      <c r="G36" s="4" t="n">
+      <c r="I36" s="4" t="n">
         <v>3832</v>
       </c>
-      <c r="H36" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I36" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="J36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7357,11 +8032,11 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="4" t="n">
         <v>542018</v>
       </c>
-      <c r="C37" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="D37" s="4" t="n">
         <v>0</v>
       </c>
@@ -7381,6 +8056,12 @@
         <v>0</v>
       </c>
       <c r="J37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7391,30 +8072,36 @@
         </is>
       </c>
       <c r="B38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C38" s="4" t="n">
         <v>-4596</v>
       </c>
-      <c r="C38" s="4" t="n">
+      <c r="D38" s="4" t="n">
+        <v>-6781</v>
+      </c>
+      <c r="E38" s="4" t="n">
         <v>-13637</v>
       </c>
-      <c r="D38" s="4" t="n">
+      <c r="F38" s="4" t="n">
         <v>-20512</v>
       </c>
-      <c r="E38" s="4" t="n">
+      <c r="G38" s="4" t="n">
         <v>-6837</v>
       </c>
-      <c r="F38" s="4" t="n">
+      <c r="H38" s="4" t="n">
         <v>-13675</v>
       </c>
-      <c r="G38" s="4" t="n">
+      <c r="I38" s="4" t="n">
         <v>-20588</v>
       </c>
-      <c r="H38" s="4" t="n">
+      <c r="J38" s="4" t="n">
         <v>-6781</v>
       </c>
-      <c r="I38" s="4" t="n">
+      <c r="K38" s="4" t="n">
         <v>-13632</v>
       </c>
-      <c r="J38" s="4" t="n">
+      <c r="L38" s="4" t="n">
         <v>-23301</v>
       </c>
     </row>
@@ -7440,15 +8127,21 @@
         <v>0</v>
       </c>
       <c r="G39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="4" t="n">
         <v>-1658</v>
       </c>
-      <c r="H39" s="4" t="n">
+      <c r="J39" s="4" t="n">
         <v>-1932</v>
       </c>
-      <c r="I39" s="4" t="n">
+      <c r="K39" s="4" t="n">
         <v>-2811</v>
       </c>
-      <c r="J39" s="4" t="n">
+      <c r="L39" s="4" t="n">
         <v>-3259</v>
       </c>
     </row>
@@ -7480,9 +8173,15 @@
         <v>0</v>
       </c>
       <c r="I40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="4" t="n">
         <v>900000</v>
       </c>
-      <c r="J40" s="4" t="n">
+      <c r="L40" s="4" t="n">
         <v>900000</v>
       </c>
     </row>
@@ -7517,6 +8216,12 @@
         <v>0</v>
       </c>
       <c r="J41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="4" t="n">
         <v>-2250</v>
       </c>
     </row>
@@ -7545,12 +8250,18 @@
         <v>0</v>
       </c>
       <c r="H42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="4" t="n">
         <v>-2195</v>
       </c>
-      <c r="I42" s="4" t="n">
+      <c r="K42" s="4" t="n">
         <v>-31581</v>
       </c>
-      <c r="J42" s="4" t="n">
+      <c r="L42" s="4" t="n">
         <v>-31581</v>
       </c>
     </row>
@@ -7570,7 +8281,7 @@
         <v>0</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>952</v>
+        <v>0</v>
       </c>
       <c r="F43" s="4" t="n">
         <v>0</v>
@@ -7579,12 +8290,18 @@
         <v>0</v>
       </c>
       <c r="H43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" s="4" t="n">
         <v>321</v>
       </c>
-      <c r="I43" s="4" t="n">
+      <c r="K43" s="4" t="n">
         <v>319</v>
       </c>
-      <c r="J43" s="4" t="n">
+      <c r="L43" s="4" t="n">
         <v>301</v>
       </c>
     </row>
@@ -7630,6 +8347,14 @@
         <f>SUM(J35:J43)</f>
         <v/>
       </c>
+      <c r="K44" s="6">
+        <f>SUM(K35:K43)</f>
+        <v/>
+      </c>
+      <c r="L44" s="6">
+        <f>SUM(L35:L43)</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -7638,31 +8363,88 @@
         </is>
       </c>
       <c r="B45" s="4" t="n">
+        <v>121</v>
+      </c>
+      <c r="C45" s="4" t="n">
         <v>158</v>
       </c>
-      <c r="C45" s="4" t="n">
+      <c r="D45" s="4" t="n">
+        <v>-181</v>
+      </c>
+      <c r="E45" s="4" t="n">
         <v>-555</v>
       </c>
-      <c r="D45" s="4" t="n">
+      <c r="F45" s="4" t="n">
         <v>-555</v>
       </c>
-      <c r="E45" s="4" t="n">
+      <c r="G45" s="4" t="n">
         <v>-722</v>
       </c>
-      <c r="F45" s="4" t="n">
+      <c r="H45" s="4" t="n">
         <v>-766</v>
       </c>
-      <c r="G45" s="4" t="n">
+      <c r="I45" s="4" t="n">
         <v>-16</v>
       </c>
-      <c r="H45" s="4" t="n">
+      <c r="J45" s="4" t="n">
         <v>1259</v>
       </c>
-      <c r="I45" s="4" t="n">
+      <c r="K45" s="4" t="n">
         <v>2214</v>
       </c>
-      <c r="J45" s="4" t="n">
+      <c r="L45" s="4" t="n">
         <v>2174</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Net Change in Cash</t>
+        </is>
+      </c>
+      <c r="B46" s="6">
+        <f>B28+B34+B44+B45</f>
+        <v/>
+      </c>
+      <c r="C46" s="6">
+        <f>C28+C34+C44+C45</f>
+        <v/>
+      </c>
+      <c r="D46" s="6">
+        <f>D28+D34+D44+D45</f>
+        <v/>
+      </c>
+      <c r="E46" s="6">
+        <f>E28+E34+E44+E45</f>
+        <v/>
+      </c>
+      <c r="F46" s="6">
+        <f>F28+F34+F44+F45</f>
+        <v/>
+      </c>
+      <c r="G46" s="6">
+        <f>G28+G34+G44+G45</f>
+        <v/>
+      </c>
+      <c r="H46" s="6">
+        <f>H28+H34+H44+H45</f>
+        <v/>
+      </c>
+      <c r="I46" s="6">
+        <f>I28+I34+I44+I45</f>
+        <v/>
+      </c>
+      <c r="J46" s="6">
+        <f>J28+J34+J44+J45</f>
+        <v/>
+      </c>
+      <c r="K46" s="6">
+        <f>K28+K34+K44+K45</f>
+        <v/>
+      </c>
+      <c r="L46" s="6">
+        <f>L28+L34+L44+L45</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
vault backup: 2026-04-26 16:43:04
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model.xlsx
@@ -683,7 +683,7 @@
         <v>0</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>327461</v>
+        <v>-327461</v>
       </c>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n"/>
@@ -3886,7 +3886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:M17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3901,61 +3901,67 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
+          <t>Q1 FY2022</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
           <t>Q2 FY2022</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2022</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Q1 FY2023</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2023</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2023</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Q1 FY2024</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2024</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2024</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Q1 FY2025</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2025</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2025</t>
         </is>
@@ -3968,36 +3974,39 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
+        <v>133388</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>287408</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>475640</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="E2" s="4" t="n">
         <v>259939</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="F2" s="4" t="n">
         <v>585822</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="G2" s="4" t="n">
         <v>970579</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="H2" s="4" t="n">
         <v>355708</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="I2" s="4" t="n">
         <v>757685</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="J2" s="4" t="n">
         <v>1023433</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>329276</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>1068535</v>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="M2" s="4" t="n">
         <v>1793641</v>
       </c>
     </row>
@@ -4008,36 +4017,39 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
+        <v>-79494</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>-174195</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>-283778</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="E3" s="4" t="n">
         <v>-146121</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="F3" s="4" t="n">
         <v>-313010</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="G3" s="4" t="n">
         <v>-503685</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="H3" s="4" t="n">
         <v>-173501</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="I3" s="4" t="n">
         <v>-366380</v>
       </c>
-      <c r="I3" s="4" t="n">
+      <c r="J3" s="4" t="n">
         <v>-509899</v>
       </c>
-      <c r="J3" s="4" t="n">
+      <c r="K3" s="4" t="n">
         <v>-156903</v>
       </c>
-      <c r="K3" s="4" t="n">
+      <c r="L3" s="4" t="n">
         <v>-515311</v>
       </c>
-      <c r="L3" s="4" t="n">
+      <c r="M3" s="4" t="n">
         <v>-868138</v>
       </c>
     </row>
@@ -4091,6 +4103,10 @@
         <f>L2+L3</f>
         <v/>
       </c>
+      <c r="M4" s="6">
+        <f>M2+M3</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -4099,36 +4115,39 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
+        <v>-43778</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>-90667</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="D5" s="4" t="n">
         <v>-316917</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="E5" s="4" t="n">
         <v>-68905</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>-163086</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="G5" s="4" t="n">
         <v>-259471</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>-99017</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="I5" s="4" t="n">
         <v>-213867</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="J5" s="4" t="n">
         <v>-339310</v>
       </c>
-      <c r="J5" s="4" t="n">
+      <c r="K5" s="4" t="n">
         <v>-120342</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="L5" s="4" t="n">
         <v>-358228</v>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="M5" s="4" t="n">
         <v>-563799</v>
       </c>
     </row>
@@ -4169,7 +4188,10 @@
         <v>0</v>
       </c>
       <c r="L6" s="4" t="n">
-        <v>246707</v>
+        <v>0</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>-246707</v>
       </c>
     </row>
     <row r="7">
@@ -4222,6 +4244,10 @@
         <f>L4+SUM(L5:L6)</f>
         <v/>
       </c>
+      <c r="M7" s="6">
+        <f>M4+SUM(M5:M6)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -4230,36 +4256,39 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="C8" s="4" t="n">
         <v>129</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="D8" s="4" t="n">
         <v>1579</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="E8" s="4" t="n">
         <v>4969</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="F8" s="4" t="n">
         <v>10542</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="G8" s="4" t="n">
         <v>17767</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="H8" s="4" t="n">
         <v>9640</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="I8" s="4" t="n">
         <v>20287</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="J8" s="4" t="n">
         <v>31399</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="K8" s="4" t="n">
         <v>7846</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="L8" s="4" t="n">
         <v>-6196</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="M8" s="4" t="n">
         <v>-19592</v>
       </c>
     </row>
@@ -4270,36 +4299,39 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
+        <v>-162</v>
+      </c>
+      <c r="C9" s="4" t="n">
         <v>-676</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="D9" s="4" t="n">
         <v>-930</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="E9" s="4" t="n">
         <v>-118</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="F9" s="4" t="n">
         <v>-1049</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="G9" s="4" t="n">
         <v>-1226</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="H9" s="4" t="n">
         <v>-369</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="I9" s="4" t="n">
         <v>-633</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="J9" s="4" t="n">
         <v>-356</v>
       </c>
-      <c r="J9" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="K9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4334,12 +4366,15 @@
         <v>0</v>
       </c>
       <c r="J10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="4" t="n">
         <v>1116</v>
       </c>
-      <c r="K10" s="4" t="n">
+      <c r="L10" s="4" t="n">
         <v>1658</v>
       </c>
-      <c r="L10" s="4" t="n">
+      <c r="M10" s="4" t="n">
         <v>7022</v>
       </c>
     </row>
@@ -4393,6 +4428,10 @@
         <f>L7+SUM(L8:L10)</f>
         <v/>
       </c>
+      <c r="M11" s="6">
+        <f>M7+SUM(M8:M10)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -4401,36 +4440,39 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
+        <v>-3351</v>
+      </c>
+      <c r="C12" s="4" t="n">
         <v>-6161</v>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="D12" s="4" t="n">
         <v>-41653</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="E12" s="4" t="n">
         <v>-8537</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="F12" s="4" t="n">
         <v>-26483</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="G12" s="4" t="n">
         <v>-47279</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>-14650</v>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="I12" s="4" t="n">
         <v>-39498</v>
       </c>
-      <c r="I12" s="4" t="n">
+      <c r="J12" s="4" t="n">
         <v>-41317</v>
       </c>
-      <c r="J12" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>-16574</v>
       </c>
-      <c r="K12" s="4" t="n">
+      <c r="L12" s="4" t="n">
         <v>-46184</v>
       </c>
-      <c r="L12" s="4" t="n">
+      <c r="M12" s="4" t="n">
         <v>-19167</v>
       </c>
     </row>
@@ -4484,6 +4526,10 @@
         <f>L11+L12</f>
         <v/>
       </c>
+      <c r="M13" s="6">
+        <f>M11+M12</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -4492,36 +4538,39 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
+        <v>6679</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>15838</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="D14" s="4" t="n">
         <v>-166059</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E14" s="4" t="n">
         <v>41227</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>92736</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="G14" s="4" t="n">
         <v>176685</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>77811</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="I14" s="4" t="n">
         <v>157594</v>
       </c>
-      <c r="I14" s="4" t="n">
+      <c r="J14" s="4" t="n">
         <v>163950</v>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="K14" s="4" t="n">
         <v>44419</v>
       </c>
-      <c r="K14" s="4" t="n">
+      <c r="L14" s="4" t="n">
         <v>144274</v>
       </c>
-      <c r="L14" s="4" t="n">
+      <c r="M14" s="4" t="n">
         <v>83260</v>
       </c>
     </row>
@@ -4535,33 +4584,36 @@
         <v>0</v>
       </c>
       <c r="C15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="4" t="n">
         <v>-4596</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="E15" s="4" t="n">
         <v>-6781</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="F15" s="4" t="n">
         <v>-13637</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="G15" s="4" t="n">
         <v>-20512</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="H15" s="4" t="n">
         <v>-6837</v>
       </c>
-      <c r="H15" s="4" t="n">
+      <c r="I15" s="4" t="n">
         <v>-13675</v>
       </c>
-      <c r="I15" s="4" t="n">
+      <c r="J15" s="4" t="n">
         <v>-20588</v>
       </c>
-      <c r="J15" s="4" t="n">
+      <c r="K15" s="4" t="n">
         <v>-6781</v>
       </c>
-      <c r="K15" s="4" t="n">
+      <c r="L15" s="4" t="n">
         <v>-13632</v>
       </c>
-      <c r="L15" s="4" t="n">
+      <c r="M15" s="4" t="n">
         <v>-23289</v>
       </c>
     </row>
@@ -4578,30 +4630,33 @@
         <v>0</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>2934</v>
+        <v>0</v>
       </c>
       <c r="E16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="4" t="n">
         <v>6727</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="G16" s="4" t="n">
         <v>13263</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="H16" s="4" t="n">
         <v>6128</v>
       </c>
-      <c r="H16" s="4" t="n">
+      <c r="I16" s="4" t="n">
         <v>12417</v>
       </c>
-      <c r="I16" s="4" t="n">
+      <c r="J16" s="4" t="n">
         <v>12357</v>
       </c>
-      <c r="J16" s="4" t="n">
+      <c r="K16" s="4" t="n">
         <v>3219</v>
       </c>
-      <c r="K16" s="4" t="n">
+      <c r="L16" s="4" t="n">
         <v>10703</v>
       </c>
-      <c r="L16" s="4" t="n">
+      <c r="M16" s="4" t="n">
         <v>5272</v>
       </c>
     </row>
@@ -4612,36 +4667,39 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
+        <v>6679</v>
+      </c>
+      <c r="C17" s="4" t="n">
         <v>15838</v>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="D17" s="4" t="n">
         <v>-170655</v>
       </c>
-      <c r="D17" s="4" t="n">
-        <v>31512</v>
-      </c>
       <c r="E17" s="4" t="n">
+        <v>34446</v>
+      </c>
+      <c r="F17" s="4" t="n">
         <v>72372</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="G17" s="4" t="n">
         <v>142910</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="H17" s="4" t="n">
         <v>64846</v>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="I17" s="4" t="n">
         <v>131502</v>
       </c>
-      <c r="I17" s="4" t="n">
+      <c r="J17" s="4" t="n">
         <v>131005</v>
       </c>
-      <c r="J17" s="4" t="n">
+      <c r="K17" s="4" t="n">
         <v>34419</v>
       </c>
-      <c r="K17" s="4" t="n">
+      <c r="L17" s="4" t="n">
         <v>119939</v>
       </c>
-      <c r="L17" s="4" t="n">
+      <c r="M17" s="4" t="n">
         <v>54699</v>
       </c>
     </row>
@@ -4656,7 +4714,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -4671,6 +4729,7 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4682,50 +4741,55 @@
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
+          <t>Q1 FY2023</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
           <t>Q2 FY2023</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2023</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Q4 FY2023</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Q1 FY2024</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2024</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2024</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Q4 FY2024</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Q1 FY2025</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2025</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2025</t>
         </is>
@@ -4741,33 +4805,36 @@
         <v>614159</v>
       </c>
       <c r="C2" s="4" t="n">
+        <v>595476</v>
+      </c>
+      <c r="D2" s="4" t="n">
         <v>681054</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="E2" s="4" t="n">
         <v>760022</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="F2" s="4" t="n">
         <v>755981</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="G2" s="4" t="n">
         <v>879498</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="H2" s="4" t="n">
         <v>903210</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="I2" s="4" t="n">
         <v>903748</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="J2" s="4" t="n">
         <v>890190</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>977285</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>615233</v>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="M2" s="4" t="n">
         <v>805955</v>
       </c>
     </row>
@@ -4781,7 +4848,7 @@
         <v>38768</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>0</v>
+        <v>38105</v>
       </c>
       <c r="D3" s="4" t="n">
         <v>0</v>
@@ -4808,6 +4875,9 @@
         <v>0</v>
       </c>
       <c r="L3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="4" t="n">
         <v>126508</v>
       </c>
     </row>
@@ -4821,33 +4891,36 @@
         <v>63311</v>
       </c>
       <c r="C4" s="4" t="n">
+        <v>172032</v>
+      </c>
+      <c r="D4" s="4" t="n">
         <v>197811</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="E4" s="4" t="n">
         <v>215243</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="F4" s="4" t="n">
         <v>183703</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="G4" s="4" t="n">
         <v>200117</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="H4" s="4" t="n">
         <v>262920</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="I4" s="4" t="n">
         <v>208774</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="J4" s="4" t="n">
         <v>270342</v>
       </c>
-      <c r="J4" s="4" t="n">
+      <c r="K4" s="4" t="n">
         <v>256424</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="L4" s="4" t="n">
         <v>490389</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="M4" s="4" t="n">
         <v>513682</v>
       </c>
     </row>
@@ -4861,26 +4934,26 @@
         <v>2979</v>
       </c>
       <c r="C5" s="4" t="n">
+        <v>3587</v>
+      </c>
+      <c r="D5" s="4" t="n">
         <v>3323</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="E5" s="4" t="n">
         <v>3309</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="F5" s="4" t="n">
         <v>2318</v>
       </c>
-      <c r="F5" s="4" t="n">
+      <c r="G5" s="4" t="n">
         <v>2259</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="H5" s="4" t="n">
         <v>1166</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="I5" s="4" t="n">
         <v>1025</v>
       </c>
-      <c r="I5" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="J5" s="4" t="n">
         <v>0</v>
       </c>
@@ -4888,6 +4961,9 @@
         <v>0</v>
       </c>
       <c r="L5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -4901,33 +4977,36 @@
         <v>173289</v>
       </c>
       <c r="C6" s="4" t="n">
+        <v>154280</v>
+      </c>
+      <c r="D6" s="4" t="n">
         <v>152545</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="E6" s="4" t="n">
         <v>198704</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="F6" s="4" t="n">
         <v>229275</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="G6" s="4" t="n">
         <v>197504</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="H6" s="4" t="n">
         <v>180669</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>197572</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="J6" s="4" t="n">
         <v>131165</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="K6" s="4" t="n">
         <v>141159</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="L6" s="4" t="n">
         <v>230046</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="M6" s="4" t="n">
         <v>282514</v>
       </c>
     </row>
@@ -4941,33 +5020,36 @@
         <v>11341</v>
       </c>
       <c r="C7" s="4" t="n">
+        <v>15507</v>
+      </c>
+      <c r="D7" s="4" t="n">
         <v>23398</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="E7" s="4" t="n">
         <v>23747</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="F7" s="4" t="n">
         <v>19503</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="G7" s="4" t="n">
         <v>21523</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="H7" s="4" t="n">
         <v>22900</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="I7" s="4" t="n">
         <v>38227</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="J7" s="4" t="n">
         <v>18759</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>22464</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="L7" s="4" t="n">
         <v>41420</v>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="M7" s="4" t="n">
         <v>163395</v>
       </c>
     </row>
@@ -5008,6 +5090,9 @@
         <v>14124</v>
       </c>
       <c r="L8" s="4" t="n">
+        <v>14124</v>
+      </c>
+      <c r="M8" s="4" t="n">
         <v>49520</v>
       </c>
     </row>
@@ -5061,6 +5146,10 @@
         <f>SUM(L2:L8)</f>
         <v/>
       </c>
+      <c r="M9" s="6">
+        <f>SUM(M2:M8)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -5101,6 +5190,9 @@
       <c r="L10" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="M10" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -5112,33 +5204,36 @@
         <v>10185</v>
       </c>
       <c r="C11" s="4" t="n">
+        <v>12054</v>
+      </c>
+      <c r="D11" s="4" t="n">
         <v>15892</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="E11" s="4" t="n">
         <v>21061</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="F11" s="4" t="n">
         <v>24868</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="G11" s="4" t="n">
         <v>28350</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="H11" s="4" t="n">
         <v>36282</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="I11" s="4" t="n">
         <v>38370</v>
       </c>
-      <c r="I11" s="4" t="n">
+      <c r="J11" s="4" t="n">
         <v>55602</v>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="K11" s="4" t="n">
         <v>58698</v>
       </c>
-      <c r="K11" s="4" t="n">
+      <c r="L11" s="4" t="n">
         <v>72516</v>
       </c>
-      <c r="L11" s="4" t="n">
+      <c r="M11" s="4" t="n">
         <v>80925</v>
       </c>
     </row>
@@ -5152,33 +5247,36 @@
         <v>972</v>
       </c>
       <c r="C12" s="4" t="n">
+        <v>931</v>
+      </c>
+      <c r="D12" s="4" t="n">
         <v>756</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="E12" s="4" t="n">
         <v>1152</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="F12" s="4" t="n">
         <v>1957</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="G12" s="4" t="n">
         <v>1688</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>1507</v>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="I12" s="4" t="n">
         <v>5506</v>
       </c>
-      <c r="I12" s="4" t="n">
+      <c r="J12" s="4" t="n">
         <v>21606</v>
       </c>
-      <c r="J12" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>20866</v>
       </c>
-      <c r="K12" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="L12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5192,33 +5290,36 @@
         <v>12254</v>
       </c>
       <c r="C13" s="4" t="n">
+        <v>12359</v>
+      </c>
+      <c r="D13" s="4" t="n">
         <v>12211</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="E13" s="4" t="n">
         <v>11772</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="F13" s="4" t="n">
         <v>12139</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="G13" s="4" t="n">
         <v>11741</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="H13" s="4" t="n">
         <v>11491</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="I13" s="4" t="n">
         <v>11877</v>
       </c>
-      <c r="I13" s="4" t="n">
+      <c r="J13" s="4" t="n">
         <v>12213</v>
       </c>
-      <c r="J13" s="4" t="n">
+      <c r="K13" s="4" t="n">
         <v>12444</v>
       </c>
-      <c r="K13" s="4" t="n">
+      <c r="L13" s="4" t="n">
         <v>1222115</v>
       </c>
-      <c r="L13" s="4" t="n">
+      <c r="M13" s="4" t="n">
         <v>1397819</v>
       </c>
     </row>
@@ -5232,33 +5333,36 @@
         <v>13679</v>
       </c>
       <c r="C14" s="4" t="n">
+        <v>13949</v>
+      </c>
+      <c r="D14" s="4" t="n">
         <v>13937</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E14" s="4" t="n">
         <v>13588</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>14173</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="G14" s="4" t="n">
         <v>13866</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>13730</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="I14" s="4" t="n">
         <v>14360</v>
       </c>
-      <c r="I14" s="4" t="n">
+      <c r="J14" s="4" t="n">
         <v>71582</v>
       </c>
-      <c r="J14" s="4" t="n">
+      <c r="K14" s="4" t="n">
         <v>72128</v>
       </c>
-      <c r="K14" s="4" t="n">
+      <c r="L14" s="4" t="n">
         <v>802234</v>
       </c>
-      <c r="L14" s="4" t="n">
+      <c r="M14" s="4" t="n">
         <v>914957</v>
       </c>
     </row>
@@ -5272,33 +5376,36 @@
         <v>262462</v>
       </c>
       <c r="C15" s="4" t="n">
+        <v>258931</v>
+      </c>
+      <c r="D15" s="4" t="n">
         <v>255400</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="E15" s="4" t="n">
         <v>251869</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="F15" s="4" t="n">
         <v>248338</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="G15" s="4" t="n">
         <v>244807</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="H15" s="4" t="n">
         <v>241276</v>
       </c>
-      <c r="H15" s="4" t="n">
+      <c r="I15" s="4" t="n">
         <v>237746</v>
       </c>
-      <c r="I15" s="4" t="n">
+      <c r="J15" s="4" t="n">
         <v>234215</v>
       </c>
-      <c r="J15" s="4" t="n">
+      <c r="K15" s="4" t="n">
         <v>230684</v>
       </c>
-      <c r="K15" s="4" t="n">
+      <c r="L15" s="4" t="n">
         <v>227153</v>
       </c>
-      <c r="L15" s="4" t="n">
+      <c r="M15" s="4" t="n">
         <v>784214</v>
       </c>
     </row>
@@ -5312,33 +5419,36 @@
         <v>501</v>
       </c>
       <c r="C16" s="4" t="n">
+        <v>482</v>
+      </c>
+      <c r="D16" s="4" t="n">
         <v>28373</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="E16" s="4" t="n">
         <v>30614</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="F16" s="4" t="n">
         <v>29518</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="G16" s="4" t="n">
         <v>22437</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="H16" s="4" t="n">
         <v>22727</v>
       </c>
-      <c r="H16" s="4" t="n">
+      <c r="I16" s="4" t="n">
         <v>24186</v>
       </c>
-      <c r="I16" s="4" t="n">
+      <c r="J16" s="4" t="n">
         <v>38699</v>
       </c>
-      <c r="J16" s="4" t="n">
+      <c r="K16" s="4" t="n">
         <v>38525</v>
       </c>
-      <c r="K16" s="4" t="n">
+      <c r="L16" s="4" t="n">
         <v>43158</v>
       </c>
-      <c r="L16" s="4" t="n">
+      <c r="M16" s="4" t="n">
         <v>110410</v>
       </c>
     </row>
@@ -5352,26 +5462,26 @@
         <v>208</v>
       </c>
       <c r="C17" s="4" t="n">
+        <v>191</v>
+      </c>
+      <c r="D17" s="4" t="n">
         <v>171</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="E17" s="4" t="n">
         <v>148</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="F17" s="4" t="n">
         <v>208</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="G17" s="4" t="n">
         <v>263</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="H17" s="4" t="n">
         <v>233</v>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="I17" s="4" t="n">
         <v>214</v>
       </c>
-      <c r="I17" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="J17" s="4" t="n">
         <v>0</v>
       </c>
@@ -5379,6 +5489,9 @@
         <v>0</v>
       </c>
       <c r="L17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5392,33 +5505,36 @@
         <v>263</v>
       </c>
       <c r="C18" s="4" t="n">
+        <v>263</v>
+      </c>
+      <c r="D18" s="4" t="n">
         <v>254</v>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="E18" s="4" t="n">
         <v>265</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="F18" s="4" t="n">
         <v>291</v>
       </c>
-      <c r="F18" s="4" t="n">
+      <c r="G18" s="4" t="n">
         <v>7963</v>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="H18" s="4" t="n">
         <v>6653</v>
       </c>
-      <c r="H18" s="4" t="n">
+      <c r="I18" s="4" t="n">
         <v>8594</v>
       </c>
-      <c r="I18" s="4" t="n">
+      <c r="J18" s="4" t="n">
         <v>8384</v>
       </c>
-      <c r="J18" s="4" t="n">
+      <c r="K18" s="4" t="n">
         <v>14717</v>
       </c>
-      <c r="K18" s="4" t="n">
+      <c r="L18" s="4" t="n">
         <v>36755</v>
       </c>
-      <c r="L18" s="4" t="n">
+      <c r="M18" s="4" t="n">
         <v>35809</v>
       </c>
     </row>
@@ -5472,6 +5588,10 @@
         <f>L9+SUM(L10:L18)</f>
         <v/>
       </c>
+      <c r="M19" s="6">
+        <f>M9+SUM(M10:M18)</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -5480,36 +5600,39 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
-        <v>106147</v>
+        <v>107340</v>
       </c>
       <c r="C20" s="4" t="n">
+        <v>107112</v>
+      </c>
+      <c r="D20" s="4" t="n">
         <v>94313</v>
       </c>
-      <c r="D20" s="4" t="n">
+      <c r="E20" s="4" t="n">
         <v>121088</v>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="F20" s="4" t="n">
         <v>42840</v>
       </c>
-      <c r="F20" s="4" t="n">
+      <c r="G20" s="4" t="n">
         <v>40196</v>
       </c>
-      <c r="G20" s="4" t="n">
+      <c r="H20" s="4" t="n">
         <v>47423</v>
       </c>
-      <c r="H20" s="4" t="n">
+      <c r="I20" s="4" t="n">
         <v>30938</v>
       </c>
-      <c r="I20" s="4" t="n">
+      <c r="J20" s="4" t="n">
         <v>41287</v>
       </c>
-      <c r="J20" s="4" t="n">
+      <c r="K20" s="4" t="n">
         <v>61052</v>
       </c>
-      <c r="K20" s="4" t="n">
+      <c r="L20" s="4" t="n">
         <v>120962</v>
       </c>
-      <c r="L20" s="4" t="n">
+      <c r="M20" s="4" t="n">
         <v>97794</v>
       </c>
     </row>
@@ -5529,27 +5652,30 @@
         <v>0</v>
       </c>
       <c r="E21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="4" t="n">
         <v>62120</v>
       </c>
-      <c r="F21" s="4" t="n">
+      <c r="G21" s="4" t="n">
         <v>63871</v>
       </c>
-      <c r="G21" s="4" t="n">
+      <c r="H21" s="4" t="n">
         <v>79633</v>
       </c>
-      <c r="H21" s="4" t="n">
+      <c r="I21" s="4" t="n">
         <v>73024</v>
       </c>
-      <c r="I21" s="4" t="n">
+      <c r="J21" s="4" t="n">
         <v>148780</v>
       </c>
-      <c r="J21" s="4" t="n">
+      <c r="K21" s="4" t="n">
         <v>152046</v>
       </c>
-      <c r="K21" s="4" t="n">
+      <c r="L21" s="4" t="n">
         <v>225859</v>
       </c>
-      <c r="L21" s="4" t="n">
+      <c r="M21" s="4" t="n">
         <v>311768</v>
       </c>
     </row>
@@ -5560,36 +5686,39 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>1193</v>
+        <v>0</v>
       </c>
       <c r="C22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="4" t="n">
         <v>58798</v>
       </c>
-      <c r="D22" s="4" t="n">
+      <c r="E22" s="4" t="n">
         <v>58855</v>
       </c>
-      <c r="E22" s="4" t="n">
+      <c r="F22" s="4" t="n">
         <v>50424</v>
       </c>
-      <c r="F22" s="4" t="n">
+      <c r="G22" s="4" t="n">
         <v>58619</v>
       </c>
-      <c r="G22" s="4" t="n">
+      <c r="H22" s="4" t="n">
         <v>5374</v>
       </c>
-      <c r="H22" s="4" t="n">
+      <c r="I22" s="4" t="n">
         <v>739</v>
       </c>
-      <c r="I22" s="4" t="n">
+      <c r="J22" s="4" t="n">
         <v>10834</v>
       </c>
-      <c r="J22" s="4" t="n">
+      <c r="K22" s="4" t="n">
         <v>26206</v>
       </c>
-      <c r="K22" s="4" t="n">
+      <c r="L22" s="4" t="n">
         <v>21765</v>
       </c>
-      <c r="L22" s="4" t="n">
+      <c r="M22" s="4" t="n">
         <v>49590</v>
       </c>
     </row>
@@ -5603,7 +5732,7 @@
         <v>3986</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>0</v>
+        <v>1063</v>
       </c>
       <c r="D23" s="4" t="n">
         <v>0</v>
@@ -5630,6 +5759,9 @@
         <v>0</v>
       </c>
       <c r="L23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="4" t="n">
         <v>252953</v>
       </c>
     </row>
@@ -5643,33 +5775,36 @@
         <v>35977</v>
       </c>
       <c r="C24" s="4" t="n">
+        <v>68225</v>
+      </c>
+      <c r="D24" s="4" t="n">
         <v>98933</v>
       </c>
-      <c r="D24" s="4" t="n">
+      <c r="E24" s="4" t="n">
         <v>136557</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="F24" s="4" t="n">
         <v>99787</v>
       </c>
-      <c r="F24" s="4" t="n">
+      <c r="G24" s="4" t="n">
         <v>129201</v>
       </c>
-      <c r="G24" s="4" t="n">
+      <c r="H24" s="4" t="n">
         <v>156479</v>
       </c>
-      <c r="H24" s="4" t="n">
+      <c r="I24" s="4" t="n">
         <v>158810</v>
       </c>
-      <c r="I24" s="4" t="n">
+      <c r="J24" s="4" t="n">
         <v>135948</v>
       </c>
-      <c r="J24" s="4" t="n">
+      <c r="K24" s="4" t="n">
         <v>151327</v>
       </c>
-      <c r="K24" s="4" t="n">
+      <c r="L24" s="4" t="n">
         <v>200169</v>
       </c>
-      <c r="L24" s="4" t="n">
+      <c r="M24" s="4" t="n">
         <v>234068</v>
       </c>
     </row>
@@ -5683,33 +5818,36 @@
         <v>661</v>
       </c>
       <c r="C25" s="4" t="n">
+        <v>605</v>
+      </c>
+      <c r="D25" s="4" t="n">
         <v>505</v>
       </c>
-      <c r="D25" s="4" t="n">
+      <c r="E25" s="4" t="n">
         <v>628</v>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="F25" s="4" t="n">
         <v>980</v>
       </c>
-      <c r="F25" s="4" t="n">
+      <c r="G25" s="4" t="n">
         <v>821</v>
       </c>
-      <c r="G25" s="4" t="n">
+      <c r="H25" s="4" t="n">
         <v>729</v>
       </c>
-      <c r="H25" s="4" t="n">
+      <c r="I25" s="4" t="n">
         <v>1358</v>
       </c>
-      <c r="I25" s="4" t="n">
+      <c r="J25" s="4" t="n">
         <v>3265</v>
       </c>
-      <c r="J25" s="4" t="n">
+      <c r="K25" s="4" t="n">
         <v>3550</v>
       </c>
-      <c r="K25" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="L25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5723,26 +5861,26 @@
         <v>70</v>
       </c>
       <c r="C26" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="D26" s="4" t="n">
         <v>67</v>
       </c>
-      <c r="D26" s="4" t="n">
+      <c r="E26" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="F26" s="4" t="n">
         <v>59</v>
-      </c>
-      <c r="F26" s="4" t="n">
-        <v>61</v>
       </c>
       <c r="G26" s="4" t="n">
         <v>61</v>
       </c>
       <c r="H26" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="I26" s="4" t="n">
         <v>99</v>
       </c>
-      <c r="I26" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="J26" s="4" t="n">
         <v>0</v>
       </c>
@@ -5750,6 +5888,9 @@
         <v>0</v>
       </c>
       <c r="L26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5787,11 +5928,14 @@
         <v>0</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>25000</v>
+        <v>0</v>
       </c>
       <c r="L27" s="4" t="n">
         <v>25000</v>
       </c>
+      <c r="M27" s="4" t="n">
+        <v>25000</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
@@ -5803,13 +5947,13 @@
         <v>9675</v>
       </c>
       <c r="C28" s="4" t="n">
-        <v>9500</v>
+        <v>9563</v>
       </c>
       <c r="D28" s="4" t="n">
         <v>9500</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>9513</v>
+        <v>9500</v>
       </c>
       <c r="F28" s="4" t="n">
         <v>9513</v>
@@ -5827,9 +5971,12 @@
         <v>9513</v>
       </c>
       <c r="K28" s="4" t="n">
+        <v>9513</v>
+      </c>
+      <c r="L28" s="4" t="n">
         <v>16071</v>
       </c>
-      <c r="L28" s="4" t="n">
+      <c r="M28" s="4" t="n">
         <v>25557</v>
       </c>
     </row>
@@ -5843,33 +5990,36 @@
         <v>3586</v>
       </c>
       <c r="C29" s="4" t="n">
+        <v>5094</v>
+      </c>
+      <c r="D29" s="4" t="n">
         <v>7109</v>
       </c>
-      <c r="D29" s="4" t="n">
+      <c r="E29" s="4" t="n">
         <v>8826</v>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="F29" s="4" t="n">
         <v>10890</v>
       </c>
-      <c r="F29" s="4" t="n">
+      <c r="G29" s="4" t="n">
         <v>12987</v>
       </c>
-      <c r="G29" s="4" t="n">
+      <c r="H29" s="4" t="n">
         <v>13772</v>
       </c>
-      <c r="H29" s="4" t="n">
+      <c r="I29" s="4" t="n">
         <v>14979</v>
       </c>
-      <c r="I29" s="4" t="n">
+      <c r="J29" s="4" t="n">
         <v>15908</v>
       </c>
-      <c r="J29" s="4" t="n">
+      <c r="K29" s="4" t="n">
         <v>14160</v>
       </c>
-      <c r="K29" s="4" t="n">
+      <c r="L29" s="4" t="n">
         <v>49949</v>
       </c>
-      <c r="L29" s="4" t="n">
+      <c r="M29" s="4" t="n">
         <v>32258</v>
       </c>
     </row>
@@ -5923,6 +6073,10 @@
         <f>SUM(L20:L29)</f>
         <v/>
       </c>
+      <c r="M30" s="6">
+        <f>SUM(M20:M29)</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
@@ -5934,33 +6088,36 @@
         <v>326</v>
       </c>
       <c r="C31" s="4" t="n">
+        <v>336</v>
+      </c>
+      <c r="D31" s="4" t="n">
         <v>249</v>
       </c>
-      <c r="D31" s="4" t="n">
+      <c r="E31" s="4" t="n">
         <v>512</v>
       </c>
-      <c r="E31" s="4" t="n">
+      <c r="F31" s="4" t="n">
         <v>955</v>
       </c>
-      <c r="F31" s="4" t="n">
+      <c r="G31" s="4" t="n">
         <v>850</v>
       </c>
-      <c r="G31" s="4" t="n">
+      <c r="H31" s="4" t="n">
         <v>762</v>
       </c>
-      <c r="H31" s="4" t="n">
+      <c r="I31" s="4" t="n">
         <v>4193</v>
       </c>
-      <c r="I31" s="4" t="n">
+      <c r="J31" s="4" t="n">
         <v>16674</v>
       </c>
-      <c r="J31" s="4" t="n">
+      <c r="K31" s="4" t="n">
         <v>16152</v>
       </c>
-      <c r="K31" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="L31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -5974,26 +6131,26 @@
         <v>162</v>
       </c>
       <c r="C32" s="4" t="n">
+        <v>156</v>
+      </c>
+      <c r="D32" s="4" t="n">
         <v>147</v>
       </c>
-      <c r="D32" s="4" t="n">
+      <c r="E32" s="4" t="n">
         <v>135</v>
       </c>
-      <c r="E32" s="4" t="n">
+      <c r="F32" s="4" t="n">
         <v>193</v>
       </c>
-      <c r="F32" s="4" t="n">
+      <c r="G32" s="4" t="n">
         <v>245</v>
       </c>
-      <c r="G32" s="4" t="n">
+      <c r="H32" s="4" t="n">
         <v>228</v>
       </c>
-      <c r="H32" s="4" t="n">
+      <c r="I32" s="4" t="n">
         <v>189</v>
       </c>
-      <c r="I32" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="J32" s="4" t="n">
         <v>0</v>
       </c>
@@ -6001,6 +6158,9 @@
         <v>0</v>
       </c>
       <c r="L32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6014,26 +6174,26 @@
         <v>15919</v>
       </c>
       <c r="C33" s="4" t="n">
+        <v>19250</v>
+      </c>
+      <c r="D33" s="4" t="n">
         <v>2333</v>
       </c>
-      <c r="D33" s="4" t="n">
+      <c r="E33" s="4" t="n">
         <v>2249</v>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="F33" s="4" t="n">
         <v>2880</v>
       </c>
-      <c r="F33" s="4" t="n">
+      <c r="G33" s="4" t="n">
         <v>2248</v>
       </c>
-      <c r="G33" s="4" t="n">
+      <c r="H33" s="4" t="n">
         <v>2201</v>
       </c>
-      <c r="H33" s="4" t="n">
+      <c r="I33" s="4" t="n">
         <v>2275</v>
       </c>
-      <c r="I33" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="J33" s="4" t="n">
         <v>0</v>
       </c>
@@ -6041,6 +6201,9 @@
         <v>0</v>
       </c>
       <c r="L33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6078,9 +6241,12 @@
         <v>0</v>
       </c>
       <c r="K34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="4" t="n">
         <v>862917</v>
       </c>
-      <c r="L34" s="4" t="n">
+      <c r="M34" s="4" t="n">
         <v>861472</v>
       </c>
     </row>
@@ -6094,33 +6260,36 @@
         <v>179788</v>
       </c>
       <c r="C35" s="4" t="n">
+        <v>175275</v>
+      </c>
+      <c r="D35" s="4" t="n">
         <v>171745</v>
       </c>
-      <c r="D35" s="4" t="n">
+      <c r="E35" s="4" t="n">
         <v>169370</v>
       </c>
-      <c r="E35" s="4" t="n">
+      <c r="F35" s="4" t="n">
         <v>167227</v>
       </c>
-      <c r="F35" s="4" t="n">
+      <c r="G35" s="4" t="n">
         <v>164849</v>
       </c>
-      <c r="G35" s="4" t="n">
+      <c r="H35" s="4" t="n">
         <v>162471</v>
       </c>
-      <c r="H35" s="4" t="n">
+      <c r="I35" s="4" t="n">
         <v>160092</v>
       </c>
-      <c r="I35" s="4" t="n">
+      <c r="J35" s="4" t="n">
         <v>157714</v>
       </c>
-      <c r="J35" s="4" t="n">
+      <c r="K35" s="4" t="n">
         <v>155336</v>
       </c>
-      <c r="K35" s="4" t="n">
+      <c r="L35" s="4" t="n">
         <v>156135</v>
       </c>
-      <c r="L35" s="4" t="n">
+      <c r="M35" s="4" t="n">
         <v>387432</v>
       </c>
     </row>
@@ -6152,15 +6321,18 @@
         <v>0</v>
       </c>
       <c r="I36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="4" t="n">
         <v>2541</v>
       </c>
-      <c r="J36" s="4" t="n">
+      <c r="K36" s="4" t="n">
         <v>2574</v>
       </c>
-      <c r="K36" s="4" t="n">
+      <c r="L36" s="4" t="n">
         <v>25002</v>
       </c>
-      <c r="L36" s="4" t="n">
+      <c r="M36" s="4" t="n">
         <v>24431</v>
       </c>
     </row>
@@ -6214,6 +6386,10 @@
         <f>L30+SUM(L31:L36)</f>
         <v/>
       </c>
+      <c r="M37" s="6">
+        <f>M30+SUM(M31:M36)</f>
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
@@ -6252,6 +6428,9 @@
         <v>824488</v>
       </c>
       <c r="L38" s="4" t="n">
+        <v>824488</v>
+      </c>
+      <c r="M38" s="4" t="n">
         <v>1760275</v>
       </c>
     </row>
@@ -6274,13 +6453,13 @@
         <v>77</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>78</v>
       </c>
       <c r="H39" s="4" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I39" s="4" t="n">
         <v>79</v>
@@ -6289,11 +6468,14 @@
         <v>79</v>
       </c>
       <c r="K39" s="4" t="n">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="L39" s="4" t="n">
         <v>101</v>
       </c>
+      <c r="M39" s="4" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
@@ -6305,33 +6487,36 @@
         <v>280668</v>
       </c>
       <c r="C40" s="4" t="n">
+        <v>279872</v>
+      </c>
+      <c r="D40" s="4" t="n">
         <v>278980</v>
       </c>
-      <c r="D40" s="4" t="n">
+      <c r="E40" s="4" t="n">
         <v>277980</v>
       </c>
-      <c r="E40" s="4" t="n">
+      <c r="F40" s="4" t="n">
         <v>276717</v>
       </c>
-      <c r="F40" s="4" t="n">
+      <c r="G40" s="4" t="n">
         <v>281247</v>
       </c>
-      <c r="G40" s="4" t="n">
+      <c r="H40" s="4" t="n">
         <v>286173</v>
       </c>
-      <c r="H40" s="4" t="n">
+      <c r="I40" s="4" t="n">
         <v>292576</v>
       </c>
-      <c r="I40" s="4" t="n">
+      <c r="J40" s="4" t="n">
         <v>297579</v>
       </c>
-      <c r="J40" s="4" t="n">
+      <c r="K40" s="4" t="n">
         <v>300877</v>
       </c>
-      <c r="K40" s="4" t="n">
+      <c r="L40" s="4" t="n">
         <v>1028384</v>
       </c>
-      <c r="L40" s="4" t="n">
+      <c r="M40" s="4" t="n">
         <v>1035021</v>
       </c>
     </row>
@@ -6345,33 +6530,36 @@
         <v>-1881</v>
       </c>
       <c r="C41" s="4" t="n">
+        <v>-1287</v>
+      </c>
+      <c r="D41" s="4" t="n">
         <v>-1877</v>
       </c>
-      <c r="D41" s="4" t="n">
+      <c r="E41" s="4" t="n">
         <v>-2541</v>
       </c>
-      <c r="E41" s="4" t="n">
+      <c r="F41" s="4" t="n">
         <v>-701</v>
       </c>
-      <c r="F41" s="4" t="n">
+      <c r="G41" s="4" t="n">
         <v>-2055</v>
       </c>
-      <c r="G41" s="4" t="n">
+      <c r="H41" s="4" t="n">
         <v>-2363</v>
       </c>
-      <c r="H41" s="4" t="n">
+      <c r="I41" s="4" t="n">
         <v>-338</v>
       </c>
-      <c r="I41" s="4" t="n">
+      <c r="J41" s="4" t="n">
         <v>-3250</v>
       </c>
-      <c r="J41" s="4" t="n">
+      <c r="K41" s="4" t="n">
         <v>-1001</v>
       </c>
-      <c r="K41" s="4" t="n">
+      <c r="L41" s="4" t="n">
         <v>2178</v>
       </c>
-      <c r="L41" s="4" t="n">
+      <c r="M41" s="4" t="n">
         <v>2508</v>
       </c>
     </row>
@@ -6385,33 +6573,36 @@
         <v>-238772</v>
       </c>
       <c r="C42" s="4" t="n">
+        <v>-197627</v>
+      </c>
+      <c r="D42" s="4" t="n">
         <v>-146118</v>
       </c>
-      <c r="D42" s="4" t="n">
+      <c r="E42" s="4" t="n">
         <v>-62169</v>
       </c>
-      <c r="E42" s="4" t="n">
+      <c r="F42" s="4" t="n">
         <v>-12053</v>
       </c>
-      <c r="F42" s="4" t="n">
+      <c r="G42" s="4" t="n">
         <v>58921</v>
       </c>
-      <c r="G42" s="4" t="n">
+      <c r="H42" s="4" t="n">
         <v>131866</v>
       </c>
-      <c r="H42" s="4" t="n">
+      <c r="I42" s="4" t="n">
         <v>131309</v>
       </c>
-      <c r="I42" s="4" t="n">
+      <c r="J42" s="4" t="n">
         <v>105521</v>
       </c>
-      <c r="J42" s="4" t="n">
+      <c r="K42" s="4" t="n">
         <v>143159</v>
       </c>
-      <c r="K42" s="4" t="n">
+      <c r="L42" s="4" t="n">
         <v>236163</v>
       </c>
-      <c r="L42" s="4" t="n">
+      <c r="M42" s="4" t="n">
         <v>165480</v>
       </c>
     </row>
@@ -6465,6 +6656,10 @@
         <f>SUM(L38:L42)</f>
         <v/>
       </c>
+      <c r="M43" s="6">
+        <f>SUM(M38:M42)</f>
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
@@ -6514,6 +6709,10 @@
       </c>
       <c r="L44" s="6">
         <f>L37+L43</f>
+        <v/>
+      </c>
+      <c r="M44" s="6">
+        <f>M37+M43</f>
         <v/>
       </c>
     </row>
@@ -6528,7 +6727,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6543,61 +6742,67 @@
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr"/>
       <c r="B1" s="2" t="inlineStr">
         <is>
+          <t>Q1 FY2022</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
           <t>Q2 FY2022</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2022</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Q1 FY2023</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2023</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2023</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Q1 FY2024</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2024</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2024</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Q1 FY2025</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Q2 FY2025</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Q3 FY2025</t>
         </is>
@@ -6610,36 +6815,39 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
+        <v>6679</v>
+      </c>
+      <c r="C2" s="4" t="n">
         <v>15838</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="D2" s="4" t="n">
         <v>-166059</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="E2" s="4" t="n">
         <v>41227</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="F2" s="4" t="n">
         <v>92736</v>
       </c>
-      <c r="F2" s="4" t="n">
+      <c r="G2" s="4" t="n">
         <v>176685</v>
       </c>
-      <c r="G2" s="4" t="n">
+      <c r="H2" s="4" t="n">
         <v>77811</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="I2" s="4" t="n">
         <v>157594</v>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="J2" s="4" t="n">
         <v>163950</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="K2" s="4" t="n">
         <v>44419</v>
       </c>
-      <c r="K2" s="4" t="n">
+      <c r="L2" s="4" t="n">
         <v>144274</v>
       </c>
-      <c r="L2" s="4" t="n">
+      <c r="M2" s="4" t="n">
         <v>83260</v>
       </c>
     </row>
@@ -6650,23 +6858,23 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
+        <v>245</v>
+      </c>
+      <c r="C3" s="4" t="n">
         <v>556</v>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="D3" s="4" t="n">
         <v>952</v>
       </c>
-      <c r="D3" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="E3" s="4" t="n">
+        <v>404</v>
+      </c>
+      <c r="F3" s="4" t="n">
         <v>953</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="G3" s="4" t="n">
         <v>1676</v>
       </c>
-      <c r="G3" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="H3" s="4" t="n">
         <v>0</v>
       </c>
@@ -6680,6 +6888,9 @@
         <v>0</v>
       </c>
       <c r="L3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6690,23 +6901,23 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
+        <v>141</v>
+      </c>
+      <c r="C4" s="4" t="n">
         <v>275</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="D4" s="4" t="n">
         <v>402</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="E4" s="4" t="n">
+        <v>145</v>
+      </c>
+      <c r="F4" s="4" t="n">
         <v>294</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="G4" s="4" t="n">
         <v>445</v>
       </c>
-      <c r="G4" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="H4" s="4" t="n">
         <v>0</v>
       </c>
@@ -6720,6 +6931,9 @@
         <v>0</v>
       </c>
       <c r="L4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6733,11 +6947,11 @@
         <v>0</v>
       </c>
       <c r="C5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="4" t="n">
         <v>2379</v>
       </c>
-      <c r="D5" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="E5" s="4" t="n">
         <v>0</v>
       </c>
@@ -6760,6 +6974,9 @@
         <v>0</v>
       </c>
       <c r="L5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6776,7 +6993,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>549</v>
+        <v>0</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>0</v>
@@ -6785,21 +7002,24 @@
         <v>0</v>
       </c>
       <c r="G6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4" t="n">
         <v>1229</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="I6" s="4" t="n">
         <v>2648</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="J6" s="4" t="n">
         <v>4888</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="K6" s="4" t="n">
         <v>2611</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="L6" s="4" t="n">
         <v>11730</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="M6" s="4" t="n">
         <v>20516</v>
       </c>
     </row>
@@ -6810,36 +7030,39 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
+        <v>455</v>
+      </c>
+      <c r="C7" s="4" t="n">
         <v>466</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="D7" s="4" t="n">
         <v>705</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="E7" s="4" t="n">
         <v>837</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="F7" s="4" t="n">
         <v>1088</v>
       </c>
-      <c r="F7" s="4" t="n">
+      <c r="G7" s="4" t="n">
         <v>1880</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="H7" s="4" t="n">
         <v>2250</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="I7" s="4" t="n">
         <v>4072</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="J7" s="4" t="n">
         <v>4279</v>
       </c>
-      <c r="J7" s="4" t="n">
+      <c r="K7" s="4" t="n">
         <v>2077</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="L7" s="4" t="n">
         <v>5529</v>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="M7" s="4" t="n">
         <v>3226</v>
       </c>
     </row>
@@ -6853,33 +7076,36 @@
         <v>0</v>
       </c>
       <c r="C8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="4" t="n">
         <v>2354</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="E8" s="4" t="n">
         <v>3531</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="F8" s="4" t="n">
         <v>7062</v>
       </c>
-      <c r="F8" s="4" t="n">
+      <c r="G8" s="4" t="n">
         <v>10593</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="H8" s="4" t="n">
         <v>3531</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="I8" s="4" t="n">
         <v>7062</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="J8" s="4" t="n">
         <v>10593</v>
       </c>
-      <c r="J8" s="4" t="n">
+      <c r="K8" s="4" t="n">
         <v>3531</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="L8" s="4" t="n">
         <v>7062</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="M8" s="4" t="n">
         <v>13391</v>
       </c>
     </row>
@@ -6890,36 +7116,39 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
+        <v>2596</v>
+      </c>
+      <c r="C9" s="4" t="n">
         <v>331</v>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="D9" s="4" t="n">
         <v>1078</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="E9" s="4" t="n">
         <v>1672</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="F9" s="4" t="n">
         <v>-3888</v>
       </c>
-      <c r="F9" s="4" t="n">
+      <c r="G9" s="4" t="n">
         <v>2677</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="H9" s="4" t="n">
         <v>2386</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="I9" s="4" t="n">
         <v>11554</v>
       </c>
-      <c r="I9" s="4" t="n">
+      <c r="J9" s="4" t="n">
         <v>17118</v>
       </c>
-      <c r="J9" s="4" t="n">
+      <c r="K9" s="4" t="n">
         <v>5337</v>
       </c>
-      <c r="K9" s="4" t="n">
+      <c r="L9" s="4" t="n">
         <v>15262</v>
       </c>
-      <c r="L9" s="4" t="n">
+      <c r="M9" s="4" t="n">
         <v>22313</v>
       </c>
     </row>
@@ -6939,27 +7168,30 @@
         <v>0</v>
       </c>
       <c r="E10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="4" t="n">
         <v>191</v>
       </c>
-      <c r="F10" s="4" t="n">
+      <c r="G10" s="4" t="n">
         <v>195</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="H10" s="4" t="n">
         <v>-8</v>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="I10" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="I10" s="4" t="n">
+      <c r="J10" s="4" t="n">
         <v>126</v>
       </c>
-      <c r="J10" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="K10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6970,36 +7202,39 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
+        <v>4310</v>
+      </c>
+      <c r="C11" s="4" t="n">
         <v>8517</v>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="D11" s="4" t="n">
         <v>14780</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="E11" s="4" t="n">
         <v>5507</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="F11" s="4" t="n">
         <v>11242</v>
       </c>
-      <c r="F11" s="4" t="n">
+      <c r="G11" s="4" t="n">
         <v>16221</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="H11" s="4" t="n">
         <v>3563</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="I11" s="4" t="n">
         <v>8309</v>
       </c>
-      <c r="I11" s="4" t="n">
+      <c r="J11" s="4" t="n">
         <v>13685</v>
       </c>
-      <c r="J11" s="4" t="n">
+      <c r="K11" s="4" t="n">
         <v>5029</v>
       </c>
-      <c r="K11" s="4" t="n">
+      <c r="L11" s="4" t="n">
         <v>11463</v>
       </c>
-      <c r="L11" s="4" t="n">
+      <c r="M11" s="4" t="n">
         <v>18847</v>
       </c>
     </row>
@@ -7010,36 +7245,39 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
+        <v>2561</v>
+      </c>
+      <c r="C12" s="4" t="n">
         <v>1072</v>
       </c>
-      <c r="C12" s="4" t="n">
+      <c r="D12" s="4" t="n">
         <v>31329</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="E12" s="4" t="n">
         <v>2873</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="F12" s="4" t="n">
         <v>-41044</v>
       </c>
-      <c r="F12" s="4" t="n">
+      <c r="G12" s="4" t="n">
         <v>-44303</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="H12" s="4" t="n">
         <v>6450</v>
       </c>
-      <c r="H12" s="4" t="n">
+      <c r="I12" s="4" t="n">
         <v>6112</v>
       </c>
-      <c r="I12" s="4" t="n">
+      <c r="J12" s="4" t="n">
         <v>4727</v>
       </c>
-      <c r="J12" s="4" t="n">
+      <c r="K12" s="4" t="n">
         <v>269</v>
       </c>
-      <c r="K12" s="4" t="n">
+      <c r="L12" s="4" t="n">
         <v>-4161</v>
       </c>
-      <c r="L12" s="4" t="n">
+      <c r="M12" s="4" t="n">
         <v>-71408</v>
       </c>
     </row>
@@ -7050,36 +7288,39 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="C13" s="4" t="n">
         <v>602</v>
       </c>
-      <c r="C13" s="4" t="n">
+      <c r="D13" s="4" t="n">
         <v>1007</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="E13" s="4" t="n">
         <v>69</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="F13" s="4" t="n">
         <v>206</v>
       </c>
-      <c r="F13" s="4" t="n">
+      <c r="G13" s="4" t="n">
         <v>258</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="H13" s="4" t="n">
         <v>369</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="I13" s="4" t="n">
         <v>633</v>
       </c>
-      <c r="I13" s="4" t="n">
+      <c r="J13" s="4" t="n">
         <v>356</v>
       </c>
-      <c r="J13" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="K13" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7117,11 +7358,14 @@
         <v>0</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>13800</v>
+        <v>0</v>
       </c>
       <c r="L14" s="4" t="n">
         <v>13800</v>
       </c>
+      <c r="M14" s="4" t="n">
+        <v>13800</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -7133,33 +7377,36 @@
         <v>0</v>
       </c>
       <c r="C15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="E15" s="4" t="n">
         <v>-4</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="F15" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F15" s="4" t="n">
+      <c r="G15" s="4" t="n">
         <v>-2</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="H15" s="4" t="n">
         <v>-7672</v>
       </c>
-      <c r="H15" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="I15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="J15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" s="4" t="n">
         <v>-1014</v>
       </c>
-      <c r="K15" s="4" t="n">
+      <c r="L15" s="4" t="n">
         <v>-257</v>
       </c>
-      <c r="L15" s="4" t="n">
+      <c r="M15" s="4" t="n">
         <v>1964</v>
       </c>
     </row>
@@ -7170,36 +7417,39 @@
         </is>
       </c>
       <c r="B16" s="4" t="n">
+        <v>-34420</v>
+      </c>
+      <c r="C16" s="4" t="n">
         <v>-27920</v>
       </c>
-      <c r="C16" s="4" t="n">
+      <c r="D16" s="4" t="n">
         <v>-78967</v>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="E16" s="4" t="n">
         <v>-109639</v>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="F16" s="4" t="n">
         <v>-135600</v>
       </c>
-      <c r="F16" s="4" t="n">
+      <c r="G16" s="4" t="n">
         <v>-153271</v>
       </c>
-      <c r="G16" s="4" t="n">
+      <c r="H16" s="4" t="n">
         <v>-18664</v>
       </c>
-      <c r="H16" s="4" t="n">
+      <c r="I16" s="4" t="n">
         <v>-82213</v>
       </c>
-      <c r="I16" s="4" t="n">
+      <c r="J16" s="4" t="n">
         <v>-26529</v>
       </c>
-      <c r="J16" s="4" t="n">
+      <c r="K16" s="4" t="n">
         <v>11841</v>
       </c>
-      <c r="K16" s="4" t="n">
+      <c r="L16" s="4" t="n">
         <v>-143153</v>
       </c>
-      <c r="L16" s="4" t="n">
+      <c r="M16" s="4" t="n">
         <v>-164133</v>
       </c>
     </row>
@@ -7210,36 +7460,39 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
+        <v>4531</v>
+      </c>
+      <c r="C17" s="4" t="n">
         <v>28753</v>
       </c>
-      <c r="C17" s="4" t="n">
+      <c r="D17" s="4" t="n">
         <v>36211</v>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="E17" s="4" t="n">
         <v>17338</v>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="F17" s="4" t="n">
         <v>24632</v>
       </c>
-      <c r="F17" s="4" t="n">
+      <c r="G17" s="4" t="n">
         <v>-28092</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="H17" s="4" t="n">
         <v>29386</v>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="I17" s="4" t="n">
         <v>37052</v>
       </c>
-      <c r="I17" s="4" t="n">
+      <c r="J17" s="4" t="n">
         <v>14585</v>
       </c>
-      <c r="J17" s="4" t="n">
+      <c r="K17" s="4" t="n">
         <v>4794</v>
       </c>
-      <c r="K17" s="4" t="n">
+      <c r="L17" s="4" t="n">
         <v>23039</v>
       </c>
-      <c r="L17" s="4" t="n">
+      <c r="M17" s="4" t="n">
         <v>31132</v>
       </c>
     </row>
@@ -7250,36 +7503,39 @@
         </is>
       </c>
       <c r="B18" s="4" t="n">
+        <v>3513</v>
+      </c>
+      <c r="C18" s="4" t="n">
         <v>1257</v>
       </c>
-      <c r="C18" s="4" t="n">
+      <c r="D18" s="4" t="n">
         <v>1459</v>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="E18" s="4" t="n">
         <v>-4166</v>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="F18" s="4" t="n">
         <v>-12058</v>
       </c>
-      <c r="F18" s="4" t="n">
+      <c r="G18" s="4" t="n">
         <v>-12406</v>
       </c>
-      <c r="G18" s="4" t="n">
+      <c r="H18" s="4" t="n">
         <v>-2076</v>
       </c>
-      <c r="H18" s="4" t="n">
+      <c r="I18" s="4" t="n">
         <v>-3469</v>
       </c>
-      <c r="I18" s="4" t="n">
+      <c r="J18" s="4" t="n">
         <v>-20261</v>
       </c>
-      <c r="J18" s="4" t="n">
+      <c r="K18" s="4" t="n">
         <v>-3687</v>
       </c>
-      <c r="K18" s="4" t="n">
+      <c r="L18" s="4" t="n">
         <v>-20645</v>
       </c>
-      <c r="L18" s="4" t="n">
+      <c r="M18" s="4" t="n">
         <v>-142920</v>
       </c>
     </row>
@@ -7290,23 +7546,23 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
+        <v>5552</v>
+      </c>
+      <c r="C19" s="4" t="n">
         <v>-7176</v>
       </c>
-      <c r="C19" s="4" t="n">
+      <c r="D19" s="4" t="n">
         <v>-3050</v>
       </c>
-      <c r="D19" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="E19" s="4" t="n">
+        <v>182</v>
+      </c>
+      <c r="F19" s="4" t="n">
         <v>-12491</v>
       </c>
-      <c r="F19" s="4" t="n">
+      <c r="G19" s="4" t="n">
         <v>14652</v>
       </c>
-      <c r="G19" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="H19" s="4" t="n">
         <v>0</v>
       </c>
@@ -7320,6 +7576,9 @@
         <v>0</v>
       </c>
       <c r="L19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7330,11 +7589,11 @@
         </is>
       </c>
       <c r="B20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="4" t="n">
         <v>488</v>
       </c>
-      <c r="C20" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="D20" s="4" t="n">
         <v>0</v>
       </c>
@@ -7348,18 +7607,21 @@
         <v>0</v>
       </c>
       <c r="H20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="4" t="n">
         <v>-6362</v>
       </c>
-      <c r="I20" s="4" t="n">
+      <c r="J20" s="4" t="n">
         <v>-5303</v>
       </c>
-      <c r="J20" s="4" t="n">
+      <c r="K20" s="4" t="n">
         <v>-1552</v>
       </c>
-      <c r="K20" s="4" t="n">
+      <c r="L20" s="4" t="n">
         <v>-468</v>
       </c>
-      <c r="L20" s="4" t="n">
+      <c r="M20" s="4" t="n">
         <v>-275</v>
       </c>
     </row>
@@ -7376,7 +7638,7 @@
         <v>0</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>-19712</v>
+        <v>0</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>0</v>
@@ -7385,21 +7647,24 @@
         <v>0</v>
       </c>
       <c r="G21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="4" t="n">
         <v>-3013</v>
       </c>
-      <c r="H21" s="4" t="n">
+      <c r="I21" s="4" t="n">
         <v>3950</v>
       </c>
-      <c r="I21" s="4" t="n">
+      <c r="J21" s="4" t="n">
         <v>-12259</v>
       </c>
-      <c r="J21" s="4" t="n">
+      <c r="K21" s="4" t="n">
         <v>11679</v>
       </c>
-      <c r="K21" s="4" t="n">
+      <c r="L21" s="4" t="n">
         <v>20789</v>
       </c>
-      <c r="L21" s="4" t="n">
+      <c r="M21" s="4" t="n">
         <v>4081</v>
       </c>
     </row>
@@ -7416,7 +7681,7 @@
         <v>0</v>
       </c>
       <c r="D22" s="4" t="n">
-        <v>12643</v>
+        <v>0</v>
       </c>
       <c r="E22" s="4" t="n">
         <v>0</v>
@@ -7425,21 +7690,24 @@
         <v>0</v>
       </c>
       <c r="G22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4" t="n">
         <v>1998</v>
       </c>
-      <c r="H22" s="4" t="n">
+      <c r="I22" s="4" t="n">
         <v>17760</v>
       </c>
-      <c r="I22" s="4" t="n">
+      <c r="J22" s="4" t="n">
         <v>11151</v>
       </c>
-      <c r="J22" s="4" t="n">
+      <c r="K22" s="4" t="n">
         <v>-8673</v>
       </c>
-      <c r="K22" s="4" t="n">
+      <c r="L22" s="4" t="n">
         <v>-7013</v>
       </c>
-      <c r="L22" s="4" t="n">
+      <c r="M22" s="4" t="n">
         <v>32961</v>
       </c>
     </row>
@@ -7450,36 +7718,39 @@
         </is>
       </c>
       <c r="B23" s="4" t="n">
+        <v>765</v>
+      </c>
+      <c r="C23" s="4" t="n">
         <v>1820</v>
       </c>
-      <c r="C23" s="4" t="n">
+      <c r="D23" s="4" t="n">
         <v>32590</v>
       </c>
-      <c r="D23" s="4" t="n">
-        <v>8759</v>
-      </c>
       <c r="E23" s="4" t="n">
+        <v>1508</v>
+      </c>
+      <c r="F23" s="4" t="n">
         <v>61128</v>
       </c>
-      <c r="F23" s="4" t="n">
+      <c r="G23" s="4" t="n">
         <v>62901</v>
       </c>
-      <c r="G23" s="4" t="n">
+      <c r="H23" s="4" t="n">
         <v>10344</v>
       </c>
-      <c r="H23" s="4" t="n">
+      <c r="I23" s="4" t="n">
         <v>-42094</v>
       </c>
-      <c r="I23" s="4" t="n">
+      <c r="J23" s="4" t="n">
         <v>-45537</v>
       </c>
-      <c r="J23" s="4" t="n">
+      <c r="K23" s="4" t="n">
         <v>13705</v>
       </c>
-      <c r="K23" s="4" t="n">
+      <c r="L23" s="4" t="n">
         <v>12927</v>
       </c>
-      <c r="L23" s="4" t="n">
+      <c r="M23" s="4" t="n">
         <v>42433</v>
       </c>
     </row>
@@ -7490,36 +7761,39 @@
         </is>
       </c>
       <c r="B24" s="4" t="n">
+        <v>12190</v>
+      </c>
+      <c r="C24" s="4" t="n">
         <v>17512</v>
       </c>
-      <c r="C24" s="4" t="n">
+      <c r="D24" s="4" t="n">
         <v>24213</v>
       </c>
-      <c r="D24" s="4" t="n">
+      <c r="E24" s="4" t="n">
         <v>32248</v>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="F24" s="4" t="n">
         <v>62995</v>
       </c>
-      <c r="F24" s="4" t="n">
+      <c r="G24" s="4" t="n">
         <v>100580</v>
       </c>
-      <c r="G24" s="4" t="n">
+      <c r="H24" s="4" t="n">
         <v>29414</v>
       </c>
-      <c r="H24" s="4" t="n">
+      <c r="I24" s="4" t="n">
         <v>56692</v>
       </c>
-      <c r="I24" s="4" t="n">
+      <c r="J24" s="4" t="n">
         <v>59023</v>
       </c>
-      <c r="J24" s="4" t="n">
+      <c r="K24" s="4" t="n">
         <v>15379</v>
       </c>
-      <c r="K24" s="4" t="n">
+      <c r="L24" s="4" t="n">
         <v>64221</v>
       </c>
-      <c r="L24" s="4" t="n">
+      <c r="M24" s="4" t="n">
         <v>83276</v>
       </c>
     </row>
@@ -7533,19 +7807,19 @@
         <v>0</v>
       </c>
       <c r="C25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="4" t="n">
         <v>115551</v>
       </c>
-      <c r="D25" s="4" t="n">
+      <c r="E25" s="4" t="n">
         <v>-2923</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>-3986</v>
       </c>
       <c r="F25" s="4" t="n">
         <v>-3986</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>-248</v>
+        <v>-3986</v>
       </c>
       <c r="H25" s="4" t="n">
         <v>-248</v>
@@ -7554,12 +7828,15 @@
         <v>-248</v>
       </c>
       <c r="J25" s="4" t="n">
-        <v>0</v>
+        <v>-248</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="4" t="n">
         <v>252953</v>
       </c>
     </row>
@@ -7570,36 +7847,39 @@
         </is>
       </c>
       <c r="B26" s="4" t="n">
+        <v>-78</v>
+      </c>
+      <c r="C26" s="4" t="n">
         <v>-95</v>
       </c>
-      <c r="C26" s="4" t="n">
+      <c r="D26" s="4" t="n">
         <v>-126</v>
       </c>
-      <c r="D26" s="4" t="n">
+      <c r="E26" s="4" t="n">
         <v>-15</v>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="F26" s="4" t="n">
         <v>-38</v>
       </c>
-      <c r="F26" s="4" t="n">
+      <c r="G26" s="4" t="n">
         <v>-64</v>
       </c>
-      <c r="G26" s="4" t="n">
+      <c r="H26" s="4" t="n">
         <v>-23</v>
       </c>
-      <c r="H26" s="4" t="n">
+      <c r="I26" s="4" t="n">
         <v>-34</v>
       </c>
-      <c r="I26" s="4" t="n">
+      <c r="J26" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="J26" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="K26" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7613,33 +7893,36 @@
         <v>0</v>
       </c>
       <c r="C27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="4" t="n">
         <v>154103</v>
       </c>
-      <c r="D27" s="4" t="n">
+      <c r="E27" s="4" t="n">
         <v>-4625</v>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="F27" s="4" t="n">
         <v>-8219</v>
       </c>
-      <c r="F27" s="4" t="n">
+      <c r="G27" s="4" t="n">
         <v>-10593</v>
       </c>
-      <c r="G27" s="4" t="n">
+      <c r="H27" s="4" t="n">
         <v>-2378</v>
       </c>
-      <c r="H27" s="4" t="n">
+      <c r="I27" s="4" t="n">
         <v>-4757</v>
       </c>
-      <c r="I27" s="4" t="n">
+      <c r="J27" s="4" t="n">
         <v>-7135</v>
       </c>
-      <c r="J27" s="4" t="n">
+      <c r="K27" s="4" t="n">
         <v>-2378</v>
       </c>
-      <c r="K27" s="4" t="n">
+      <c r="L27" s="4" t="n">
         <v>-7320</v>
       </c>
-      <c r="L27" s="4" t="n">
+      <c r="M27" s="4" t="n">
         <v>233463</v>
       </c>
     </row>
@@ -7693,6 +7976,10 @@
         <f>SUM(L2:L27)</f>
         <v/>
       </c>
+      <c r="M28" s="6">
+        <f>SUM(M2:M27)</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
@@ -7701,13 +7988,13 @@
         </is>
       </c>
       <c r="B29" s="4" t="n">
-        <v>2592</v>
+        <v>0</v>
       </c>
       <c r="C29" s="4" t="n">
         <v>2592</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>3233</v>
+        <v>2592</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>3233</v>
@@ -7716,7 +8003,7 @@
         <v>3233</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>0</v>
+        <v>3233</v>
       </c>
       <c r="H29" s="4" t="n">
         <v>0</v>
@@ -7731,6 +8018,9 @@
         <v>0</v>
       </c>
       <c r="L29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7741,36 +8031,39 @@
         </is>
       </c>
       <c r="B30" s="4" t="n">
+        <v>-742</v>
+      </c>
+      <c r="C30" s="4" t="n">
         <v>-2456</v>
       </c>
-      <c r="C30" s="4" t="n">
+      <c r="D30" s="4" t="n">
         <v>-3477</v>
       </c>
-      <c r="D30" s="4" t="n">
+      <c r="E30" s="4" t="n">
         <v>-2253</v>
       </c>
-      <c r="E30" s="4" t="n">
+      <c r="F30" s="4" t="n">
         <v>-6810</v>
       </c>
-      <c r="F30" s="4" t="n">
+      <c r="G30" s="4" t="n">
         <v>-12687</v>
       </c>
-      <c r="G30" s="4" t="n">
+      <c r="H30" s="4" t="n">
         <v>-4525</v>
       </c>
-      <c r="H30" s="4" t="n">
+      <c r="I30" s="4" t="n">
         <v>-13739</v>
       </c>
-      <c r="I30" s="4" t="n">
+      <c r="J30" s="4" t="n">
         <v>-17983</v>
       </c>
-      <c r="J30" s="4" t="n">
+      <c r="K30" s="4" t="n">
         <v>-6944</v>
       </c>
-      <c r="K30" s="4" t="n">
+      <c r="L30" s="4" t="n">
         <v>-15194</v>
       </c>
-      <c r="L30" s="4" t="n">
+      <c r="M30" s="4" t="n">
         <v>-25539</v>
       </c>
     </row>
@@ -7802,17 +8095,20 @@
         <v>0</v>
       </c>
       <c r="I31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="4" t="n">
         <v>-3000</v>
       </c>
-      <c r="J31" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="K31" s="4" t="n">
-        <v>-5000</v>
+        <v>0</v>
       </c>
       <c r="L31" s="4" t="n">
         <v>-5000</v>
       </c>
+      <c r="M31" s="4" t="n">
+        <v>-5000</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
@@ -7848,9 +8144,12 @@
         <v>0</v>
       </c>
       <c r="K32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="4" t="n">
         <v>-1256351</v>
       </c>
-      <c r="L32" s="4" t="n">
+      <c r="M32" s="4" t="n">
         <v>-1278769</v>
       </c>
     </row>
@@ -7891,6 +8190,9 @@
         <v>0</v>
       </c>
       <c r="L33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="4" t="n">
         <v>30617</v>
       </c>
     </row>
@@ -7944,6 +8246,10 @@
         <f>SUM(L29:L33)</f>
         <v/>
       </c>
+      <c r="M34" s="6">
+        <f>SUM(M29:M33)</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -7952,36 +8258,39 @@
         </is>
       </c>
       <c r="B35" s="4" t="n">
+        <v>-20</v>
+      </c>
+      <c r="C35" s="4" t="n">
         <v>-37</v>
       </c>
-      <c r="C35" s="4" t="n">
+      <c r="D35" s="4" t="n">
         <v>-49</v>
       </c>
-      <c r="D35" s="4" t="n">
+      <c r="E35" s="4" t="n">
         <v>-11</v>
       </c>
-      <c r="E35" s="4" t="n">
+      <c r="F35" s="4" t="n">
         <v>-22</v>
       </c>
-      <c r="F35" s="4" t="n">
+      <c r="G35" s="4" t="n">
         <v>-33</v>
       </c>
-      <c r="G35" s="4" t="n">
+      <c r="H35" s="4" t="n">
         <v>-15</v>
       </c>
-      <c r="H35" s="4" t="n">
+      <c r="I35" s="4" t="n">
         <v>-30</v>
       </c>
-      <c r="I35" s="4" t="n">
+      <c r="J35" s="4" t="n">
         <v>-46</v>
       </c>
-      <c r="J35" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="K35" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7992,36 +8301,39 @@
         </is>
       </c>
       <c r="B36" s="4" t="n">
+        <v>810</v>
+      </c>
+      <c r="C36" s="4" t="n">
         <v>1260</v>
       </c>
-      <c r="C36" s="4" t="n">
+      <c r="D36" s="4" t="n">
         <v>3104</v>
       </c>
-      <c r="D36" s="4" t="n">
+      <c r="E36" s="4" t="n">
         <v>478</v>
       </c>
-      <c r="E36" s="4" t="n">
+      <c r="F36" s="4" t="n">
         <v>707</v>
       </c>
-      <c r="F36" s="4" t="n">
+      <c r="G36" s="4" t="n">
         <v>1603</v>
       </c>
-      <c r="G36" s="4" t="n">
+      <c r="H36" s="4" t="n">
         <v>967</v>
       </c>
-      <c r="H36" s="4" t="n">
+      <c r="I36" s="4" t="n">
         <v>1147</v>
       </c>
-      <c r="I36" s="4" t="n">
+      <c r="J36" s="4" t="n">
         <v>3832</v>
       </c>
-      <c r="J36" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="K36" s="4" t="n">
         <v>0</v>
       </c>
       <c r="L36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8035,11 +8347,11 @@
         <v>0</v>
       </c>
       <c r="C37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="4" t="n">
         <v>542018</v>
       </c>
-      <c r="D37" s="4" t="n">
-        <v>0</v>
-      </c>
       <c r="E37" s="4" t="n">
         <v>0</v>
       </c>
@@ -8062,6 +8374,9 @@
         <v>0</v>
       </c>
       <c r="L37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -8075,33 +8390,36 @@
         <v>0</v>
       </c>
       <c r="C38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="4" t="n">
         <v>-4596</v>
       </c>
-      <c r="D38" s="4" t="n">
+      <c r="E38" s="4" t="n">
         <v>-6781</v>
       </c>
-      <c r="E38" s="4" t="n">
+      <c r="F38" s="4" t="n">
         <v>-13637</v>
       </c>
-      <c r="F38" s="4" t="n">
+      <c r="G38" s="4" t="n">
         <v>-20512</v>
       </c>
-      <c r="G38" s="4" t="n">
+      <c r="H38" s="4" t="n">
         <v>-6837</v>
       </c>
-      <c r="H38" s="4" t="n">
+      <c r="I38" s="4" t="n">
         <v>-13675</v>
       </c>
-      <c r="I38" s="4" t="n">
+      <c r="J38" s="4" t="n">
         <v>-20588</v>
       </c>
-      <c r="J38" s="4" t="n">
+      <c r="K38" s="4" t="n">
         <v>-6781</v>
       </c>
-      <c r="K38" s="4" t="n">
+      <c r="L38" s="4" t="n">
         <v>-13632</v>
       </c>
-      <c r="L38" s="4" t="n">
+      <c r="M38" s="4" t="n">
         <v>-23301</v>
       </c>
     </row>
@@ -8133,15 +8451,18 @@
         <v>0</v>
       </c>
       <c r="I39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="4" t="n">
         <v>-1658</v>
       </c>
-      <c r="J39" s="4" t="n">
+      <c r="K39" s="4" t="n">
         <v>-1932</v>
       </c>
-      <c r="K39" s="4" t="n">
+      <c r="L39" s="4" t="n">
         <v>-2811</v>
       </c>
-      <c r="L39" s="4" t="n">
+      <c r="M39" s="4" t="n">
         <v>-3259</v>
       </c>
     </row>
@@ -8179,11 +8500,14 @@
         <v>0</v>
       </c>
       <c r="K40" s="4" t="n">
-        <v>900000</v>
+        <v>0</v>
       </c>
       <c r="L40" s="4" t="n">
         <v>900000</v>
       </c>
+      <c r="M40" s="4" t="n">
+        <v>900000</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
@@ -8222,6 +8546,9 @@
         <v>0</v>
       </c>
       <c r="L41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="4" t="n">
         <v>-2250</v>
       </c>
     </row>
@@ -8256,14 +8583,17 @@
         <v>0</v>
       </c>
       <c r="J42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" s="4" t="n">
         <v>-2195</v>
-      </c>
-      <c r="K42" s="4" t="n">
-        <v>-31581</v>
       </c>
       <c r="L42" s="4" t="n">
         <v>-31581</v>
       </c>
+      <c r="M42" s="4" t="n">
+        <v>-31581</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
@@ -8296,12 +8626,15 @@
         <v>0</v>
       </c>
       <c r="J43" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" s="4" t="n">
         <v>321</v>
       </c>
-      <c r="K43" s="4" t="n">
+      <c r="L43" s="4" t="n">
         <v>319</v>
       </c>
-      <c r="L43" s="4" t="n">
+      <c r="M43" s="4" t="n">
         <v>301</v>
       </c>
     </row>
@@ -8355,6 +8688,10 @@
         <f>SUM(L35:L43)</f>
         <v/>
       </c>
+      <c r="M44" s="6">
+        <f>SUM(M35:M43)</f>
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
@@ -8363,36 +8700,39 @@
         </is>
       </c>
       <c r="B45" s="4" t="n">
+        <v>104</v>
+      </c>
+      <c r="C45" s="4" t="n">
         <v>121</v>
       </c>
-      <c r="C45" s="4" t="n">
+      <c r="D45" s="4" t="n">
         <v>158</v>
       </c>
-      <c r="D45" s="4" t="n">
+      <c r="E45" s="4" t="n">
         <v>-181</v>
-      </c>
-      <c r="E45" s="4" t="n">
-        <v>-555</v>
       </c>
       <c r="F45" s="4" t="n">
         <v>-555</v>
       </c>
       <c r="G45" s="4" t="n">
+        <v>-555</v>
+      </c>
+      <c r="H45" s="4" t="n">
         <v>-722</v>
       </c>
-      <c r="H45" s="4" t="n">
+      <c r="I45" s="4" t="n">
         <v>-766</v>
       </c>
-      <c r="I45" s="4" t="n">
+      <c r="J45" s="4" t="n">
         <v>-16</v>
       </c>
-      <c r="J45" s="4" t="n">
+      <c r="K45" s="4" t="n">
         <v>1259</v>
       </c>
-      <c r="K45" s="4" t="n">
+      <c r="L45" s="4" t="n">
         <v>2214</v>
       </c>
-      <c r="L45" s="4" t="n">
+      <c r="M45" s="4" t="n">
         <v>2174</v>
       </c>
     </row>
@@ -8444,6 +8784,10 @@
       </c>
       <c r="L46" s="6">
         <f>L28+L34+L44+L45</f>
+        <v/>
+      </c>
+      <c r="M46" s="6">
+        <f>M28+M34+M44+M45</f>
         <v/>
       </c>
     </row>

</xml_diff>